<commit_message>
fix: failed to generate json for some news
Added method="json_schema" to LangChain.model.with_structured_output
</commit_message>
<xml_diff>
--- a/data/Annotazioni_1_with_factoids.xlsx
+++ b/data/Annotazioni_1_with_factoids.xlsx
@@ -552,7 +552,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>['Istat explained a few days ago that contractual wages grew by 0.8%', 'Istat explained a few days ago that the inflation rate was 5.2%', 'Due to the 0.8% wage growth and 5.2% inflation, there will be a loss of purchasing power of almost five points in 2022', 'The law provides for the re-evaluation of the maintenance allowance following separation or divorce', 'The re-evaluation of the maintenance allowance protects the recipient by adjusting the amount due to the economically weaker spouse or children to the average cost of living', 'The revaluation of the maintenance allowance must be carried out every year according to the ISTAT indices', "The revaluation of the maintenance allowance must always be applied regardless of agreement by the spouses or by a judge's judgment of separation or divorce", 'For the revaluation, the index of consumer prices of the families of workers and employees must be used', 'The index of consumer prices used for revaluation references the Istat index published compared to the month of the first payment of the maintenance allowance decided by the court of the previous year', 'If the maintenance allowance fails to adapt, the rule allows requesting arrears for the last 5 years', 'Starting in 2022, the indexation mechanism was re-introduced', 'The indexation mechanism re-evaluates pension amounts for allowances and coupons', 'Pensioners receiving a monthly allowance up to 4 times the social allowance (about 2,000 euros) will receive a full revaluation compared to inflation', 'Pensioners receiving between 4 and 5 times the social allowance will receive a 90% increase compared to inflation', 'Istat established that the inflation index for 2022 will be 1.9 percent', 'In 2023, the cheques will recover the price growth recorded in 2022', 'The revaluation, according to current estimates, will be around 7% in 2023', 'Property owners can attach the rent allowance to the trend of inflation', 'Rules for liquidations provide that the TFR, excluding the share gained in the year, will increase every year', 'The TFR increase is calculated using a fixed rate of 1.5% plus 75% of the increase of the index of consumer prices for the families of workers and employees (3/4 of the rate of inflation)', 'The index of consumer prices increase for the families of workers and employees is established by Istat compared to December of the previous year', 'If the revaluation rate is applied for fractions of a year, the increase in the Istat index must be calculated from the month of termination of the employment relationship compared to December of the previous year']</t>
+          <t>['Pensioners, beneficiaries of a maintenance allowance in the event of divorce, and tenants of a rent may try to avoid the price race.', 'Public and private employees (unless there are specific agreements on the contract) and self-employed will maintain their wages.', 'Istat explained on 2022-07-02 that contractual wages grew by 0.8%.', 'Istat explained on 2022-07-02 that the inflation rate was 5.2%.', 'Due to the 0.8% wage growth and 5.2% inflation rate, there will be a loss of purchasing power of almost five points on 2022-01-01.', 'The law provides for the re-evaluation of the maintenance allowance in the event of separation or divorce.', 'The re-evaluation protects the recipient by adjusting the amount due to the economically weaker spouse or children to the average cost of living.', 'The revaluation must be carried out each year according to the ISTAT indices.', 'The revaluation must always be applied, regardless of agreement by the spouses or by the judge.', 'For the revaluation, the index of consumer prices of the families of workers and employees shall be used.', 'The index used for revaluation references the index published by Istat compared to the month of the first payment of the maintenance allowance decided by the court of the previous year.', 'If the maintenance allowance fails to adapt, the rule allows requesting arrears for the last 5 years.', 'Pensioners will also have a protective shield.', 'The indexation mechanism was re-introduced from on 2022-01-01 to re-evaluate pension amounts for allowances and coupons.', 'Pensioners receiving a monthly allowance up to 4 times the social allowance (about 2,000 euros) will receive a full revaluation compared to inflation.', 'Pensioners receiving between 4 and 5 times the social allowance will receive a 90% increase compared to inflation.', 'Istat established that the inflation index for on 2022-01-01, which will be based on adjustments referred to 2021, will be 1.9 percent.', 'In 2023, the cheques will recover the price growth recorded in 2022.', 'The revaluation, according to current estimates, will be around 7%.', 'Property owners can attach the rent allowance to the trend of inflation.', 'Regarding liquidations, the rules provide that the TFR, excluding the share gained in the year, will increase each year.', 'The TFR increase is calculated using a fixed rate of 1.5%.', 'The TFR increase also uses 75% of the increase of the index of consumer prices for the families of workers and employees (3/4 of the rate of inflation), established by Istat compared to December of the previous year.', 'If the revaluation rate is applied by fractions of the year, the increase in the ISTAT index must be calculated from the month of termination of the employment relationship compared to December of the previous year.', 'If inflation is 2%, 75% is 1.5%.', 'The TFR must be re-evaluated by 3% (1.5% plus 1.5%) in the example provided.']</t>
         </is>
       </c>
     </row>
@@ -620,7 +620,7 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>["The government's move on the IMU returns to December in masked form as a down payment of the service tax.", 'The treasury is hunting 3 billion to avoid the increase of the estimated tax in October.', 'The operation-maquillage of the tax on the house is expected to arrive in November.', 'The holding on the financial law is at risk due to the alarm at the Quirinal.', 'The President of Naples consulted with the Alphanus and Epiphans secretaries while the PDL threatened a crisis.', 'Angela Merkel was the clear winner in the popular vote in the German elections.', 'An electoral law that many insist on exporting to Italy will not allow Italy to govern itself.', 'A new large coalition appears on the horizon in Germany.', 'The last series of agreements, run in 2005, resulted from an agreement signed after weeks of negotiation.', 'The legislative program was more than 300 pages long.', 'The legislative program exceeded the "manifesto" of the electoral prodians of 2006.', 'The great coalition was born with a half-hour investiture speech from the President-in-Office.', "The President-in-Office's speech promised everything and more, denying any budgetary constraint.", 'Decision-making paralysis occurred previously, even more animated than in Germany.', 'The government is now acting only in the dream sphere or in that of accounting tricks.', 'The update note to the Def, presented a few days ago by the executive, proposes macroeconomic scenarios from dreamy late summer.', 'The proposed macroeconomic scenarios suggest that Italy should grow in the next three years at a rate twice that of potential.', 'The proposed macroeconomic scenarios tear the estimates of international organizations.', 'The proposed macroeconomic scenarios do not require doing anything to make such a sudden change of pace possible.', 'These scenarios include the coexistence of high inflation (a GDP deflator of 2%) with a further fall in household consumption and rising unemployment.', 'The three phenomena (high inflation, fall in consumption, rising unemployment) are difficult to understand how they can be realized simultaneously.', 'The scenarios allow drawing up tables where the debt ratio and GDP never rise above 130% of gross domestic product.', 'Institutional fund managers cannot be convinced to invest in Italy by these unrealistic scenarios.', "These scenarios risk weakening Italy's negotiating position at the Community level.", 'Accounting engineering is intended to revalue the shares held by banks at the banks of Italy.', 'The shares held by banks at the banks of Italy were a legacy of when the banks were public.', 'The banks would see their capital position strengthened through the accounting engineering process.', 'The Treasury would receive a contribution for the gains achieved through accounting engineering.', 'Taxpayers risk paying a very high bill because a central bank cannot be owned by private banks.', 'A special commission of essays was set up because there are no market references for the transaction.', 'The country risks finishing in the hands of the troika, day after day, without realizing it, by using dreams and accounting engineering.', 'It was hard to get back from a debt of 120 percent.', 'It is much more difficult to reduce the debt from 130 percent and growing.', 'If the government does not want to be remembered for giving national sovereignty, the government must find a program agreement.', 'The program agreement must open negotiations at Brussels.', 'The agreement should be sculpted into the law of stability.', "The law of stability's philosophy is tackling emergencies with long-term reforms.", 'Refinancing the supplementary fund by way of derogation should provide for the gradual overrun of this institution.', 'The supplementary fund should provide wage supplements for those working less than EUR 5 per hour.', 'The supplementary fund should provide a way to facilitate labor mobility and increase employment.', 'Any new access to the coffin will have to be blocked by way of derogation.', 'The blocking of new access to the coffin must start with that required for former party employees by a very large parliamentary coalition.', 'Ordinary social shock absorbers will be available for other workers.', 'Increasing VAT, possibly limited to luxury goods only, could be offset by a cut in the tax wedge.', 'Indirect taxes increase the difference between labor costs and purchasing power of wages.', 'Measures to cut expenditure should be implemented gradually.', 'One can start by dismantling the bureaucracy created by the federalism of the league.', 'The federalism of the league created duplications, uncontrolled local spending, and an excess of power centers.', 'The directing booth should protect the government from the raging attacks of those affected by the cuts.', 'Including these measures in the Stability Act makes it possible to open negotiations with Brussels.', 'Negotiations with Brussels also include deficits of more than 3% over the coming years.']</t>
+          <t>["The government's move on the IMU returns to December in masked form.", 'The government uses the IMU move as a down payment of the service tax.', 'The Treasury is hunting 3 billion to avoid the increase of the estimated tax on 2013-10-25.', 'The operation-maquillage of the tax on the house is expected to arrive in November.', 'The holding on the financial law is at risk at the Quirinal.', 'The Napolitan President consulted with the Alphanus and Epiphans secretaries.', 'The PDL threatens a crisis again.', 'Angela Merkel was the clear winner in the popular vote in the German elections.', 'An electoral law that many insist on exporting to Italy will not allow Italy to govern itself.', 'A new large koalition appears on the horizon.', 'The last koalition series ran in the year 2005.', 'The legislative program of the koalition was more than 300 pages long.', "The legislative program exceeded the 'manifesto' of the electoral prodians of 2006.", 'The Great Coalition promised itself everything and more, denying any budgetary constraint.', 'The update note to the DEF, presented by the executive, proposes macroeconomic scenarios.', 'The macroeconomic scenarios propose growth in the next three years at a rate twice that of potential.', 'The proposed growth rate tears the estimates of international organizations.', 'The scenarios include high inflation (a GDP deflator of 2%).', 'The scenarios include a further fall in household consumption.', 'The scenarios include rising unemployment.', 'The scenarios may be used to draw up tables where the debt ratio and GDP never rise above 130% of gross domestic product.', "The unrealistic scenarios risk weakening Italy's negotiating position at Community level.", 'Accounting engineering is intended to revalue the shares held by banks at the banks of Italy.', 'The revaluation would strengthen the capital position of the banks.', 'The Treasury would receive a contribution for the gains achieved through accounting engineering.', 'Taxpayers risk paying a high bill if taxpayers have to buy back the shares.', 'The country risks finishing in the hands of the Troika.', 'It was hard to get back from a debt of 120 percent.', 'It is much more difficult to reduce debt from 130 percent and growing.', 'The government must find a program agreement to open negotiations at Bruxelles.', 'The agreement should be sculpted into the law of stability.', "The law of stability's philosophy is tackling emergencies with long-term reforms.", 'Refinancing the supplementary fund by way of derogation should provide for the gradual overrun of the institution.', 'The fund should provide wage supplements for those working less than EUR 5 per hour.', 'Any new access to the coffin must be blocked by way of derogation.', 'The blocking of new access must start with that required for the former party employees by a very large parliamentary coalition.', 'The increase in VAT, possibly limited to luxury goods only, could be offset by a cut in the tax wedge.', 'Indirect taxes increase the difference between labor costs and purchasing power of wages.', 'Measures to cut expenditure should be implemented gradually.', 'One can start by dismantling the bureaucracy created by the federalism of the league.', 'The federalism of the league created duplications, uncontrolled local spending, and an excess of power centers.', 'Including these measures in the Stability Act makes it possible to open negotiations with Bruxelles.', 'These negotiations can include deficits of more than 3% over the coming years.']</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>['The recovery is expected to be shy, feeble, and pregnant with downside risks', 'Small businesses, especially those in the south, are left on the margins', 'Consumption is languishing', 'The number of unemployed people is expected to increase in 2015', 'Inflation is continuing to decrease', 'The economic bulletin of the Bank of Italy, published on 2014-01-18, is more cautious than ever', 'The quarterly diffusion of the economic bulletin coincides with two important news regarding PIL', "Commissioner Olli Rehn is confident in the country's rehabilitation capacity", 'Commissioner Olli Rehn asked to push ahead with disengagement and spending review', 'Commissioner Olli Rehn suggested that Italy can achieve more flexibility on budgetary rules', 'Flexibility on budgetary rules is an indispensable condition for releasing resources for investment', 'On issues related to the commissioner and the minister of the economy, Fabrizio Saccomanni, there was a breakfast on 2014-01-17', 'The EU is reviewing the calculation of the GDP', 'The EU is moving investments in research and development from the expenditure box (a liability) to the investments category', 'Extrapolations suggest the benefit of the GDP calculation review will be between 1% and 2%', 'The GDP calculation review will have non-negligible effects on the deficit-PIL ratio', 'The GDP calculation review will affect the consolidation of the accounts and the relationships with Brussels', 'The document of the Bank of Italy is anchored only on a technical-analytic ground', 'The macro projections developed by the economists place the year-end GDP growth at 0.7%', 'The macro projections developed by the economists predict that the GDP growth will rise to 1% in 2015', "The government's estimates for year-end GDP growth are 1% and 1.7% (for 2015)", "The Bank of Italy's GDP estimates are much smaller than the government's estimates", 'The unemployment rate is projected to rise to 12.9% in 2015', 'The Bank of Italy warns that only the recovery of domestic demand can extend the recovery to the labor market', 'Risks to growth currently remain downward-oriented', 'The recovery of investment may be delayed if conditions for access to credit remain restrictive longer than expected', 'The recovery of investment may be delayed if payments of commercial debts of public administrations differ', 'The risk of general deflation is judged to be moderate', 'The fall in inflation could be more pronounced and persistent than expected', 'The fall in inflation could be more pronounced and persistent if the weakness of demand reflects expectations', 'The confidence of enterprises is improving', 'Industrial activity is picking up after being diminished almost without interruptions from summer of 2011', 'Small enterprises, especially in the south, remain on the margins of the process', 'The decline in consumption of families diminished in the third quarter of 2013', 'Italians do not spend on 2014-01-18', 'Consumption continues to be restrained by the weakness of disposable income', 'Consumption continues to be restrained by difficult labor market conditions', 'The Italian bank noted that the recovery of trust since the beginning of 2013 was interrupted in the fourth quarter', 'The Italian bank changed its internal organization to include 8 departments, services, and divisions under the Directory']</t>
+          <t>['Small businesses, especially those in the south, are left on the margins.', 'Consumption is languishing.', 'The unemployed will increase in 2015.', 'Inflation continues to decrease.', 'The economic bulletin of the bank of Italy was published on 2014-01-18.', 'The quarterly diffusion of the economic bulletin coincided with two important news items regarding PIL.', "Commissioner Olli Rehn is confident in the country's rehabilitation capacity.", 'Commissioner Olli Rehn asked to push ahead with disengagement and spending review.', 'Commissioner Olli Rehn suggests that Italy can achieve more flexibility on budgetary rules.', 'Flexibility on budgetary rules is an indispensable condition for releasing resources for investment.', 'On 2014-01-17, there was a breakfast between Commissioner Olli Rehn and the minister of the economy, Fabrizio Saccomanni.', 'The UE is reviewing the calculation of the GDP.', 'The UE is moving investments in research and development from the expenditure box (a liability) to the investments category.', 'The benefit of the GDP calculation review is expected to be between 1% and 2%.', 'The benefit will have effects on the deficit-PIL ratio.', 'These ratios affect the consolidation of the accounts and the relationships with Bruxelles.', 'The macro projections developed by the bank of Italy place the year-end GDP growth at 0.7%.', "The bank of Italy's estimates are smaller than the government's estimates for year-end GDP growth.", 'The government estimates GDP growth at 1.7% for the second year.', 'The unemployment rate will rise to 12.9% in 2015.', 'The bank of Italy warns that only the recovery of domestic demand can extend the recovery to the labor market.', 'Risks to growth remain downward-oriented.', 'The recovery of investment may be delayed if conditions for access to credit remain restrictive longer than expected.', 'The recovery of investment may be delayed if payments of commercial debts of public administrations differ.', 'The risk of general deflation is judged to be moderate.', 'The fall in inflation could be more pronounced and persistent than expected if the weakness of demand reflects expectations.', 'Enterprise confidence is improving.', 'Industrial activity is picking up after being diminished almost without interruptions from summer of 2011.', 'The background is varied depending on the category of enterprises and their location.', 'Small enterprises, especially in the south, remain on the margins of the process.', 'The decline in consumption of families diminished in the third quarter of 2013.', 'Italians do not spend on 2014-01-18.', 'Consumption is restrained by the weakness of disposable income.', 'Consumption is restrained by difficult labor market conditions.', 'The bank of Italy notes that the recovery of trust since the beginning of 2013 was interrupted in the fourth quarter.', 'The bank of Italy changed its internal organization.', 'The bank of Italy structured its organization under the Directory, 8 departments, services and divisions.']</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['On 2021-09-20, Giuseppe Chestnut, managing director of Bench BPM, stated that moratorium loans fell from over 16 billion euros to 4.8 billion euros.', 'Giuseppe Chestnut stated that almost 75% of the customers exposed to the 4.8 billion euros have good ratings.', 'Moratorium credits increased from 280 billion euros in March 2020 to 147 billion euros in December 2020.', 'Moratorium credits decreased to 71 billion euros in September 2021.', 'The Italian economy sees GDP growing to over 6% per annum on 2021-10-18.', 'Ferrara Ferruccio, founder and president of Negentropy Capital Partners, signed one of the first transactions of acquisition of bad debts with Pimco and Deutsche Bank in 2011.', 'The COVID-19 pandemic lengthened the times of recovery.', 'Bank exposures increased in the 18 months leading up to 2021-10-18.', 'The total amount of non-performing loans (NPL) and unprovisioned troubled payments (UTP) in Italy is around 500 billion euros on 2021-10-18.', 'Of the 500 billion euros in Italy, about 180 billion euros are UTP.', 'Of the 500 billion euros in Italy, about 120 billion euros are NPL still within the banking perimeters.', 'The remaining 200 billion euros have emerged from the perimeter of the banks and are held in specialized funds.', 'In 2021, the value of the portfolios sold by the banks was about 34 billion euros.', 'The value of the UTP reached 11 billion euros in 2021.', 'Banks are ready to sell NPL for 26 billion euros from 2021-10-18 to the end of the year.', 'Bank Ifis, in its September report, predicted that new credit deteriorated on households and resident companies would grow by about 70 billion euros between 2022 and 2023.', 'Bank Ifis noted that the increase in the rate of deterioration would be driven by the enterprise component.', 'Bank Ifis predicted that the stock of the credits deteriorated gross would contract in 2021.', 'The contraction of the stock of the credits deteriorated gross in 2021 will reduce the NPE ratio below the target by 5% as required by the BCE.', 'The impact on employment is expected to increase from 2022.', 'The public hand plays an important role in the bad loans market through AMCO and GACS.', 'GACS, the public guarantees on the securitization of suffering, was introduced by a decree of February 2016.', 'The European Union granted a further 12-month extension for GACS in 2021.', 'Bank Ifis expects approximately 7 billion euros of new guaranteed transactions based on the GACS extension.', 'The total transaction value assisted by GACS since 2016 is expected to reach 94 billion euros.', 'The top four Italian operators concentrating the GACS gross book value are Dovale, Prelios, Cerved, and Land Credit.', 'Ferrara emphasized that Negentropy controls portfolios for approximately 3 billion euros of GBV.', 'When a credit institution places an asset for sale, up to 25-30 operators are invited to participate in the purchase.', 'The increase in the number of operators led to an upward revision of prices in the bad loans market.', 'In 2021, 125 thousand judicial auctions were estimated in Italy.', 'The number of judicial auctions in 2021 decreased by 39 percent compared to the pre-pandemic period.', 'The courts suspended over 120 thousand auctions.', 'The suspended auctions resulted in operations of at least 13 billion euros blocked in the courtrooms.']</t>
         </is>
       </c>
     </row>
@@ -812,7 +812,7 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['A letter requires 1 sheet plus an envelope.', 'An application requires 4 sheets.', 'Instructions require 2 sheets.', 'Photocopies attached to the application require 2 sheets (or 4 sheets if necessary delegation).', 'The estimated population is 1,300,000.', 'The minimum sheets used per application is 9 sheets plus an envelope.', 'The total estimated sheets needed is 11,700,000 sheets.', 'The total estimated sheets are equal to 23,400 rismes of paper of 500 sheets.', 'The number of bags forgotten is 1,300,000.', 'Claudia Ceroni in Roma was dazzled by an increase in VAT on an unnecessary asset (sky).', 'The author convinced parents to improve the insulation of the roof and install sanitary panels, condensing boiler, and thermostatic valves for about 10,000 euros.', 'The author and boyfriend spent about 50,000 euros on additional insulation and fixtures for their new home.', 'The deduction for renovations is no longer certain.', 'The deduction rate may be reduced from 55% to 35%.', 'The 4% rate on loans fixed by the Government of Luciano is expected to keep the interest rate on variable rate loans below 4% for 2009.', 'Mr Boeri wrote in the newspaper at the newsstands on 2008-12-01 questioning the lack of a measure for fixed rate loans.', 'The BCE rate cut is expected to bring the Euribor to little more than 3%.', 'The variable rate loan will be 3% (Euribor) plus an average spread of 1%, totaling 4%.', 'The author predicts a variable rate of 3.5% in 2009.', 'The headline on page 19 of Republic of on 2008-12-01 stated that the yo-yo was the most important part of the fight against crime for TG1.', "TG1 did not give account in the edition of the 20 of 2008-11-29 of the review on the fight against the mafias organized by 'politically incorrect' to reindeer housewife (Bologna).", 'The conference on mafias took place a few hundred meters from the yo-yo championship.']</t>
         </is>
       </c>
     </row>
@@ -876,7 +876,7 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>['A study by the national consumer union ranked cities based on the greatest annual increases in cost of living.', 'The data for the ranking of cities was drawn up from Istat in January 2023.', 'Perugia and Terni are among the top six most expensive cities.', 'The cost of light and gas in Perugia increased by 85.8%.', 'The small difference in cost of living between Perugia and Terni indicates that the cost of living is uniform throughout the region.', 'An average Italian family spends 1,157 euros annually on the cost of living in Perugia.', 'The survey compares the change in electricity and gas prices over the last 3 years at the national level.', 'The survey compares the free market with the protected market for electricity and gas prices.', 'The free market price of light increased by more than double (129%) compared to the protected market price between June 2021 and January 2023.', 'As of December 2021, the protected market price of gas decreased by 7.4%.', 'From January 2020 to January 2023, the free market price of light jumped 262.8%.', 'From January 2020 to January 2023, the protected market price of light increased by more than 115.8%.', 'In January 2023, the rise in electricity, gas, and other fuels in Italy was 67.3% compared to a year earlier.', 'An average family spends 907.50 euros annually on electricity, gas, and other fuels in Italy.', 'Some cities spend almost 90 percent of the average family spending on electricity, gas, and other fuels.', 'In Alexandria, electricity, gas, and diesel costs rose by 88.6% in January 2022.', 'The cost in Vercelli (Piemonte) increased by 87.1%.', 'The cost in Olbia-Tempio increased by more than 51%.', 'The cost in Benevento increased by 53.1%.', 'The cost in Trieste increased by 54.6%.', 'The cost in Pordenone and Udine increased by 54.7%.', 'The CGIA of Mestre conducted a study on the impact of inflation on family purchasing power.', 'The loss of purchasing power in Umbria due to inflation in the two years 2022-2023 could amount to almost six thousand euros per household.', 'Bank deposits in Italy amounted to 14.5 billion euros at the end of 2021.', 'The total estimated loss of purchasing power in Umbria across 2022 and 2023 was 2.1 billion euros.', 'The CGIA estimates the loss of purchasing power for Perugia at over 1.6 billion euros (approximately 5,746 euros per family).']</t>
+          <t>['A study by the national consumer union ranked cities based on annual increases, using data from Istat from January 2023.', 'Perugia and Terni were ranked among the top six most expensive cities.', 'The cost of light and gas in Perugia increased by 85.8%.', 'The average annual cost of living for a family in Perugia is 1,157 euros.', 'The survey compares the change in electricity and gas prices over the last 3 years, comparing free and protected markets.', 'From June 2021 to January 2023, the protected market light in Italy rose by 108.4%.', 'The protected market gas price decreased by 7.4% since December 2021.', 'From January 2020 to January 2023, the protected market light jumped 115.8%.', 'In January, the rise in electricity, gas, and other fuels in Italy was 67.3% compared to a year earlier.', 'The average annual cost of electricity, gas, and other fuels for a family in Italy is 907.50 euros.', 'In Alexandria, electricity, gas, and diesel costs increased by 88.6% in January 2022.', 'Vercelli (Piemonte) saw an increase of 87.1%.', 'Biella saw an increase of 86.1%.', 'Power (the city less tartassata) saw an increase of 35.2%.', 'Olbia-Tempio saw an increase of 51%.', 'Gorizia saw an increase of 51.7%.', 'Benevento saw an increase of 53.1%.', 'Caserta saw an increase of 53.5%.', 'Trieste saw an increase of 54.6%.', 'Pordenone and Udine saw an increase of 54.7%.', 'The CGIA of Mestre conducted a study on the weight of family purchasing power regarding inflation.', 'The loss of purchasing power in Umbria over the two years 2022-2023 could amount to almost 6,000 euros per household.', 'The estimate for the loss of purchasing power in Umbria in 2022 was 1.2 billion euros.', 'The total estimated loss of purchasing power in Umbria over the two years was 2.1 billion euros.', 'Bank deposits at the end of 2021 amounted to 14.5 billion euros.', 'For Perugia, the loss of purchasing power could amount to over 1.6 billion euros.']</t>
         </is>
       </c>
     </row>
@@ -936,7 +936,7 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>['The tax package to stimulate the American economy in a severe crisis had the support of the Federal Reserve President Bernanke on 2008-10-20', 'The central bank considers a further cut in rates in the short-term future of the economy due to low inflation from the recession', 'Bernanke, who spoke before the chamber budget committee, stated that the credit crisis is hitting the economy because Americans find it hard to find money for their activities', 'The governor told the Members that the idea of a tax package seems appropriate because the economy is likely to be weak for several quarters and there is a risk of a prolonged slowdown', 'The political free way brought a tax drug law to the agenda in the country one hour after the technical support statements', 'Bernanke, the spokesman of the Dana Perino president, echoed that the Bush administration is open to ideas that could stimulate the economy and help get out of the downward spiral faster', 'The Bush administration will only be open if there are ideas that really stimulate the economy', 'The governor of the Fed stated that Congress, which is responsible for approving a second tax package after the one passed at the beginning of the year, should include measures to facilitate access to credit for consumers, homeowners, and those interested in borrowing', 'The governor of the Fed believes that measures to facilitate access to credit for consumers, homeowners, and those interested in borrowing could promote economic growth and job creation', 'The Dow Jones index rose above 9000 points, with a rise of 4.67%', 'The Nasdaq rose by 3.43% to 1,700 points', 'The dollar strengthened against the euro, falling to 1.33 dollars from 1.34 at the start', 'London rose by 5.41%', 'Paris rose by 3.56%', 'Madrid rose by 2.99%', 'Milan rose by 2.65%', 'Frankfurt rose by 1.12%', 'Bernanke hinted at a new rate cut at the end of October meeting of the Fed to boost stock exchange purchases', 'Federal bonds are 100% reduced by 25 cents', 'Federal bonds could also be reduced by half a point, similar to the previous reduction made by all banks', 'The use of public expenditure to combat the threat of depression dominates the fate of the American budget', 'Paul Krugman wrote in the New York Times about massive injections of state money in the banks', 'Bernanke admitted that the current deficit is wide but not inappropriate given the nature of the emergency', 'Bernanke stated that the current deficit is unavoidable given the loss of tax revenues', 'Bernanke is aware that every tax action inevitably involves trade and may burden future generations', 'Bernanke accepted the inevitability of intervention', 'The governor predicted that the pace of economic activity will remain below the growth potential for several quarters', 'The governor predicted that the slowdown in investment and business spending will extend to the major sectors']</t>
+          <t>['A new package to be voted on in Congress to stimulate the American economy in severe crisis was supported by the President of the Federal Reserve, Bernanke, and the President Bush on 2008-10-20.', 'The central bank takes into account a further cut in rates in the short-term future of the economy due to low inflation from the recession.', 'Bernanke stated that the credit crisis is hitting the economy because Americans find it hard to find money for their activities.', 'The governor told Members that the idea of a tax package seems appropriate because the economy is likely to be weak for several quarters and there is a risk of a prolonged slowdown.', 'One hour after these statements of technical support, the political free way came to the agenda of a tax drug law bis in the country.', 'Bernanke, the spokesman of the President Bush, echoed that the Bush administration is open to ideas that could stimulate the economy and help the United States get out of the downward spiral faster.', 'The governor of the Fed stated that Congress should include measures to facilitate access to credit for consumers, homeowners, and those interested in borrowing in a second tax package.', 'The governor of the Fed believes that these actions could promote economic growth and job creation.', 'Wall Street expanded earnings after the promise of central bank stimulus and the availability of President Bush.', 'The Dow Jones index rose above 9000 points, with a rise of 4.67%.', 'The Nasdaq earned 3.43% to 1,700 points.', 'The dollar strengthened against the euro, coming down to 1.33 dollars from 1.34 at the start.', 'London rose by 5.41%.', 'Paris rose by 3.56%.', 'Madrid rose by 2.99%.', 'Milan rose by 2.65%.', 'Frankfurt rose by 1.12%.', 'Bernanke hinted that a new cut of rates could happen at the meeting of the end of October of the Fed.', 'Federal bonds are 100% reduced by 25 cents.', 'Federal bonds could also be half a point, like the previous one made together by all banks.', 'Paul Krugman wrote in the New York Times, invoking massive injections of state money in the banks.', 'Bernanke admitted that the current deficit is wide but not inappropriate given the nature of the emergency.', 'Bernanke stated that the current deficit is not avoidable given the loss of tax revenues.', 'Bernanke is aware that every tax action inevitably involves trade.', 'Bernanke stated that tax actions may be heavy on future generations.', 'The governor predicted that the pace of economic activity will remain below the growth potential for several quarters.', 'The governor predicted that the slowdown in investment and business spending will extend to the major sectors.']</t>
         </is>
       </c>
     </row>
@@ -996,7 +996,7 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['If saving could be put on income with a one percentage point remuneration, households would have earned 30 billion, which is almost 2% of gross domestic product.', 'The saving rate of Italian households relative to disposable income grew by 50% in the year.', 'The yield of savings, excluding investments in listed companies, remained low, close to zero.', 'Each percentage point of remuneration, given the size of financial assets in the hands of households, is estimated at around €30 billion.', '2% of GDP is the size of a good government budget maneuver of the past.', 'The key theme of the annual report of the president of the CONSOB, Paolo Savona, is the protection of savings.', 'Savings in deposits have been stationary in the last two years.', 'Cryptocurrencies and bitcoins threaten savings in deposits.', 'The speculative effect triggered by cryptocurrencies and bitcoins seems similar to what happened before 2008 with subprime mortgages.', 'The diffusion of virtual tools caused the emergence of technological platforms.', 'The market segments are rapidly evolving.', 'Before the 2008 crisis, derivative contracts developed to a size of ten times the global GDP.', 'Something similar to the pre-2008 derivative contract development is foreseeable in the market for virtual monetary and financial products, especially encrypted ones.', 'Paolo Savona recalled that one bitcoin recently bought a large electric car.', 'The bitcoin subsequently lost half of its purchasing power.', 'For the President CONSOB, financial informatics is a prodigious lamp.', 'Authorities cannot bring back the change because it acts in the controllable immaterial sphere by changing the information exchange protocol.', 'Changing the information exchange protocol fragments the unity of the world market.', 'Fragmenting the unity of the world market reduces the international competitiveness test.', 'Traditional supervisory instruments are no longer sufficient.', 'According to Paolo Savona, the authorities may intervene using the advantages of digitized techniques under current conditions.', 'The action of the authorities will be more effective if the authorities cooperate with each other.', "Italy's issue is sensitive due to a constitutional rule that tasks the public with encouraging and protecting savings in all its forms.", 'The constitutional rule also tasks the public with regulating, coordinating, and controlling the exercise of credit.', 'Paolo Savona explained that it would be improper to assign a content that embraces virtual instruments to the specification of savings and credit without specific regulation.', 'The original blockchain is impenetrable regarding hacking techniques.', 'The blockchain used by other cryptocurrencies is not impenetrable.', 'There is a call to proceed quickly with adjustment systems.', 'Paolo Savona stated that the lack of adequate safeguards (standards and bodies) leads to a worsening of market transparency.', 'Market transparency is the basis for the legality and rational choices of operators.', 'These techniques allow shielding for criminal activities, including tax evasion, money laundering, terrorist financing, and kidnapping.', "Paolo Savona recalled CONSOB's activity in darkening hundreds of websites in Italy that illegally collected savings.", 'Paolo Savona hopes for an international solution for cybersecurity.', 'The solution to cybersecurity requires close international cooperation.', 'The solution to cybersecurity cannot be achieved at the national level.', 'The part of the Bretton Woods agreement concerning the interchangeability between different national currencies did not pass the test of international cooperation.', 'Technological innovations applied to finance re-proposed the urgency of relaunching the Bretton Woods agreement.', 'The president of CONSOB re-launched the proposal for unification of the single text of finance and the single bank text.', 'The president of CONSOB suggested a more tightened collaboration between the Italian authorities.', 'Paolo Savona explained that Italy needs to activate structures of formal consultation between governing bodies and independent authorities.', 'These structures must give a unitary address to choices regarding European and international initiatives.', 'A first step would be the transposition of the 2011 recommendation of the European Systemic Risk Board.', 'This transposition would create a single national counterpart responsible for macro-prudential stability.', 'The Bank of Italy would maintain a central role due to its participation in the euro system.', 'Close coordination between the three independent supervisory authorities (CONSOB, IVASS, and COVIP), with the participation of the Ministry of Economic Affairs, would be ensured.', 'Public debt has grown greatly to cope with economic and social difficulties.', 'Confidence in the response capacity of the Italian economy has grown.', 'The growth in confidence resulted from the ECB acquiring significant volumes of public bonds.', 'The growth in confidence resulted from the European Commission temporarily suspending the Stability Pact and launching the next generation EU plan.', 'The speaker agrees on the assessments regarding the structural improvement of the real growth rate.', 'The speaker stated that a change in pace is necessary.', 'Paolo Savona said that continuing the relaunching of productive activity requires integrating past decisions.', 'The integration must stimulate the venture capital of enterprises to improve their leverage and make them available for new initiatives.', 'The reform of the tax offers an important occasion to consider productive authorities on the same plane as ethical ones in distribution equity appraisals.']</t>
         </is>
       </c>
     </row>
@@ -1060,7 +1060,7 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['Stefano Lepri, governor of Roma, stated that the financial crisis is passing on to enterprises and families.', 'Mario Dragons, governor of the Bank of Italia, stated that the credit paid by the banks has not diminished for now.', 'Mario Dragons stated that the situation can change quickly.', 'Consumption is falling.', 'The product declined in the second quarter.', 'Negative signals for the next quarters arrived after the decline of the product in the second quarter.', 'To stem negative effects, Silvio Berlusconi accepted the proposal of Confindustria.', 'The proposal was to open a discussion table between government, enterprises, and banks.', 'Minister Claudio Scajola added that state guarantees on corporate debts are being studied.', 'Mario Dragons reassured the Italian banks during the audition to the Senate.', 'Mario Dragons stated that the capitalization of the major Italian banks remains sufficient on 2008-10-22.', 'Mario Dragons stated that the Italian banks could absorb a shock, even if losses from the Lehman bankruptcy reached the worst assumptions.', 'The banks suffered on the stock exchange due to a sentence of the President of the Council that was partly misunderstood.', 'Silvio Berlusconi made open stock exchange comments on listed companies in Naples.', 'Silvio Berlusconi stated that two or three banks, in addition to Unicredit, might have advantages in increasing their capital.', 'The prices of the major banks fell in the first press headlines.', 'The prices of the major banks returned later.', 'The clearing up on the financial markets confirmed on 2008-10-21 that the yield was below 5% of the three-month Euribor rate.', 'Mario Dragons assured that the Italian banks have only partially shared errors and distortions of the world financial system.', 'Mario Dragons stated that the world financial system errors and distortions originated mainly in the United States.', 'Mario Dragons stated that the Italian bank has consistently given a strict interpretation of European standards.', 'Mario Dragons stated that the public opinion tendency to involve central banks in reproach is not present in the euro area or Italy.', 'Mario Dragons recalled that warnings about the imbalances of the international financial system were repeatedly given in several interventions, especially in autumn 2006.', 'Mario Dragons summarized that while the moment, mechanism, and scale of the crisis could not be predicted, the accumulating tensions were visible.', 'Banks or other intermediaries who gave Lehman Brothers securities savers will not have to leave them alone.', 'New rules on transparency in the relationship between banks and customers will be ready at the beginning of next year.', 'Better regulation of derivatives and other innovative financial products will be needed globally.', 'New rules must prevent banks from taking risks that are too exposed to their capital.', 'Mario Dragons concluded that Italy does not come out badly from the financial crisis.', 'Mario Dragons stated that the effects of the crisis on the real economy add to pre-existing structural weaknesses.', 'The International Monetary Fund confirmed a forecast decline in gross product of -0.1% in 2008.', 'Alessandro Leiold, head of the European department of IMF, warned that reacting with state aid would not be the right answer.', 'Alessandro Leiold recommended better liberalizations.']</t>
         </is>
       </c>
     </row>
@@ -1120,7 +1120,7 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>['Mortgage applications are being lowered.', 'Requirements to obtain mortgages are being raised.', 'The credit crunch is increasing.', 'Goldman Sachs explained in a report that the credit crunch is the most intense since the sovereign debt crisis.', 'The increase in interest rates by the European Central Bank (ECB) is substantially impacting households.', 'According to the last Francoforte bank lending survey, the contraction in demand for housing loans was minus 21% in the fourth quarter of 2022.', 'The last Francoforte bank lending survey reported that demand for consumer credit and other loans to households decreased sharply in net terms.', 'The decrease in demand for consumer credit and other loans to households was less severe than the decrease for building loans, according to the last Francoforte bank lending survey.', 'Goldman Sachs stated that the current scenario represents a substantial further tightening of credit standards applied to households and businesses.', 'The uncertain prospects of the economy weigh mainly on the credit standards applied to households and businesses.', 'The cost of funds and the liquidity position contribute increasingly to the credit standards applied to households and businesses.', 'On 2023-02-02, the situation was destined to worsen due to the rising cost of money, according to the hawks.', 'The Federal Reserve (Fed) has a hard line for the whole 2023 BCE rates.', 'The European Central Bank (ECB) explained that the net decline in demand for real estate loans was mainly determined by the deterioration of the real estate market prospects.', 'Banks forecast a further net decrease in demand for loans to enterprises in the first quarter of 2023.', 'Banks estimate a persistent and strong net decline in demand for loans to households for the first quarter of 2023, according to Francoforte.', 'Goldman Sachs expects a decrease in credit concession and a reduction in demand for other loans of equal magnitude.', 'The expected decrease and reduction in demand for personal loans and other loans are compared to what was observed in the last four months of the year.', 'The current phenomenon is spread evenly across the euro area, unlike the crisis that hit the eurozone a decade ago.']</t>
+          <t>['Mortgage applications are being lowered.', 'Requirements to obtain mortgages are being raised.', 'The credit crunch is increasing.', 'Goldman Sachs explained in a report that the current credit crunch is the most intense since the sovereign debt crisis.', 'The increase in interest rates by the European Central Bank (ECB) is substantially impacting households.', 'According to the last Francoforte bank lending survey, the contraction in demand for housing loans in the fourth quarter of 2022 was minus 21%.', 'The demand for consumer credit and other loans to households decreased sharply in net terms.', 'The decrease in demand for consumer credit and other loans to households was less severe than the decrease for building loans.', 'Goldman Sachs stated that the scenario represents a substantial further tightening of credit standards.', 'These credit standards apply to households and businesses.', 'The uncertain prospects of the economy weigh mainly on the credit standards.', 'The cost of funds and the liquidity position are contributing more and more to the credit standards.', 'The European Central Bank (ECB) explains that the net decline in demand for real estate loans was determined by the general level of interest rates.', 'The net decline in demand for real estate loans was also determined by lower consumer confidence.', 'The net decline in demand for real estate loans was also determined by the deterioration of the prospects of the real estate market.', 'In the first quarter of 2023, banks forecast a further net decrease in demand for loans to enterprises.', 'Francoforte notes that banks estimate a persistent and strong net decline in demand for loans to households in the first quarter of 2023.', 'Goldman Sachs confirmed that it expects a decrease in credit concession.', 'Goldman Sachs expects a reduction in demand for personal loans.', 'These reductions are expected to be of equal magnitude compared to the last four months of the year.', 'The current phenomenon is spread evenly across the euro area.', 'The current phenomenon differs from the crisis that hit the eurozone a decade ago.']</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: prevent italian names to be translated in english
That was accomplished adding spaCy library. This partially solved the issue.
</commit_message>
<xml_diff>
--- a/data/Annotazioni_1_with_factoids.xlsx
+++ b/data/Annotazioni_1_with_factoids.xlsx
@@ -542,17 +542,17 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>pensioners, beneficiaries of a maintenance allowance in the event of divorce and tenants of a rent may try not to get lost by the crazy price race. but public and private employees (unless there are specific agreements on the contract) and self-employed will remain on the stake with their wages. So much so that, as Istat explained a few days ago, with contractual wages growing only by 0.8% and an inflation rate of 5.2%, this year there will be a loss of purchasing power of almost five points. But the shield won't be so bad for everyone, as I said. the law, for example, provides for the re-evaluation of the maintenance allowance, in the event of separation or divorce, in order to protect the recipient, adjusting the amount due to the economically weaker spouse or children to the average cost of living. the revaluation must be carried out each year according to the ISTAT indices and must always be applied, in any case, whether or not it has been agreed by the spouses in the agreement or by the judge by the judgment of separation or divorce. for the revaluation, the index of consumer prices of the families of workers and employees shall be used, taking as a reference the index published by the Istat as compared to the month of the first payment of the maintenance allowance decided by the court of the previous year. in the event of failure to adapt, the rule also provides for the possibility of requesting arrears for the last 5 years. Pensioners will also have a protective shield. from this year the indexation mechanism has been re-introduced which re-evaluates the pension amounts for allowances and coupons. Thus pensioners who receive a monthly allowance up to 4 times the social allowance (about 2,000 euros) will have a full revaluation of the amount compared to inflation, pensioners who receive between 4 and 5 times the allowance will have 90% increase compared to inflation; pensioners who receive more than 5 times the social allowance will have 75% increase compared to inflation. Istat has established that, for this year, the inflation index on which the adjustments referred to 2021 will be based will be 1.9 percent. but in 2023 the cheques will recover the price growth recorded in 2022 and the revaluation, according to current estimates, will be around 7%. even the owners of a property will be able to attach the rent allowance to the trend of inflation, while, in terms of liquidations, the rules provide that the tfr, with the exception of the share gained in the year, will be increased each year with the application of a fixed rate of 1.5% and 75% of the increase of the index of consumer prices for the families of workers and employees (3/4 of the rate of inflation), established by the Istat, compared to December of the previous year. in the case of application of the revaluation rate by fractions of the year, the increase in the ist index shall be that resulting in the month of termination of the employment relationship compared to that in December of the previous year. For example: if inflation is 2%: 75% is 1.5%, to which the fixed rate must be added. therefore the tfr must be re-evaluated by 3%, equal to 1,5% plus 1,5%. bunch michele</t>
+          <t>pensioners, beneficiaries of a maintenance allowance in the event of divorce and tenants of a rent may try not to get lost by the crazy price race. but public and private employees (unless there are specific agreements on the contract) and self-employed will remain on the stake with their wages. So much so that, as Istat explained a few days ago, with contractual wages growing only by 0.8% and an inflation rate of 5.2%, this year there will be a loss of purchasing power of almost five points. But the shield won't be so bad for everyone, as I said. the law, for example, provides for the re-evaluation of the maintenance allowance, in the event of separation or divorce, in order to protect the recipient, adjusting the amount due to the economically weaker spouse or children to the average cost of living. the revaluation must be carried out each year according to the ISTAT indices and must always be applied, in any case, whether or not it has been agreed by the spouses in the agreement or by the judge by the judgment of separation or divorce. for the revaluation, the index of consumer prices of the families of workers and employees shall be used, taking as a reference the index published by the Istat as compared to the month of the first payment of the maintenance allowance decided by the court of the previous year. in the event of failure to adapt, the rule also provides for the possibility of requesting arrears for the last 5 years. Pensioners will also have a protective shield. from this year the indexation mechanism has been re-introduced which re-evaluates the pension amounts for allowances and coupons. Thus pensioners who receive a monthly allowance up to 4 times the social allowance (about 2,000 euros) will have a full revaluation of the amount compared to inflation, pensioners who receive between 4 and 5 times the allowance will have 90% increase compared to inflation; pensioners who receive more than 5 times the social allowance will have 75% increase compared to inflation. Istat has established that, for this year, the inflation index on which the adjustments referred to 2021 will be based will be 1.9 percent. but in 2023 the cheques will recover the price growth recorded in 2022 and the revaluation, according to current estimates, will be around 7%. even the owners of a property will be able to attach the rent allowance to the trend of inflation, while, in terms of liquidations, the rules provide that the tfr, with the exception of the share gained in the year, will be increased each year with the application of a fixed rate of 1.5% and 75% of the increase of the index of consumer prices for the families of workers and employees (3/4 of the rate of inflation), established by the Istat, compared to December of the previous year. in the case of application of the revaluation rate by fractions of the year, the increase in the ist index shall be that resulting in the month of termination of the employment relationship compared to that in December of the previous year. For example: if inflation is 2%: 75% is 1.5%, to which the fixed rate must be added. therefore the tfr must be re-evaluated by 3%, equal to 1,5% plus 1,5%. michele di branco</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>Observation date: 2022-07-02 00:00:00. pensioners, beneficiaries of a maintenance allowance in the event of divorce and tenants of a rent may try not to get lost by the crazy price race. but public and private employees (unless there are specific agreements on the contract) and self-employed will remain on the stake with their wages. So much so that, as Istat explained a few days ago, with contractual wages growing only by 0.8% and an inflation rate of 5.2%, this year there will be a loss of purchasing power of almost five points. But the shield won't be so bad for everyone, as I said. the law, for example, provides for the re-evaluation of the maintenance allowance, in the event of separation or divorce, in order to protect the recipient, adjusting the amount due to the economically weaker spouse or children to the average cost of living. the revaluation must be carried out each year according to the ISTAT indices and must always be applied, in any case, whether or not it has been agreed by the spouses in the agreement or by the judge by the judgment of separation or divorce. for the revaluation, the index of consumer prices of the families of workers and employees shall be used, taking as a reference the index published by the Istat as compared to the month of the first payment of the maintenance allowance decided by the court of the previous year. in the event of failure to adapt, the rule also provides for the possibility of requesting arrears for the last 5 years. Pensioners will also have a protective shield. from this year the indexation mechanism has been re-introduced which re-evaluates the pension amounts for allowances and coupons. Thus pensioners who receive a monthly allowance up to 4 times the social allowance (about 2,000 euros) will have a full revaluation of the amount compared to inflation, pensioners who receive between 4 and 5 times the allowance will have 90% increase compared to inflation; pensioners who receive more than 5 times the social allowance will have 75% increase compared to inflation. Istat has established that, for this year, the inflation index on which the adjustments referred to 2021 will be based will be 1.9 percent. but in 2023 the cheques will recover the price growth recorded in 2022 and the revaluation, according to current estimates, will be around 7%. even the owners of a property will be able to attach the rent allowance to the trend of inflation, while, in terms of liquidations, the rules provide that the tfr, with the exception of the share gained in the year, will be increased each year with the application of a fixed rate of 1.5% and 75% of the increase of the index of consumer prices for the families of workers and employees (3/4 of the rate of inflation), established by the Istat, compared to December of the previous year. in the case of application of the revaluation rate by fractions of the year, the increase in the ist index shall be that resulting in the month of termination of the employment relationship compared to that in December of the previous year. For example: if inflation is 2%: 75% is 1.5%, to which the fixed rate must be added. therefore the tfr must be re-evaluated by 3%, equal to 1,5% plus 1,5%. bunch michele</t>
+          <t>Observation date: 2022-07-02 00:00:00. pensioners, beneficiaries of a maintenance allowance in the event of divorce and tenants of a rent may try not to get lost by the crazy price race. but public and private employees (unless there are specific agreements on the contract) and self-employed will remain on the stake with their wages. So much so that, as Istat explained a few days ago, with contractual wages growing only by 0.8% and an inflation rate of 5.2%, this year there will be a loss of purchasing power of almost five points. But the shield won't be so bad for everyone, as I said. the law, for example, provides for the re-evaluation of the maintenance allowance, in the event of separation or divorce, in order to protect the recipient, adjusting the amount due to the economically weaker spouse or children to the average cost of living. the revaluation must be carried out each year according to the ISTAT indices and must always be applied, in any case, whether or not it has been agreed by the spouses in the agreement or by the judge by the judgment of separation or divorce. for the revaluation, the index of consumer prices of the families of workers and employees shall be used, taking as a reference the index published by the Istat as compared to the month of the first payment of the maintenance allowance decided by the court of the previous year. in the event of failure to adapt, the rule also provides for the possibility of requesting arrears for the last 5 years. Pensioners will also have a protective shield. from this year the indexation mechanism has been re-introduced which re-evaluates the pension amounts for allowances and coupons. Thus pensioners who receive a monthly allowance up to 4 times the social allowance (about 2,000 euros) will have a full revaluation of the amount compared to inflation, pensioners who receive between 4 and 5 times the allowance will have 90% increase compared to inflation; pensioners who receive more than 5 times the social allowance will have 75% increase compared to inflation. Istat has established that, for this year, the inflation index on which the adjustments referred to 2021 will be based will be 1.9 percent. but in 2023 the cheques will recover the price growth recorded in 2022 and the revaluation, according to current estimates, will be around 7%. even the owners of a property will be able to attach the rent allowance to the trend of inflation, while, in terms of liquidations, the rules provide that the tfr, with the exception of the share gained in the year, will be increased each year with the application of a fixed rate of 1.5% and 75% of the increase of the index of consumer prices for the families of workers and employees (3/4 of the rate of inflation), established by the Istat, compared to December of the previous year. in the case of application of the revaluation rate by fractions of the year, the increase in the ist index shall be that resulting in the month of termination of the employment relationship compared to that in December of the previous year. For example: if inflation is 2%: 75% is 1.5%, to which the fixed rate must be added. therefore the tfr must be re-evaluated by 3%, equal to 1,5% plus 1,5%. michele di branco</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>['Pensioners, beneficiaries of a maintenance allowance in the event of divorce, and tenants of a rent may try to avoid the price race.', 'Public and private employees (unless there are specific agreements on the contract) and self-employed will maintain their wages.', 'Istat explained on 2022-07-02 that contractual wages grew by 0.8%.', 'Istat explained on 2022-07-02 that the inflation rate was 5.2%.', 'Due to the 0.8% wage growth and 5.2% inflation rate, there will be a loss of purchasing power of almost five points on 2022-01-01.', 'The law provides for the re-evaluation of the maintenance allowance in the event of separation or divorce.', 'The re-evaluation protects the recipient by adjusting the amount due to the economically weaker spouse or children to the average cost of living.', 'The revaluation must be carried out each year according to the ISTAT indices.', 'The revaluation must always be applied, regardless of agreement by the spouses or by the judge.', 'For the revaluation, the index of consumer prices of the families of workers and employees shall be used.', 'The index used for revaluation references the index published by Istat compared to the month of the first payment of the maintenance allowance decided by the court of the previous year.', 'If the maintenance allowance fails to adapt, the rule allows requesting arrears for the last 5 years.', 'Pensioners will also have a protective shield.', 'The indexation mechanism was re-introduced from on 2022-01-01 to re-evaluate pension amounts for allowances and coupons.', 'Pensioners receiving a monthly allowance up to 4 times the social allowance (about 2,000 euros) will receive a full revaluation compared to inflation.', 'Pensioners receiving between 4 and 5 times the social allowance will receive a 90% increase compared to inflation.', 'Istat established that the inflation index for on 2022-01-01, which will be based on adjustments referred to 2021, will be 1.9 percent.', 'In 2023, the cheques will recover the price growth recorded in 2022.', 'The revaluation, according to current estimates, will be around 7%.', 'Property owners can attach the rent allowance to the trend of inflation.', 'Regarding liquidations, the rules provide that the TFR, excluding the share gained in the year, will increase each year.', 'The TFR increase is calculated using a fixed rate of 1.5%.', 'The TFR increase also uses 75% of the increase of the index of consumer prices for the families of workers and employees (3/4 of the rate of inflation), established by Istat compared to December of the previous year.', 'If the revaluation rate is applied by fractions of the year, the increase in the ISTAT index must be calculated from the month of termination of the employment relationship compared to December of the previous year.', 'If inflation is 2%, 75% is 1.5%.', 'The TFR must be re-evaluated by 3% (1.5% plus 1.5%) in the example provided.']</t>
+          <t>['Public and private employees (unless there are specific agreements on the contract) and self-employed will retain their wages.', 'Istat explained that contractual wages grew by 0.8%.', 'The inflation rate is 5.2%.', 'on 2022-01-01, there will be a loss of purchasing power of almost five points.', 'The law provides for the re-evaluation of the maintenance allowance in the event of separation or divorce.', 'The re-evaluation protects the recipient.', 'The law adjusts the amount due to the economically weaker spouse or children to the average cost of living.', 'The revaluation must be carried out each year according to the ISTAT indices.', 'The revaluation must always be applied.', 'The revaluation applies regardless of agreement by the spouses.', 'The revaluation applies regardless of judgment by the judge of separation or divorce.', 'For the revaluation, the index of consumer prices of the families of workers and employees shall be used.', 'The index used for revaluation references the index published by Istat compared to the month of the first payment of the maintenance allowance decided by the court of the previous year.', 'If the maintenance allowance fails to adapt, the rule allows requesting arrears for the last 5 years.', 'From on 2022-01-01, the indexation mechanism was re-introduced.', 'The indexation mechanism re-evaluates pension amounts for allowances and coupons.', 'Pensioners receiving a monthly allowance up to 4 times the social allowance (about 2,000 euros) will receive a full revaluation compared to inflation.', 'Pensioners receiving between 4 and 5 times the social allowance will receive a 90% increase compared to inflation.', 'Istat established that the inflation index for on 2022-01-01 will be 1.9 percent.', 'In 2023, the cheques will recover the price growth recorded in 2022.', 'The revaluation, according to current estimates, will be around 7%.', 'Property owners can attach the rent allowance to the trend of inflation.', 'Regarding liquidations, the rules provide that the TFR (with the exception of the share gained in the year) will be increased each year.', 'The TFR increase applies a fixed rate of 1.5%.', 'The TFR increase also applies 75% of the increase of the index of consumer prices for the families of workers and employees.', 'The index of consumer prices increase is established by Istat compared to December of the previous year.', 'If the revaluation rate is applied by fractions of the year, the increase in the ISTAT index must be calculated.', 'The calculation compares the month of termination of the employment relationship to December of the previous year.', 'If inflation is 2%, 75% is 1.5%.', 'The TFR must be re-evaluated by 3% (1.5% plus 1.5%).']</t>
         </is>
       </c>
     </row>
@@ -610,17 +610,17 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>- the government's move on the imu, which returns to December in masked form, as a down payment of the service tax. the treasury is hunting 3 billion to avoid the increase of the estimated tax in October but the operation-maquillage of the tax on the house is expected to arrive in November. And at the quirinal, now the alarm goes off. the holding on the financial law is at risk. consultation of the Napolitan President with the alphanus and epiphans secretaries while the pdl threatens a crisis again. The German elections had a very clear winner in the popular vote, Angela Merkel. But an electoral law that many insist on exporting to us will not allow it to govern itself. Thus a new large koalition appears on the horizon. the last of the series, ran the year 2005, resulted from an agreement signed after weeks of negotiation. the legislative programme was more than 300 pages long, it also exceeded the "manifesto" of the electoral prodians of 2006. Like that, he remained dead letter. Our great coalition was born with a half-hour investiture speech from the President-in-Office. It promised itself everything and more, denying any budgetary constraint. Then there was the same decision-making paralysis, even more animated than in Germany: quarrels raging on live TV as soon as it had to clash with budgetary constraints. They don't forgive. Unlike the Germans, we cannot afford decision-making paralysis. The government is now acting only in the dream sphere or in that of accounting tricks. the update note to the def presented a few days ago by our executive proposes macroeconomic scenarios from dreamy late summer. We should grow in the next three years at a rate twice that of potential, tearing the estimates of international organisations, without doing anything to make such a sudden change of pace possible. These scenarios include the coexistence of high inflation (a GDP deflator of 2%) with a further fall in household consumption and rising unemployment. It is difficult to understand how the three phenomena can be realized simultaneously. They may be used to draw up tables in which the debt ratio and GDP never rises above 130% of gross domestic product, but these unrealistic scenarios cannot convince institutional fund managers to invest in our country. If anything, they risk weakening our negotiating position at Community level. We already hear the objections to bruxelles: "If things are destined to go so well, why should we give you the room for manoeuvre that you ask us for?" accounting engineering has also been added to false optimism. is intended to revalue the shares held by banks at the banks of Italy, a legacy of when the banks were public. with banks that would see their capital position strengthened. the treasure which would receive a contribution for the gains thus achieved. It is less happy for taxpayers who will one day have to buy back these shares because a central bank cannot be owned by private banks. They risk paying a very salty bill because the price will presumably be very high. would be in the interest of both banks and the Treasury. and there are no market references, so much so that a special commission of essays has been set up. As he puts his head under the sand with dreams and accounting engineering, the country risks finishing, day after day, in the hands of the troika, without even realizing it. It was hard to get back from a debt of 120 percent. it is much more difficult to do so from a debt to 130 percent and growing. If this government does not want to be remembered for what has given national sovereignty, it must find a programme agreement on the basis of which to open a negotiation at bruxelles. the agreement should be sculpted into the law of stability. its philosophy of tackling emergencies with long-term reforms. For example, the refinancing of the supplementary fund by way of derogation should provide for the gradual overrun of this institution, with wage supplements for those working less than EUR 5 per hour, a way to facilitate labour mobility and increase employment. Any new access to the coffin will have to be blocked by way of derogation, starting with that required for the former party employees by a very large parliamentary coalition. As with other workers, ordinary social shock absorbers will be available. Another example: the increase in VAT, possibly limited to luxury goods only, could be offset by a cut in the tax wedge, since indirect taxes increase the difference between labour costs and purchasing power of wages. then there should be measures to cut expenditure, which could be implemented gradually, but with actions already approved. One can start from dismantling the bureaucracy created by the federalism of the league, which has created duplications, uncontrolled local spending and an excess of power centers. a few examples: how to justify the sponsorship offered by the Sardinian region to the Cagliari football team? What are 45 port authorities for? Can we not reduce the number of prefectures and really abolish the provinces? Needless to say, cutting this waste is also politically expensive. The directing booth should serve to protect the government from the raging attacks to which it will be subjected by those affected by the cuts. With these measures included in the Stability Act it is possible to open negotiations with bruxelles which also include deficits of more than 3% over the coming years. But it will take a compact government, not a company whose survival is questioned every day.</t>
+          <t>- the government's move on the imu, which returns to December in masked form, as a down payment of the service tax. the treasury is hunting 3 billion to avoid the increase of the estimated tax in October but the operation-maquillage of the tax on the house is expected to arrive in November. And at the quirinal, now the alarm goes off. the holding on the financial law is at risk. President napolitano consultations with the alphanus and epiphans secretaries while the pdl threatens a crisis again. The German elections had a very clear winner in the popular vote, angela merkel. But an electoral law that many insist on exporting to us will not allow it to govern itself. Thus a new large koalition appears on the horizon. the last of the series, ran the year 2005, resulted from an agreement signed after weeks of negotiation. the legislative programme was more than 300 pages long, it also exceeded the "manifesto" of the electoral prodians of 2006. Like that, he remained dead letter. Our great coalition was born with a half-hour investiture speech from the President-in-Office. It promised itself everything and more, denying any budgetary constraint. Then there was the same decision-making paralysis, even more animated than in Germany: quarrels raging on live TV as soon as it had to clash with budgetary constraints. They don't forgive. Unlike the Germans, we cannot afford decision-making paralysis. The government is now acting only in the dream sphere or in that of accounting tricks. the update note to the def presented a few days ago by our executive proposes macroeconomic scenarios from dreamy late summer. We should grow in the next three years at a rate twice that of potential, tearing the estimates of international organisations, without doing anything to make such a sudden change of pace possible. These scenarios include the coexistence of high inflation (a GDP deflator of 2%) with a further fall in household consumption and rising unemployment. It is difficult to understand how the three phenomena can be realized simultaneously. They may be used to draw up tables in which the debt ratio and GDP never rises above 130% of gross domestic product, but these unrealistic scenarios cannot convince institutional fund managers to invest in our country. If anything, they risk weakening our negotiating position at Community level. We already hear the objections to bruxelles: "If things are destined to go so well, why should we give you the room for manoeuvre that you ask us for?" accounting engineering has also been added to false optimism. is intended to revalue the shares held by banks at the banks of Italy, a legacy of when the banks were public. with banks that would see their capital position strengthened. the treasure which would receive a contribution for the gains thus achieved. It is less happy for taxpayers who will one day have to buy back these shares because a central bank cannot be owned by private banks. They risk paying a very salty bill because the price will presumably be very high. would be in the interest of both banks and the Treasury. and there are no market references, so much so that a special commission of essays has been set up. As he puts his head under the sand with dreams and accounting engineering, the country risks finishing, day after day, in the hands of the troika, without even realizing it. It was hard to get back from a debt of 120 percent. it is much more difficult to do so from a debt to 130 percent and growing. If this government does not want to be remembered for what has given national sovereignty, it must find a programme agreement on the basis of which to open a negotiation at bruxelles. the agreement should be sculpted into the law of stability. its philosophy of tackling emergencies with long-term reforms. For example, the refinancing of the supplementary fund by way of derogation should provide for the gradual overrun of this institution, with wage supplements for those working less than EUR 5 per hour, a way to facilitate labour mobility and increase employment. Any new access to the coffin will have to be blocked by way of derogation, starting with that required for the former party employees by a very large parliamentary coalition. As with other workers, ordinary social shock absorbers will be available. Another example: the increase in VAT, possibly limited to luxury goods only, could be offset by a cut in the tax wedge, since indirect taxes increase the difference between labour costs and purchasing power of wages. then there should be measures to cut expenditure, which could be implemented gradually, but with actions already approved. One can start from dismantling the bureaucracy created by the federalism of the league, which has created duplications, uncontrolled local spending and an excess of power centers. a few examples: how to justify the sponsorship offered by the Sardinian region to the football team of the cagliari? What are 45 port authorities for? Can we not reduce the number of prefectures and really abolish the provinces? Needless to say, cutting this waste is also politically expensive. The directing booth should serve to protect the government from the raging attacks to which it will be subjected by those affected by the cuts. With these measures included in the Stability Act it is possible to open negotiations with bruxelles which also include deficits of more than 3% over the coming years. But it will take a compact government, not a company whose survival is questioned every day.</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Observation date: 2013-09-25 00:00:00. - the government's move on the imu, which returns to December in masked form, as a down payment of the service tax. the treasury is hunting 3 billion to avoid the increase of the estimated tax in October but the operation-maquillage of the tax on the house is expected to arrive in November. And at the quirinal, now the alarm goes off. the holding on the financial law is at risk. consultation of the Napolitan President with the alphanus and epiphans secretaries while the pdl threatens a crisis again. The German elections had a very clear winner in the popular vote, Angela Merkel. But an electoral law that many insist on exporting to us will not allow it to govern itself. Thus a new large koalition appears on the horizon. the last of the series, ran the year 2005, resulted from an agreement signed after weeks of negotiation. the legislative programme was more than 300 pages long, it also exceeded the "manifesto" of the electoral prodians of 2006. Like that, he remained dead letter. Our great coalition was born with a half-hour investiture speech from the President-in-Office. It promised itself everything and more, denying any budgetary constraint. Then there was the same decision-making paralysis, even more animated than in Germany: quarrels raging on live TV as soon as it had to clash with budgetary constraints. They don't forgive. Unlike the Germans, we cannot afford decision-making paralysis. The government is now acting only in the dream sphere or in that of accounting tricks. the update note to the def presented a few days ago by our executive proposes macroeconomic scenarios from dreamy late summer. We should grow in the next three years at a rate twice that of potential, tearing the estimates of international organisations, without doing anything to make such a sudden change of pace possible. These scenarios include the coexistence of high inflation (a GDP deflator of 2%) with a further fall in household consumption and rising unemployment. It is difficult to understand how the three phenomena can be realized simultaneously. They may be used to draw up tables in which the debt ratio and GDP never rises above 130% of gross domestic product, but these unrealistic scenarios cannot convince institutional fund managers to invest in our country. If anything, they risk weakening our negotiating position at Community level. We already hear the objections to bruxelles: "If things are destined to go so well, why should we give you the room for manoeuvre that you ask us for?" accounting engineering has also been added to false optimism. is intended to revalue the shares held by banks at the banks of Italy, a legacy of when the banks were public. with banks that would see their capital position strengthened. the treasure which would receive a contribution for the gains thus achieved. It is less happy for taxpayers who will one day have to buy back these shares because a central bank cannot be owned by private banks. They risk paying a very salty bill because the price will presumably be very high. would be in the interest of both banks and the Treasury. and there are no market references, so much so that a special commission of essays has been set up. As he puts his head under the sand with dreams and accounting engineering, the country risks finishing, day after day, in the hands of the troika, without even realizing it. It was hard to get back from a debt of 120 percent. it is much more difficult to do so from a debt to 130 percent and growing. If this government does not want to be remembered for what has given national sovereignty, it must find a programme agreement on the basis of which to open a negotiation at bruxelles. the agreement should be sculpted into the law of stability. its philosophy of tackling emergencies with long-term reforms. For example, the refinancing of the supplementary fund by way of derogation should provide for the gradual overrun of this institution, with wage supplements for those working less than EUR 5 per hour, a way to facilitate labour mobility and increase employment. Any new access to the coffin will have to be blocked by way of derogation, starting with that required for the former party employees by a very large parliamentary coalition. As with other workers, ordinary social shock absorbers will be available. Another example: the increase in VAT, possibly limited to luxury goods only, could be offset by a cut in the tax wedge, since indirect taxes increase the difference between labour costs and purchasing power of wages. then there should be measures to cut expenditure, which could be implemented gradually, but with actions already approved. One can start from dismantling the bureaucracy created by the federalism of the league, which has created duplications, uncontrolled local spending and an excess of power centers. a few examples: how to justify the sponsorship offered by the Sardinian region to the Cagliari football team? What are 45 port authorities for? Can we not reduce the number of prefectures and really abolish the provinces? Needless to say, cutting this waste is also politically expensive. The directing booth should serve to protect the government from the raging attacks to which it will be subjected by those affected by the cuts. With these measures included in the Stability Act it is possible to open negotiations with bruxelles which also include deficits of more than 3% over the coming years. But it will take a compact government, not a company whose survival is questioned every day.</t>
+          <t>Observation date: 2013-09-25 00:00:00. - the government's move on the imu, which returns to December in masked form, as a down payment of the service tax. the treasury is hunting 3 billion to avoid the increase of the estimated tax in October but the operation-maquillage of the tax on the house is expected to arrive in November. And at the quirinal, now the alarm goes off. the holding on the financial law is at risk. President napolitano consultations with the alphanus and epiphans secretaries while the pdl threatens a crisis again. The German elections had a very clear winner in the popular vote, angela merkel. But an electoral law that many insist on exporting to us will not allow it to govern itself. Thus a new large koalition appears on the horizon. the last of the series, ran the year 2005, resulted from an agreement signed after weeks of negotiation. the legislative programme was more than 300 pages long, it also exceeded the "manifesto" of the electoral prodians of 2006. Like that, he remained dead letter. Our great coalition was born with a half-hour investiture speech from the President-in-Office. It promised itself everything and more, denying any budgetary constraint. Then there was the same decision-making paralysis, even more animated than in Germany: quarrels raging on live TV as soon as it had to clash with budgetary constraints. They don't forgive. Unlike the Germans, we cannot afford decision-making paralysis. The government is now acting only in the dream sphere or in that of accounting tricks. the update note to the def presented a few days ago by our executive proposes macroeconomic scenarios from dreamy late summer. We should grow in the next three years at a rate twice that of potential, tearing the estimates of international organisations, without doing anything to make such a sudden change of pace possible. These scenarios include the coexistence of high inflation (a GDP deflator of 2%) with a further fall in household consumption and rising unemployment. It is difficult to understand how the three phenomena can be realized simultaneously. They may be used to draw up tables in which the debt ratio and GDP never rises above 130% of gross domestic product, but these unrealistic scenarios cannot convince institutional fund managers to invest in our country. If anything, they risk weakening our negotiating position at Community level. We already hear the objections to bruxelles: "If things are destined to go so well, why should we give you the room for manoeuvre that you ask us for?" accounting engineering has also been added to false optimism. is intended to revalue the shares held by banks at the banks of Italy, a legacy of when the banks were public. with banks that would see their capital position strengthened. the treasure which would receive a contribution for the gains thus achieved. It is less happy for taxpayers who will one day have to buy back these shares because a central bank cannot be owned by private banks. They risk paying a very salty bill because the price will presumably be very high. would be in the interest of both banks and the Treasury. and there are no market references, so much so that a special commission of essays has been set up. As he puts his head under the sand with dreams and accounting engineering, the country risks finishing, day after day, in the hands of the troika, without even realizing it. It was hard to get back from a debt of 120 percent. it is much more difficult to do so from a debt to 130 percent and growing. If this government does not want to be remembered for what has given national sovereignty, it must find a programme agreement on the basis of which to open a negotiation at bruxelles. the agreement should be sculpted into the law of stability. its philosophy of tackling emergencies with long-term reforms. For example, the refinancing of the supplementary fund by way of derogation should provide for the gradual overrun of this institution, with wage supplements for those working less than EUR 5 per hour, a way to facilitate labour mobility and increase employment. Any new access to the coffin will have to be blocked by way of derogation, starting with that required for the former party employees by a very large parliamentary coalition. As with other workers, ordinary social shock absorbers will be available. Another example: the increase in VAT, possibly limited to luxury goods only, could be offset by a cut in the tax wedge, since indirect taxes increase the difference between labour costs and purchasing power of wages. then there should be measures to cut expenditure, which could be implemented gradually, but with actions already approved. One can start from dismantling the bureaucracy created by the federalism of the league, which has created duplications, uncontrolled local spending and an excess of power centers. a few examples: how to justify the sponsorship offered by the Sardinian region to the football team of the cagliari? What are 45 port authorities for? Can we not reduce the number of prefectures and really abolish the provinces? Needless to say, cutting this waste is also politically expensive. The directing booth should serve to protect the government from the raging attacks to which it will be subjected by those affected by the cuts. With these measures included in the Stability Act it is possible to open negotiations with bruxelles which also include deficits of more than 3% over the coming years. But it will take a compact government, not a company whose survival is questioned every day.</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>["The government's move on the IMU returns to December in masked form.", 'The government uses the IMU move as a down payment of the service tax.', 'The Treasury is hunting 3 billion to avoid the increase of the estimated tax on 2013-10-25.', 'The operation-maquillage of the tax on the house is expected to arrive in November.', 'The holding on the financial law is at risk at the Quirinal.', 'The Napolitan President consulted with the Alphanus and Epiphans secretaries.', 'The PDL threatens a crisis again.', 'Angela Merkel was the clear winner in the popular vote in the German elections.', 'An electoral law that many insist on exporting to Italy will not allow Italy to govern itself.', 'A new large koalition appears on the horizon.', 'The last koalition series ran in the year 2005.', 'The legislative program of the koalition was more than 300 pages long.', "The legislative program exceeded the 'manifesto' of the electoral prodians of 2006.", 'The Great Coalition promised itself everything and more, denying any budgetary constraint.', 'The update note to the DEF, presented by the executive, proposes macroeconomic scenarios.', 'The macroeconomic scenarios propose growth in the next three years at a rate twice that of potential.', 'The proposed growth rate tears the estimates of international organizations.', 'The scenarios include high inflation (a GDP deflator of 2%).', 'The scenarios include a further fall in household consumption.', 'The scenarios include rising unemployment.', 'The scenarios may be used to draw up tables where the debt ratio and GDP never rise above 130% of gross domestic product.', "The unrealistic scenarios risk weakening Italy's negotiating position at Community level.", 'Accounting engineering is intended to revalue the shares held by banks at the banks of Italy.', 'The revaluation would strengthen the capital position of the banks.', 'The Treasury would receive a contribution for the gains achieved through accounting engineering.', 'Taxpayers risk paying a high bill if taxpayers have to buy back the shares.', 'The country risks finishing in the hands of the Troika.', 'It was hard to get back from a debt of 120 percent.', 'It is much more difficult to reduce debt from 130 percent and growing.', 'The government must find a program agreement to open negotiations at Bruxelles.', 'The agreement should be sculpted into the law of stability.', "The law of stability's philosophy is tackling emergencies with long-term reforms.", 'Refinancing the supplementary fund by way of derogation should provide for the gradual overrun of the institution.', 'The fund should provide wage supplements for those working less than EUR 5 per hour.', 'Any new access to the coffin must be blocked by way of derogation.', 'The blocking of new access must start with that required for the former party employees by a very large parliamentary coalition.', 'The increase in VAT, possibly limited to luxury goods only, could be offset by a cut in the tax wedge.', 'Indirect taxes increase the difference between labor costs and purchasing power of wages.', 'Measures to cut expenditure should be implemented gradually.', 'One can start by dismantling the bureaucracy created by the federalism of the league.', 'The federalism of the league created duplications, uncontrolled local spending, and an excess of power centers.', 'Including these measures in the Stability Act makes it possible to open negotiations with Bruxelles.', 'These negotiations can include deficits of more than 3% over the coming years.']</t>
+          <t>['The government planned a move on the IMU.', 'The IMU move was scheduled for December.', 'The IMU move was structured as a down payment of the service tax.', 'The Treasury was seeking 3 billion to avoid an increase in the estimated tax.', 'The tax operation (maquillage) on the house was expected to arrive in November.', 'President Napolitano consulted with the Alphanus secretary.', 'The PDL threatened a crisis.', 'Angela Merkel was the clear winner in the popular vote in the German elections.', 'A new large coalition appeared on the horizon.', 'The last coalition series ran in the year 2005.', 'The coalition resulted from an agreement signed after weeks of negotiation.', 'The legislative program was more than 300 pages long.', "The legislative program exceeded the 'manifesto' of the electoral prodians of 2006.", 'The great coalition was born with a half-hour investiture speech from the President-in-Office.', 'The great coalition promised everything and more.', 'The great coalition denied any budgetary constraint.', 'Decision-making paralysis occurred.', 'The paralysis was animated when it had to clash with budgetary constraints.', 'The government is acting only in the dream sphere or in that of accounting tricks.', 'The update note to the DEF was presented by the executive.', 'The update note proposed macroeconomic scenarios.', 'The scenarios suggested growth in the next three years at a rate twice that of potential.', 'The scenarios contradicted the estimates of international organizations.', 'The scenarios include high inflation (a GDP deflator of 2%).', 'The scenarios include a further fall in household consumption.', 'The scenarios include rising unemployment.', 'The scenarios allow drawing up tables where the debt ratio and GDP never rise above 130% of gross domestic product.', "These unrealistic scenarios risk weakening the country's negotiating position at Community level.", 'Objections were heard regarding the room for maneuver requested from Bruxelles.', 'Accounting engineering was intended to revalue shares held by banks at the banks of Italy.', 'These shares were a legacy of when the banks were public.', 'Banks would see their capital position strengthened due to accounting engineering.', 'A special commission of essays was set up because there were no market references.', 'The country risks falling into the hands of the troika.', 'It was hard to get back from a debt of 120 percent.', 'It is much more difficult to recover from a debt of 130 percent and growing.', 'The government must find a program agreement to open negotiations at Bruxelles.', 'The agreement should be sculpted into the law of stability.', "The law of stability's philosophy is tackling emergencies with long-term reforms.", 'Refinancing the supplementary fund by way of derogation should provide for the gradual overrun of the institution.', 'The fund should provide wage supplements for those working less than EUR 5 per hour.', 'This measure aims to facilitate labor mobility and increase employment.', 'Any new access to the coffin must be blocked by way of derogation.', 'The blocking must start with the access required for former party employees by a very large parliamentary coalition.', 'Ordinary social shock absorbers will be available for workers.', 'An increase in VAT, possibly limited to luxury goods only, could be offset by a cut in the tax wedge.', 'Indirect taxes increase the difference between labor costs and purchasing power of wages.', 'Measures should be implemented to cut expenditure.', 'The cuts should start with dismantling the bureaucracy created by the federalism of the league.', 'The federalism of the league created duplications, uncontrolled local spending, and an excess of power centers.', 'The text questioned the justification of the sponsorship offered by the Sardinian region to the Cagliari football team.', 'The text questioned the purpose of 45 port authorities.', 'The text suggested reducing the number of prefectures and abolishing the provinces.', 'The Stability Act measures allow opening negotiations with Bruxelles.', 'These negotiations include deficits of more than 3% over the coming years.']</t>
         </is>
       </c>
     </row>
@@ -674,17 +674,17 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>- needless to be deceived: the recovery will be shy, feeble and pregnant with downside risks. small businesses, especially those in the south, are left on the margins; consumption is languishing. and, above all, the unemployed also increase in 2015 and inflation continues to decrease. is more cautious than ever the economic bulletin of the bank of Italy, the first of the new year. its diffusion, on a quarterly basis, coincides this time with two important news in the matter of pil. the first: Commissioner Olli Rehn is confident in the country's rehabilitation capacity, asks to push ahead with disengagement and spending review, and suggests that Italy can achieve more flexibility on budgetary rules, which is an indispensable condition for releasing resources for investment. For the record: on these and other issues yesterday there was a breakfast between the commissioner and the minister of the economy, fabrizio saccomanni. the second news reveals that the ue is reviewing the calculation of the GDP, moving the investments in research and development from the expenditure box, therefore a liability, to that of the investments. According to extrapolations the benefit will be between 1 and 2%, with not negligible effects also for the purposes of the deficitpil and debt-pil ratio and, therefore, of the consolidation of the accounts and of the relationships with bruxelles. the document of the bank of Italy, of course, remains anchored only on the technical-analytic ground. Thus, the macro projections developed by these economists place the year-end GDP growth of 0.7%, and then rise to 1% in 2015. are therefore much smaller estimates than those of the government (1 and 1.7% respectively). They are small shots up in a slow European context. the effects on employment are not yet visible: this year the unemployment rate will be nailed to 12.8% and the next year will rise to 12.9%. Only the recovery of domestic demand will be able to extend the recovery to the labour market, warns the bank of Italy. At the moment, however, the risks to growth remain downward-oriented, the recovery of investment may be delayed, especially if the conditions for access to credit remain restrictive longer than expected or if payments of commercial debts of public administrations differ. and the risk of general deflation rests on everything: this danger is judged to be moderate. but the fall in inflation could be more pronounced and persistent than expected, especially if the weakness of demand reflected expectations. In short, as the president of the ECB himself recently recalled, "it is still early to sing victory" , better to stay on the ground. The general picture, in fact, remains in the dark. the confidence of the enterprises sure, is improving, the industrial activity is picking up breath after being diminished almost without interruptions from summer of 2011. but the background is very varied depending on the category of enterprises and their location: small ones, especially in the south, remain on the margins of the process. in the same way, if it is true that in the third quarter of 2013 the decline in consumption of the families has also diminished, it is true that today Italians do not spend. consumption continues to be restrained both by the weakness of disposable income and by difficult labour market conditions. The Italian bank also notes that the recovery of trust since the beginning of 2013 has been interrupted in the fourth quarter. At the same time, it changes its internal organization: under the Directory, 8 departments, services and divisions. © confidential reproduction</t>
+          <t>- needless to be deceived: the recovery will be shy, feeble and pregnant with downside risks. small businesses, especially those in the south, are left on the margins; consumption is languishing. and, above all, the unemployed also increase in 2015 and inflation continues to decrease. is more cautious than ever the economic bulletin of the banca d'italia, the first of the new year. its diffusion, on a quarterly basis, coincides this time with two important news in the matter of pil. the first: Commissioner ue, olli rehn, is confident in the country's rehabilitation capacity, asks to push on disposal and spending review and causes the hypothesis that Italy can obtain more flexibility on budgetary rules, an indispensable condition for freeing resources to be allocated to investments. For the record: on these and other issues yesterday there was a breakfast between the commissioner and the minister of the economy, fabrizio saccomanni. the second news reveals that the ue is reviewing the calculation of the GDP, moving the investments in research and development from the expenditure box, therefore a liability, to that of the investments. According to extrapolations the benefit will be between 1 and 2%, with not negligible effects also for the purposes of the deficitpil and debt-pil ratio and, therefore, of the consolidation of the accounts and of the relationships with bruxelles. the document of the banca d'italia, of course, remains anchored only on the technical-analytic ground. Thus, the macro projections developed by these economists place the year-end GDP growth of 0.7%, and then rise to 1% in 2015. are therefore much smaller estimates than those of the government (1 and 1.7% respectively). They are small shots up in a slow European context. the effects on employment are not yet visible: this year the unemployment rate will be nailed to 12.8% and the next year will rise to 12.9%. Only the recovery of domestic demand will be able to extend the recovery to the labour market, warns the banca d'italia. At the moment, however, the risks to growth remain downward-oriented, the recovery of investment may be delayed, especially if the conditions for access to credit remain restrictive longer than expected or if payments of commercial debts of public administrations differ. and the risk of general deflation rests on everything: this danger is judged to be moderate. but the fall in inflation could be more pronounced and persistent than expected, especially if the weakness of demand reflected expectations. In short, as the president of the ECB himself recently recalled, "it is still early to sing victory" , better to stay on the ground. The general picture, in fact, remains in the dark. the confidence of the enterprises sure, is improving, the industrial activity is picking up breath after being diminished almost without interruptions from summer of 2011. but the background is very varied depending on the category of enterprises and their location: small ones, especially in the south, remain on the margins of the process. in the same way, if it is true that in the third quarter of 2013 the decline in consumption of the families has also diminished, it is true that today Italians do not spend. consumption continues to be restrained both by the weakness of disposable income and by difficult labour market conditions. the banca d'italia also notes that the recovery of trust since the beginning of 2013 has been interrupted in the fourth quarter. At the same time, it changes its internal organization: under the Directory, 8 departments, services and divisions. © confidential reproduction</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>Observation date: 2014-01-18 00:00:00. - needless to be deceived: the recovery will be shy, feeble and pregnant with downside risks. small businesses, especially those in the south, are left on the margins; consumption is languishing. and, above all, the unemployed also increase in 2015 and inflation continues to decrease. is more cautious than ever the economic bulletin of the bank of Italy, the first of the new year. its diffusion, on a quarterly basis, coincides this time with two important news in the matter of pil. the first: Commissioner Olli Rehn is confident in the country's rehabilitation capacity, asks to push ahead with disengagement and spending review, and suggests that Italy can achieve more flexibility on budgetary rules, which is an indispensable condition for releasing resources for investment. For the record: on these and other issues yesterday there was a breakfast between the commissioner and the minister of the economy, fabrizio saccomanni. the second news reveals that the ue is reviewing the calculation of the GDP, moving the investments in research and development from the expenditure box, therefore a liability, to that of the investments. According to extrapolations the benefit will be between 1 and 2%, with not negligible effects also for the purposes of the deficitpil and debt-pil ratio and, therefore, of the consolidation of the accounts and of the relationships with bruxelles. the document of the bank of Italy, of course, remains anchored only on the technical-analytic ground. Thus, the macro projections developed by these economists place the year-end GDP growth of 0.7%, and then rise to 1% in 2015. are therefore much smaller estimates than those of the government (1 and 1.7% respectively). They are small shots up in a slow European context. the effects on employment are not yet visible: this year the unemployment rate will be nailed to 12.8% and the next year will rise to 12.9%. Only the recovery of domestic demand will be able to extend the recovery to the labour market, warns the bank of Italy. At the moment, however, the risks to growth remain downward-oriented, the recovery of investment may be delayed, especially if the conditions for access to credit remain restrictive longer than expected or if payments of commercial debts of public administrations differ. and the risk of general deflation rests on everything: this danger is judged to be moderate. but the fall in inflation could be more pronounced and persistent than expected, especially if the weakness of demand reflected expectations. In short, as the president of the ECB himself recently recalled, "it is still early to sing victory" , better to stay on the ground. The general picture, in fact, remains in the dark. the confidence of the enterprises sure, is improving, the industrial activity is picking up breath after being diminished almost without interruptions from summer of 2011. but the background is very varied depending on the category of enterprises and their location: small ones, especially in the south, remain on the margins of the process. in the same way, if it is true that in the third quarter of 2013 the decline in consumption of the families has also diminished, it is true that today Italians do not spend. consumption continues to be restrained both by the weakness of disposable income and by difficult labour market conditions. The Italian bank also notes that the recovery of trust since the beginning of 2013 has been interrupted in the fourth quarter. At the same time, it changes its internal organization: under the Directory, 8 departments, services and divisions. © confidential reproduction</t>
+          <t>Observation date: 2014-01-18 00:00:00. - needless to be deceived: the recovery will be shy, feeble and pregnant with downside risks. small businesses, especially those in the south, are left on the margins; consumption is languishing. and, above all, the unemployed also increase in 2015 and inflation continues to decrease. is more cautious than ever the economic bulletin of the banca d'italia, the first of the new year. its diffusion, on a quarterly basis, coincides this time with two important news in the matter of pil. the first: Commissioner ue, olli rehn, is confident in the country's rehabilitation capacity, asks to push on disposal and spending review and causes the hypothesis that Italy can obtain more flexibility on budgetary rules, an indispensable condition for freeing resources to be allocated to investments. For the record: on these and other issues yesterday there was a breakfast between the commissioner and the minister of the economy, fabrizio saccomanni. the second news reveals that the ue is reviewing the calculation of the GDP, moving the investments in research and development from the expenditure box, therefore a liability, to that of the investments. According to extrapolations the benefit will be between 1 and 2%, with not negligible effects also for the purposes of the deficitpil and debt-pil ratio and, therefore, of the consolidation of the accounts and of the relationships with bruxelles. the document of the banca d'italia, of course, remains anchored only on the technical-analytic ground. Thus, the macro projections developed by these economists place the year-end GDP growth of 0.7%, and then rise to 1% in 2015. are therefore much smaller estimates than those of the government (1 and 1.7% respectively). They are small shots up in a slow European context. the effects on employment are not yet visible: this year the unemployment rate will be nailed to 12.8% and the next year will rise to 12.9%. Only the recovery of domestic demand will be able to extend the recovery to the labour market, warns the banca d'italia. At the moment, however, the risks to growth remain downward-oriented, the recovery of investment may be delayed, especially if the conditions for access to credit remain restrictive longer than expected or if payments of commercial debts of public administrations differ. and the risk of general deflation rests on everything: this danger is judged to be moderate. but the fall in inflation could be more pronounced and persistent than expected, especially if the weakness of demand reflected expectations. In short, as the president of the ECB himself recently recalled, "it is still early to sing victory" , better to stay on the ground. The general picture, in fact, remains in the dark. the confidence of the enterprises sure, is improving, the industrial activity is picking up breath after being diminished almost without interruptions from summer of 2011. but the background is very varied depending on the category of enterprises and their location: small ones, especially in the south, remain on the margins of the process. in the same way, if it is true that in the third quarter of 2013 the decline in consumption of the families has also diminished, it is true that today Italians do not spend. consumption continues to be restrained both by the weakness of disposable income and by difficult labour market conditions. the banca d'italia also notes that the recovery of trust since the beginning of 2013 has been interrupted in the fourth quarter. At the same time, it changes its internal organization: under the Directory, 8 departments, services and divisions. © confidential reproduction</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>['Small businesses, especially those in the south, are left on the margins.', 'Consumption is languishing.', 'The unemployed will increase in 2015.', 'Inflation continues to decrease.', 'The economic bulletin of the bank of Italy was published on 2014-01-18.', 'The quarterly diffusion of the economic bulletin coincided with two important news items regarding PIL.', "Commissioner Olli Rehn is confident in the country's rehabilitation capacity.", 'Commissioner Olli Rehn asked to push ahead with disengagement and spending review.', 'Commissioner Olli Rehn suggests that Italy can achieve more flexibility on budgetary rules.', 'Flexibility on budgetary rules is an indispensable condition for releasing resources for investment.', 'On 2014-01-17, there was a breakfast between Commissioner Olli Rehn and the minister of the economy, Fabrizio Saccomanni.', 'The UE is reviewing the calculation of the GDP.', 'The UE is moving investments in research and development from the expenditure box (a liability) to the investments category.', 'The benefit of the GDP calculation review is expected to be between 1% and 2%.', 'The benefit will have effects on the deficit-PIL ratio.', 'These ratios affect the consolidation of the accounts and the relationships with Bruxelles.', 'The macro projections developed by the bank of Italy place the year-end GDP growth at 0.7%.', "The bank of Italy's estimates are smaller than the government's estimates for year-end GDP growth.", 'The government estimates GDP growth at 1.7% for the second year.', 'The unemployment rate will rise to 12.9% in 2015.', 'The bank of Italy warns that only the recovery of domestic demand can extend the recovery to the labor market.', 'Risks to growth remain downward-oriented.', 'The recovery of investment may be delayed if conditions for access to credit remain restrictive longer than expected.', 'The recovery of investment may be delayed if payments of commercial debts of public administrations differ.', 'The risk of general deflation is judged to be moderate.', 'The fall in inflation could be more pronounced and persistent than expected if the weakness of demand reflects expectations.', 'Enterprise confidence is improving.', 'Industrial activity is picking up after being diminished almost without interruptions from summer of 2011.', 'The background is varied depending on the category of enterprises and their location.', 'Small enterprises, especially in the south, remain on the margins of the process.', 'The decline in consumption of families diminished in the third quarter of 2013.', 'Italians do not spend on 2014-01-18.', 'Consumption is restrained by the weakness of disposable income.', 'Consumption is restrained by difficult labor market conditions.', 'The bank of Italy notes that the recovery of trust since the beginning of 2013 was interrupted in the fourth quarter.', 'The bank of Italy changed its internal organization.', 'The bank of Italy structured its organization under the Directory, 8 departments, services and divisions.']</t>
+          <t>['Small businesses, especially those in the south, are left on the margins.', 'Consumption is languishing.', 'The unemployed will increase in 2015.', 'Inflation continues to decrease.', "The economic bulletin of the banca d'italia was published on 2014-01-18.", 'The quarterly diffusion of the economic bulletin coincides with two important news regarding PIL.', "Commissioner UE, Olli Rehn, is confident in Italy's rehabilitation capacity.", 'Commissioner UE, Olli Rehn, asks to push on disposal and spending review.', 'Commissioner UE, Olli Rehn, caused the hypothesis that Italy can obtain more flexibility on budgetary rules.', 'Obtaining flexibility on budgetary rules is an indispensable condition for freeing resources to be allocated to investments.', 'On 2014-01-17, there was a breakfast between Commissioner UE and the Minister of the Economy, Fabrizio Saccomanni.', 'The UE is reviewing the calculation of the GDP.', 'The UE is moving investments in research and development from the expenditure box (a liability) to the investments category.', 'The benefit of the GDP calculation review is expected to be between 1% and 2%.', 'The benefit will have non-negligible effects on the deficit-PIL ratio.', "The document of the banca d'italia remains anchored only on the technical-analytic ground.", "The macro projections developed by the banca d'italia place the year-end GDP growth at 0.7%.", "The banca d'italia's estimates are smaller than the government's estimates for year-end GDP growth.", 'The unemployment rate will rise to 12.9% in 2015.', "The banca d'italia warns that only the recovery of domestic demand will extend the recovery to the labor market.", 'Risks to growth remain downward-oriented.', 'The recovery of investment may be delayed if conditions for access to credit remain restrictive longer than expected.', 'The risk of general deflation is judged to be moderate.', 'The fall in inflation could be more pronounced and persistent than expected.', 'The confidence of the enterprises is improving.', 'Industrial activity is picking up breath after being diminished from summer of 2011.', 'Small enterprises, especially in the south, remain on the margins of the process.', 'The decline in consumption of families diminished in the third quarter of 2013.', 'Italians do not spend on 2014-01-18.', 'Consumption is restrained by the weakness of disposable income.', 'Consumption is restrained by difficult labor market conditions.', "The banca d'italia notes that the recovery of trust since the beginning of 2013 was interrupted in the fourth quarter.", "The banca d'italia changed its internal organization.", "The banca d'italia's internal organization includes 8 departments, services, and divisions under the Directory."]</t>
         </is>
       </c>
     </row>
@@ -738,17 +738,17 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>the optimism on 20 September last, on these pages, the managing director of bench bpm, juseppe chestnut, had said confidently about the holding of the recovery phase. "We," said chestnut referring to moratorias, "we have fallen from over 16 billion euros to 4.8 billion euros, which means that customers have resumed to repay the loans. almost 75% of the customers exposed to those 4.8 billion have good ratings and we are confident. are very comforting data. but despite the optimism of chestnut, the concern for the maintenance of the system is concrete. While it is true that moratorium credits increased from 280 billion in March 2020 to 147 billion in December 2020 to 71 billion in September 2021, the deadline for support measures is seen as the real great test for the Italian economy, which today sees GDP growing to over 6% per annum, but which has to face this curve by elbow. The first half of 2022 seems thus destined to bring to the surface what has been kept aside so far. This is a happy moment for the Italian economy - explains ferrara ferruccio, founder and president of negentropy capital partners, who signed together with pimco and deutsche bank one of the very first transactions of acquisition of bad debts in the distant 2011 -. After very heavy months, the bouncing is bringing back optimism and this is a fantastic medicine for the economy. But the time will soon come when we will have to deal with the past and for businesses to resume payments due to banks and now in moratorium. there are different reactivitys depending on the industrial sectors, but the underlying condition remains fairly heavy. also because Italy has reached the pandemic with a complicated financial situation and a fractional growth compared to the major European competitors, this should not be forgotten. the covid has lengthened the times of recovery and it is undeniable that in the last eighteen months the bank exposures have increased. Today, in Italy, the total amount of non-performing loans, i.e. the sum of npl and utp, whose distinction is however very thin and often depends on bank to bank, is around € 500 billion in total. This is a very considerable figure, which makes Italy the first European market for this type of position, one of the world's first. of these 500 billion, about 180 billion are utp and about 120 billion are the npl still within the banking perimeters. The remaining 200 billion have not disappeared. have emerged from the perimeter of the banks and therefore no longer represent a structural theme for the credit industry, burdened also by the needs imposed by the calendar provisioning, but they are in the portfolios of specialized funds. From the point of view of the Italian economy, however, little change... in 2021 the value of the portfolios sold by the banks will be about 34 billion (1.5 billion only from mps if the transfer to unicredit were to take place), increasing in 2020, as well as the utp, which will reach 11 billion. from here to the end of the year they are ready to be sold npl for 26 billion. last month, bank ifis in the usual September report on the sector, wrote: "in the two-year period 2022-2023 the new credit deteriorated on households and resident companies is expected to grow (about 70 billion euros in the two years), without however reaching the peak of 2013. the increase in the rate of deterioration will be driven by the enterprise component but the bank led by Frederick geertman has also emphasized the positive effect of the measures of the government: in 2021 the stock of the credits deteriorated gross is previewed in contraction. This will reduce the npe ratio below the target by 5% as required by the bce. The impact on employment is expected to increase from 2022 and will reach 5.9% in 2023 , when the protection network laid down by the executive will now be put behind it. on the market for bad loans, an important role is played by the public hand, both through the subsidiary amco and through the gacs, the public guarantees on the securitisation of suffering, introduced by a decree of February 2016 several times, extended. On the basis of the further 12-month extension granted by the European Union in 2021, bank ifis expects approximately €7 billion of new guaranteed transactions, bringing the total transaction since 2016 to €94 billion. seven services engaged in operations assisted by gacs so far, with 80% of the value, i.e. the gross book value (gBV), the gross book value, concentrated among the top four Italian operators: dovalue, prelios, cerved and land credit. the operators are the attention of the operators on the Italian market is very high - emphasizes ferrara, that with negentropy controls portfolios for approximately 3 billion euros of gbv - and it demonstrates the fact that today when a credit institution places for sale one of its assets are up to 25-30 the operators invited to participate to the purchase. the increase in the number of operators has also led to an upward revision of prices: to make room among many competitors there are those who have bought at very aggressive levels in the past and the increase in the average value of transactions has done well to the bank's balance sheets. Now it remains to understand what 2022 will be like, but it is difficult to predict: I hope that support for the business system will be abandoned only gradually, this would help to maintain the sectors most exposed so far such as manufacturing, fashion, tourism and catering. the system of loans and loans is based on real guarantees, in the vast majority of cases, real estate. again in this case the covid has left its mark: in 2021 125 thousand judicial auctions are estimated in Italy, a decrease of 39 percent compared to before the pandemic. the courts have suspended over 120 thousand auctions and result in operations of at least 13 billion euros blocked in the courtrooms. even these waiting for the restart. © Reserved reproduction npl with this acronym means non-performing loans , i.e. non-performing loans, impaired loans. i.e., loans that are not repaid to banks by companies, which thus are in default utp under the terms unlikely to pay (utp) are the probable defaults, i.e. exposures for which the bank is unlikely to fully fulfil its contractual obligations past two, are exposures or payments that have expired or are insurmountable over a period of more than 90 days. It is the first step of the crisis, which can evolve in car and then in npl</t>
+          <t>the optimism on 20 September last, on these pages, the managing director of bench bpm, giuseppe castagna, had said confidently about the holding of the recovery phase. "We," said chestnut referring to moratorias, "we have fallen from over 16 billion euros to 4.8 billion euros, which means that customers have resumed to repay the loans. almost 75% of the customers exposed to those 4.8 billion have good ratings and we are confident. are very comforting data. but despite the optimism of chestnut, the concern for the maintenance of the system is concrete. While it is true that moratorium credits increased from 280 billion in March 2020 to 147 billion in December 2020 to 71 billion in September 2021, the deadline for support measures is seen as the real great test for the Italian economy, which today sees GDP growing to over 6% per annum, but which has to face this curve by elbow. The first half of 2022 seems thus destined to bring to the surface what has been kept aside so far. This is a happy moment for the Italian economy - explains ferruccio ferrara, founder and president of negentropy capital partners, who signed together with pimco and deutsche bank one of the very first transactions of acquisition of bad loans in the distant 2011 -. After very heavy months, the bouncing is bringing back optimism and this is a fantastic medicine for the economy. But the time will soon come when we will have to deal with the past and for businesses to resume payments due to banks and now in moratorium. there are different reactivitys depending on the industrial sectors, but the underlying condition remains fairly heavy. also because Italy has reached the pandemic with a complicated financial situation and a fractional growth compared to the major European competitors, this should not be forgotten. the covid has lengthened the recovery times and it is undeniable that in the last eighteen months the bank exposures have increased. Today, in Italy, the total amount of non-performing loans, i.e. the sum of npl and utp, whose distinction is however very thin and often depends on bank to bank, is around € 500 billion in total. This is a very considerable figure, which makes Italy the first European market for this type of position, one of the world's first. of these 500 billion, about 180 billion are utp and about 120 billion are the npl still within the banking perimeters. The remaining 200 billion have not disappeared. have emerged from the perimeter of the banks and therefore no longer represent a structural theme for the credit industry, burdened also by the needs imposed by the calendar provisioning, but they are in the portfolios of specialized funds. From the point of view of the Italian economy, however, little change... in 2021 the value of the portfolios sold by the banks will be about 34 billion (1.5 billion only from mps if the transfer to unicredit were to take place), increasing in 2020, as well as the utp, which will reach 11 billion. from here to the end of the year they are ready to be sold npl for 26 billion. last month, bank ifis in the usual September report on the sector, wrote: "in the two-year period 2022-2023 the new credit deteriorated on households and resident companies is expected to grow (about 70 billion euros in the two years), without however reaching the peak of 2013. the increase in the rate of deterioration will be driven by the enterprise component but the bank led by frederick geertman has also emphasized the positive effect of the measures of the government: in 2021 the stock of the credits deteriorated gross is previewed in contraction. This will reduce the npe ratio below the target by 5% as required by the bce. The impact on employment is expected to increase from 2022 and will reach 5.9% in 2023 , when the protection network laid down by the executive will now be put behind it. on the market for bad loans, an important role is played by the public hand, both through the subsidiary amco and through the gacs, the public guarantees on the securitisation of suffering, introduced by a decree of February 2016 several times, extended. On the basis of the further extension of 12 months granted by unione europea during 2021, bank ifis expects approximately 7 billion euros of new guaranteed transactions, bringing to 94 billion euros the total transaction since 2016. seven services engaged in operations assisted by gacs so far, with 80% of the value, i.e. gross book value (gBV), the gross book value, concentrated among the first four Italian operators: dovalue, prelios, cerved and land credit. the operators are the attention of the operators on the Italian market is very high - emphasizes ferrara, that with negentropy controls portfolios for approximately 3 billion euros of gbv - and it demonstrates the fact that today when a credit institution places for sale one of its assets are up to 25-30 the operators invited to participate to the purchase. the increase in the number of operators has also led to an upward revision of prices: to make room among many competitors there are those who have bought at very aggressive levels in the past and the increase in the average value of transactions has done well to the bank's balance sheets. Now it remains to understand what 2022 will be like, but it is difficult to predict: I hope that support for the business system will be abandoned only gradually, this would help to maintain the sectors most exposed so far such as manufacturing, fashion, tourism and catering. the system of loans and loans is based on real guarantees, in the vast majority of cases, real estate. again in this case the covid has left its mark: in 2021 125 thousand judicial auctions are estimated in Italy, a decrease of 39 percent compared to before the pandemic. the courts have suspended over 120 thousand auctions and result in operations of at least 13 billion euros blocked in the courtrooms. even these waiting for the restart. © Reserved reproduction npl with this acronym means non-performing loans , i.e. non-performing loans, impaired loans. i.e., loans that are not repaid to banks by companies, which thus are in default utp under the terms unlikely to pay (utp) are the probable defaults, i.e. exposures for which the bank is unlikely to fully fulfil its contractual obligations past two, are exposures or payments that have expired or are insurmountable over a period of more than 90 days. It is the first step of the crisis, which can evolve in car and then in npl</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>Observation date: 2021-10-18 00:00:00. the optimism on 20 September last, on these pages, the managing director of bench bpm, juseppe chestnut, had said confidently about the holding of the recovery phase. "We," said chestnut referring to moratorias, "we have fallen from over 16 billion euros to 4.8 billion euros, which means that customers have resumed to repay the loans. almost 75% of the customers exposed to those 4.8 billion have good ratings and we are confident. are very comforting data. but despite the optimism of chestnut, the concern for the maintenance of the system is concrete. While it is true that moratorium credits increased from 280 billion in March 2020 to 147 billion in December 2020 to 71 billion in September 2021, the deadline for support measures is seen as the real great test for the Italian economy, which today sees GDP growing to over 6% per annum, but which has to face this curve by elbow. The first half of 2022 seems thus destined to bring to the surface what has been kept aside so far. This is a happy moment for the Italian economy - explains ferrara ferruccio, founder and president of negentropy capital partners, who signed together with pimco and deutsche bank one of the very first transactions of acquisition of bad debts in the distant 2011 -. After very heavy months, the bouncing is bringing back optimism and this is a fantastic medicine for the economy. But the time will soon come when we will have to deal with the past and for businesses to resume payments due to banks and now in moratorium. there are different reactivitys depending on the industrial sectors, but the underlying condition remains fairly heavy. also because Italy has reached the pandemic with a complicated financial situation and a fractional growth compared to the major European competitors, this should not be forgotten. the covid has lengthened the times of recovery and it is undeniable that in the last eighteen months the bank exposures have increased. Today, in Italy, the total amount of non-performing loans, i.e. the sum of npl and utp, whose distinction is however very thin and often depends on bank to bank, is around € 500 billion in total. This is a very considerable figure, which makes Italy the first European market for this type of position, one of the world's first. of these 500 billion, about 180 billion are utp and about 120 billion are the npl still within the banking perimeters. The remaining 200 billion have not disappeared. have emerged from the perimeter of the banks and therefore no longer represent a structural theme for the credit industry, burdened also by the needs imposed by the calendar provisioning, but they are in the portfolios of specialized funds. From the point of view of the Italian economy, however, little change... in 2021 the value of the portfolios sold by the banks will be about 34 billion (1.5 billion only from mps if the transfer to unicredit were to take place), increasing in 2020, as well as the utp, which will reach 11 billion. from here to the end of the year they are ready to be sold npl for 26 billion. last month, bank ifis in the usual September report on the sector, wrote: "in the two-year period 2022-2023 the new credit deteriorated on households and resident companies is expected to grow (about 70 billion euros in the two years), without however reaching the peak of 2013. the increase in the rate of deterioration will be driven by the enterprise component but the bank led by Frederick geertman has also emphasized the positive effect of the measures of the government: in 2021 the stock of the credits deteriorated gross is previewed in contraction. This will reduce the npe ratio below the target by 5% as required by the bce. The impact on employment is expected to increase from 2022 and will reach 5.9% in 2023 , when the protection network laid down by the executive will now be put behind it. on the market for bad loans, an important role is played by the public hand, both through the subsidiary amco and through the gacs, the public guarantees on the securitisation of suffering, introduced by a decree of February 2016 several times, extended. On the basis of the further 12-month extension granted by the European Union in 2021, bank ifis expects approximately €7 billion of new guaranteed transactions, bringing the total transaction since 2016 to €94 billion. seven services engaged in operations assisted by gacs so far, with 80% of the value, i.e. the gross book value (gBV), the gross book value, concentrated among the top four Italian operators: dovalue, prelios, cerved and land credit. the operators are the attention of the operators on the Italian market is very high - emphasizes ferrara, that with negentropy controls portfolios for approximately 3 billion euros of gbv - and it demonstrates the fact that today when a credit institution places for sale one of its assets are up to 25-30 the operators invited to participate to the purchase. the increase in the number of operators has also led to an upward revision of prices: to make room among many competitors there are those who have bought at very aggressive levels in the past and the increase in the average value of transactions has done well to the bank's balance sheets. Now it remains to understand what 2022 will be like, but it is difficult to predict: I hope that support for the business system will be abandoned only gradually, this would help to maintain the sectors most exposed so far such as manufacturing, fashion, tourism and catering. the system of loans and loans is based on real guarantees, in the vast majority of cases, real estate. again in this case the covid has left its mark: in 2021 125 thousand judicial auctions are estimated in Italy, a decrease of 39 percent compared to before the pandemic. the courts have suspended over 120 thousand auctions and result in operations of at least 13 billion euros blocked in the courtrooms. even these waiting for the restart. © Reserved reproduction npl with this acronym means non-performing loans , i.e. non-performing loans, impaired loans. i.e., loans that are not repaid to banks by companies, which thus are in default utp under the terms unlikely to pay (utp) are the probable defaults, i.e. exposures for which the bank is unlikely to fully fulfil its contractual obligations past two, are exposures or payments that have expired or are insurmountable over a period of more than 90 days. It is the first step of the crisis, which can evolve in car and then in npl</t>
+          <t>Observation date: 2021-10-18 00:00:00. the optimism on 20 September last, on these pages, the managing director of bench bpm, giuseppe castagna, had said confidently about the holding of the recovery phase. "We," said chestnut referring to moratorias, "we have fallen from over 16 billion euros to 4.8 billion euros, which means that customers have resumed to repay the loans. almost 75% of the customers exposed to those 4.8 billion have good ratings and we are confident. are very comforting data. but despite the optimism of chestnut, the concern for the maintenance of the system is concrete. While it is true that moratorium credits increased from 280 billion in March 2020 to 147 billion in December 2020 to 71 billion in September 2021, the deadline for support measures is seen as the real great test for the Italian economy, which today sees GDP growing to over 6% per annum, but which has to face this curve by elbow. The first half of 2022 seems thus destined to bring to the surface what has been kept aside so far. This is a happy moment for the Italian economy - explains ferruccio ferrara, founder and president of negentropy capital partners, who signed together with pimco and deutsche bank one of the very first transactions of acquisition of bad loans in the distant 2011 -. After very heavy months, the bouncing is bringing back optimism and this is a fantastic medicine for the economy. But the time will soon come when we will have to deal with the past and for businesses to resume payments due to banks and now in moratorium. there are different reactivitys depending on the industrial sectors, but the underlying condition remains fairly heavy. also because Italy has reached the pandemic with a complicated financial situation and a fractional growth compared to the major European competitors, this should not be forgotten. the covid has lengthened the recovery times and it is undeniable that in the last eighteen months the bank exposures have increased. Today, in Italy, the total amount of non-performing loans, i.e. the sum of npl and utp, whose distinction is however very thin and often depends on bank to bank, is around € 500 billion in total. This is a very considerable figure, which makes Italy the first European market for this type of position, one of the world's first. of these 500 billion, about 180 billion are utp and about 120 billion are the npl still within the banking perimeters. The remaining 200 billion have not disappeared. have emerged from the perimeter of the banks and therefore no longer represent a structural theme for the credit industry, burdened also by the needs imposed by the calendar provisioning, but they are in the portfolios of specialized funds. From the point of view of the Italian economy, however, little change... in 2021 the value of the portfolios sold by the banks will be about 34 billion (1.5 billion only from mps if the transfer to unicredit were to take place), increasing in 2020, as well as the utp, which will reach 11 billion. from here to the end of the year they are ready to be sold npl for 26 billion. last month, bank ifis in the usual September report on the sector, wrote: "in the two-year period 2022-2023 the new credit deteriorated on households and resident companies is expected to grow (about 70 billion euros in the two years), without however reaching the peak of 2013. the increase in the rate of deterioration will be driven by the enterprise component but the bank led by frederick geertman has also emphasized the positive effect of the measures of the government: in 2021 the stock of the credits deteriorated gross is previewed in contraction. This will reduce the npe ratio below the target by 5% as required by the bce. The impact on employment is expected to increase from 2022 and will reach 5.9% in 2023 , when the protection network laid down by the executive will now be put behind it. on the market for bad loans, an important role is played by the public hand, both through the subsidiary amco and through the gacs, the public guarantees on the securitisation of suffering, introduced by a decree of February 2016 several times, extended. On the basis of the further extension of 12 months granted by unione europea during 2021, bank ifis expects approximately 7 billion euros of new guaranteed transactions, bringing to 94 billion euros the total transaction since 2016. seven services engaged in operations assisted by gacs so far, with 80% of the value, i.e. gross book value (gBV), the gross book value, concentrated among the first four Italian operators: dovalue, prelios, cerved and land credit. the operators are the attention of the operators on the Italian market is very high - emphasizes ferrara, that with negentropy controls portfolios for approximately 3 billion euros of gbv - and it demonstrates the fact that today when a credit institution places for sale one of its assets are up to 25-30 the operators invited to participate to the purchase. the increase in the number of operators has also led to an upward revision of prices: to make room among many competitors there are those who have bought at very aggressive levels in the past and the increase in the average value of transactions has done well to the bank's balance sheets. Now it remains to understand what 2022 will be like, but it is difficult to predict: I hope that support for the business system will be abandoned only gradually, this would help to maintain the sectors most exposed so far such as manufacturing, fashion, tourism and catering. the system of loans and loans is based on real guarantees, in the vast majority of cases, real estate. again in this case the covid has left its mark: in 2021 125 thousand judicial auctions are estimated in Italy, a decrease of 39 percent compared to before the pandemic. the courts have suspended over 120 thousand auctions and result in operations of at least 13 billion euros blocked in the courtrooms. even these waiting for the restart. © Reserved reproduction npl with this acronym means non-performing loans , i.e. non-performing loans, impaired loans. i.e., loans that are not repaid to banks by companies, which thus are in default utp under the terms unlikely to pay (utp) are the probable defaults, i.e. exposures for which the bank is unlikely to fully fulfil its contractual obligations past two, are exposures or payments that have expired or are insurmountable over a period of more than 90 days. It is the first step of the crisis, which can evolve in car and then in npl</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>['On 2021-09-20, Giuseppe Chestnut, managing director of Bench BPM, stated that moratorium loans fell from over 16 billion euros to 4.8 billion euros.', 'Giuseppe Chestnut stated that almost 75% of the customers exposed to the 4.8 billion euros have good ratings.', 'Moratorium credits increased from 280 billion euros in March 2020 to 147 billion euros in December 2020.', 'Moratorium credits decreased to 71 billion euros in September 2021.', 'The Italian economy sees GDP growing to over 6% per annum on 2021-10-18.', 'Ferrara Ferruccio, founder and president of Negentropy Capital Partners, signed one of the first transactions of acquisition of bad debts with Pimco and Deutsche Bank in 2011.', 'The COVID-19 pandemic lengthened the times of recovery.', 'Bank exposures increased in the 18 months leading up to 2021-10-18.', 'The total amount of non-performing loans (NPL) and unprovisioned troubled payments (UTP) in Italy is around 500 billion euros on 2021-10-18.', 'Of the 500 billion euros in Italy, about 180 billion euros are UTP.', 'Of the 500 billion euros in Italy, about 120 billion euros are NPL still within the banking perimeters.', 'The remaining 200 billion euros have emerged from the perimeter of the banks and are held in specialized funds.', 'In 2021, the value of the portfolios sold by the banks was about 34 billion euros.', 'The value of the UTP reached 11 billion euros in 2021.', 'Banks are ready to sell NPL for 26 billion euros from 2021-10-18 to the end of the year.', 'Bank Ifis, in its September report, predicted that new credit deteriorated on households and resident companies would grow by about 70 billion euros between 2022 and 2023.', 'Bank Ifis noted that the increase in the rate of deterioration would be driven by the enterprise component.', 'Bank Ifis predicted that the stock of the credits deteriorated gross would contract in 2021.', 'The contraction of the stock of the credits deteriorated gross in 2021 will reduce the NPE ratio below the target by 5% as required by the BCE.', 'The impact on employment is expected to increase from 2022.', 'The public hand plays an important role in the bad loans market through AMCO and GACS.', 'GACS, the public guarantees on the securitization of suffering, was introduced by a decree of February 2016.', 'The European Union granted a further 12-month extension for GACS in 2021.', 'Bank Ifis expects approximately 7 billion euros of new guaranteed transactions based on the GACS extension.', 'The total transaction value assisted by GACS since 2016 is expected to reach 94 billion euros.', 'The top four Italian operators concentrating the GACS gross book value are Dovale, Prelios, Cerved, and Land Credit.', 'Ferrara emphasized that Negentropy controls portfolios for approximately 3 billion euros of GBV.', 'When a credit institution places an asset for sale, up to 25-30 operators are invited to participate in the purchase.', 'The increase in the number of operators led to an upward revision of prices in the bad loans market.', 'In 2021, 125 thousand judicial auctions were estimated in Italy.', 'The number of judicial auctions in 2021 decreased by 39 percent compared to the pre-pandemic period.', 'The courts suspended over 120 thousand auctions.', 'The suspended auctions resulted in operations of at least 13 billion euros blocked in the courtrooms.']</t>
+          <t>['On 2021-10-18, Giuseppe Castagna, managing director of Bench BPM, expressed optimism about the holding of the recovery phase on 2021-09-20.', 'Chestnut stated that the amount fell from over 16 billion euros to 4.8 billion euros.', 'Chestnut stated that almost 75% of customers exposed to 4.8 billion euros have good ratings.', 'Moratorium credits increased from 280 billion euros in March 2020 to 147 billion euros in December 2020.', 'Moratorium credits decreased to 71 billion euros in September 2021.', 'The Italian economy sees GDP growing to over 6% per annum on 2021-10-18.', 'Ferruccio Ferrara, founder and president of Negentropy Capital Partners, signed one of the first transactions of acquisition of bad loans with Pimco and Deutsche Bank in 2011.', 'The COVID-19 pandemic lengthened recovery times.', 'Bank exposures increased in the eighteen months preceding 2021-10-18.', 'The total amount of non-performing loans (NPL) and utp in Italy is around € 500 billion on 2021-10-18.', 'Of the 500 billion euros in non-performing loans and utp, about 180 billion euros are utp.', 'Of the 500 billion euros, about 120 billion euros are NPL still within the banking perimeters.', 'The remaining 200 billion euros have emerged from the perimeter of the banks and are held in specialized funds.', 'In 2021, the value of portfolios sold by the banks is projected to be about 34 billion euros.', 'The value of utp is projected to reach 11 billion euros in 2021.', 'Banks are ready to sell NPL for 26 billion euros from 2021-10-18 to the end of the year.', 'Bank Ifis, in its September report, predicted that new credit deteriorated on households and resident companies would grow by about 70 billion euros between 2022 and 2023.', 'The bank led by Frederick Geertman predicted that the stock of credits deteriorated gross would contract in 2021.', 'This contraction is expected to reduce the NPE ratio below the target by 5% as required by the BCE.', 'The impact on employment is expected to increase from 2022.', 'The public hand plays an important role in the bad loans market through the subsidiary AMCO and through GACS.', 'GACS are public guarantees on the securitization of suffering, introduced by a decree in February 2016.', 'Bank Ifis expects approximately 7 billion euros of new guaranteed transactions based on a 12-month extension granted by the European Union during 2021.', 'The total transaction amount since 2016 is expected to reach 94 billion euros.', 'Seven services have been engaged in operations assisted by GACS.', '80% of the gross book value (gBV) of these operations is concentrated among the first four Italian operators: Dovale, Prelios, Cerved, and Land Credit.', 'Ferraara emphasized that Negentropy controls portfolios for approximately 3 billion euros of gBV.', 'When a credit institution places an asset for sale, up to 25-30 operators are invited to participate in the purchase.', 'The increase in the number of operators led to an upward revision of prices.', 'In 2021, 125 thousand judicial auctions are estimated in Italy.', 'The number of judicial auctions in 2021 represents a 39 percent decrease compared to the pre-pandemic period.', 'The courts suspended over 120 thousand auctions, resulting in operations of at least 13 billion euros blocked in the courtrooms.']</t>
         </is>
       </c>
     </row>
@@ -802,17 +802,17 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>. not within the scope of the measure but on the manner in which it is granted. there is a letter to be sent: 1 sheet (plus envelope). an application is made: 4 sheets. the instructions: 2 sheets. photocopies to be attached to the application: 2 sheets (or 4 if necessary delegation). In the best case for each application, at least 9 sheets (plus envelope) will be used, multiplied by the estimated population of 1.300,000, making 11,700,000 sheets ( Eleven million and seven hundred thousand sheets) which, to give an idea, are equal to 23,400 rismes of paper of 500 sheets. I forgot the 1,300,000 bags. I wonder, but has the Ministry of Simplification not been established? the deductions lost on building renovations claudia ceroni roma dazzled by an increase in VAT on an unnecessary asset (sky) is neglecting a much more serious problem than the new decree launched on Friday. I am 30 years old, I am a construction engineer, in light of the incentives we knew to be certain I convinced my parents to intervene on their home improving the insulation of the roof and installing sanitary panels for sanitary use, condensing boiler, thermostatic valves, for a total of about 10,000 euros. along with my boyfriend we spent about 50,000 euros in additional insulation of the roof and fixtures that meet the energy efficiency requirements, for our new home, spending about 50,000 euros additional, with the belief that you could access the deduction. This deduction no longer exists, or at least it is not certain or will be reduced from 55% at present to 35%. I would like our Minister Tremonti and the staff of the President of the Council to answer these two simple questions: who will repay us for this non-refund that, at the time of the intervention, was considered certain? I believe that we are not very far from a scam, if by it we mean what is quoted by the demaur: "made committed by those who make illicit profits to the detriment of others, having misled them with artifices and tricks." It is enough to replace artificial and defrauded by laws and decrees, which makes the fact even more serious. the 4% rate on loans fixed by the Government of Luciano at paola lux101065@hotmail.com in the government's maneuver is expected that, for 2009, the interest rate on variable rate loans will not exceed 4%. Damn it! Even a far-left government wouldn't have thought that. Mr Boeri, in the newspaper at the newsstands yesterday, wonders (rhetorically I presume) why such a measure is not also envisaged for fixed rate loans. simply because with the next cut of the bce rate to 2.75%, if not less, the euribor will initially quota little more than 3%, added an average spread of 1%, and here is that 4% will be the rate that the banks will have to apply on the loans at variable rate. benefit for families virtually zero. If we apply the principle also to fixed-rate loans with interest rates well above 4%, we would run the risk of really helping families! If we then consider that in 2009 we could also reach a variable rate of 3.5%. This 4% rate would be a way like another to help those who really need it: banks. the news about the mafias and the choices of the tg1 pine caserta secretary of editorial staff of the tg1 kind director, on page 19 Republic of yesterday headlines: "for tg1 the yo-yo most important of the fight against crime" because the tg1 did not give account, in the edition of the 20 of Saturday, of the review on the fight against the mafias organized by 'politically incorrect' to reindeer housewife (bologna). the meeting was certainly relevant but, to see, also the national edition of your newspaper decided not to give news of the convention on mafias. Republic has limited itself to bringing back the protest of rita purse. What the editorial secretary of the tg1 omits to say is that the conference on mafias took place a few hundred meters from the yo-yo championship: this is the reason for the controversy raised by the purse. 2lette_13563977rb1</t>
+          <t>. not within the scope of the measure but on the manner in which it is granted. there is a letter to be sent: 1 sheet (plus envelope). an application is made: 4 sheets. the instructions: 2 sheets. photocopies to be attached to the application: 2 sheets (or 4 if necessary delegation). In the best case for each application, at least 9 sheets (plus envelope) will be used, multiplied by the estimated population of 1.300,000, making 11,700,000 sheets ( Eleven million and seven hundred thousand sheets) which, to give an idea, are equal to 23,400 rismes of paper of 500 sheets. I forgot the 1,300,000 bags. I wonder, but has the Ministry of Simplification not been established? the deductions lost on the construction renovations claudia ceroni roma dazzled by an increase of VAT on an unnecessary asset (sky) is neglecting a much more serious problem than the new decree launched on Friday. I am 30 years old, I am a construction engineer, in light of the incentives we knew to be certain I convinced my parents to intervene on their home improving the insulation of the roof and installing sanitary panels for sanitary use, condensing boiler, thermostatic valves, for a total of about 10,000 euros. along with my boyfriend we spent about 50,000 euros in additional insulation of the roof and fixtures that meet the energy efficiency requirements, for our new home, spending about 50,000 euros additional, with the belief that you could access the deduction. This deduction no longer exists, or at least it is not certain or will be reduced from 55% at present to 35%. I would like our Minister Tremonti and the staff of the President of the Council to answer these two simple questions: who will repay us for this non-refund that, at the time of the intervention, was considered certain? I believe that we are not very far from a scam, if by it we mean what is quoted by the demaur: "made committed by those who make illicit profits to the detriment of others, having misled them with artifices and tricks." It is enough to replace artificial and defrauded by laws and decrees, which makes the fact even more serious. the 4% interest rate on loans fixed by the Government of paola lux101065@hotmail.com in the government's manoeuvre is expected that the interest rate on variable rate loans will not exceed 4% in 2009. Damn it! Even a far-left government wouldn't have thought that. tito boeri, in the newspaper at the newsstands yesterday, is asked (retorically I presume) why this measure is not also provided for fixed rate loans. simply because with the next cut of the bce rate to 2.75%, if not less, the euribor will initially quota little more than 3%, added an average spread of 1%, and here is that 4% will be the rate that the banks will have to apply on the loans at variable rate. benefit for families virtually zero. If we apply the principle also to fixed-rate loans with interest rates well above 4%, we would run the risk of really helping families! If we then consider that in 2009 we could also reach a variable rate of 3.5%. This 4% rate would be a way like another to help those who really need it: banks. the news about the mafias and the choices of the tg1 pine caserta secretary of editorial staff of the tg1 kind director, on page 19 Republic of yesterday headlines: "for tg1 the yo-yo most important of the fight against crime" because the tg1 did not give account, in the edition of the 20 of Saturday, of the review on the fight against the mafias organized by 'politically incorrect' to reindeer housewife (bologna). the meeting was certainly relevant but, to see, also the national edition of your newspaper decided not to give news of the convention on mafias. Republic limited itself to reporting the protest of rita borsellino. What the editorial secretary of the tg1 omits to say is that the conference on mafias took place a few hundred meters from the yo-yo championship: this is the reason for the controversy raised by the purse. 2lette_13563977rb1</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>Observation date: 2008-12-02 00:00:00. . not within the scope of the measure but on the manner in which it is granted. there is a letter to be sent: 1 sheet (plus envelope). an application is made: 4 sheets. the instructions: 2 sheets. photocopies to be attached to the application: 2 sheets (or 4 if necessary delegation). In the best case for each application, at least 9 sheets (plus envelope) will be used, multiplied by the estimated population of 1.300,000, making 11,700,000 sheets ( Eleven million and seven hundred thousand sheets) which, to give an idea, are equal to 23,400 rismes of paper of 500 sheets. I forgot the 1,300,000 bags. I wonder, but has the Ministry of Simplification not been established? the deductions lost on building renovations claudia ceroni roma dazzled by an increase in VAT on an unnecessary asset (sky) is neglecting a much more serious problem than the new decree launched on Friday. I am 30 years old, I am a construction engineer, in light of the incentives we knew to be certain I convinced my parents to intervene on their home improving the insulation of the roof and installing sanitary panels for sanitary use, condensing boiler, thermostatic valves, for a total of about 10,000 euros. along with my boyfriend we spent about 50,000 euros in additional insulation of the roof and fixtures that meet the energy efficiency requirements, for our new home, spending about 50,000 euros additional, with the belief that you could access the deduction. This deduction no longer exists, or at least it is not certain or will be reduced from 55% at present to 35%. I would like our Minister Tremonti and the staff of the President of the Council to answer these two simple questions: who will repay us for this non-refund that, at the time of the intervention, was considered certain? I believe that we are not very far from a scam, if by it we mean what is quoted by the demaur: "made committed by those who make illicit profits to the detriment of others, having misled them with artifices and tricks." It is enough to replace artificial and defrauded by laws and decrees, which makes the fact even more serious. the 4% rate on loans fixed by the Government of Luciano at paola lux101065@hotmail.com in the government's maneuver is expected that, for 2009, the interest rate on variable rate loans will not exceed 4%. Damn it! Even a far-left government wouldn't have thought that. Mr Boeri, in the newspaper at the newsstands yesterday, wonders (rhetorically I presume) why such a measure is not also envisaged for fixed rate loans. simply because with the next cut of the bce rate to 2.75%, if not less, the euribor will initially quota little more than 3%, added an average spread of 1%, and here is that 4% will be the rate that the banks will have to apply on the loans at variable rate. benefit for families virtually zero. If we apply the principle also to fixed-rate loans with interest rates well above 4%, we would run the risk of really helping families! If we then consider that in 2009 we could also reach a variable rate of 3.5%. This 4% rate would be a way like another to help those who really need it: banks. the news about the mafias and the choices of the tg1 pine caserta secretary of editorial staff of the tg1 kind director, on page 19 Republic of yesterday headlines: "for tg1 the yo-yo most important of the fight against crime" because the tg1 did not give account, in the edition of the 20 of Saturday, of the review on the fight against the mafias organized by 'politically incorrect' to reindeer housewife (bologna). the meeting was certainly relevant but, to see, also the national edition of your newspaper decided not to give news of the convention on mafias. Republic has limited itself to bringing back the protest of rita purse. What the editorial secretary of the tg1 omits to say is that the conference on mafias took place a few hundred meters from the yo-yo championship: this is the reason for the controversy raised by the purse. 2lette_13563977rb1</t>
+          <t>Observation date: 2008-12-02 00:00:00. . not within the scope of the measure but on the manner in which it is granted. there is a letter to be sent: 1 sheet (plus envelope). an application is made: 4 sheets. the instructions: 2 sheets. photocopies to be attached to the application: 2 sheets (or 4 if necessary delegation). In the best case for each application, at least 9 sheets (plus envelope) will be used, multiplied by the estimated population of 1.300,000, making 11,700,000 sheets ( Eleven million and seven hundred thousand sheets) which, to give an idea, are equal to 23,400 rismes of paper of 500 sheets. I forgot the 1,300,000 bags. I wonder, but has the Ministry of Simplification not been established? the deductions lost on the construction renovations claudia ceroni roma dazzled by an increase of VAT on an unnecessary asset (sky) is neglecting a much more serious problem than the new decree launched on Friday. I am 30 years old, I am a construction engineer, in light of the incentives we knew to be certain I convinced my parents to intervene on their home improving the insulation of the roof and installing sanitary panels for sanitary use, condensing boiler, thermostatic valves, for a total of about 10,000 euros. along with my boyfriend we spent about 50,000 euros in additional insulation of the roof and fixtures that meet the energy efficiency requirements, for our new home, spending about 50,000 euros additional, with the belief that you could access the deduction. This deduction no longer exists, or at least it is not certain or will be reduced from 55% at present to 35%. I would like our Minister Tremonti and the staff of the President of the Council to answer these two simple questions: who will repay us for this non-refund that, at the time of the intervention, was considered certain? I believe that we are not very far from a scam, if by it we mean what is quoted by the demaur: "made committed by those who make illicit profits to the detriment of others, having misled them with artifices and tricks." It is enough to replace artificial and defrauded by laws and decrees, which makes the fact even more serious. the 4% interest rate on loans fixed by the Government of paola lux101065@hotmail.com in the government's manoeuvre is expected that the interest rate on variable rate loans will not exceed 4% in 2009. Damn it! Even a far-left government wouldn't have thought that. tito boeri, in the newspaper at the newsstands yesterday, is asked (retorically I presume) why this measure is not also provided for fixed rate loans. simply because with the next cut of the bce rate to 2.75%, if not less, the euribor will initially quota little more than 3%, added an average spread of 1%, and here is that 4% will be the rate that the banks will have to apply on the loans at variable rate. benefit for families virtually zero. If we apply the principle also to fixed-rate loans with interest rates well above 4%, we would run the risk of really helping families! If we then consider that in 2009 we could also reach a variable rate of 3.5%. This 4% rate would be a way like another to help those who really need it: banks. the news about the mafias and the choices of the tg1 pine caserta secretary of editorial staff of the tg1 kind director, on page 19 Republic of yesterday headlines: "for tg1 the yo-yo most important of the fight against crime" because the tg1 did not give account, in the edition of the 20 of Saturday, of the review on the fight against the mafias organized by 'politically incorrect' to reindeer housewife (bologna). the meeting was certainly relevant but, to see, also the national edition of your newspaper decided not to give news of the convention on mafias. Republic limited itself to reporting the protest of rita borsellino. What the editorial secretary of the tg1 omits to say is that the conference on mafias took place a few hundred meters from the yo-yo championship: this is the reason for the controversy raised by the purse. 2lette_13563977rb1</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>['A letter requires 1 sheet plus an envelope.', 'An application requires 4 sheets.', 'Instructions require 2 sheets.', 'Photocopies attached to the application require 2 sheets (or 4 sheets if necessary delegation).', 'The estimated population is 1,300,000.', 'The minimum sheets used per application is 9 sheets plus an envelope.', 'The total estimated sheets needed is 11,700,000 sheets.', 'The total estimated sheets are equal to 23,400 rismes of paper of 500 sheets.', 'The number of bags forgotten is 1,300,000.', 'Claudia Ceroni in Roma was dazzled by an increase in VAT on an unnecessary asset (sky).', 'The author convinced parents to improve the insulation of the roof and install sanitary panels, condensing boiler, and thermostatic valves for about 10,000 euros.', 'The author and boyfriend spent about 50,000 euros on additional insulation and fixtures for their new home.', 'The deduction for renovations is no longer certain.', 'The deduction rate may be reduced from 55% to 35%.', 'The 4% rate on loans fixed by the Government of Luciano is expected to keep the interest rate on variable rate loans below 4% for 2009.', 'Mr Boeri wrote in the newspaper at the newsstands on 2008-12-01 questioning the lack of a measure for fixed rate loans.', 'The BCE rate cut is expected to bring the Euribor to little more than 3%.', 'The variable rate loan will be 3% (Euribor) plus an average spread of 1%, totaling 4%.', 'The author predicts a variable rate of 3.5% in 2009.', 'The headline on page 19 of Republic of on 2008-12-01 stated that the yo-yo was the most important part of the fight against crime for TG1.', "TG1 did not give account in the edition of the 20 of 2008-11-29 of the review on the fight against the mafias organized by 'politically incorrect' to reindeer housewife (Bologna).", 'The conference on mafias took place a few hundred meters from the yo-yo championship.']</t>
+          <t>['A letter requires 1 sheet plus an envelope.', 'An application requires 4 sheets.', 'The instructions require 2 sheets.', 'Photocopies attached to the application require 2 sheets, or 4 sheets if necessary delegation is required.', 'In the best case for each application, at least 9 sheets plus an envelope will be used.', 'The estimated population is 1,300,000.', 'The total estimated sheets required is 11,700,000 sheets.', 'The total estimated sheets required are equal to 23,400 rismes of paper of 500 sheets.', "The Ministry of Simplification's establishment status is questioned.", 'The increase of VAT on an unnecessary asset (sky) is neglecting a problem more serious than the new decree launched on 2008-11-30.', 'The construction renovations intervention by the parents required approximately 10,000 euros.', 'The additional insulation and fixtures for the new home cost approximately 50,000 euros.', 'The deduction for construction renovations is no longer certain.', 'The deduction percentage may be reduced from 55% to 35%.', 'The 4% interest rate on loans fixed by the Government is expected to keep the interest rate on variable rate loans below 4% in 2009.', 'Tito Boeri was asked in the newspaper at the newsstands on 2008-12-01 why a measure was not provided for fixed rate loans.', "The headline on page 19 of the Republic newspaper on 2008-12-01 stated: 'for tg1 the yo-yo most important of the fight against crime.'", "The TG1 did not give account, in the edition of 2008-12-06, of the review on the fight against the mafias organized by 'politically incorrect' to Reindeer Housewife (Bologna).", 'The conference on mafias took place a few hundred meters from the yo-yo championship.', 'This proximity is the reason for the controversy raised by the purse.']</t>
         </is>
       </c>
     </row>
@@ -866,17 +866,17 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>It says a study of the national consumer union that has lined up the ranking of the cities with the greatest annual increases, drawing up the data from Istat last January. so Perugia and terni end up in the top six of the most expensive cities touching the podium. in particular in Perugia the cost of light and gas has had an increase of 85.8%: while terni stops at 85.4%. a minimum delta between the two capitals indicating that the stag is, in fact, uniform throughout the region. in particular considering how much an Italian family spends on average the Perugia stagata is equal to 1,157 euros on an annual basis; while that for a ternan family is equal to 1,152 euros. a derby that ends substantially in parity (there are only 5 euros of difference) and win it does not lead to carousels or parties with scarves and flags. At national level, however, the survey compares the change in electricity and gas prices over the last 3 years, comparing the free market with the protected market. from June 2021, before the increases taken from July to January 2023, the light of the free market in Italy rose by 248.3% compared to 108.4% of the protected, more than double (+129%), while considering the first useful figure of the gas detected by the Istat, December 2021, the free since then has increased by 141.1% against a decrease of 7.4% of the protected. In 3 years, from January 2020 to January 2023, free light jumped 262,8%, compared to more than 115,8% of the protected market. for electricity, gas and other fuels, item that includes gas, light (free and protected market), diesel for heating and solid fuels, if in Italy the rise in January was 67.3% compared to a year earlier, with a family stag equal on average to 907,50 euros on an annual basis, in some cities it has almost 90 percent. the comparison does not console the fact that Umbria is at the foot of the podium, also because the distance with those who conquer the highest step is reduced. In Alexandria, electricity, gas and diesel costs fly 88.6% on January 2022. the piemonte fills with vercelli that inserts a plus 87,1% and biella with more 86,1%. on the other side of the ranking, the city less tartassata is power with more 35.2%. in second place aosta with more than 50.8%. on the lowest step of the podium of the virtuous cities olbia-temple with more 51%. followed by Napoli (+51.4%), Gorizia (+51.7%), Benevento (+53.1%), seventh caserta (+53.5%), then Avellino (+53.7%) and Trieste (+54.6%). They close the top ten pordenone and udine, ex aequo with +54.7%. the other classifies another study on the price run comes from the office studies of the cgia of mestre which indicates the weight of the purchasing power of the families regarding the inflation that goes in the rush. in the two years 2022-2023 could amount to almost six thousand euros per household the loss of purchasing power in Umbria due to inflation. the estimate is based on data from the Italian bank, Istat and the European Commission. against bank deposits that, at the end of 2021, amounted to 14.5 billion euros, in Umbria in 2022 the estimated loss of purchasing power amounts to 1.2 billion euros while in 2023, complicit in a slowdown in inflation, 885 million euros for a total of 2.1 billion euros. At provincial level the figure of the cgia says that for that of Perugia the loss of purchasing power could amount to beyond 1,6 billion euros (almost 5,746 to family) while in that of terni to 536 million (5,251 to family). Here the gap is more clear than what happens for increases in electricity and gas bills. Blessed luke</t>
+          <t>It says a study of the national consumer union that has lined up the ranking of the cities with the greatest annual increases, drawing up the data from Istat last January. so Perugia and terni end up in the top six of the most expensive cities touching the podium. in particular in Perugia the cost of light and gas has had an increase of 85.8%: while terni stops at 85.4%. a minimum delta between the two capitals indicating that the stag is, in fact, uniform throughout the region. in particular considering how much an Italian family spends on average the Perugia stagata is equal to 1,157 euros on an annual basis; while that for a ternan family is equal to 1,152 euros. a derby that ends substantially in parity (there are only 5 euros of difference) and win it does not lead to carousels or parties with scarves and flags. At national level, however, the survey compares the change in electricity and gas prices over the last 3 years, comparing the free market with the protected market. from June 2021, before the increases taken from July to January 2023, the light of the free market in Italy rose by 248.3% compared to 108.4% of the protected, more than double (+129%), while considering the first useful figure of the gas detected by the Istat, December 2021, the free since then has increased by 141.1% against a decrease of 7.4% of the protected. In 3 years, from January 2020 to January 2023, free light jumped 262,8%, compared to more than 115,8% of the protected market. for electricity, gas and other fuels, item that includes gas, light (free and protected market), diesel for heating and solid fuels, if in Italy the rise in January was 67.3% compared to a year earlier, with a family stag equal on average to 907,50 euros on an annual basis, in some cities it has almost 90 percent. the comparison does not console the fact that Umbria is at the foot of the podium, also because the distance with those who conquer the highest step is reduced. In Alexandria, electricity, gas and diesel costs fly 88.6% on January 2022. the piemonte fills with vercelli that inserts a plus 87,1% and biella with more 86,1%. on the other side of the ranking, the city less tartassata is power with more 35.2%. in second place aosta with more than 50.8%. on the lowest step of the podium of the virtuous cities olbia-temple with more 51%. followed by Napoli (+51.4%), Gorizia (+51.7%), Benevento (+53.1%), seventh caserta (+53.5%), then Avellino (+53.7%) and Trieste (+54.6%). They close the top ten pordenone and udine, ex aequo with +54.7%. the other classifies another study on the price run comes from the office studies of the cgia of mestre which indicates the weight of the purchasing power of the families regarding the inflation that goes in the rush. in the two years 2022-2023 could amount to almost six thousand euros per household the loss of purchasing power in Umbria due to inflation. the estimate is based on the data of banca d'italia, istat and commissione europea. against bank deposits that, at the end of 2021, amounted to 14.5 billion euros, in Umbria in 2022 the estimated loss of purchasing power amounts to 1.2 billion euros while in 2023, complicit in a slowdown in inflation, 885 million euros for a total of 2.1 billion euros. At provincial level the figure of the cgia says that for that of Perugia the loss of purchasing power could amount to beyond 1,6 billion euros (almost 5,746 to family) while in that of terni to 536 million (5,251 to family). Here the gap is more clear than what happens for increases in electricity and gas bills. luca benedetti</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>Observation date: 2023-02-26 00:00:00. It says a study of the national consumer union that has lined up the ranking of the cities with the greatest annual increases, drawing up the data from Istat last January. so Perugia and terni end up in the top six of the most expensive cities touching the podium. in particular in Perugia the cost of light and gas has had an increase of 85.8%: while terni stops at 85.4%. a minimum delta between the two capitals indicating that the stag is, in fact, uniform throughout the region. in particular considering how much an Italian family spends on average the Perugia stagata is equal to 1,157 euros on an annual basis; while that for a ternan family is equal to 1,152 euros. a derby that ends substantially in parity (there are only 5 euros of difference) and win it does not lead to carousels or parties with scarves and flags. At national level, however, the survey compares the change in electricity and gas prices over the last 3 years, comparing the free market with the protected market. from June 2021, before the increases taken from July to January 2023, the light of the free market in Italy rose by 248.3% compared to 108.4% of the protected, more than double (+129%), while considering the first useful figure of the gas detected by the Istat, December 2021, the free since then has increased by 141.1% against a decrease of 7.4% of the protected. In 3 years, from January 2020 to January 2023, free light jumped 262,8%, compared to more than 115,8% of the protected market. for electricity, gas and other fuels, item that includes gas, light (free and protected market), diesel for heating and solid fuels, if in Italy the rise in January was 67.3% compared to a year earlier, with a family stag equal on average to 907,50 euros on an annual basis, in some cities it has almost 90 percent. the comparison does not console the fact that Umbria is at the foot of the podium, also because the distance with those who conquer the highest step is reduced. In Alexandria, electricity, gas and diesel costs fly 88.6% on January 2022. the piemonte fills with vercelli that inserts a plus 87,1% and biella with more 86,1%. on the other side of the ranking, the city less tartassata is power with more 35.2%. in second place aosta with more than 50.8%. on the lowest step of the podium of the virtuous cities olbia-temple with more 51%. followed by Napoli (+51.4%), Gorizia (+51.7%), Benevento (+53.1%), seventh caserta (+53.5%), then Avellino (+53.7%) and Trieste (+54.6%). They close the top ten pordenone and udine, ex aequo with +54.7%. the other classifies another study on the price run comes from the office studies of the cgia of mestre which indicates the weight of the purchasing power of the families regarding the inflation that goes in the rush. in the two years 2022-2023 could amount to almost six thousand euros per household the loss of purchasing power in Umbria due to inflation. the estimate is based on data from the Italian bank, Istat and the European Commission. against bank deposits that, at the end of 2021, amounted to 14.5 billion euros, in Umbria in 2022 the estimated loss of purchasing power amounts to 1.2 billion euros while in 2023, complicit in a slowdown in inflation, 885 million euros for a total of 2.1 billion euros. At provincial level the figure of the cgia says that for that of Perugia the loss of purchasing power could amount to beyond 1,6 billion euros (almost 5,746 to family) while in that of terni to 536 million (5,251 to family). Here the gap is more clear than what happens for increases in electricity and gas bills. Blessed luke</t>
+          <t>Observation date: 2023-02-26 00:00:00. It says a study of the national consumer union that has lined up the ranking of the cities with the greatest annual increases, drawing up the data from Istat last January. so Perugia and terni end up in the top six of the most expensive cities touching the podium. in particular in Perugia the cost of light and gas has had an increase of 85.8%: while terni stops at 85.4%. a minimum delta between the two capitals indicating that the stag is, in fact, uniform throughout the region. in particular considering how much an Italian family spends on average the Perugia stagata is equal to 1,157 euros on an annual basis; while that for a ternan family is equal to 1,152 euros. a derby that ends substantially in parity (there are only 5 euros of difference) and win it does not lead to carousels or parties with scarves and flags. At national level, however, the survey compares the change in electricity and gas prices over the last 3 years, comparing the free market with the protected market. from June 2021, before the increases taken from July to January 2023, the light of the free market in Italy rose by 248.3% compared to 108.4% of the protected, more than double (+129%), while considering the first useful figure of the gas detected by the Istat, December 2021, the free since then has increased by 141.1% against a decrease of 7.4% of the protected. In 3 years, from January 2020 to January 2023, free light jumped 262,8%, compared to more than 115,8% of the protected market. for electricity, gas and other fuels, item that includes gas, light (free and protected market), diesel for heating and solid fuels, if in Italy the rise in January was 67.3% compared to a year earlier, with a family stag equal on average to 907,50 euros on an annual basis, in some cities it has almost 90 percent. the comparison does not console the fact that Umbria is at the foot of the podium, also because the distance with those who conquer the highest step is reduced. In Alexandria, electricity, gas and diesel costs fly 88.6% on January 2022. the piemonte fills with vercelli that inserts a plus 87,1% and biella with more 86,1%. on the other side of the ranking, the city less tartassata is power with more 35.2%. in second place aosta with more than 50.8%. on the lowest step of the podium of the virtuous cities olbia-temple with more 51%. followed by Napoli (+51.4%), Gorizia (+51.7%), Benevento (+53.1%), seventh caserta (+53.5%), then Avellino (+53.7%) and Trieste (+54.6%). They close the top ten pordenone and udine, ex aequo with +54.7%. the other classifies another study on the price run comes from the office studies of the cgia of mestre which indicates the weight of the purchasing power of the families regarding the inflation that goes in the rush. in the two years 2022-2023 could amount to almost six thousand euros per household the loss of purchasing power in Umbria due to inflation. the estimate is based on the data of banca d'italia, istat and commissione europea. against bank deposits that, at the end of 2021, amounted to 14.5 billion euros, in Umbria in 2022 the estimated loss of purchasing power amounts to 1.2 billion euros while in 2023, complicit in a slowdown in inflation, 885 million euros for a total of 2.1 billion euros. At provincial level the figure of the cgia says that for that of Perugia the loss of purchasing power could amount to beyond 1,6 billion euros (almost 5,746 to family) while in that of terni to 536 million (5,251 to family). Here the gap is more clear than what happens for increases in electricity and gas bills. luca benedetti</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>['A study by the national consumer union ranked cities based on annual increases, using data from Istat from January 2023.', 'Perugia and Terni were ranked among the top six most expensive cities.', 'The cost of light and gas in Perugia increased by 85.8%.', 'The average annual cost of living for a family in Perugia is 1,157 euros.', 'The survey compares the change in electricity and gas prices over the last 3 years, comparing free and protected markets.', 'From June 2021 to January 2023, the protected market light in Italy rose by 108.4%.', 'The protected market gas price decreased by 7.4% since December 2021.', 'From January 2020 to January 2023, the protected market light jumped 115.8%.', 'In January, the rise in electricity, gas, and other fuels in Italy was 67.3% compared to a year earlier.', 'The average annual cost of electricity, gas, and other fuels for a family in Italy is 907.50 euros.', 'In Alexandria, electricity, gas, and diesel costs increased by 88.6% in January 2022.', 'Vercelli (Piemonte) saw an increase of 87.1%.', 'Biella saw an increase of 86.1%.', 'Power (the city less tartassata) saw an increase of 35.2%.', 'Olbia-Tempio saw an increase of 51%.', 'Gorizia saw an increase of 51.7%.', 'Benevento saw an increase of 53.1%.', 'Caserta saw an increase of 53.5%.', 'Trieste saw an increase of 54.6%.', 'Pordenone and Udine saw an increase of 54.7%.', 'The CGIA of Mestre conducted a study on the weight of family purchasing power regarding inflation.', 'The loss of purchasing power in Umbria over the two years 2022-2023 could amount to almost 6,000 euros per household.', 'The estimate for the loss of purchasing power in Umbria in 2022 was 1.2 billion euros.', 'The total estimated loss of purchasing power in Umbria over the two years was 2.1 billion euros.', 'Bank deposits at the end of 2021 amounted to 14.5 billion euros.', 'For Perugia, the loss of purchasing power could amount to over 1.6 billion euros.']</t>
+          <t>['A study by the national consumer union ranked cities based on annual increases.', 'The data for the ranking came from Istat for January 2023.', 'Perugia and Terni are among the top six most expensive cities.', 'The cost of light and gas in Perugia increased by 85.8%.', 'The average annual spending of an Italian family in Perugia is 1,157 euros.', 'The survey compared changes in electricity and gas prices over three years.', 'The survey compared the free market and the protected market for electricity and gas prices.', 'From June 2021 to January 2023, the protected market light in Italy rose by 108.4%.', 'The protected market gas price, according to Istat data from December 2021, decreased by 7.4%.', 'From January 2020 to January 2023, free light jumped 262.8%.', 'From January 2020 to January 2023, the protected market light jumped by more than 115.8%.', 'In January 2023, the rise in electricity, gas, and other fuels in Italy was 67.3% compared to the previous year.', 'The average annual family spending on electricity, gas, and other fuels in Italy is 907.50 euros.', 'Umbria is at the bottom of the ranking.', 'The cost of electricity, gas, and diesel in Alexandria increased by 88.6% in January 2022.', 'Vercelli (Piemonte) saw an increase of 87.1%.', 'Biella saw an increase of 86.1%.', 'Potenza saw an increase of 35.2%.', 'Olbia-Tempio saw an increase of more than 51%.', 'Benevento saw an increase of 53.1%.', 'Caserta saw an increase of 53.5%.', 'Trieste saw an increase of 54.6%.', 'Pordenone and Udine both increased by 54.7%.', 'The CGIA of Mestre conducted a study on the purchasing power loss due to inflation.', 'The loss of purchasing power in Umbria over the two years 2022-2023 could amount to almost 6,000 euros per household.', "The estimate for the purchasing power loss is based on data from Banca d'Italia, Istat, and the European Commission.", 'Bank deposits in Italy at the end of 2021 amounted to 14.5 billion euros.', 'The total estimated loss of purchasing power in Umbria over 2022 and 2023 was 2.1 billion euros.', 'The CGIA estimates the loss of purchasing power for Perugia at almost 5,746 euros per family.', 'The CGIA estimates the loss of purchasing power for Terni at 536 million euros.']</t>
         </is>
       </c>
     </row>
@@ -926,17 +926,17 @@
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
-          <t>. the closure of the major international exchanges. The development of the dow Jones (continued on page 5) glaucous new york magazine a new package to be voted on in Congress to stimulate the American economy in severe crisis yesterday had the support of the president of the federal reserve bernanke well, and a conditional green light from the president bush. In the short-term future of the economy, the central bank also takes into account a further cut in rates, thanks to low inflation from the recession. For Bernanke, who spoke before the chamber budget committee, the credit crisis "is hitting the economy" because the Americans find it hard to find money for their activities. "with an economy likely to be weak for several quarters still and the risk of a prolonged slowdown, the idea of a tax package seems appropriate in this situation," said the governor to Members, refusing to define the ideal entity for him to intervene. One hour after these statements of technical support, the political free way has come to the agenda of a tax drug law bis in the country. the Bush administration "is open to ideas that could stimulate the economy and help us get out of this downward spiral faster," echoed Bernanke the spokesman of the Dana Perino president. but the ok will only be there if they will be ideas that "really stimulate the economy." the congress, which is responsible for approving a second tax package after the one passed at the beginning of the year which gave very limited benefits, according to the governor of the fed "should include measures to facilitate access to credit for consumers, homeowners and in general those interested in borrowing. These actions could be particularly effective," he dared, "to promote economic growth and job creation." Wall street, which had already started positive, expanded earnings after the promise of central bank stimulus and the availability of bush. the dowjones index has risen above quota 9000 points, with a rise of 4.67%, well also the nasdaq that has earned 3,43% to 1,700 points, while the dollar has strengthened against the euro, coming down to 1.33 dollars from 1.34 of the start. Europe also runs, where London shines (+5, 41%), followed by Paris (+3,56%), Madrid (+2,99%), and Milan (+2, 65%). more cautious francoforte (+1.12%). to give breath to the purchases on the stock exchange, it has also contributed the hint of Bernanke to a new cut of the rates at the meeting of the end of October of the fed. federal bonds are 100% reduced by 25 cents, but 46% could also be half a point, like the previous one made together by all banks. The fate of the American budget, however, is no longer a problem for anyone, in these world moonlights where the use of public expenditure to embarrass the threat of depression is dominated. the new nobel prize of the economy Paul Krugman wrote it on the new York times, invoking massive injections of state money in the banks and the same Bernanke mentioned it in his speech: "the current deficit is wide," admitted," but not inappropriate given the nature of the emergency that we are facing and not avoidable given the loss of tax revenues." Bernanke is aware that "every tax action inevitably involves trade" and may "heavy on future generations," but he accepted the inevitability of intervention. Without defining recession as the current state of the economy, the governor predicted that "the pace of economic activity will remain below the growth potential for several quarters, and that the slowdown in investment and business spending will extend to the major sectors."</t>
+          <t>. the closure of the major international exchanges. the development of the dow jones (follows on page 5) glauco maggi new york a new package to be voted in Congress to stimulate the American economy in severe crisis yesterday had the support of the president of the federal reserve bernanke, and a conditional green light from the presidente bush. In the short-term future of the economy, the central bank also takes into account a further cut in rates, thanks to low inflation from the recession. For Bernanke, who spoke before the budget committee of the camera, the credit crisis "is hitting the economy" because the Americans struggle to find money for their activities. "with an economy likely to be weak for several quarters still and the risk of a prolonged slowdown, the idea of a tax package seems appropriate in this situation," said the governor to Members, refusing to define the ideal entity for him to intervene. One hour after these statements of technical support, the political free way has come to the agenda of a tax drug law bis in the country. The amministrazione bush "is open to ideas that could stimulate the economy and help us get out of this downward spiral faster," echoed Bernanke the spokesman of the Dana Perino president. but the ok will only be there if they will be ideas that "really stimulate the economy." the congress, which is responsible for approving a second tax package after the one passed at the beginning of the year that gave very limited benefits, according to the governor of the fed "should include measures to facilitate access to credit for consumers, homeowners and in general those interested in borrowing. These actions could be particularly effective," he dared, "to promote economic growth and job creation." wall street, which had already started positive, expanded earnings after the promise of central bank stimulus and the availability of bush. the dowjones index has risen above quota 9000 points, with a rise of 4.67%, well also the nasdaq that has earned 3,43% to 1,700 points, while the dollar has strengthened against the euro, coming down to 1.33 dollars from 1.34 of the start. Europe also runs, where London shines (+5, 41%), followed by Paris (+3,56%), Madrid (+2,99%), and Milan (+2, 65%). more cautious francoforte (+1.12%). to give breath to the purchases on the stock exchange, it has also contributed the hint of Bernanke to a new cut of the rates at the meeting of the end October of the fed. federal bonds are 100% reduced by 25 cents, but 46% could also be half a point, like the previous one made together by all banks. The fate of the American budget, however, is no longer a problem for anyone, in these world moonlights where the use of public expenditure to embarrass the threat of depression is dominated. the new nobel prize of the economy Paul Krugman wrote it on the new york times, invoking massive injections of state money in the banks and the same Bernanke mentioned it in his speech: "the current deficit is wide," admitted," but not inappropriate given the nature of the emergency that we are facing and not avoidable given the loss of tax revenues." Bernanke is aware that "every tax action inevitably involves trade" and may "heavy on future generations," but he accepted the inevitability of intervention. Without defining recession as the current state of the economy, the governor predicted that "the pace of economic activity will remain below the growth potential for several quarters, and that the slowdown in investment and business spending will extend to the major sectors."</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>Observation date: 2008-10-21 00:00:00. . the closure of the major international exchanges. The development of the dow Jones (continued on page 5) glaucous new york magazine a new package to be voted on in Congress to stimulate the American economy in severe crisis yesterday had the support of the president of the federal reserve bernanke well, and a conditional green light from the president bush. In the short-term future of the economy, the central bank also takes into account a further cut in rates, thanks to low inflation from the recession. For Bernanke, who spoke before the chamber budget committee, the credit crisis "is hitting the economy" because the Americans find it hard to find money for their activities. "with an economy likely to be weak for several quarters still and the risk of a prolonged slowdown, the idea of a tax package seems appropriate in this situation," said the governor to Members, refusing to define the ideal entity for him to intervene. One hour after these statements of technical support, the political free way has come to the agenda of a tax drug law bis in the country. the Bush administration "is open to ideas that could stimulate the economy and help us get out of this downward spiral faster," echoed Bernanke the spokesman of the Dana Perino president. but the ok will only be there if they will be ideas that "really stimulate the economy." the congress, which is responsible for approving a second tax package after the one passed at the beginning of the year which gave very limited benefits, according to the governor of the fed "should include measures to facilitate access to credit for consumers, homeowners and in general those interested in borrowing. These actions could be particularly effective," he dared, "to promote economic growth and job creation." Wall street, which had already started positive, expanded earnings after the promise of central bank stimulus and the availability of bush. the dowjones index has risen above quota 9000 points, with a rise of 4.67%, well also the nasdaq that has earned 3,43% to 1,700 points, while the dollar has strengthened against the euro, coming down to 1.33 dollars from 1.34 of the start. Europe also runs, where London shines (+5, 41%), followed by Paris (+3,56%), Madrid (+2,99%), and Milan (+2, 65%). more cautious francoforte (+1.12%). to give breath to the purchases on the stock exchange, it has also contributed the hint of Bernanke to a new cut of the rates at the meeting of the end of October of the fed. federal bonds are 100% reduced by 25 cents, but 46% could also be half a point, like the previous one made together by all banks. The fate of the American budget, however, is no longer a problem for anyone, in these world moonlights where the use of public expenditure to embarrass the threat of depression is dominated. the new nobel prize of the economy Paul Krugman wrote it on the new York times, invoking massive injections of state money in the banks and the same Bernanke mentioned it in his speech: "the current deficit is wide," admitted," but not inappropriate given the nature of the emergency that we are facing and not avoidable given the loss of tax revenues." Bernanke is aware that "every tax action inevitably involves trade" and may "heavy on future generations," but he accepted the inevitability of intervention. Without defining recession as the current state of the economy, the governor predicted that "the pace of economic activity will remain below the growth potential for several quarters, and that the slowdown in investment and business spending will extend to the major sectors."</t>
+          <t>Observation date: 2008-10-21 00:00:00. . the closure of the major international exchanges. the development of the dow jones (follows on page 5) glauco maggi new york a new package to be voted in Congress to stimulate the American economy in severe crisis yesterday had the support of the president of the federal reserve bernanke, and a conditional green light from the presidente bush. In the short-term future of the economy, the central bank also takes into account a further cut in rates, thanks to low inflation from the recession. For Bernanke, who spoke before the budget committee of the camera, the credit crisis "is hitting the economy" because the Americans struggle to find money for their activities. "with an economy likely to be weak for several quarters still and the risk of a prolonged slowdown, the idea of a tax package seems appropriate in this situation," said the governor to Members, refusing to define the ideal entity for him to intervene. One hour after these statements of technical support, the political free way has come to the agenda of a tax drug law bis in the country. The amministrazione bush "is open to ideas that could stimulate the economy and help us get out of this downward spiral faster," echoed Bernanke the spokesman of the Dana Perino president. but the ok will only be there if they will be ideas that "really stimulate the economy." the congress, which is responsible for approving a second tax package after the one passed at the beginning of the year that gave very limited benefits, according to the governor of the fed "should include measures to facilitate access to credit for consumers, homeowners and in general those interested in borrowing. These actions could be particularly effective," he dared, "to promote economic growth and job creation." wall street, which had already started positive, expanded earnings after the promise of central bank stimulus and the availability of bush. the dowjones index has risen above quota 9000 points, with a rise of 4.67%, well also the nasdaq that has earned 3,43% to 1,700 points, while the dollar has strengthened against the euro, coming down to 1.33 dollars from 1.34 of the start. Europe also runs, where London shines (+5, 41%), followed by Paris (+3,56%), Madrid (+2,99%), and Milan (+2, 65%). more cautious francoforte (+1.12%). to give breath to the purchases on the stock exchange, it has also contributed the hint of Bernanke to a new cut of the rates at the meeting of the end October of the fed. federal bonds are 100% reduced by 25 cents, but 46% could also be half a point, like the previous one made together by all banks. The fate of the American budget, however, is no longer a problem for anyone, in these world moonlights where the use of public expenditure to embarrass the threat of depression is dominated. the new nobel prize of the economy Paul Krugman wrote it on the new york times, invoking massive injections of state money in the banks and the same Bernanke mentioned it in his speech: "the current deficit is wide," admitted," but not inappropriate given the nature of the emergency that we are facing and not avoidable given the loss of tax revenues." Bernanke is aware that "every tax action inevitably involves trade" and may "heavy on future generations," but he accepted the inevitability of intervention. Without defining recession as the current state of the economy, the governor predicted that "the pace of economic activity will remain below the growth potential for several quarters, and that the slowdown in investment and business spending will extend to the major sectors."</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>['A new package to be voted on in Congress to stimulate the American economy in severe crisis was supported by the President of the Federal Reserve, Bernanke, and the President Bush on 2008-10-20.', 'The central bank takes into account a further cut in rates in the short-term future of the economy due to low inflation from the recession.', 'Bernanke stated that the credit crisis is hitting the economy because Americans find it hard to find money for their activities.', 'The governor told Members that the idea of a tax package seems appropriate because the economy is likely to be weak for several quarters and there is a risk of a prolonged slowdown.', 'One hour after these statements of technical support, the political free way came to the agenda of a tax drug law bis in the country.', 'Bernanke, the spokesman of the President Bush, echoed that the Bush administration is open to ideas that could stimulate the economy and help the United States get out of the downward spiral faster.', 'The governor of the Fed stated that Congress should include measures to facilitate access to credit for consumers, homeowners, and those interested in borrowing in a second tax package.', 'The governor of the Fed believes that these actions could promote economic growth and job creation.', 'Wall Street expanded earnings after the promise of central bank stimulus and the availability of President Bush.', 'The Dow Jones index rose above 9000 points, with a rise of 4.67%.', 'The Nasdaq earned 3.43% to 1,700 points.', 'The dollar strengthened against the euro, coming down to 1.33 dollars from 1.34 at the start.', 'London rose by 5.41%.', 'Paris rose by 3.56%.', 'Madrid rose by 2.99%.', 'Milan rose by 2.65%.', 'Frankfurt rose by 1.12%.', 'Bernanke hinted that a new cut of rates could happen at the meeting of the end of October of the Fed.', 'Federal bonds are 100% reduced by 25 cents.', 'Federal bonds could also be half a point, like the previous one made together by all banks.', 'Paul Krugman wrote in the New York Times, invoking massive injections of state money in the banks.', 'Bernanke admitted that the current deficit is wide but not inappropriate given the nature of the emergency.', 'Bernanke stated that the current deficit is not avoidable given the loss of tax revenues.', 'Bernanke is aware that every tax action inevitably involves trade.', 'Bernanke stated that tax actions may be heavy on future generations.', 'The governor predicted that the pace of economic activity will remain below the growth potential for several quarters.', 'The governor predicted that the slowdown in investment and business spending will extend to the major sectors.']</t>
+          <t>['A new package to be voted in Congress to stimulate the American economy was discussed on 2008-10-20.', 'The proposal for the tax package had the support of the Federal Reserve President, Bernanke.', 'The proposal for the tax package received a conditional green light from President Bush.', 'The central bank considers a further cut in rates due to low inflation from the recession.', 'Bernanke stated that the credit crisis is hitting the economy because Americans struggle to find money for their activities.', 'Bernanke stated that the idea of a tax package seems appropriate given the risk of a prolonged slowdown and an economy likely to be weak for several quarters.', 'One hour after the technical support statements, the political free way was added to the agenda of a tax drug law bis in the country.', 'The administration of Bush is open to ideas that could stimulate the economy and help the country get out of the downward spiral faster, according to Bernanke.', 'The administration of Bush will only proceed if there are ideas that really stimulate the economy.', 'The Congress is responsible for approving a second tax package.', 'The governor of the Fed recommended that the second tax package should include measures to facilitate access to credit for consumers, homeowners, and those interested in borrowing.', 'The governor of the Fed stated that these actions could promote economic growth and job creation.', 'Wall Street expanded earnings after the promise of central bank stimulus and the availability of Bush.', 'The Dow Jones index rose above 9000 points, with a rise of 4.67%.', 'The Nasdaq index rose 3.43% to 1,700 points.', 'The dollar strengthened against the euro, coming down to 1.33 dollars from 1.34 at the start.', 'London rose 5.41% on the stock exchange.', 'Paris rose 3.56% on the stock exchange.', 'Francoforte rose 1.12% on the stock exchange.', "Bernanke's hint of a new rate cut at the end of October contributed to purchases on the stock exchange.", 'Federal bonds are reduced by 25 cents.', 'Federal bonds could also be reduced by half a point.', 'Paul Krugman wrote about the new Nobel Prize of the economy in the New York Times.', 'Bernanke admitted that the current deficit is wide but not inappropriate given the nature of the emergency.', 'Bernanke stated that the pace of economic activity will remain below the growth potential for several quarters.', 'Bernanke predicted that the slowdown in investment and business spending will extend to the major sectors.']</t>
         </is>
       </c>
     </row>
@@ -986,17 +986,17 @@
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
-          <t>If, on the other hand, there had been the ability to put that saving on income even with a remuneration of one percentage point, households would have earned a total of 30 billion, almost 2% of gross domestic product. The saving rate of Italian households relative to disposable income grew by 50% in the year but, where savings invested in listed companies are excluded, its yield remained rather low, close to zero. Given the size of financial assets in the hands of households, each percentage point of remuneration can be estimated at around €30 billion, almost 2% of GDP being the size of a good government budget maneuver of the past. the key theme of the annual report of the president of the consob, Paolo Savona, is the main asset that the authority he leads intends to protect: savings. but this has been stationary on the deposits in the last two years. and is now threatened by a shadow that stretches on international markets and that is very difficult to control: they are the sirens of cryptocurrencies and bitcoins. a phenomenon in strong growth and increasingly difficult to keep under control. so much as to push savannah to launch an alarm: the speculative effect that they are triggering seems very similar to what happened before 2008 with subprime mortgages. The diffusion of virtual tools has called for the emergence of the already mentioned technological platforms These new market segments are rapidly evolving and experience before the 2008 crisis seems to be repeated when derivative contracts developed to a size of ten times the global GDP, taking complex forms that received a high rating. Even with the necessary distinctions, it is foreseeable that something similar is happening in the market for virtual monetary and financial products, especially encrypted, is happening. Savona recalled that only one bitcoin has recently had the opportunity to buy a large electric car and soon after lost half of its purchasing power. For the President consob \l'informatica finanziale is a prodigious lamp from which the genius came out. the authorities will not be able to bring it back in, because it acts in the controllable immaterial sphere only by changing the information exchange protocol, i.e. by fragmenting the unity of the world market and thus reducing the international competitiveness test. Traditional supervisory instruments are no longer sufficient. under the current conditions, according to Savona, the authorities may also intervene using the advantages of digitised techniques their action will be more effective if they cooperate with each other. For Italy, the issue is even more sensitive because of the constitutional rule that confers on the public the task of encouraging and protecting savings in all its forms and of regulating, coordinating and controlling the exercise of credit. It would be improper, he explained, if it were to be assigned to the specification of the savings in all its forms and to the credit to be protected a content that would also embrace the virtual instruments, without switching from a specific regulation. These currencies are pivoting on blockchains. As far as it is known about the state of hacking techniques, the original blockchain is impenetrable, while the one used by other cryptocurrency is not, it has chiosato. and once again there is a call to proceed quickly with adjustment systems. "Without adequate safeguards (standards and bodies) " he said - this leads to a worsening of market transparency, which is the basis for the legality and rational choices of operators. Among the well-known negative effects is the shielding that these techniques allow criminal activities, such as tax evasion, money laundering, terrorist financing and kidnapping. Savona has remembered the activity of consob in darkening in italy hundreds of websites that illegally collected savings. But in this context, it's a bit like emptying the sea with your hands. Mr Savona obviously hopes for an international solution. The issue of cybersecurity covers even broader political issues, the solution of which cannot be achieved at national level and requires close international cooperation, i.e. the emergence of a global public good, as were the fmi, l'onu and wto. the part of the Bretton Woods agreement closest to the solutions to the problem raised here of the interchangeability between different national currencies did not bear the test of international cooperation, but the technological innovations applied to finance re-proposed the urgency of its relaunch in a topical key, he said. the president consob has also re-launched the proposal of unification of the single text of finance and the single bank text and then suggest a more tightened collaboration between the Italian authorities. "To this end, it is necessary to activate in Italy structures of formal consultation between governing bodies and independent authorities that give a unitary address to the choices in the matter, also in view of the position to assume in front of the European and international initiatives in progress," he explained -. A first step would be the transposition of the 2011 recommendation of the European Systemic Risk Board, which would give life to a single national counterpart that bears responsibility for macro-preudential stability. The Bank of Italy would maintain a central role, justified by its participation in the euro system around which European finance is currently based, but close coordination between the three independent supervisory authorities (consob, ivass and covip), with the participation of the Ministry of Economic Affairs, would be ensured. In order to cope with economic and social difficulties, public debt has grown greatly, even in forms other than those which an emerging state would have required. However, confidence in the response capacity of the Italian economy has grown. This result is also the result of decisions taken by the ECB to acquire significant volumes of public bonds and by the European Commission to suspend, albeit temporarily, the Stability Pact and launch the next generation eu plan. We agree on the assessments given for all these decisions on the structural improvement of our real growth rate. But now we need to change the pace. However, for the continuation of the phase of relaunching the productive activity it is necessary to integrate the decisions taken so far in order to stimulate the venture capital of the enterprises in order to improve their leverage and make them more available to undertake new initiatives, Savona said, according to which it offers an important occasion the reform of the tax demanded for a long time, above all, the task is assigned to it to consider the productive authorities on the same plane as those ethical ones in the appraisals of the distribution equity. click to view the image</t>
+          <t>If, on the other hand, there had been the ability to put that saving on income even with a remuneration of one percentage point, households would have earned a total of 30 billion, almost 2% of gross domestic product. The savings rate of Italian households compared to disposable income increased by 50%, but where the savings invested in listed companies are excluded, its return remained rather low, close to zero. Given the size of financial assets in the hands of households, each percentage point of remuneration can be estimated at around €30 billion, almost 2% of GDP being the size of a good government budget maneuver of the past. the key theme of the annual report of the president of the consob, paolo savona, is the main asset that the authority he leads intends to protect: savings. but this has been stationary on the deposits in the last two years. and is now threatened by a shadow that stretches on international markets and that is very difficult to control: they are the sirens of cryptocurrencies and bitcoins. a phenomenon in strong growth and increasingly difficult to keep under control. so much as to push savannah to launch an alarm: the speculative effect that they are triggering seems very similar to what happened before 2008 with subprime mortgages. The diffusion of virtual tools has called for the emergence of the already mentioned technological platforms These new market segments are rapidly evolving and experience before the 2008 crisis seems to be repeated when derivative contracts developed to a size of ten times the global GDP, taking complex forms that received a high rating. Even with the necessary distinctions, it is foreseeable that something similar is happening in the market for virtual monetary and financial products, especially encrypted, is happening. Savona recalled that only one bitcoin has recently had the opportunity to buy a large electric car and soon after lost half of its purchasing power. For the President consob \l'informatica finanziale is a prodigious lamp from which the genius came out. the authorities will not be able to bring it back in, because it acts in the controllable immaterial sphere only by changing the information exchange protocol, i.e. by fragmenting the unity of the world market and thus reducing the international competitiveness test. Traditional supervisory instruments are no longer sufficient. under the current conditions, according to Savona, the authorities may also intervene using the advantages of digitised techniques their action will be more effective if they cooperate with each other. For Italy, the issue is even more sensitive because of the constitutional rule that confers on the public the task of encouraging and protecting savings in all its forms and of regulating, coordinating and controlling the exercise of credit. It would be improper, he explained, if it were to be assigned to the specification of the savings in all its forms and to the credit to be protected a content that would also embrace the virtual instruments, without switching from a specific regulation. These currencies are pivoting on blockchains. As far as it is known about the state of hacking techniques, the original blockchain is impenetrable, while the one used by other cryptocurrency is not, it has chiosato. and once again there is a call to proceed quickly with adjustment systems. "Without adequate safeguards (standards and bodies) " he said - this leads to a worsening of market transparency, which is the basis for the legality and rational choices of operators. Among the well-known negative effects is the shielding that these techniques allow criminal activities, such as tax evasion, money laundering, terrorist financing and kidnapping. Savona has remembered the activity of consob in darkening in italy hundreds of websites that illegally collected savings. But in this context, it's a bit like emptying the sea with your hands. Mr Savona obviously hopes for an international solution. The issue of cybersecurity embraces even broader political issues, the solution of which cannot be achieved at national level and requires close international collaboration, i.e. the emergence of a global public good, as were the fmi, the onu and the wto. the part of the Bretton Woods agreement closest to the solutions to the problem raised here of the interchangeability between different national currencies did not bear the test of international cooperation, but the technological innovations applied to finance re-proposed the urgency of its relaunch in a topical key, he said. the president consob has also re-launched the proposal of unification of the single text of finance and the single bank text and then suggest a more tightened collaboration between the Italian authorities. "To this end, it is necessary to activate in Italy structures of formal consultation between governing bodies and independent authorities that give a unitary address to the choices in the matter, also in view of the position to assume in front of the European and international initiatives in progress," he explained -. A first step would be the transposition of the 2011 recommendation of the European Systemic Risk Board, which would give life to a single national counterpart that bears responsibility for macro-preudential stability. banca d’italia would maintain a central role, justified by its participation in the euro system around which European finance is currently based, but close coordination between the three independent supervisory authorities (consob, ivass and covip), with the participation of the Ministry of Economic Affairs, would be ensured. In order to cope with economic and social difficulties, public debt has grown greatly, even in forms other than those which an emerging state would have required. However, confidence in the response capacity of the Italian economy has grown. This result is also the result of decisions taken by the ECB to purchase significant volumes of public bonds and by the commissione europea to suspend, albeit temporarily, the Stability Pact and launch the next generation eu plan. We agree on the assessments given for all these decisions on the structural improvement of our real growth rate. But now we need to change the pace. However, for the continuation of the phase of relaunching the productive activity it is necessary to integrate the decisions taken so far in order to stimulate the venture capital of the enterprises in order to improve their leverage and make them more available to undertake new initiatives, Savona said, according to which it offers an important occasion the reform of the tax demanded for a long time, above all, the task is assigned to it to consider the productive authorities on the same plane as those ethical ones in the appraisals of the distribution equity. click to view the image</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>Observation date: 2021-06-14 00:00:00. If, on the other hand, there had been the ability to put that saving on income even with a remuneration of one percentage point, households would have earned a total of 30 billion, almost 2% of gross domestic product. The saving rate of Italian households relative to disposable income grew by 50% in the year but, where savings invested in listed companies are excluded, its yield remained rather low, close to zero. Given the size of financial assets in the hands of households, each percentage point of remuneration can be estimated at around €30 billion, almost 2% of GDP being the size of a good government budget maneuver of the past. the key theme of the annual report of the president of the consob, Paolo Savona, is the main asset that the authority he leads intends to protect: savings. but this has been stationary on the deposits in the last two years. and is now threatened by a shadow that stretches on international markets and that is very difficult to control: they are the sirens of cryptocurrencies and bitcoins. a phenomenon in strong growth and increasingly difficult to keep under control. so much as to push savannah to launch an alarm: the speculative effect that they are triggering seems very similar to what happened before 2008 with subprime mortgages. The diffusion of virtual tools has called for the emergence of the already mentioned technological platforms These new market segments are rapidly evolving and experience before the 2008 crisis seems to be repeated when derivative contracts developed to a size of ten times the global GDP, taking complex forms that received a high rating. Even with the necessary distinctions, it is foreseeable that something similar is happening in the market for virtual monetary and financial products, especially encrypted, is happening. Savona recalled that only one bitcoin has recently had the opportunity to buy a large electric car and soon after lost half of its purchasing power. For the President consob \l'informatica finanziale is a prodigious lamp from which the genius came out. the authorities will not be able to bring it back in, because it acts in the controllable immaterial sphere only by changing the information exchange protocol, i.e. by fragmenting the unity of the world market and thus reducing the international competitiveness test. Traditional supervisory instruments are no longer sufficient. under the current conditions, according to Savona, the authorities may also intervene using the advantages of digitised techniques their action will be more effective if they cooperate with each other. For Italy, the issue is even more sensitive because of the constitutional rule that confers on the public the task of encouraging and protecting savings in all its forms and of regulating, coordinating and controlling the exercise of credit. It would be improper, he explained, if it were to be assigned to the specification of the savings in all its forms and to the credit to be protected a content that would also embrace the virtual instruments, without switching from a specific regulation. These currencies are pivoting on blockchains. As far as it is known about the state of hacking techniques, the original blockchain is impenetrable, while the one used by other cryptocurrency is not, it has chiosato. and once again there is a call to proceed quickly with adjustment systems. "Without adequate safeguards (standards and bodies) " he said - this leads to a worsening of market transparency, which is the basis for the legality and rational choices of operators. Among the well-known negative effects is the shielding that these techniques allow criminal activities, such as tax evasion, money laundering, terrorist financing and kidnapping. Savona has remembered the activity of consob in darkening in italy hundreds of websites that illegally collected savings. But in this context, it's a bit like emptying the sea with your hands. Mr Savona obviously hopes for an international solution. The issue of cybersecurity covers even broader political issues, the solution of which cannot be achieved at national level and requires close international cooperation, i.e. the emergence of a global public good, as were the fmi, l'onu and wto. the part of the Bretton Woods agreement closest to the solutions to the problem raised here of the interchangeability between different national currencies did not bear the test of international cooperation, but the technological innovations applied to finance re-proposed the urgency of its relaunch in a topical key, he said. the president consob has also re-launched the proposal of unification of the single text of finance and the single bank text and then suggest a more tightened collaboration between the Italian authorities. "To this end, it is necessary to activate in Italy structures of formal consultation between governing bodies and independent authorities that give a unitary address to the choices in the matter, also in view of the position to assume in front of the European and international initiatives in progress," he explained -. A first step would be the transposition of the 2011 recommendation of the European Systemic Risk Board, which would give life to a single national counterpart that bears responsibility for macro-preudential stability. The Bank of Italy would maintain a central role, justified by its participation in the euro system around which European finance is currently based, but close coordination between the three independent supervisory authorities (consob, ivass and covip), with the participation of the Ministry of Economic Affairs, would be ensured. In order to cope with economic and social difficulties, public debt has grown greatly, even in forms other than those which an emerging state would have required. However, confidence in the response capacity of the Italian economy has grown. This result is also the result of decisions taken by the ECB to acquire significant volumes of public bonds and by the European Commission to suspend, albeit temporarily, the Stability Pact and launch the next generation eu plan. We agree on the assessments given for all these decisions on the structural improvement of our real growth rate. But now we need to change the pace. However, for the continuation of the phase of relaunching the productive activity it is necessary to integrate the decisions taken so far in order to stimulate the venture capital of the enterprises in order to improve their leverage and make them more available to undertake new initiatives, Savona said, according to which it offers an important occasion the reform of the tax demanded for a long time, above all, the task is assigned to it to consider the productive authorities on the same plane as those ethical ones in the appraisals of the distribution equity. click to view the image</t>
+          <t>Observation date: 2021-06-14 00:00:00. If, on the other hand, there had been the ability to put that saving on income even with a remuneration of one percentage point, households would have earned a total of 30 billion, almost 2% of gross domestic product. The savings rate of Italian households compared to disposable income increased by 50%, but where the savings invested in listed companies are excluded, its return remained rather low, close to zero. Given the size of financial assets in the hands of households, each percentage point of remuneration can be estimated at around €30 billion, almost 2% of GDP being the size of a good government budget maneuver of the past. the key theme of the annual report of the president of the consob, paolo savona, is the main asset that the authority he leads intends to protect: savings. but this has been stationary on the deposits in the last two years. and is now threatened by a shadow that stretches on international markets and that is very difficult to control: they are the sirens of cryptocurrencies and bitcoins. a phenomenon in strong growth and increasingly difficult to keep under control. so much as to push savannah to launch an alarm: the speculative effect that they are triggering seems very similar to what happened before 2008 with subprime mortgages. The diffusion of virtual tools has called for the emergence of the already mentioned technological platforms These new market segments are rapidly evolving and experience before the 2008 crisis seems to be repeated when derivative contracts developed to a size of ten times the global GDP, taking complex forms that received a high rating. Even with the necessary distinctions, it is foreseeable that something similar is happening in the market for virtual monetary and financial products, especially encrypted, is happening. Savona recalled that only one bitcoin has recently had the opportunity to buy a large electric car and soon after lost half of its purchasing power. For the President consob \l'informatica finanziale is a prodigious lamp from which the genius came out. the authorities will not be able to bring it back in, because it acts in the controllable immaterial sphere only by changing the information exchange protocol, i.e. by fragmenting the unity of the world market and thus reducing the international competitiveness test. Traditional supervisory instruments are no longer sufficient. under the current conditions, according to Savona, the authorities may also intervene using the advantages of digitised techniques their action will be more effective if they cooperate with each other. For Italy, the issue is even more sensitive because of the constitutional rule that confers on the public the task of encouraging and protecting savings in all its forms and of regulating, coordinating and controlling the exercise of credit. It would be improper, he explained, if it were to be assigned to the specification of the savings in all its forms and to the credit to be protected a content that would also embrace the virtual instruments, without switching from a specific regulation. These currencies are pivoting on blockchains. As far as it is known about the state of hacking techniques, the original blockchain is impenetrable, while the one used by other cryptocurrency is not, it has chiosato. and once again there is a call to proceed quickly with adjustment systems. "Without adequate safeguards (standards and bodies) " he said - this leads to a worsening of market transparency, which is the basis for the legality and rational choices of operators. Among the well-known negative effects is the shielding that these techniques allow criminal activities, such as tax evasion, money laundering, terrorist financing and kidnapping. Savona has remembered the activity of consob in darkening in italy hundreds of websites that illegally collected savings. But in this context, it's a bit like emptying the sea with your hands. Mr Savona obviously hopes for an international solution. The issue of cybersecurity embraces even broader political issues, the solution of which cannot be achieved at national level and requires close international collaboration, i.e. the emergence of a global public good, as were the fmi, the onu and the wto. the part of the Bretton Woods agreement closest to the solutions to the problem raised here of the interchangeability between different national currencies did not bear the test of international cooperation, but the technological innovations applied to finance re-proposed the urgency of its relaunch in a topical key, he said. the president consob has also re-launched the proposal of unification of the single text of finance and the single bank text and then suggest a more tightened collaboration between the Italian authorities. "To this end, it is necessary to activate in Italy structures of formal consultation between governing bodies and independent authorities that give a unitary address to the choices in the matter, also in view of the position to assume in front of the European and international initiatives in progress," he explained -. A first step would be the transposition of the 2011 recommendation of the European Systemic Risk Board, which would give life to a single national counterpart that bears responsibility for macro-preudential stability. banca d’italia would maintain a central role, justified by its participation in the euro system around which European finance is currently based, but close coordination between the three independent supervisory authorities (consob, ivass and covip), with the participation of the Ministry of Economic Affairs, would be ensured. In order to cope with economic and social difficulties, public debt has grown greatly, even in forms other than those which an emerging state would have required. However, confidence in the response capacity of the Italian economy has grown. This result is also the result of decisions taken by the ECB to purchase significant volumes of public bonds and by the commissione europea to suspend, albeit temporarily, the Stability Pact and launch the next generation eu plan. We agree on the assessments given for all these decisions on the structural improvement of our real growth rate. But now we need to change the pace. However, for the continuation of the phase of relaunching the productive activity it is necessary to integrate the decisions taken so far in order to stimulate the venture capital of the enterprises in order to improve their leverage and make them more available to undertake new initiatives, Savona said, according to which it offers an important occasion the reform of the tax demanded for a long time, above all, the task is assigned to it to consider the productive authorities on the same plane as those ethical ones in the appraisals of the distribution equity. click to view the image</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>['If saving could be put on income with a one percentage point remuneration, households would have earned 30 billion, which is almost 2% of gross domestic product.', 'The saving rate of Italian households relative to disposable income grew by 50% in the year.', 'The yield of savings, excluding investments in listed companies, remained low, close to zero.', 'Each percentage point of remuneration, given the size of financial assets in the hands of households, is estimated at around €30 billion.', '2% of GDP is the size of a good government budget maneuver of the past.', 'The key theme of the annual report of the president of the CONSOB, Paolo Savona, is the protection of savings.', 'Savings in deposits have been stationary in the last two years.', 'Cryptocurrencies and bitcoins threaten savings in deposits.', 'The speculative effect triggered by cryptocurrencies and bitcoins seems similar to what happened before 2008 with subprime mortgages.', 'The diffusion of virtual tools caused the emergence of technological platforms.', 'The market segments are rapidly evolving.', 'Before the 2008 crisis, derivative contracts developed to a size of ten times the global GDP.', 'Something similar to the pre-2008 derivative contract development is foreseeable in the market for virtual monetary and financial products, especially encrypted ones.', 'Paolo Savona recalled that one bitcoin recently bought a large electric car.', 'The bitcoin subsequently lost half of its purchasing power.', 'For the President CONSOB, financial informatics is a prodigious lamp.', 'Authorities cannot bring back the change because it acts in the controllable immaterial sphere by changing the information exchange protocol.', 'Changing the information exchange protocol fragments the unity of the world market.', 'Fragmenting the unity of the world market reduces the international competitiveness test.', 'Traditional supervisory instruments are no longer sufficient.', 'According to Paolo Savona, the authorities may intervene using the advantages of digitized techniques under current conditions.', 'The action of the authorities will be more effective if the authorities cooperate with each other.', "Italy's issue is sensitive due to a constitutional rule that tasks the public with encouraging and protecting savings in all its forms.", 'The constitutional rule also tasks the public with regulating, coordinating, and controlling the exercise of credit.', 'Paolo Savona explained that it would be improper to assign a content that embraces virtual instruments to the specification of savings and credit without specific regulation.', 'The original blockchain is impenetrable regarding hacking techniques.', 'The blockchain used by other cryptocurrencies is not impenetrable.', 'There is a call to proceed quickly with adjustment systems.', 'Paolo Savona stated that the lack of adequate safeguards (standards and bodies) leads to a worsening of market transparency.', 'Market transparency is the basis for the legality and rational choices of operators.', 'These techniques allow shielding for criminal activities, including tax evasion, money laundering, terrorist financing, and kidnapping.', "Paolo Savona recalled CONSOB's activity in darkening hundreds of websites in Italy that illegally collected savings.", 'Paolo Savona hopes for an international solution for cybersecurity.', 'The solution to cybersecurity requires close international cooperation.', 'The solution to cybersecurity cannot be achieved at the national level.', 'The part of the Bretton Woods agreement concerning the interchangeability between different national currencies did not pass the test of international cooperation.', 'Technological innovations applied to finance re-proposed the urgency of relaunching the Bretton Woods agreement.', 'The president of CONSOB re-launched the proposal for unification of the single text of finance and the single bank text.', 'The president of CONSOB suggested a more tightened collaboration between the Italian authorities.', 'Paolo Savona explained that Italy needs to activate structures of formal consultation between governing bodies and independent authorities.', 'These structures must give a unitary address to choices regarding European and international initiatives.', 'A first step would be the transposition of the 2011 recommendation of the European Systemic Risk Board.', 'This transposition would create a single national counterpart responsible for macro-prudential stability.', 'The Bank of Italy would maintain a central role due to its participation in the euro system.', 'Close coordination between the three independent supervisory authorities (CONSOB, IVASS, and COVIP), with the participation of the Ministry of Economic Affairs, would be ensured.', 'Public debt has grown greatly to cope with economic and social difficulties.', 'Confidence in the response capacity of the Italian economy has grown.', 'The growth in confidence resulted from the ECB acquiring significant volumes of public bonds.', 'The growth in confidence resulted from the European Commission temporarily suspending the Stability Pact and launching the next generation EU plan.', 'The speaker agrees on the assessments regarding the structural improvement of the real growth rate.', 'The speaker stated that a change in pace is necessary.', 'Paolo Savona said that continuing the relaunching of productive activity requires integrating past decisions.', 'The integration must stimulate the venture capital of enterprises to improve their leverage and make them available for new initiatives.', 'The reform of the tax offers an important occasion to consider productive authorities on the same plane as ethical ones in distribution equity appraisals.']</t>
+          <t>['If savings could be put on income with a one percentage point remuneration, households would have earned 30 billion, which is almost 2% of gross domestic product.', 'The savings rate of Italian households compared to disposable income increased by 50%.', 'The return on savings, excluding investments in listed companies, remained low, close to zero.', 'Each percentage point of remuneration on household financial assets is estimated at around €30 billion.', 'This amount (€30 billion, almost 2% of GDP) is the size of a good government budget maneuver of the past.', 'The key theme of the annual report of the president of Consob, Paolo Savona, is protecting savings.', 'Savings have been stationary on deposits in the last two years.', 'Cryptocurrencies and bitcoins threaten savings in international markets.', 'The growth of cryptocurrencies is strong and increasingly difficult to control.', 'Paolo Savona launched an alarm because the speculative effect triggered by cryptocurrencies is similar to what happened before 2008 with subprime mortgages.', 'The diffusion of virtual tools caused the emergence of technological platforms.', 'Before the 2008 crisis, derivative contracts developed to a size of ten times the global GDP.', 'Something similar to the pre-2008 derivative market development is happening in the market for virtual monetary and financial products.', 'Paolo Savona recalled that one bitcoin recently bought a large electric car.', 'The purchasing power of that bitcoin was lost by half soon after the purchase.', 'For the President of Consob, financial informatics is a prodigious lamp.', 'Authorities cannot control the immaterial sphere because it changes the information exchange protocol.', 'Changing the information exchange protocol fragments the unity of the world market.', 'Traditional supervisory instruments are no longer sufficient.', 'Italy has a constitutional rule that requires the public to encourage and protect savings in all forms.', 'The constitutional rule also requires the public to regulate, coordinate, and control the exercise of credit.', 'It would be improper to assign the protection of savings and credit to a content that embraces virtual instruments without specific regulation.', 'Cryptocurrencies operate on blockchains.', 'The original blockchain is impenetrable regarding hacking techniques.', 'The blockchain used by other cryptocurrencies is vulnerable to hacking.', 'There is a call to proceed quickly with adjustment systems.', 'Without adequate safeguards (standards and bodies), market transparency worsens.', 'Market transparency is the basis for the legality and rational choices of operators.', 'These techniques allow criminal activities, including tax evasion, money laundering, terrorist financing, and kidnapping.', 'Mr. Savona hopes for an international solution for cybersecurity.', 'Solving the issue of cybersecurity requires close international collaboration and cannot be achieved at the national level.', 'Technological innovations applied to finance re-proposed the urgency of relaunching the Bretton Woods agreement.', 'The president of Consob re-launched the proposal to unify the single text of finance and the single bank text.', 'The president of Consob suggested tighter collaboration among Italian authorities.', 'Italy needs to activate structures of formal consultation between governing bodies and independent authorities.', 'These structures must provide a unitary address for choices regarding European and international initiatives.', 'A first step is transposing the 2011 recommendation of the European Systemic Risk Board.', 'Transposing the recommendation would create a single national counterpart responsible for macro-prudential stability.', 'Banca d’Italia would maintain a central role due to its participation in the euro system.', 'Close coordination between Consob, IVASS, Covip, and the Ministry of Economic Affairs would be ensured.', 'Public debt has grown greatly to cope with economic and social difficulties.', 'Confidence in the response capacity of the Italian economy has grown.', 'The ECB purchased significant volumes of public bonds.', 'The Commissione Europea temporarily suspended the Stability Pact and launched the next generation EU plan.', 'To continue relaunching productive activity, it is necessary to stimulate venture capital of enterprises.', 'The reform of the tax is needed to improve enterprise leverage and availability for new initiatives.', 'The reform of the tax must consider productive authorities on the same plane as ethical ones when appraising distribution equity.']</t>
         </is>
       </c>
     </row>
@@ -1050,17 +1050,17 @@
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr">
         <is>
-          <t>. the words of the governor Stefano lepri roma the financial crisis begins to pass on to the enterprises and the families; for now the credit paid by the banks has not diminished, says the governor of the bank of italia mario dragons, "the situation, however, can change quickly." consumption is falling. After the decline of the product in the second quarter, "negative signals for the next quarters" arrive. to stem the negative effects, silvio berlusconi has accepted the proposal of the confindustria to open a discussion table between government, enterprises and banks. It will call him just back from the trip to China: "we ask that banks do not miss their support for investment and consumption." The promise is to find "important funds" in the budget. and Minister Claudio Scajola added: state guarantees on corporate debts are being studied, as is the case with banks. Dragons in his audition to the Senate first wanted to reassure the Italian banks: "thanks to strict laws and a firm vigilance action, there is not that extended 'banking system shadow' in which elsewhere the crisis has found origin and food" . today "the capitalisation of the major Italian banks remains sufficient" , even if the losses from the Lehman bankruptcy reached the worst of the assumptions "such a shock could be absorbed" . However, the banks suffered on the stock exchange, due to a sentence of the president of the council that was partly misunderstood. again, and always in Naples as the first time on eni and enel, Berlusconi let himself run away with open stock exchange comments on listed companies. According to the official statement, he said: "Maybe two or three banks in addition to unicredit will have advantages in increasing their capital, naturally finding the means on the market." In the first press headlines, the prices of the major banks fell, and then they returned a little later. the clearing up on the financial markets confirmed yesterday with the tyron below 5% of the three-month euribor rate, reference point for variable-rate home loans. the Italian banks, assures the governor, "have only partially shared errors and distortions" of the world financial system, originated mainly in the United States. the European standards "the Italian bank has consistently given a strict interpretation." Dragons is well aware that public opinion tends to involve central banks in reproach. makes it clear that this can be justified in the uses, where there has been a "capture of the regulator" (in simple terms wall street influenced too much the government and the federal reserve) and in other countries; it is not in the euro area and especially in Italy. "alarms, over time, were not lacking," he recalls: "not least those who speak to you had repeatedly drawn attention to the imbalances of the international financial system," in several interventions, especially in autumn 2006; the trouble is that "in quiet times the warnings are often ignored." "They could not be predicted - he summarizes - neither the moment, nor the precise mechanism, nor the scale of the crisis; but one could well see the tensions that were accumulating." banks or other intermediaries who have given Lehman Brothers securities savers "will not have to leave them alone." new rules on transparency in the relationship between banks and customers will be ready at the beginning of next year. in the world, better regulation of derivatives and other innovative financial products will be needed to clean up. new rules will have to prevent banks from taking risks that are too exposed to their capital. "All in all, Italy does not come out badly" from the financial crisis, the governor concludes; but the effects of the crisis on the real economy "add to pre-existing structural weaknesses." The same judgment comes from the International Monetary Fund, which confirms the forecast decline in gross product both in 2008 (-0.1%) and in 2009 (-0.2%). but to react with state aid would not be the right answer, warns the head of the European department of fmi alessandro leiold: "better liberalisations."</t>
+          <t>. the words of the governor Stefano hari roma the financial crisis begins to pass on to the enterprises and the families; for now the credit paid by the banks has not diminished, says the governor of the bank of Italy mario draghi, "the situation, however, can change quickly." consumption is falling. After the decline of the product in the second quarter, "negative signals for the next quarters" arrive. To stem the negative effects, silvio berlusconi has accepted the Confindustria's proposal to open a discussion table between government, business and banks. It will call him just back from the trip to China: "we ask that banks do not miss their support for investment and consumption." The promise is to find "important funds" in the budget. and Minister claudio scajola added: state guarantees on corporate debts are being studied, as is the case with banks. Dragons in his audition to the Senate first wanted to reassure the Italian banks: "thanks to strict laws and a firm vigilance action, there is not that extended 'banking system shadow' in which elsewhere the crisis has found origin and food" . today "the capitalisation of the major Italian banks remains sufficient" , even if the losses from the Lehman bankruptcy reached the worst of the assumptions "such a shock could be absorbed" . However, the banks suffered on the stock exchange, due to a sentence of the president of the council that was partly misunderstood. again, and always in Naples as the first time on eni and enel, berlusconi let himself run away with open stock exchange comments on listed companies. According to the official statement, he said: "Maybe two or three banks in addition to unicredit will have advantages in increasing their capital, naturally finding the means on the market." In the first press headlines, the prices of the major banks fell, and then they returned a little later. the clearing up on the financial markets confirmed yesterday with the tyron below 5% of the three-month euribor rate, reference point for variable-rate home loans. the Italian banks, assures the governor, "have only partially shared errors and distortions" of the world financial system, originated mainly in the United States. of the European standards "banca d'italia has consistently given a strict interpretation." Dragons is well aware that public opinion tends to involve central banks in reproach. makes it clear that this can be justified in the uses, where there has been a "capture of the regulator" (in simple terms wall street influenced too much the government and the federal reserve) and in other countries; it is not in the euro area and especially in Italy. "alarms, over time, were not lacking," he recalls: "not least those who speak to you had repeatedly drawn attention to the imbalances of the international financial system," in several interventions, especially in autumn 2006; the trouble is that "in quiet times the warnings are often ignored." "They could not be predicted - he summarizes - neither the moment, nor the precise mechanism, nor the scale of the crisis; but one could well see the tensions that were accumulating." banks or other intermediaries who have given Lehman Brothers securities savers "will not have to leave them alone." new rules on transparency in the relationship between banks and customers will be ready at the beginning of next year. in the world, better regulation of derivatives and other innovative financial products will be needed to clean up. new rules will have to prevent banks from taking risks that are too exposed to their capital. "All in all, Italy does not come out badly" from the financial crisis, the governor concludes; but the effects of the crisis on the real economy "add to pre-existing structural weaknesses." The same judgment comes from the International Monetary Fund, which confirms the forecast decline in gross product both in 2008 (-0.1%) and in 2009 (-0.2%). but to react with state aid would not be the right answer, warns the head of the European department of the fmi alessandro leipold: "better liberalisations."</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>Observation date: 2008-10-22 00:00:00. . the words of the governor Stefano lepri roma the financial crisis begins to pass on to the enterprises and the families; for now the credit paid by the banks has not diminished, says the governor of the bank of italia mario dragons, "the situation, however, can change quickly." consumption is falling. After the decline of the product in the second quarter, "negative signals for the next quarters" arrive. to stem the negative effects, silvio berlusconi has accepted the proposal of the confindustria to open a discussion table between government, enterprises and banks. It will call him just back from the trip to China: "we ask that banks do not miss their support for investment and consumption." The promise is to find "important funds" in the budget. and Minister Claudio Scajola added: state guarantees on corporate debts are being studied, as is the case with banks. Dragons in his audition to the Senate first wanted to reassure the Italian banks: "thanks to strict laws and a firm vigilance action, there is not that extended 'banking system shadow' in which elsewhere the crisis has found origin and food" . today "the capitalisation of the major Italian banks remains sufficient" , even if the losses from the Lehman bankruptcy reached the worst of the assumptions "such a shock could be absorbed" . However, the banks suffered on the stock exchange, due to a sentence of the president of the council that was partly misunderstood. again, and always in Naples as the first time on eni and enel, Berlusconi let himself run away with open stock exchange comments on listed companies. According to the official statement, he said: "Maybe two or three banks in addition to unicredit will have advantages in increasing their capital, naturally finding the means on the market." In the first press headlines, the prices of the major banks fell, and then they returned a little later. the clearing up on the financial markets confirmed yesterday with the tyron below 5% of the three-month euribor rate, reference point for variable-rate home loans. the Italian banks, assures the governor, "have only partially shared errors and distortions" of the world financial system, originated mainly in the United States. the European standards "the Italian bank has consistently given a strict interpretation." Dragons is well aware that public opinion tends to involve central banks in reproach. makes it clear that this can be justified in the uses, where there has been a "capture of the regulator" (in simple terms wall street influenced too much the government and the federal reserve) and in other countries; it is not in the euro area and especially in Italy. "alarms, over time, were not lacking," he recalls: "not least those who speak to you had repeatedly drawn attention to the imbalances of the international financial system," in several interventions, especially in autumn 2006; the trouble is that "in quiet times the warnings are often ignored." "They could not be predicted - he summarizes - neither the moment, nor the precise mechanism, nor the scale of the crisis; but one could well see the tensions that were accumulating." banks or other intermediaries who have given Lehman Brothers securities savers "will not have to leave them alone." new rules on transparency in the relationship between banks and customers will be ready at the beginning of next year. in the world, better regulation of derivatives and other innovative financial products will be needed to clean up. new rules will have to prevent banks from taking risks that are too exposed to their capital. "All in all, Italy does not come out badly" from the financial crisis, the governor concludes; but the effects of the crisis on the real economy "add to pre-existing structural weaknesses." The same judgment comes from the International Monetary Fund, which confirms the forecast decline in gross product both in 2008 (-0.1%) and in 2009 (-0.2%). but to react with state aid would not be the right answer, warns the head of the European department of fmi alessandro leiold: "better liberalisations."</t>
+          <t>Observation date: 2008-10-22 00:00:00. . the words of the governor Stefano hari roma the financial crisis begins to pass on to the enterprises and the families; for now the credit paid by the banks has not diminished, says the governor of the bank of Italy mario draghi, "the situation, however, can change quickly." consumption is falling. After the decline of the product in the second quarter, "negative signals for the next quarters" arrive. To stem the negative effects, silvio berlusconi has accepted the Confindustria's proposal to open a discussion table between government, business and banks. It will call him just back from the trip to China: "we ask that banks do not miss their support for investment and consumption." The promise is to find "important funds" in the budget. and Minister claudio scajola added: state guarantees on corporate debts are being studied, as is the case with banks. Dragons in his audition to the Senate first wanted to reassure the Italian banks: "thanks to strict laws and a firm vigilance action, there is not that extended 'banking system shadow' in which elsewhere the crisis has found origin and food" . today "the capitalisation of the major Italian banks remains sufficient" , even if the losses from the Lehman bankruptcy reached the worst of the assumptions "such a shock could be absorbed" . However, the banks suffered on the stock exchange, due to a sentence of the president of the council that was partly misunderstood. again, and always in Naples as the first time on eni and enel, berlusconi let himself run away with open stock exchange comments on listed companies. According to the official statement, he said: "Maybe two or three banks in addition to unicredit will have advantages in increasing their capital, naturally finding the means on the market." In the first press headlines, the prices of the major banks fell, and then they returned a little later. the clearing up on the financial markets confirmed yesterday with the tyron below 5% of the three-month euribor rate, reference point for variable-rate home loans. the Italian banks, assures the governor, "have only partially shared errors and distortions" of the world financial system, originated mainly in the United States. of the European standards "banca d'italia has consistently given a strict interpretation." Dragons is well aware that public opinion tends to involve central banks in reproach. makes it clear that this can be justified in the uses, where there has been a "capture of the regulator" (in simple terms wall street influenced too much the government and the federal reserve) and in other countries; it is not in the euro area and especially in Italy. "alarms, over time, were not lacking," he recalls: "not least those who speak to you had repeatedly drawn attention to the imbalances of the international financial system," in several interventions, especially in autumn 2006; the trouble is that "in quiet times the warnings are often ignored." "They could not be predicted - he summarizes - neither the moment, nor the precise mechanism, nor the scale of the crisis; but one could well see the tensions that were accumulating." banks or other intermediaries who have given Lehman Brothers securities savers "will not have to leave them alone." new rules on transparency in the relationship between banks and customers will be ready at the beginning of next year. in the world, better regulation of derivatives and other innovative financial products will be needed to clean up. new rules will have to prevent banks from taking risks that are too exposed to their capital. "All in all, Italy does not come out badly" from the financial crisis, the governor concludes; but the effects of the crisis on the real economy "add to pre-existing structural weaknesses." The same judgment comes from the International Monetary Fund, which confirms the forecast decline in gross product both in 2008 (-0.1%) and in 2009 (-0.2%). but to react with state aid would not be the right answer, warns the head of the European department of the fmi alessandro leipold: "better liberalisations."</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>['Stefano Lepri (Governor of Roma) stated that the financial crisis is passing on to enterprises and families.', 'Mario Dragons (Governor of the Bank of Italia) stated that credit paid by the banks has not diminished for now.', 'Mario Dragons stated that the situation can change quickly.', 'Consumption is falling.', 'The product declined in the second quarter.', 'Negative signals for the next quarters arrived after the decline of the product in the second quarter.', 'To stem negative effects, Silvio Berlusconi accepted the proposal of Confindustria.', 'The proposal was to open a discussion table between government, enterprises, and banks.', 'Minister Claudio Scajola added that state guarantees on corporate debts are being studied.', 'Mario Dragons reassured the Italian banks during the audition to the Senate.', 'Mario Dragons stated that the capitalization of the major Italian banks remains sufficient on 2008-10-22.', 'Mario Dragons stated that the Italian banks could absorb a shock, even if losses from the Lehman bankruptcy reached the worst assumptions.', 'The banks suffered on the stock exchange due to a sentence of the President of the Council that was partly misunderstood.', 'Silvio Berlusconi made open stock exchange comments on listed companies in Naples.', 'Silvio Berlusconi stated that two or three banks, in addition to Unicredit, might have advantages in increasing their capital.', 'The prices of the major banks fell in the first press headlines.', 'The prices of the major banks returned later.', 'The clearing up on the financial markets confirmed on 2008-10-21 that the yield was below 5% of the three-month Euribor rate.', 'Mario Dragons assured that the Italian banks have only partially shared errors and distortions of the world financial system.', 'Mario Dragons stated that the world financial system errors and distortions originated mainly in the United States.', 'Mario Dragons stated that the Italian bank has consistently given a strict interpretation of European standards.', 'Mario Dragons stated that the public opinion tendency to involve central banks in reproach is not present in the euro area or Italy.', 'Mario Dragons recalled that warnings about the imbalances of the international financial system were repeatedly given in several interventions, especially in autumn 2006.', 'Mario Dragons summarized that while the moment, mechanism, and scale of the crisis could not be predicted, the accumulating tensions were visible.', 'New rules on transparency in the relationship between banks and customers will be ready at the beginning of next year.', 'Better regulation of derivatives and other innovative financial products will be needed globally.', 'New rules must prevent banks from taking risks that are too exposed to their capital.', 'Mario Dragons concluded that the effects of the crisis on the real economy add to pre-existing structural weaknesses.', 'The International Monetary Fund confirmed a forecast decline in gross product of -0.1% in 2008.', 'Alessandro Leiold (head of the European department of IMF) warned that reacting with state aid would not be the right answer.', 'Alessandro Leiold recommended better liberalizations.']</t>
+          <t>['Mario Draghi, the governor of the Bank of Italy, stated that the financial crisis was passing to enterprises and families.', 'Mario Draghi stated that the credit paid by the banks had not diminished for now.', 'Mario Draghi stated that the situation could change quickly.', 'Consumption is falling.', 'The product declined in the second quarter.', 'Negative signals for the next quarters arrived.', "Silvio Berlusconi accepted Confindustria's proposal.", 'The proposal was to open a discussion table between government, business, and banks.', 'Claudio Scajola added that state guarantees on corporate debts are being studied.', 'Mario Draghi reassured the Italian banks during the audition to the Senate.', 'Mario Draghi stated that the capitalization of the major Italian banks remains sufficient on 2008-10-22.', 'Mario Draghi stated that the major Italian banks could absorb a shock, even if losses from the Lehman bankruptcy reached the worst assumptions.', 'The banks suffered on the stock exchange due to a sentence of the president of the council.', 'Silvio Berlusconi made open stock exchange comments on listed companies in Naples.', 'Silvio Berlusconi stated that two or three banks, in addition to Unicredit, might have advantages in increasing their capital.', 'The clearing up on the financial markets confirmed on 2008-10-21 that the Euribor rate was below 5%.', 'Mario Draghi assured that the Italian banks partially shared errors and distortions of the world financial system.', "Mario Draghi stated that the world financial system's errors and distortions originated mainly in the United States.", 'Mario Draghi recalled that alarms regarding the imbalances of the international financial system were not lacking.', 'Mario Draghi noted that the warnings were often ignored in quiet times.', 'Banks or other intermediaries who gave Lehman Brothers securities savers will not have to leave them alone.', 'New rules on transparency in the relationship between banks and customers will be ready at the beginning of next year.', 'Better regulation of derivatives and other innovative financial products will be needed globally.', 'New rules must prevent banks from taking risks too exposed to their capital.', 'Mario Draghi concluded that Italy does not come out badly from the financial crisis.', 'The effects of the crisis on the real economy add to pre-existing structural weaknesses.', 'The International Monetary Fund confirmed a forecast decline in gross product in 2008 (-0.1%).', 'Alessandro Leipold warned that reacting with state aid would not be the right answer.', 'Alessandro Leipold advised better liberalizations.']</t>
         </is>
       </c>
     </row>
@@ -1110,17 +1110,17 @@
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr">
         <is>
-          <t>. They lower mortgage applications, raise the requirements to obtain them, and increase the credit crunch. The latter, explains goldman sachs in a report is the most intense since the sovereign debt crisis. The increase in interest rates by the European Central Bank (ECB) is beginning to impact on households and businesses in a substantial way. According to the last francoforte bank lending survey, in the fourth quarter of 2022, the contraction in demand for housing loans, minus 21%, was the strongest ever recorded, and demand for consumer credit and other loans to households decreased sharply in net terms, although to a lesser extent than for building loans. a scenario that, according to goldman sachs, represents a substantial further tightening of the credit standards (i.e. those applied to households and businesses), on which the uncertain prospects of the economy weigh mainly but to which the cost of funds and the liquidity position contribute more and more. read also-hard line of the fed for the whole 2023 bce rates, today is the day of the hawks the situation is destined to worsen along with the rises of the cost of the money. As the ECB explains, the net decline in demand for real estate loans was mainly determined by the general level of interest rates, the lower consumer confidence and the deterioration of the prospects of the real estate market. In the first quarter of 2023, banks forecast a further net decrease in demand for loans to enterprises. For loans to households, notes francoforte, banks estimate a persistent and strong net decline in demand for the first quarter of 2023. a picture also confirmed by goldman sachs, who expects a decrease in the credit concession and a reduction in demand, both for personal loans and loans, of equal magnitude, compared to what observed in the last four months of the year. Unlike the crisis that hit the eurozone a decade ago, in this case the phenomenon is spread evenly across the euro area.</t>
+          <t>. They lower mortgage applications, raise the requirements to obtain them, and increase the credit crunch. The latter, explains goldman sachs in a report is the most intense since the sovereign debt crisis. the increase in interest rates by the banca centrale europea (bce) begins to impact on households and businesses in a substantial way. According to the last francoforte bank lending survey, in the fourth quarter of 2022, the contraction in demand for housing loans, minus 21%, was the strongest ever recorded, and demand for consumer credit and other loans to households decreased sharply in net terms, although to a lesser extent than for building loans. a scenario that, according to goldman sachs, represents a substantial further tightening of the credit standards (i.e. those applied to households and enterprises), on which the uncertain prospects of the economy mainly weigh but to which the cost of the funds and the liquidity position contribute more and more. read also-hard line of the fed for the whole 2023 bce rates, today is the day of the hawks the situation is destined to worsen along with the rises of the cost of the money. As the ECB explains, the net decline in demand for real estate loans was mainly determined by the general level of interest rates, the lower consumer confidence and the deterioration of the prospects of the real estate market. In the first quarter of 2023, banks forecast a further net decrease in demand for loans to enterprises. For loans to households, notes francoforte, banks estimate a persistent and strong net decline in demand for the first quarter of 2023. a picture also confirmed by goldman sachs, which expects a decrease in the credit concession and a reduction in demand, both for personal loans and loans, of equal magnitude, compared to what observed in the last four months of the year. Unlike the crisis that hit the eurozone a decade ago, in this case the phenomenon is spread evenly across the euro area.</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>Observation date: 2023-02-02 00:00:00. . They lower mortgage applications, raise the requirements to obtain them, and increase the credit crunch. The latter, explains goldman sachs in a report is the most intense since the sovereign debt crisis. The increase in interest rates by the European Central Bank (ECB) is beginning to impact on households and businesses in a substantial way. According to the last francoforte bank lending survey, in the fourth quarter of 2022, the contraction in demand for housing loans, minus 21%, was the strongest ever recorded, and demand for consumer credit and other loans to households decreased sharply in net terms, although to a lesser extent than for building loans. a scenario that, according to goldman sachs, represents a substantial further tightening of the credit standards (i.e. those applied to households and businesses), on which the uncertain prospects of the economy weigh mainly but to which the cost of funds and the liquidity position contribute more and more. read also-hard line of the fed for the whole 2023 bce rates, today is the day of the hawks the situation is destined to worsen along with the rises of the cost of the money. As the ECB explains, the net decline in demand for real estate loans was mainly determined by the general level of interest rates, the lower consumer confidence and the deterioration of the prospects of the real estate market. In the first quarter of 2023, banks forecast a further net decrease in demand for loans to enterprises. For loans to households, notes francoforte, banks estimate a persistent and strong net decline in demand for the first quarter of 2023. a picture also confirmed by goldman sachs, who expects a decrease in the credit concession and a reduction in demand, both for personal loans and loans, of equal magnitude, compared to what observed in the last four months of the year. Unlike the crisis that hit the eurozone a decade ago, in this case the phenomenon is spread evenly across the euro area.</t>
+          <t>Observation date: 2023-02-02 00:00:00. . They lower mortgage applications, raise the requirements to obtain them, and increase the credit crunch. The latter, explains goldman sachs in a report is the most intense since the sovereign debt crisis. the increase in interest rates by the banca centrale europea (bce) begins to impact on households and businesses in a substantial way. According to the last francoforte bank lending survey, in the fourth quarter of 2022, the contraction in demand for housing loans, minus 21%, was the strongest ever recorded, and demand for consumer credit and other loans to households decreased sharply in net terms, although to a lesser extent than for building loans. a scenario that, according to goldman sachs, represents a substantial further tightening of the credit standards (i.e. those applied to households and enterprises), on which the uncertain prospects of the economy mainly weigh but to which the cost of the funds and the liquidity position contribute more and more. read also-hard line of the fed for the whole 2023 bce rates, today is the day of the hawks the situation is destined to worsen along with the rises of the cost of the money. As the ECB explains, the net decline in demand for real estate loans was mainly determined by the general level of interest rates, the lower consumer confidence and the deterioration of the prospects of the real estate market. In the first quarter of 2023, banks forecast a further net decrease in demand for loans to enterprises. For loans to households, notes francoforte, banks estimate a persistent and strong net decline in demand for the first quarter of 2023. a picture also confirmed by goldman sachs, which expects a decrease in the credit concession and a reduction in demand, both for personal loans and loans, of equal magnitude, compared to what observed in the last four months of the year. Unlike the crisis that hit the eurozone a decade ago, in this case the phenomenon is spread evenly across the euro area.</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>['Mortgage applications are being lowered.', 'Requirements to obtain mortgages are being raised.', 'The credit crunch is increasing.', 'Goldman Sachs explained in a report that the current credit crunch is the most intense since the sovereign debt crisis.', 'The increase in interest rates by the European Central Bank (ECB) is substantially impacting households.', 'According to the last Francoforte bank lending survey, the contraction in demand for housing loans was minus 21% in the fourth quarter of 2022.', 'Demand for consumer credit and other loans to households decreased sharply in net terms in the fourth quarter of 2022.', 'The decrease in demand for consumer credit and other loans to households was less severe than the decrease for building loans.', 'Goldman Sachs stated that the scenario represents a substantial further tightening of credit standards applied to households and businesses.', 'The cost of funds and the liquidity position are contributing more and more to the tightening of credit standards.', 'The European Central Bank (ECB) explained that the net decline in demand for real estate loans was determined by the general level of interest rates.', 'The net decline in demand for real estate loans was determined by lower consumer confidence.', 'The net decline in demand for real estate loans was determined by the deterioration of the prospects of the real estate market.', 'Banks forecast a further net decrease in demand for loans to enterprises in the first quarter of 2023.', 'Francoforte notes that banks estimate a persistent and strong net decline in demand for loans to households in the first quarter of 2023.', 'Goldman Sachs expects a decrease in the credit concession.', 'Goldman Sachs expects a reduction in demand for loans of equal magnitude to personal loans.', 'The reduction in demand is compared to what was observed in the last four months of the year.', 'The current phenomenon is spread evenly across the euro area.', 'The current phenomenon contrasts with the crisis that hit the eurozone a decade ago.']</t>
+          <t>['Financial Authorities lower mortgage applications.', 'Financial Authorities raise the requirements to obtain mortgage applications.', 'Financial Authorities increase the credit crunch.', 'Goldman Sachs explains in a report that the credit crunch is the most intense since the sovereign debt crisis.', 'The increase in interest rates by the Banca Centrale Europea (BCE) begins to impact households in a substantial way.', 'According to the last Francoforte Bank Lending Survey, the contraction in demand for housing loans was minus 21% in the fourth quarter of 2022.', 'According to the last Francoforte Bank Lending Survey, demand for consumer credit and other loans to households decreased sharply in net terms.', 'The decrease in demand for consumer credit and other loans to households was less than the decrease for building loans.', 'Goldman Sachs states that the scenario represents a substantial further tightening of the credit standards applied to households and enterprises.', 'The cost of funds and the liquidity position contribute more and more to the tightening of credit standards.', 'The situation is destined to worsen along with the rises of the cost of money.', 'The ECB explains that the net decline in demand for real estate loans was mainly determined by the deterioration of the prospects of the real estate market.', 'In the first quarter of 2023, banks forecast a further net decrease in demand for loans to enterprises.', 'Francoforte notes that banks estimate a persistent and strong net decline in demand for loans to households in the first quarter of 2023.', 'Goldman Sachs expects a decrease in the credit concession.', 'Goldman Sachs expects a reduction in demand for loans of equal magnitude to personal loans.', 'The expected reduction in demand for personal loans and loans is compared to the last four months of the year.', 'The current phenomenon is spread evenly across the euro area.', 'The current phenomenon is different from the crisis that hit the eurozone a decade ago.']</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: TranslationService now can evaluate news Sentiment
+ removed useless env vars for MarianMT
+ overloaded the _translate_single_text() method to be compatible for news with and without sentiment
</commit_message>
<xml_diff>
--- a/data/Annotazioni_1_with_factoids.xlsx
+++ b/data/Annotazioni_1_with_factoids.xlsx
@@ -542,25 +542,17 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Pensioners, beneficiaries of spousal support following divorce, and landlords of rental properties may attempt to avoid being overwhelmed by the rapid increase in prices. However, public and private employees (unless specific contractual agreements exist) and the self-employed will see their salaries stagnate. Indeed, as Istat explained a few days ago, with contractual wages growing by only 0.8% and an inflation rate of 5.2%, this translates to a loss of purchasing power equivalent to nearly five percentage points this year. However, this protection is not universal, and the outlook remains concerning.
-The law, for example, provides for the revaluation of spousal support, in the event of separation or divorce, with the aim of protecting the recipient by adjusting the amount owed to the economically weaker spouse or children according to the average cost of living. This revaluation must be carried out every year according to Istat indices and must be applied always and forever, regardless of whether the spouses agreed to it or if the judge ruled on it in the separation or divorce decree. For the revaluation, the Consumer Price Index for working and salaried households is used, taking as reference the index published by Istat relative to the month of the first payment of the spousal support decided by the court in the previous year. In case of failure to adjust, the rule also provides for the possibility of claiming arrears for the last 5 years.
-Even pensioners will have a protective shield. Since this year, the indexation mechanism has been reintroduced, which revalues pension amounts for different brackets and tiers. Thus, pensioners who receive a monthly payment up to 4 times the social allowance (about 2,000 euros) will receive a full revaluation of the amount relative to inflation; pensioners who receive between 4 and 5 times the allowance will receive a 90% increase relative to inflation; and pensioners who receive more than 5 times the social allowance will receive a 75% increase relative to inflation. Istat has established that, for this year, the inflation index on which the adjustments will be based, however, refers to 2021, and will be 1.9 percent. But in 2023, the payments will recover the price growth recorded in 2022, and the revaluation, based on current estimates, could reach around 7%.
-Property owners can also link their rental payments to the trend of inflation, while, regarding liquidations, the rules provide that the TFR (Trattamento di Fine Rapporto, or Italian severance pay), excluding the amount accrued in the current year, will be increased every year by applying a fixed rate of 1.5% and 75% of the increase in the Consumer Price Index for working and salaried households (3/4 of the inflation rate), determined by Istat, relative to the month of December of the previous year. In case of applying the revaluation rate for fractions of a year, the increase in the Istat index is that resulting in the month of termination of the employment relationship compared to that of December of the previous year. Example: if inflation is at 2%: 75% equals 1.5%, to which the fixed rate is added. Therefore, the TFR must be revalued by 3%, equal to 1.5% plus 1.5%.
-Michele di Branco</t>
+          <t>Pensioners, beneficiaries of maintenance payments following divorce, and landlords can try to avoid being overwhelmed by the crazy run of prices. However, public and private employees (unless there are specific contractual agreements) and the self-employed will see their wages stagnate. In fact, as Istat explained a few days ago, with contractual wages growing by only 0.8% and an inflation rate of 5.2%, there will be a loss of purchasing power of nearly five points this year. The shield, however, is not for everyone, and, as stated, things will not go well for all. The law, for example, provides for the revaluation of maintenance payments in the event of separation or divorce, in order to protect the recipient by adjusting the amount owed to the economically weaker spouse or children according to the average cost of living. This revaluation must be carried out every year according to Istat indices and must be applied always and forever, regardless of whether the spouses agreed to it or if the judge ruled on the separation or divorce. For revaluation, the Consumer Price Index (CPI) for working-class families is used, referencing the index published by Istat relative to the month of the first payment of the maintenance payment decided by the court in the previous year. In case of failure to adjust, the rule also provides for the possibility of claiming back pay for the last 5 years. Even pensioners will have a protective shield. Since this year, the indexation mechanism has been reintroduced, revaluing pension amounts for different tiers and brackets. Thus, pensioners who receive a monthly allowance up to 4 times the social allowance (about 2,000 euros) will receive a full revaluation of the amount relative to inflation; pensioners who receive between 4 and 5 times the allowance will receive a 90% increase relative to inflation; and pensioners who receive more than 5 times the social allowance will receive a 75% increase relative to inflation. Istat has established that, for this year, the inflation index used for these adjustments, however, refers to 2021, and will be 1.9 percent. But in 2023, the allowances will recover the price growth recorded in 2022, and the revaluation, based on current estimates, could reach around 7%. Property owners can also link their rental payments to inflation, while, regarding severance pay, the rules provide that the TFR (end-of-service benefit), excluding the amount accrued in the current year, will be increased every year by applying a fixed rate of 1.5% and 75% of the increase in the CPI for working-class families (3/4 of the inflation rate), determined by Istat, relative to the month of December of the previous year. In case of applying the revaluation rate for fractions of a year, the increase in the Istat index is that resulting in the month the employment relationship ceases compared to that of December of the previous year. Example: if inflation is at 2%: 75% equals 1.5%, to which the fixed rate is added. Therefore, the TFR must be revalued by 3%, equal to 1.5% plus 1.5%. Michele di Branco</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>Observation date: 2022-07-02 00:00:00. Pensioners, beneficiaries of spousal support following divorce, and landlords of rental properties may attempt to avoid being overwhelmed by the rapid increase in prices. However, public and private employees (unless specific contractual agreements exist) and the self-employed will see their salaries stagnate. Indeed, as Istat explained a few days ago, with contractual wages growing by only 0.8% and an inflation rate of 5.2%, this translates to a loss of purchasing power equivalent to nearly five percentage points this year. However, this protection is not universal, and the outlook remains concerning.
-The law, for example, provides for the revaluation of spousal support, in the event of separation or divorce, with the aim of protecting the recipient by adjusting the amount owed to the economically weaker spouse or children according to the average cost of living. This revaluation must be carried out every year according to Istat indices and must be applied always and forever, regardless of whether the spouses agreed to it or if the judge ruled on it in the separation or divorce decree. For the revaluation, the Consumer Price Index for working and salaried households is used, taking as reference the index published by Istat relative to the month of the first payment of the spousal support decided by the court in the previous year. In case of failure to adjust, the rule also provides for the possibility of claiming arrears for the last 5 years.
-Even pensioners will have a protective shield. Since this year, the indexation mechanism has been reintroduced, which revalues pension amounts for different brackets and tiers. Thus, pensioners who receive a monthly payment up to 4 times the social allowance (about 2,000 euros) will receive a full revaluation of the amount relative to inflation; pensioners who receive between 4 and 5 times the allowance will receive a 90% increase relative to inflation; and pensioners who receive more than 5 times the social allowance will receive a 75% increase relative to inflation. Istat has established that, for this year, the inflation index on which the adjustments will be based, however, refers to 2021, and will be 1.9 percent. But in 2023, the payments will recover the price growth recorded in 2022, and the revaluation, based on current estimates, could reach around 7%.
-Property owners can also link their rental payments to the trend of inflation, while, regarding liquidations, the rules provide that the TFR (Trattamento di Fine Rapporto, or Italian severance pay), excluding the amount accrued in the current year, will be increased every year by applying a fixed rate of 1.5% and 75% of the increase in the Consumer Price Index for working and salaried households (3/4 of the inflation rate), determined by Istat, relative to the month of December of the previous year. In case of applying the revaluation rate for fractions of a year, the increase in the Istat index is that resulting in the month of termination of the employment relationship compared to that of December of the previous year. Example: if inflation is at 2%: 75% equals 1.5%, to which the fixed rate is added. Therefore, the TFR must be revalued by 3%, equal to 1.5% plus 1.5%.
-Michele di Branco</t>
+          <t>Observation date: 2022-07-02 00:00:00. Pensioners, beneficiaries of maintenance payments following divorce, and landlords can try to avoid being overwhelmed by the crazy run of prices. However, public and private employees (unless there are specific contractual agreements) and the self-employed will see their wages stagnate. In fact, as Istat explained a few days ago, with contractual wages growing by only 0.8% and an inflation rate of 5.2%, there will be a loss of purchasing power of nearly five points this year. The shield, however, is not for everyone, and, as stated, things will not go well for all. The law, for example, provides for the revaluation of maintenance payments in the event of separation or divorce, in order to protect the recipient by adjusting the amount owed to the economically weaker spouse or children according to the average cost of living. This revaluation must be carried out every year according to Istat indices and must be applied always and forever, regardless of whether the spouses agreed to it or if the judge ruled on the separation or divorce. For revaluation, the Consumer Price Index (CPI) for working-class families is used, referencing the index published by Istat relative to the month of the first payment of the maintenance payment decided by the court in the previous year. In case of failure to adjust, the rule also provides for the possibility of claiming back pay for the last 5 years. Even pensioners will have a protective shield. Since this year, the indexation mechanism has been reintroduced, revaluing pension amounts for different tiers and brackets. Thus, pensioners who receive a monthly allowance up to 4 times the social allowance (about 2,000 euros) will receive a full revaluation of the amount relative to inflation; pensioners who receive between 4 and 5 times the allowance will receive a 90% increase relative to inflation; and pensioners who receive more than 5 times the social allowance will receive a 75% increase relative to inflation. Istat has established that, for this year, the inflation index used for these adjustments, however, refers to 2021, and will be 1.9 percent. But in 2023, the allowances will recover the price growth recorded in 2022, and the revaluation, based on current estimates, could reach around 7%. Property owners can also link their rental payments to inflation, while, regarding severance pay, the rules provide that the TFR (end-of-service benefit), excluding the amount accrued in the current year, will be increased every year by applying a fixed rate of 1.5% and 75% of the increase in the CPI for working-class families (3/4 of the inflation rate), determined by Istat, relative to the month of December of the previous year. In case of applying the revaluation rate for fractions of a year, the increase in the Istat index is that resulting in the month the employment relationship ceases compared to that of December of the previous year. Example: if inflation is at 2%: 75% equals 1.5%, to which the fixed rate is added. Therefore, the TFR must be revalued by 3%, equal to 1.5% plus 1.5%. Michele di Branco</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>['Pensioners, beneficiaries of spousal support following divorce, and landlords of rental properties may attempt to avoid being overwhelmed by the rapid increase in prices.', 'Public and private employees (unless specific contractual agreements exist) and the self-employed will see their salaries stagnate.', 'Istat explained that contractual wages grew by 0.8%.', 'Istat explained that the inflation rate was 5.2%.', 'The combination of 0.8% wage growth and 5.2% inflation translates to a loss of purchasing power equivalent to nearly five percentage points on 2022-01-01.', 'The law provides for the revaluation of spousal support in the event of separation or divorce.', 'The revaluation aims to protect the recipient by adjusting the amount owed to the economically weaker spouse or children according to the average cost of living.', 'The revaluation must be carried out every year according to Istat indices.', 'The revaluation must be applied always and forever, regardless of the agreement of the spouses or the ruling of the judge.', 'The Consumer Price Index for working and salaried households is used for the revaluation.', 'The index used for revaluation is relative to the month of the first payment of the spousal support decided by the court in the previous year.', 'If spousal support fails to adjust, the rule allows claiming arrears for the last 5 years.', 'The indexation mechanism has been reintroduced since 2022-07-02.', 'The indexation mechanism revalues pension amounts for different brackets and tiers.', 'Pensioners receiving a monthly payment up to 4 times the social allowance (about 2,000 euros) will receive a full revaluation relative to inflation.', 'Pensioners receiving more than 5 times the social allowance will receive a 75% increase relative to inflation.', 'Istat established that the inflation index for the adjustments refers to 2021.', 'The inflation index established by Istat for the adjustments will be 1.9 percent.', 'In 2023, the payments will recover the price growth recorded in 2022.', 'The revaluation, based on current estimates, could reach around 7%.', 'Property owners can link their rental payments to the trend of inflation.', 'The rules for liquidations state that the TFR (Trattamento di Fine Rapporto, or Italian severance pay), excluding the amount accrued in the current year, will be increased every year.', 'The TFR increase is calculated by applying a fixed rate of 1.5% and 75% of the increase in the Consumer Price Index for working and salaried households.', 'The Consumer Price Index increase is determined by Istat relative to the month of December of the previous year.', 'If applying the revaluation rate for fractions of a year, the Istat index increase compares the month of termination of the employment relationship to December of the previous year.', 'If inflation is 2%, 75% equals 1.5%.', 'The TFR must be revalued by 3% (1.5% fixed rate + 1.5% calculated rate).']</t>
+          <t>['Public and private employees (unless there are specific contractual agreements) and the self-employed will see their wages stagnate.', 'Istat explained on 2022-06-28 that contractual wages grew by 0.8%.', 'Istat explained on 2022-06-28 that the inflation rate was 5.2%.', 'The combination of 0.8% wage growth and 5.2% inflation will result in a loss of purchasing power of nearly five points in 2022.', 'The law provides for the revaluation of maintenance payments following separation or divorce.', 'The revaluation protects the recipient by adjusting the amount owed to the economically weaker spouse or children according to the average cost of living.', 'The revaluation of maintenance payments must be carried out every year according to Istat indices.', 'The revaluation must be applied always and forever, regardless of whether the spouses agreed to it or if the judge ruled on the separation or divorce.', 'The Consumer Price Index (CPI) for working-class families is used for maintenance revaluation.', 'The CPI references the index published by Istat relative to the month of the first payment of the maintenance payment decided by the court in the previous year.', 'If adjustment fails, the rule allows claiming back pay for the last 5 years.', 'The indexation mechanism for pensions was reintroduced in 2022.', 'Pensioners receiving a monthly allowance up to 4 times the social allowance (about 2,000 euros) will receive a full revaluation of the amount relative to inflation.', 'Pensioners receiving between 4 and 5 times the social allowance will receive a 90% increase relative to inflation.', 'Istat established that the inflation index used for pension adjustments in 2022 refers to 2021 and will be 1.9 percent.', 'The allowances will recover the price growth recorded in 2022 in 2023.', 'The revaluation for pensions could reach around 7% based on current estimates.', 'Property owners can link their rental payments to inflation.', 'Rules regarding severance pay state that the TFR (end-of-service benefit), excluding the amount accrued in the current year, will be increased every year.', 'The TFR increase is calculated by applying a fixed rate of 1.5% and 75% of the increase in the CPI for working-class families (3/4 of the inflation rate), determined by Istat.', 'The TFR calculation references the month of December of the previous year.', 'If applying the revaluation rate for fractions of a year, the increase in the Istat index compares the month the employment relationship ceases to December of the previous year.']</t>
         </is>
       </c>
     </row>
@@ -618,35 +610,17 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>The government's move on the *imu* (local property tax) is being implemented, returning in a disguised form this December as an advance payment for the "service tax." The Treasury is searching for 3 billion [euros] to avoid the VAT increase scheduled for October, but this operation concerning the house tax is expected to arrive in November. Meanwhile, alarm bells are ringing at the *Quirinale*. The stability of the financial law is at risk. The consultations of President Napolitano with secretaries Alfano and Epifani are underway, while the *Pdl* threatens a new crisis.
-Regarding *Angela Merkel*, the German elections saw a clear winner in the popular vote. However, an electoral law that many insist on exporting to us will not allow her to govern alone. A new *Große Koalition* (Grand Coalition) thus looms on the horizon. The last one, the series, which ran in 2005, resulted from an agreement signed after weeks of negotiations. The legislative program was over 300 pages, exceeding in length even Prodi's 2006 electoral "manifesto." Like that one, it remained a dead letter. Our great coalition was born from a half-hour inauguration speech by the acting president. Everything was promised, with no budgetary constraints mentioned. Then came the same decision paralysis, albeit more animated than in Germany: furious arguments broadcast live on TV as soon as they had to confront budgetary constraints. Those do not forgive. Unlike the Germans, we cannot afford decision paralysis.
-The current government now acts only in the realm of dreams or through accounting maneuvers. The update note to the DEF (Stability Pact) presented a few days ago by our executive proposes macroeconomic scenarios straight out of a late summer dream. We should grow over the next three years at a rate double the potential rate, shattering the estimates of international organizations, without having done anything to make such a sharp change of pace possible. These scenarios contemplate the coexistence of high inflation (a GDP deflator of 2 percent), a further decline in household consumption, and rising unemployment. It is difficult to understand how these three phenomena can materialize simultaneously.
-Perhaps they will be used to draw tables in which the public debt-to-GDP ratio never rises above 130 percent of the gross domestic product, but these unrealistic scenarios cannot convince institutional fund managers to invest in our country. On the contrary, they risk weakening our negotiating position at the community level. We are already hearing the objections in *Bruxelles*: "If things are destined to go so well, why should we grant you the maneuvering space you ask for?"
-To the false optimism has been added financial engineering. There is talk of revaluing the shares held by banks at *Banca d'Italia*, a legacy from when banks were public. The banks are pleased to see their equity position strengthened. The Treasury is pleased to receive a contribution from the resulting capital gains. The taxpayers, however, are less pleased, as they will one day have to repurchase these shares because a central bank cannot be owned by private banks. They risk paying a very high price, as the cost will presumably be extremely elevated. This would be in the interest of both the banks and the Treasury. And there are no market references, so much so that a dedicated commission of experts has been established.
-While the country is burying its head in the sand with dreams and financial engineering, it risks falling, day after day, into the hands of the Troika, without us even realizing it. It was difficult to return from a debt of 120 percent. It is much more difficult to do so from a debt of 130 percent and rising.
-If this government does not want to be remembered for ceding national sovereignty, it must find a program agreement on the basis of which to open negotiations in *Bruxelles*. The agreement should be enshrined in the stability law. Its philosophy is to address emergencies with long-term reforms. For example, the refinancing of the *cassa integrazione in deroga* (derogatory redundancy fund) should contemplate the gradual phasing out of this institution, with wage supplements for those working for less than 5 euros per hour—a way to facilitate labor mobility and increase employment. Every new access to the *cassa in deroga* must be blocked, starting with that requested for former party employees by a very large parliamentary coalition. They will be able, like other workers, to access ordinary social safety nets.
-Another example: the VAT increase could be avoided, possibly restricted only to luxury goods, coupled with a reduction of the tax wedge, given that indirect taxes increase the difference between labor costs and the purchasing power of wages. There should then be measures to cut spending, which could be implemented gradually, but with already approved interventions.
-We could start by dismantling the bureaucracy created by the *Lega*'s federalism, which has created duplications, uncontrolled local spending, and an excess of centers of power. Some examples: how to justify the sponsorship offered by the *Regione Sardegna* to the *Cagliari* football team? What are the 45 port authorities for? And can the staffing levels of the prefectures be reduced, and the provinces truly abolished? It is unnecessary to point out that cutting these waste areas is politically costly.
-The steering committee (*cabina di regia*) should really serve to protect the government from the fierce attacks it will face from those affected by the cuts. With these measures included in the stability law, it is possible to open negotiations with *Bruxelles* that also contemplate deficits exceeding 3 percent in the coming years. But it will require a cohesive government—not a mere collection of parties whose survival is questioned every day.</t>
+          <t>The government's move on the IMU property tax is triggered, which returns in a disguised form this December, serving as an advance payment for a 'service tax.' The Treasury is scrambling for 3 billion [euros] to avoid the planned VAT increase in October, but this 'makeup operation' concerning the housing tax is expected to arrive in November. And now, alarm bells are ringing at the Quirinale [Prime Minister's residence]. The stability of the Finance Law is at risk. The President's consultations with Secretaries Alfano and Epifani take place while the PDL threatens another crisis. In Germany, Angela Merkel has seen a clear winner in the popular vote. However, an electoral law that many insist on exporting here will not allow her to govern alone. A new, large coalition thus looms on the horizon. The last one, the series, in 2005, resulted from an agreement signed after weeks of negotiations. The legislative program was over 300 pages, exceeding in length even Prodi's 2006 electoral manifesto. Like that, it remained dead letter. Our great coalition was born from a half-hour investiture speech by the acting president. Everything and more was promised, denying any budgetary constraints. Then came the same decision paralysis, albeit more animated than in Germany: furious arguments broadcast live on TV as soon as they had to confront budgetary constraints. Those do not forgive. Unlike the Germans, we cannot afford decision paralysis. The current government now acts only in the realm of dreams or in that of accounting tricks. The update note to the Stability Pact, presented a few days ago by our executive, proposes macroeconomic scenarios straight out of a late summer dream. We should grow in the next three years at a rate double the potential rate, shattering the estimates of international organizations, without having done anything to make such a sharp change of pace possible. These scenarios contemplate the coexistence of high inflation (a GDP deflator of 2 percent), a further drop in household consumption, and rising unemployment. It is difficult to understand how these three phenomena can materialize simultaneously. Perhaps they will be used to draw tables in which the public debt-to-GDP ratio never rises above 130 percent. But these unrealistic scenarios cannot convince institutional fund managers to invest in our country. On the contrary, they risk weakening our negotiating position at the community level. We are already hearing the objections in Brussels: 'If things are destined to go so well, why should we grant you the room for maneuver you ask for?' To the false optimism has been added accounting engineering. They plan to revalue the shares held by banks at the Bank of Italy, a legacy from when banks were public. The banks are pleased to see their equity position strengthened. The Treasury is pleased to receive a contribution from the realized capital gains. The taxpayers, however, are less pleased, as they will one day have to repurchase these shares because a central bank cannot be owned by private banks. They risk paying a very high price because the price will presumably be very high. This would be in the interest of both the banks and the Treasury. And there are no market references, so much so that a special commission of experts has been established. While they bury their heads in the sand with dreams and accounting engineering, the country risks ending, day after day, in the hands of the Troika, without us even realizing it. It was difficult to return from a debt of 120 percent. It is much more difficult to do so from a debt of 130 percent and rising. If this government does not want to be remembered for ceding national sovereignty, it must find a program agreement on the basis of which to open negotiations with Brussels. The agreement should be enshrined in the Stability Law. Its philosophy is to address emergencies with long-term reforms. For example, the refinancing of the temporary layoff fund should contemplate the gradual phasing out of this institution, with wage supplements for those working less than 5 euros per hour, a way to facilitate labor mobility and increase employment. Every new access to the temporary fund must be blocked, starting with that requested for former party employees by a very large parliamentary coalition. They will be able, like other workers, to access ordinary social safety nets. Another example: the VAT increase could be avoided, possibly restricted only to luxury goods, with a cut to the tax wedge, given that indirect taxes increase the difference between labor costs and purchasing power of wages. There should then be spending cut measures, which could be implemented gradually, but with already approved interventions. One could start by dismantling the bureaucracy created by the Lega's federalism, which has created duplications, uncontrolled local spending, and an excess of centers of power. Some examples: how to justify the sponsorship offered by the Sardinia region to the Cagliari football team? What are 45 port authorities for? And can the staffing levels of the prefectures be reduced, and the provinces truly abolished? It is unnecessary to point out that cutting these waste items is politically costly. The steering committee should really serve to protect the government from the fierce attacks it will face from those affected by the cuts. With these measures included in the Stability Law, it is possible to open negotiations with Brussels that also contemplate deficits exceeding 3 percent in the coming years. But it will require a cohesive government, not a collection whose survival is questioned every day.</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Observation date: 2013-09-25 00:00:00. The government's move on the *imu* (local property tax) is being implemented, returning in a disguised form this December as an advance payment for the "service tax." The Treasury is searching for 3 billion [euros] to avoid the VAT increase scheduled for October, but this operation concerning the house tax is expected to arrive in November. Meanwhile, alarm bells are ringing at the *Quirinale*. The stability of the financial law is at risk. The consultations of President Napolitano with secretaries Alfano and Epifani are underway, while the *Pdl* threatens a new crisis.
-Regarding *Angela Merkel*, the German elections saw a clear winner in the popular vote. However, an electoral law that many insist on exporting to us will not allow her to govern alone. A new *Große Koalition* (Grand Coalition) thus looms on the horizon. The last one, the series, which ran in 2005, resulted from an agreement signed after weeks of negotiations. The legislative program was over 300 pages, exceeding in length even Prodi's 2006 electoral "manifesto." Like that one, it remained a dead letter. Our great coalition was born from a half-hour inauguration speech by the acting president. Everything was promised, with no budgetary constraints mentioned. Then came the same decision paralysis, albeit more animated than in Germany: furious arguments broadcast live on TV as soon as they had to confront budgetary constraints. Those do not forgive. Unlike the Germans, we cannot afford decision paralysis.
-The current government now acts only in the realm of dreams or through accounting maneuvers. The update note to the DEF (Stability Pact) presented a few days ago by our executive proposes macroeconomic scenarios straight out of a late summer dream. We should grow over the next three years at a rate double the potential rate, shattering the estimates of international organizations, without having done anything to make such a sharp change of pace possible. These scenarios contemplate the coexistence of high inflation (a GDP deflator of 2 percent), a further decline in household consumption, and rising unemployment. It is difficult to understand how these three phenomena can materialize simultaneously.
-Perhaps they will be used to draw tables in which the public debt-to-GDP ratio never rises above 130 percent of the gross domestic product, but these unrealistic scenarios cannot convince institutional fund managers to invest in our country. On the contrary, they risk weakening our negotiating position at the community level. We are already hearing the objections in *Bruxelles*: "If things are destined to go so well, why should we grant you the maneuvering space you ask for?"
-To the false optimism has been added financial engineering. There is talk of revaluing the shares held by banks at *Banca d'Italia*, a legacy from when banks were public. The banks are pleased to see their equity position strengthened. The Treasury is pleased to receive a contribution from the resulting capital gains. The taxpayers, however, are less pleased, as they will one day have to repurchase these shares because a central bank cannot be owned by private banks. They risk paying a very high price, as the cost will presumably be extremely elevated. This would be in the interest of both the banks and the Treasury. And there are no market references, so much so that a dedicated commission of experts has been established.
-While the country is burying its head in the sand with dreams and financial engineering, it risks falling, day after day, into the hands of the Troika, without us even realizing it. It was difficult to return from a debt of 120 percent. It is much more difficult to do so from a debt of 130 percent and rising.
-If this government does not want to be remembered for ceding national sovereignty, it must find a program agreement on the basis of which to open negotiations in *Bruxelles*. The agreement should be enshrined in the stability law. Its philosophy is to address emergencies with long-term reforms. For example, the refinancing of the *cassa integrazione in deroga* (derogatory redundancy fund) should contemplate the gradual phasing out of this institution, with wage supplements for those working for less than 5 euros per hour—a way to facilitate labor mobility and increase employment. Every new access to the *cassa in deroga* must be blocked, starting with that requested for former party employees by a very large parliamentary coalition. They will be able, like other workers, to access ordinary social safety nets.
-Another example: the VAT increase could be avoided, possibly restricted only to luxury goods, coupled with a reduction of the tax wedge, given that indirect taxes increase the difference between labor costs and the purchasing power of wages. There should then be measures to cut spending, which could be implemented gradually, but with already approved interventions.
-We could start by dismantling the bureaucracy created by the *Lega*'s federalism, which has created duplications, uncontrolled local spending, and an excess of centers of power. Some examples: how to justify the sponsorship offered by the *Regione Sardegna* to the *Cagliari* football team? What are the 45 port authorities for? And can the staffing levels of the prefectures be reduced, and the provinces truly abolished? It is unnecessary to point out that cutting these waste areas is politically costly.
-The steering committee (*cabina di regia*) should really serve to protect the government from the fierce attacks it will face from those affected by the cuts. With these measures included in the stability law, it is possible to open negotiations with *Bruxelles* that also contemplate deficits exceeding 3 percent in the coming years. But it will require a cohesive government—not a mere collection of parties whose survival is questioned every day.</t>
+          <t>Observation date: 2013-09-25 00:00:00. The government's move on the IMU property tax is triggered, which returns in a disguised form this December, serving as an advance payment for a 'service tax.' The Treasury is scrambling for 3 billion [euros] to avoid the planned VAT increase in October, but this 'makeup operation' concerning the housing tax is expected to arrive in November. And now, alarm bells are ringing at the Quirinale [Prime Minister's residence]. The stability of the Finance Law is at risk. The President's consultations with Secretaries Alfano and Epifani take place while the PDL threatens another crisis. In Germany, Angela Merkel has seen a clear winner in the popular vote. However, an electoral law that many insist on exporting here will not allow her to govern alone. A new, large coalition thus looms on the horizon. The last one, the series, in 2005, resulted from an agreement signed after weeks of negotiations. The legislative program was over 300 pages, exceeding in length even Prodi's 2006 electoral manifesto. Like that, it remained dead letter. Our great coalition was born from a half-hour investiture speech by the acting president. Everything and more was promised, denying any budgetary constraints. Then came the same decision paralysis, albeit more animated than in Germany: furious arguments broadcast live on TV as soon as they had to confront budgetary constraints. Those do not forgive. Unlike the Germans, we cannot afford decision paralysis. The current government now acts only in the realm of dreams or in that of accounting tricks. The update note to the Stability Pact, presented a few days ago by our executive, proposes macroeconomic scenarios straight out of a late summer dream. We should grow in the next three years at a rate double the potential rate, shattering the estimates of international organizations, without having done anything to make such a sharp change of pace possible. These scenarios contemplate the coexistence of high inflation (a GDP deflator of 2 percent), a further drop in household consumption, and rising unemployment. It is difficult to understand how these three phenomena can materialize simultaneously. Perhaps they will be used to draw tables in which the public debt-to-GDP ratio never rises above 130 percent. But these unrealistic scenarios cannot convince institutional fund managers to invest in our country. On the contrary, they risk weakening our negotiating position at the community level. We are already hearing the objections in Brussels: 'If things are destined to go so well, why should we grant you the room for maneuver you ask for?' To the false optimism has been added accounting engineering. They plan to revalue the shares held by banks at the Bank of Italy, a legacy from when banks were public. The banks are pleased to see their equity position strengthened. The Treasury is pleased to receive a contribution from the realized capital gains. The taxpayers, however, are less pleased, as they will one day have to repurchase these shares because a central bank cannot be owned by private banks. They risk paying a very high price because the price will presumably be very high. This would be in the interest of both the banks and the Treasury. And there are no market references, so much so that a special commission of experts has been established. While they bury their heads in the sand with dreams and accounting engineering, the country risks ending, day after day, in the hands of the Troika, without us even realizing it. It was difficult to return from a debt of 120 percent. It is much more difficult to do so from a debt of 130 percent and rising. If this government does not want to be remembered for ceding national sovereignty, it must find a program agreement on the basis of which to open negotiations with Brussels. The agreement should be enshrined in the Stability Law. Its philosophy is to address emergencies with long-term reforms. For example, the refinancing of the temporary layoff fund should contemplate the gradual phasing out of this institution, with wage supplements for those working less than 5 euros per hour, a way to facilitate labor mobility and increase employment. Every new access to the temporary fund must be blocked, starting with that requested for former party employees by a very large parliamentary coalition. They will be able, like other workers, to access ordinary social safety nets. Another example: the VAT increase could be avoided, possibly restricted only to luxury goods, with a cut to the tax wedge, given that indirect taxes increase the difference between labor costs and purchasing power of wages. There should then be spending cut measures, which could be implemented gradually, but with already approved interventions. One could start by dismantling the bureaucracy created by the Lega's federalism, which has created duplications, uncontrolled local spending, and an excess of centers of power. Some examples: how to justify the sponsorship offered by the Sardinia region to the Cagliari football team? What are 45 port authorities for? And can the staffing levels of the prefectures be reduced, and the provinces truly abolished? It is unnecessary to point out that cutting these waste items is politically costly. The steering committee should really serve to protect the government from the fierce attacks it will face from those affected by the cuts. With these measures included in the Stability Law, it is possible to open negotiations with Brussels that also contemplate deficits exceeding 3 percent in the coming years. But it will require a cohesive government, not a collection whose survival is questioned every day.</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>["The government's move on the imu (local property tax) is being implemented on 2013-09-25.", 'The imu move will return in a disguised form in December 2013 as an advance payment for the "service tax."', 'The Treasury is searching for 3 billion euros.', 'The Treasury needs 3 billion euros to avoid the VAT increase scheduled for October 2013.', 'The operation concerning the house tax is expected to arrive in November 2013.', 'Alarm bells are ringing at the Quirinale.', 'The stability of the financial law is at risk.', 'Consultations of President Napolitano with secretaries Alfano and Epifani are underway.', 'The Pdl threatens a new crisis.', 'The German elections saw a clear winner in the popular vote for Angela Merkel.', 'An electoral law that many insist on exporting to Italy will not allow Angela Merkel to govern alone.', 'A new Große Koalition (Grand Coalition) looms on the horizon.', 'The last Große Koalition ran in 2005.', 'The legislative program of the last Große Koalition exceeded 300 pages.', 'The legislative program of the last Große Koalition was longer than Prodi\'s 2006 electoral "manifesto."', 'The great coalition was born from a half-hour inauguration speech by the acting president.', 'The great coalition promised everything without mentioning budgetary constraints.', 'The update note to the DEF (Stability Pact) was presented on 2013-09-20 by the executive.', 'The executive proposes macroeconomic scenarios for the Stability Pact.', 'The proposed scenarios suggest growth over the next three years at a rate double the potential rate.', 'The proposed scenarios shatter the estimates of international organizations.', 'The scenarios contemplate high inflation (a GDP deflator of 2 percent).', 'The scenarios contemplate a further decline in household consumption.', 'The scenarios contemplate rising unemployment.', "The scenarios risk weakening Italy's negotiating position at the community level.", 'Objections are being heard in Bruxelles regarding the proposed scenarios.', 'Financial engineering has been added to the false optimism.', "There is talk of revaluing the shares held by banks at Banca d'Italia.", 'The banks are pleased to see their equity position strengthened.', 'The Treasury is pleased to receive a contribution from the resulting capital gains.', 'Taxpayers will eventually have to repurchase the shares.', 'A central bank cannot be owned by private banks.', 'The cost of repurchasing the shares will presumably be extremely elevated.', 'A dedicated commission of experts has been established because there are no market references.', 'Italy risks falling into the hands of the Troika.', 'It was difficult to return from a debt of 120 percent.', 'It is much more difficult to return from a debt of 130 percent and rising.', 'The government must find a program agreement to open negotiations in Bruxelles.', 'The program agreement should be enshrined in the stability law.', 'The philosophy of the agreement is to address emergencies with long-term reforms.', 'The refinancing of the cassa integrazione in deroga should contemplate the gradual phasing out of this institution.', 'The phasing out should include wage supplements for those working for less than 5 euros per hour.', 'Blocking every new access to the cassa in deroga is necessary.', 'The VAT increase could be avoided, possibly restricted only to luxury goods.', 'The VAT increase could be coupled with a reduction of the tax wedge.', 'Measures to cut spending should be implemented gradually.', 'The steering committee (cabina di regia) should protect the government from fierce attacks.', 'Including these measures in the stability law allows negotiations with Bruxelles that contemplate deficits exceeding 3 percent.', 'Opening negotiations with Bruxelles requires a cohesive government.']</t>
+          <t>["The government's move on the IMU property tax is triggered.", 'The move on the IMU property tax returns in a disguised form in December 2013.', "The disguised form serves as an advance payment for a 'service tax.'", 'The Treasury is scrambling for 3 billion euros.', 'The Treasury needs the money to avoid the planned VAT increase in October 2013.', "A 'makeup operation' concerning the housing tax is expected to arrive in November 2013.", "Alarm bells are ringing at the Quirinale [Prime Minister's residence].", 'The stability of the Finance Law is at risk.', "The President's consultations with Secretaries Alfano and Epifani take place.", 'The PDL threatens another crisis.', 'In Germany, Angela Merkel saw a clear winner in the popular vote.', 'An electoral law that many insist on exporting here will not allow Angela Merkel to govern alone.', 'A new, large coalition looms on the horizon.', 'The last coalition in 2005 resulted from an agreement signed after weeks of negotiations.', 'The legislative program from 2005 was over 300 pages.', "The legislative program from 2005 exceeded in length even Prodi's 2006 electoral manifesto.", 'The legislative program from 2005 remained a dead letter.', 'The great coalition was born from a half-hour investiture speech by the acting president.', 'The current government acts only in the realm of dreams or in that of accounting tricks.', 'The executive presented an update note to the Stability Pact a few days ago.', 'The update note to the Stability Pact proposes macroeconomic scenarios.', 'The scenarios propose growth in the next three years at a rate double the potential rate.', 'The scenarios contemplate the coexistence of high inflation (a GDP deflator of 2 percent).', 'The scenarios contemplate a further drop in household consumption.', 'The scenarios contemplate rising unemployment.', 'The scenarios might be used to draw tables where the public debt-to-GDP ratio never rises above 130 percent.', 'The unrealistic scenarios cannot convince institutional fund managers to invest in the country.', 'The scenarios risk weakening the negotiating position of the country at the community level.', 'The plan involves revaluing the shares held by banks at the Bank of Italy.', 'The banks are pleased to see their equity position strengthened.', 'The Treasury is pleased to receive a contribution from the realized capital gains.', 'The taxpayers will one day have to repurchase these shares.', 'A central bank cannot be owned by private banks.', 'The taxpayers risk paying a very high price.', 'A special commission of experts has been established because there are no market references.', 'The country risks ending in the hands of the Troika.', 'It was difficult to return from a debt of 120 percent.', 'It is much more difficult to return from a debt of 130 percent and rising.', 'The government must find a program agreement to open negotiations with Brussels.', 'The program agreement should be enshrined in the Stability Law.', 'The philosophy of the Stability Law is to address emergencies with long-term reforms.', 'Refinancing the temporary layoff fund should contemplate the gradual phasing out of this institution.', 'The phasing out should include wage supplements for those working less than 5 euros per hour.', 'This measure aims to facilitate labor mobility and increase employment.', 'Every new access to the temporary fund must be blocked.', 'The blocking must start with the access requested for former party employees by a very large parliamentary coalition.', 'Former party employees will be able to access ordinary social safety nets.', 'The VAT increase could be restricted only to luxury goods.', 'The VAT increase could involve a cut to the tax wedge.', 'Indirect taxes increase the difference between labor costs and purchasing power of wages.', 'Spending cut measures should be implemented.', "Dismantling the bureaucracy created by the Lega's federalism is a potential spending cut measure.", 'The steering committee should protect the government from fierce attacks.', 'The measures included in the Stability Law make it possible to open negotiations with Brussels.', 'These negotiations can contemplate deficits exceeding 3 percent in the coming years.']</t>
         </is>
       </c>
     </row>
@@ -700,17 +674,17 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>It is useless to imagine otherwise: the recovery will be timid, sluggish, and fraught with "downside risks." Small businesses, especially those in the South, are left on the sidelines; consumption is languishing. Furthermore, the number of unemployed people is increasing even in 2015, and inflation continues to decline. The economic bulletin from the Banca d'Italia, the first of the new year, is more cautious than ever. Its quarterly release coincides this time with two significant pieces of news regarding the PIL. The first: the UE Commissioner, Olli Rehn, is confident in the country's ability to recover, calling for a push on dismissals and a spending review, and suggesting the hypothesis that Italia could obtain more "flexibility" on budgetary rules, a condition indispensable for freeing up resources for investment. For the record: yesterday, the Commissioner held a breakfast meeting with the Minister of Economy, Fabrizio Saccomanni, on these and other topics. The second piece of news reveals that the UE is revising the calculation of the PIL, moving investments in research and development from the expenditure category—thus a liability—to the investment category itself. According to extrapolations, the benefit will be between 1% and 2%, with non-negligible effects even for the deficit-PIL and debt-PIL ratio, and thus, for the country's fiscal consolidation and relations with Bruxelles. The Banca d'Italia document, naturally, remains anchored only on the technical-analytical ground. Thus, the macro projections elaborated by these economists place the year-end PIL growth at 0.7%, before rising to 1% in 2015. These are therefore estimates much more contained than those of the government (1% and 1.7%, respectively). They are small upward jumps, in an overall European context that is also sluggish. The effects on labor are not yet visible: this year the unemployment rate will remain stuck at 12.8%, and the following year it will rise to 12.9%. Only the recovery of domestic demand can extend the recovery to the labor market, warns the Banca d'Italia. At the moment, however, the risks to growth "remain oriented downwards"; the recovery of investments can be "delayed," especially "if access to credit conditions remain restrictive for longer than anticipated, or if public administration commercial debt payments register delays." And everything is weighed down by the risk of generalized deflation: this danger is judged to be "modest." But the fall in inflation could be "more accentuated and persistent" than expected, "especially if the weakness of demand were to reflect on expectations." In short, as the President of the BCE recently recalled, "it is still too early to sing victory," it is better to keep one's feet on the ground. The general picture, in fact, remains unclear. Business confidence, certainly, is improving, and industrial activity is regaining momentum after having decreased "almost without interruption" since the summer of 2011. But the underlying picture is very varied depending on the business category and its location: small businesses, especially in the South, remain on the margins of the process. Similarly, while it is true that the decline in household consumption also eased in the third quarter of 2013, it is also true that today Italians are not spending. Consumption continues to be constrained by both the weakness of disposable income and the difficult conditions of the labor market. The Banca d'Italia also notes that "the recovery of confidence, underway since the beginning of 2013, stopped in the fourth quarter." Via Nazionale, meanwhile, is changing its internal organization: under the Board of Directors, 8 departments, services, and divisions. © reproduction reserved</t>
+          <t>It is useless to delude oneself: the recovery will be timid, weak, and fraught with 'downside risks.' Small businesses, especially those in the south, are left on the sidelines; consumption is languishing. Furthermore, unemployment is increasing even in 2015, and inflation continues to decline. The Bank of Italy's economic bulletin, the first of the new year, is more cautious than ever. Its quarterly release coincides this time with two major pieces of news regarding GDP. The first: the EU Commissioner, Olli Rehn, is confident in the country's ability to recover, calling for increased dismissals and a spending review, and suggesting the hypothesis that Italy could obtain more 'flexibility' regarding budgetary rules—a condition essential for freeing up resources for investment. For the record: yesterday, the Commissioner held a breakfast meeting with the Minister of Economy, Fabrizio Saccomanni, on these and other topics. The second piece of news reveals that the EU is revising the calculation of GDP, moving investments in research and development from the expenditure category—thus a liability—to the investment category. According to extrapolations, the benefit will be between 1% and 2%, with non-negligible effects even for the deficit-to-GDP and debt-to-GDP ratios, and thus, for the country's fiscal consolidation and relations with Brussels. The Bank of Italy's document, naturally, remains anchored only on technical-analytical grounds. Thus, the macro projections elaborated by these economists place year-end GDP growth at 0.7%, before rising to 1% in 2015. These are therefore estimates considerably more contained than those of the government (1% and 1.7%, respectively). They are small upward jumps, within an overall sluggish European context. The effects on the labor market are not yet visible: this year the unemployment rate will remain stuck at 12.8%, and next year it will rise to 12.9%. Only the recovery of domestic demand can extend the recovery to the labor market, warns the Bank of Italy. However, at the moment, risks to growth 'remain oriented downwards'; the recovery of investments can be 'delayed,' especially 'if access to credit conditions remain restrictive for longer than anticipated, or if public administration commercial debt payments register delays.' And weighing on everything is the risk of generalized deflation: this danger is judged to be 'modest.' But the fall in inflation could be 'more accentuated and persistent' than expected, 'especially if the weakness of demand were to reflect on expectations.' In short, as the President of the ECB recently recalled, 'it is still too early to celebrate victory'; it is better to keep one's feet on the ground. The general picture, in fact, remains unclear. While business confidence is certainly improving, industrial activity is regaining momentum after having decreased 'almost without interruption' since the summer of 2011. But the underlying picture is very varied depending on the type of business and its location: small businesses, especially in the south, remain on the margins of the process. Similarly, while it is true that the decline in household consumption attenuated in the third quarter of 2013, it is also true that Italians are not spending today. Consumption continues to be constrained by both weak disposable income and difficult labor market conditions. The Bank of Italy also notes that 'the recovery of confidence, which began in early 2013, stopped in the fourth quarter.' Via Nazionale, meanwhile, is changing its internal organization: under the board, 8 departments, services, and divisions. © reproduction reserved.</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>Observation date: 2014-01-18 00:00:00. It is useless to imagine otherwise: the recovery will be timid, sluggish, and fraught with "downside risks." Small businesses, especially those in the South, are left on the sidelines; consumption is languishing. Furthermore, the number of unemployed people is increasing even in 2015, and inflation continues to decline. The economic bulletin from the Banca d'Italia, the first of the new year, is more cautious than ever. Its quarterly release coincides this time with two significant pieces of news regarding the PIL. The first: the UE Commissioner, Olli Rehn, is confident in the country's ability to recover, calling for a push on dismissals and a spending review, and suggesting the hypothesis that Italia could obtain more "flexibility" on budgetary rules, a condition indispensable for freeing up resources for investment. For the record: yesterday, the Commissioner held a breakfast meeting with the Minister of Economy, Fabrizio Saccomanni, on these and other topics. The second piece of news reveals that the UE is revising the calculation of the PIL, moving investments in research and development from the expenditure category—thus a liability—to the investment category itself. According to extrapolations, the benefit will be between 1% and 2%, with non-negligible effects even for the deficit-PIL and debt-PIL ratio, and thus, for the country's fiscal consolidation and relations with Bruxelles. The Banca d'Italia document, naturally, remains anchored only on the technical-analytical ground. Thus, the macro projections elaborated by these economists place the year-end PIL growth at 0.7%, before rising to 1% in 2015. These are therefore estimates much more contained than those of the government (1% and 1.7%, respectively). They are small upward jumps, in an overall European context that is also sluggish. The effects on labor are not yet visible: this year the unemployment rate will remain stuck at 12.8%, and the following year it will rise to 12.9%. Only the recovery of domestic demand can extend the recovery to the labor market, warns the Banca d'Italia. At the moment, however, the risks to growth "remain oriented downwards"; the recovery of investments can be "delayed," especially "if access to credit conditions remain restrictive for longer than anticipated, or if public administration commercial debt payments register delays." And everything is weighed down by the risk of generalized deflation: this danger is judged to be "modest." But the fall in inflation could be "more accentuated and persistent" than expected, "especially if the weakness of demand were to reflect on expectations." In short, as the President of the BCE recently recalled, "it is still too early to sing victory," it is better to keep one's feet on the ground. The general picture, in fact, remains unclear. Business confidence, certainly, is improving, and industrial activity is regaining momentum after having decreased "almost without interruption" since the summer of 2011. But the underlying picture is very varied depending on the business category and its location: small businesses, especially in the South, remain on the margins of the process. Similarly, while it is true that the decline in household consumption also eased in the third quarter of 2013, it is also true that today Italians are not spending. Consumption continues to be constrained by both the weakness of disposable income and the difficult conditions of the labor market. The Banca d'Italia also notes that "the recovery of confidence, underway since the beginning of 2013, stopped in the fourth quarter." Via Nazionale, meanwhile, is changing its internal organization: under the Board of Directors, 8 departments, services, and divisions. © reproduction reserved</t>
+          <t>Observation date: 2014-01-18 00:00:00. It is useless to delude oneself: the recovery will be timid, weak, and fraught with 'downside risks.' Small businesses, especially those in the south, are left on the sidelines; consumption is languishing. Furthermore, unemployment is increasing even in 2015, and inflation continues to decline. The Bank of Italy's economic bulletin, the first of the new year, is more cautious than ever. Its quarterly release coincides this time with two major pieces of news regarding GDP. The first: the EU Commissioner, Olli Rehn, is confident in the country's ability to recover, calling for increased dismissals and a spending review, and suggesting the hypothesis that Italy could obtain more 'flexibility' regarding budgetary rules—a condition essential for freeing up resources for investment. For the record: yesterday, the Commissioner held a breakfast meeting with the Minister of Economy, Fabrizio Saccomanni, on these and other topics. The second piece of news reveals that the EU is revising the calculation of GDP, moving investments in research and development from the expenditure category—thus a liability—to the investment category. According to extrapolations, the benefit will be between 1% and 2%, with non-negligible effects even for the deficit-to-GDP and debt-to-GDP ratios, and thus, for the country's fiscal consolidation and relations with Brussels. The Bank of Italy's document, naturally, remains anchored only on technical-analytical grounds. Thus, the macro projections elaborated by these economists place year-end GDP growth at 0.7%, before rising to 1% in 2015. These are therefore estimates considerably more contained than those of the government (1% and 1.7%, respectively). They are small upward jumps, within an overall sluggish European context. The effects on the labor market are not yet visible: this year the unemployment rate will remain stuck at 12.8%, and next year it will rise to 12.9%. Only the recovery of domestic demand can extend the recovery to the labor market, warns the Bank of Italy. However, at the moment, risks to growth 'remain oriented downwards'; the recovery of investments can be 'delayed,' especially 'if access to credit conditions remain restrictive for longer than anticipated, or if public administration commercial debt payments register delays.' And weighing on everything is the risk of generalized deflation: this danger is judged to be 'modest.' But the fall in inflation could be 'more accentuated and persistent' than expected, 'especially if the weakness of demand were to reflect on expectations.' In short, as the President of the ECB recently recalled, 'it is still too early to celebrate victory'; it is better to keep one's feet on the ground. The general picture, in fact, remains unclear. While business confidence is certainly improving, industrial activity is regaining momentum after having decreased 'almost without interruption' since the summer of 2011. But the underlying picture is very varied depending on the type of business and its location: small businesses, especially in the south, remain on the margins of the process. Similarly, while it is true that the decline in household consumption attenuated in the third quarter of 2013, it is also true that Italians are not spending today. Consumption continues to be constrained by both weak disposable income and difficult labor market conditions. The Bank of Italy also notes that 'the recovery of confidence, which began in early 2013, stopped in the fourth quarter.' Via Nazionale, meanwhile, is changing its internal organization: under the board, 8 departments, services, and divisions. © reproduction reserved.</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>['The recovery will be timid, sluggish, and fraught with "downside risks".', 'Small businesses, especially those in the South, are left on the sidelines.', 'Consumption is languishing.', 'The number of unemployed people is increasing in 2015.', 'Inflation continues to decline.', "The Banca d'Italia economic bulletin, released on 2014-01-18, is more cautious than ever.", "The Banca d'Italia quarterly release coincides with two significant pieces of news regarding the PIL.", "Olli Rehn, the UE Commissioner, is confident in the country's ability to recover.", 'Olli Rehn called for a push on dismissals and a spending review.', 'Olli Rehn suggested that Italia could obtain more "flexibility" on budgetary rules.', 'Obtaining budgetary flexibility is indispensable for freeing up resources for investment.', 'On 2014-01-17, Olli Rehn held a breakfast meeting with Fabrizio Saccomanni, the Minister of Economy.', 'The UE is revising the calculation of the PIL.', 'The UE is moving investments in research and development from the expenditure category to the investment category.', 'The benefit of the PIL revision is estimated to be between 1% and 2%.', 'The PIL revision will have non-negligible effects on the deficit-PIL and debt-PIL ratio.', "The Banca d'Italia document remains anchored only on the technical-analytical ground.", "The Banca d'Italia macro projections place the year-end PIL growth at 0.7%.", "The Banca d'Italia macro projections estimate PIL growth will rise to 1% in 2015.", "The government's projections for year-end PIL growth are 1%.", 'The unemployment rate is projected to remain at 12.8% on 2014-01-01.', 'The unemployment rate is projected to rise to 12.9% the following year.', "The Banca d'Italia warns that only the recovery of domestic demand can extend the recovery to the labor market.", 'Risks to growth remain oriented downwards.', 'The recovery of investments can be delayed if access to credit conditions remain restrictive for longer than anticipated.', 'The recovery of investments can be delayed if public administration commercial debt payments register delays.', 'The risk of generalized deflation is judged to be "modest".', 'The fall in inflation could be "more accentuated and persistent" than expected if the weakness of demand reflects on expectations.', 'Business confidence is improving.', 'Industrial activity is regaining momentum.', 'Industrial activity decreased "almost without interruption" since the summer of 2011.', 'The underlying picture is varied depending on the business category and its location.', 'Small businesses, especially in the South, remain on the margins of the process.', 'The decline in household consumption eased in the third quarter of 2013.', 'On 2014-01-18, Italians are not spending.', 'Consumption is constrained by the weakness of disposable income.', 'Consumption is constrained by the difficult conditions of the labor market.', "The Banca d'Italia noted that the recovery of confidence, underway since the beginning of 2013, stopped in the fourth quarter.", 'Via Nazionale is changing its internal organization.', "Via Nazionale's new internal organization includes 8 departments, services, and divisions under the Board of Directors."]</t>
+          <t>['Small businesses, especially those in the south, are left on the sidelines.', 'Consumption is languishing.', 'Unemployment is increasing in 2015.', 'Inflation continues to decline.', "The Bank of Italy's economic bulletin, released on 2014-01-18, is more cautious than ever.", "The Bank of Italy's quarterly release coincides with two major pieces of news regarding GDP.", "Olli Rehn, the EU Commissioner, is confident in Italy's ability to recover.", 'Olli Rehn, the EU Commissioner, called for increased dismissals and a spending review.', "Olli Rehn, the EU Commissioner, suggested that Italy could obtain more 'flexibility' regarding budgetary rules.", 'On 2014-01-17, Olli Rehn, the Commissioner, held a breakfast meeting with Fabrizio Saccomanni, the Minister of Economy.', 'The EU is revising the calculation of GDP.', 'The EU is moving investments in research and development from the expenditure category to the investment category.', 'Extrapolations suggest the benefit of the GDP revision will be between 1% and 2%.', 'The GDP revision will have non-negligible effects on the deficit-to-GDP ratio.', 'Macro projections elaborated by the economists place year-end GDP growth at 0.7%.', "The macro projections are considerably more contained than the government's estimates for year-end GDP growth.", 'The government estimates GDP growth at 1.7% in 2015.', 'The unemployment rate is projected to remain stuck at 12.8% in 2014.', 'The Bank of Italy warns that only the recovery of domestic demand can extend the recovery to the labor market.', 'Risks to growth remain oriented downwards.', 'The recovery of investments can be delayed if access to credit conditions remain restrictive for longer than anticipated.', 'The recovery of investments can be delayed if public administration commercial debt payments register delays.', 'The risk of generalized deflation is judged to be modest.', 'The fall in inflation could be more accentuated and persistent than expected if the weakness of demand reflects on expectations.', 'Business confidence is improving.', 'Industrial activity is regaining momentum after decreasing since the summer of 2011.', 'The underlying picture is varied depending on the type of business and its location.', 'Small businesses, especially in the south, remain on the margins of the process.', 'The decline in household consumption attenuated in the third quarter of 2013.', 'Italians are not spending on 2014-01-18.', 'Weak disposable income constrains consumption.', 'Difficult labor market conditions constrain consumption.', 'The Bank of Italy notes that the recovery of confidence, which began in early 2013, stopped in the fourth quarter.', 'Via Nazionale is changing its internal organization.', 'Via Nazionale will have 8 departments, services, and divisions under the board.']</t>
         </is>
       </c>
     </row>
@@ -764,43 +738,17 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>On September 20th, the CEO of BPM, Giuseppe Castagna, expressed optimism regarding the resilience of the recovery phase. "We—" Castagna said, referring to the moratoriums—"have dropped from over 16 billion euros to 4.8 billion, which means that the clientele has resumed repaying loans. Nearly 75 percent of the clientele exposed for those 4.8 billion have good ratings, and we are confident. These are very comforting figures." However, despite Castagna's optimism, concern for the system's stability remains concrete. While it is true that credits under moratorium have fallen from 280 billion in March 2020 to 147 billion in December 2020, and then to 71 billion in September 2021, the expiration of the support measures is viewed as the true major test for the Italian economy. Today, the economy sees GDP growing by over 6 percent annually, but it must face the challenge of this sharp rebound. The first half of 2022 seems destined to bring to light what has been held back until now.
-"This is a happy moment for the Italian economy," explains Ferruccio Ferrara, founder and president of Negentropy Capital Partners, who signed one of the earliest distressed credit acquisition deals with Pimco and Deutsche Bank back in 2011. "After very heavy months, the rebound underway is bringing optimism, and this is a fantastic medicine for the economy. But the time will soon come when we will have to account for the past and for businesses to resume payments owed to banks and currently under moratorium. There are different reactivities depending on the industrial sectors, but the underlying condition remains quite heavy. This is also because Italy entered the pandemic with a complicated financial situation and fractional growth compared to major European competitors; this must not be forgotten. COVID extended the recovery times, and it is undeniable that over the last eighteen months, banking exposures have increased. Today, in Italy, the total of non-performing credits (NPL and UTP combined)—a distinction that is very subtle and often depends on the specific bank—amounts to approximately 500 billion euros. This is a truly considerable figure that makes Italy the first European market for this type of position, one of the first in the world. Of these 500 billion, about 180 billion are UTP and about 120 billion are NPL still within the banking perimeter. The remaining 200 billion have not disappeared. They have left the banking perimeter and therefore no longer represent a structural issue for the credit industry, which is also burdened by the needs imposed by scheduled provisioning (calendar provisioning), but are in the portfolios of specialized funds. From the perspective of the Italian economy, however, little changes..."
-In 2021, the value of portfolios ceded by banks will be about 34 billion (1.5 billion only from mps if the cession to Unicredit were to materialize), an increase from 2020, as will UTP, which will reach 11 billion. By the end of the year, NPLs worth 26 billion are ready to be ceded. Last month, Banca Ifis, in its usual September sector report, wrote: "In the two-year period 2022-2023, new distressed credit on households and resident businesses is expected to grow (about 70 billion euros over the two years), but without reaching the peak of 2013. The increase in the deterioration rate will be driven by the corporate component." But the bank led by Frederick Geertman also highlighted the positive effect of government measures: "In 2021, the gross distressed credit stock is expected to contract. This will reduce the NPE ratio below the 5 percent target required by the BCE. The incidence on employment is expected to increase starting in 2022 and will reach 5.9% in 2023," precisely when the safety net established by the executive will be behind them.
-In the distressed credit market, an important role is played by public hands, both through the controlled entity Amco and through the Gacs, the public guarantees on the securitization of distressed assets, introduced by a decree in February 2016 and repeatedly extended. Based on the further 12-month extension granted by the European Union during 2021, Banca Ifis forecasts about 7 billion euros in new guaranteed operations, bringing the total transacted since 2016 to 94 billion euros. Seven are the services committed in the Gacs-assisted operations realized so far, with 80 percent of the value, or the gross book value (GBV), concentrated among the first four Italian operators: Dovalue, Prelios, Cerved, and Credito Fondiario.
-"The attention of operators on the Italian market is very high," emphasizes Ferrara, who, with Negentropy, manages portfolios worth about 3 billion euros of GBV—and this is demonstrated by the fact that today, when a credit institution puts up an asset for sale, up to 25-30 operators are invited to participate in the purchase. The increase in the number of operators has also induced an upward revision of prices: to make a space among many competitors, some have bought in the past at very aggressive levels, and the increase in the average value of transactions has benefited bank balance sheets. Now it remains to understand what 2022 will bring, but it is difficult to predict: I hope that the support interventions for the business system are abandoned only gradually; this would help the resilience of sectors most exposed so far, such as manufacturing, fashion, tourism, and catering."
-The system of loans and financing relies on real guarantees, in the vast majority of cases, real estate. In this case too, COVID left its mark: in 2021, 125,000 judicial auctions are estimated in Italy, a drop of 39 percent compared to pre-pandemic levels. The courts have suspended over 120,000 auctions, and there are operations valued at at least 13 billion euros blocked in the judicial courts. These too await the restart.
-***
-**Glossary of Terms**
-**NPL (Non-Performing Loans):** Loans that are not being repaid by the borrower, or distressed credits.
-**UTP (Unlikely to Pay):** Exposures for which the bank assesses that the debtor is unlikely to fully meet its contractual obligations.
-**Moratoria:** A temporary suspension of debt payments.
-**NPE Ratio:** Non-Performing Exposure ratio (a measure of bad debt relative to total loans).
-**GBV (Gross Book Value):** The total value of assets recorded on the balance sheet before any deductions.
-**Scheduled Provisioning (Calendar Provisioning):** The process of setting aside reserves (provisions) for potential losses based on a defined schedule.</t>
+          <t>Last September 20, the CEO of Banco BPM, Giuseppe Castagna, expressed optimism regarding the resilience of the recovery phase. “We—referring to the moratoriums—have fallen from over 16 billion euros to 4.8 billion, which means that the clientele has resumed repaying loans. Nearly 75 percent of the clientele exposed for those 4.8 billion have good ratings, and we are confident. These are very encouraging figures.” However, despite Castagna’s optimism, concern for the stability of the system remains concrete. While it is true that credits under moratorium have fallen from 280 billion in March 2020 to 147 billion in December 2020, and then to 71 billion in September 2021, the expiration of the support measures is seen as the real great test for the Italian economy. Today, the economy sees GDP growing by over 6 percent annually, but it must face this sharp turn. The first half of 2022 seems destined to bring to light what has been held back until now. “This is a happy time for the Italian economy,” explains Ferruccio Ferrara, founder and president of Negentropy Capital Partners, who signed one of the earliest distressed credit acquisitions with PIMCO and Deutsche Bank back in 2011. After very difficult months, the rebound underway is bringing optimism, and this is a fantastic medicine for the economy. But the time will soon come when we will have to face the past and for businesses resume payments owed to banks and currently under moratorium. There are different levels of reactivity depending on the industrial sectors, but the underlying condition remains quite heavy. This is also because Italy entered the pandemic with a complicated financial situation and fractional growth compared to major European competitors—this cannot be forgotten. COVID extended the recovery times, and it is undeniable that over the last eighteen months, banking exposures have increased. Today, in Italy, the total amount of non-performing loans, or the combination of NPLs and UTPs—whose distinction is very subtle and often depends on the bank—stands at approximately 500 billion euros. This is a truly considerable figure, making Italy the first European market for this type of position, one of the first in the world. Of these 500 billion, about 180 billion are UTPs and about 120 billion are NPLs still within the banking perimeter. The remaining 200 billion have not disappeared. They have left the banking perimeter and therefore no longer represent a structural issue for the credit industry, which is also burdened by the needs imposed by calendar provisioning, but they are in specialized fund portfolios. From the perspective of the Italian economy, however, little changes... In 2021, the value of portfolios ceded by banks will be about 34 billion (1.5 billion only from MPS if the cession to UniCredit were to materialize), growing compared to 2020, as will UTPs, which will reach 11 billion. From here until the end of the year, NPLs worth 26 billion are ready to be ceded. Last month, Banca Ifis, in its usual September sector report, wrote: “In the two-year period 2022-2023, new distressed credit on households and businesses is expected to grow (about 70 billion euros over the two years), but without reaching the peak of 2013. The increase in the deterioration rate will be driven by the corporate component.” But the bank led by Frederick Geertman also highlighted the positive effect of government measures: “In 2021, the gross stock of distressed credits is expected to contract. This will reduce the NPE ratio below the 5 percent target required by the ECB. The incidence on employment is expected to increase starting in 2022 and will reach 5.9 percent in 2023,” precisely when the safety net provided by the executive will be behind us. In the distressed credit market, a significant role is played by public hands, both through the subsidiary Amco and through GACS, the public guarantees on the securitization of distressed assets, introduced by a decree in February 2016 and repeatedly extended. Based on the further 12-month extension granted by the European Union during 2021, Banca Ifis forecasts about 7 billion euros in new guaranteed operations, bringing the total transacted since 2016 to 94 billion euros. Seven are the services committed in GACS-assisted operations so far, with 80 percent of the value, or the gross book value (GBV), concentrated among the first four Italian operators: Dovalue, Prelios, Cerved, and Credito Fondiario. The operators “the attention of operators on the Italian market is very high,” emphasizes Ferrara, who, with Negentropy, manages portfolios worth about 3 billion euros of GBV—and this is demonstrated by the fact that today, when a credit institution puts up an asset for sale, up to 25-30 operators are invited to participate in the purchase. The increase in the number of operators has also led to an upward revision of prices: to make space among many competitors, some have bought in the past at very aggressive levels, and the increase in the average value of transactions has benefited banks' balance sheets. Now it remains to understand what 2022 will bring, but it is difficult to predict: I hope that the support measures for the business system are abandoned only gradually, as this would help the stability of sectors most exposed so far, such as manufacturing, fashion, tourism, and catering.” The system of loans and financing relies on real guarantees, in the vast majority of cases, real estate. In this case too, COVID left its mark: in 2021, 125,000 judicial auctions are estimated in Italy, a drop of 39 percent compared to pre-pandemic levels. The courts have suspended over 120,000 auctions, and there are operations for at least 13 billion euros blocked in the courts. These too await a restart. © Reproduction reserved. NPL refers to non-performing loans, or non-performing credits. UTP refers to unlikely to pay, meaning exposures for which the bank assesses it unlikely that the debtor will fully meet its contractual obligations. Past due are exposures or payments overdue for a period exceeding 90 days. It is the first stage of the crisis, which can evolve into UTP and then into NPL.</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>Observation date: 2021-10-18 00:00:00. On September 20th, the CEO of BPM, Giuseppe Castagna, expressed optimism regarding the resilience of the recovery phase. "We—" Castagna said, referring to the moratoriums—"have dropped from over 16 billion euros to 4.8 billion, which means that the clientele has resumed repaying loans. Nearly 75 percent of the clientele exposed for those 4.8 billion have good ratings, and we are confident. These are very comforting figures." However, despite Castagna's optimism, concern for the system's stability remains concrete. While it is true that credits under moratorium have fallen from 280 billion in March 2020 to 147 billion in December 2020, and then to 71 billion in September 2021, the expiration of the support measures is viewed as the true major test for the Italian economy. Today, the economy sees GDP growing by over 6 percent annually, but it must face the challenge of this sharp rebound. The first half of 2022 seems destined to bring to light what has been held back until now.
-"This is a happy moment for the Italian economy," explains Ferruccio Ferrara, founder and president of Negentropy Capital Partners, who signed one of the earliest distressed credit acquisition deals with Pimco and Deutsche Bank back in 2011. "After very heavy months, the rebound underway is bringing optimism, and this is a fantastic medicine for the economy. But the time will soon come when we will have to account for the past and for businesses to resume payments owed to banks and currently under moratorium. There are different reactivities depending on the industrial sectors, but the underlying condition remains quite heavy. This is also because Italy entered the pandemic with a complicated financial situation and fractional growth compared to major European competitors; this must not be forgotten. COVID extended the recovery times, and it is undeniable that over the last eighteen months, banking exposures have increased. Today, in Italy, the total of non-performing credits (NPL and UTP combined)—a distinction that is very subtle and often depends on the specific bank—amounts to approximately 500 billion euros. This is a truly considerable figure that makes Italy the first European market for this type of position, one of the first in the world. Of these 500 billion, about 180 billion are UTP and about 120 billion are NPL still within the banking perimeter. The remaining 200 billion have not disappeared. They have left the banking perimeter and therefore no longer represent a structural issue for the credit industry, which is also burdened by the needs imposed by scheduled provisioning (calendar provisioning), but are in the portfolios of specialized funds. From the perspective of the Italian economy, however, little changes..."
-In 2021, the value of portfolios ceded by banks will be about 34 billion (1.5 billion only from mps if the cession to Unicredit were to materialize), an increase from 2020, as will UTP, which will reach 11 billion. By the end of the year, NPLs worth 26 billion are ready to be ceded. Last month, Banca Ifis, in its usual September sector report, wrote: "In the two-year period 2022-2023, new distressed credit on households and resident businesses is expected to grow (about 70 billion euros over the two years), but without reaching the peak of 2013. The increase in the deterioration rate will be driven by the corporate component." But the bank led by Frederick Geertman also highlighted the positive effect of government measures: "In 2021, the gross distressed credit stock is expected to contract. This will reduce the NPE ratio below the 5 percent target required by the BCE. The incidence on employment is expected to increase starting in 2022 and will reach 5.9% in 2023," precisely when the safety net established by the executive will be behind them.
-In the distressed credit market, an important role is played by public hands, both through the controlled entity Amco and through the Gacs, the public guarantees on the securitization of distressed assets, introduced by a decree in February 2016 and repeatedly extended. Based on the further 12-month extension granted by the European Union during 2021, Banca Ifis forecasts about 7 billion euros in new guaranteed operations, bringing the total transacted since 2016 to 94 billion euros. Seven are the services committed in the Gacs-assisted operations realized so far, with 80 percent of the value, or the gross book value (GBV), concentrated among the first four Italian operators: Dovalue, Prelios, Cerved, and Credito Fondiario.
-"The attention of operators on the Italian market is very high," emphasizes Ferrara, who, with Negentropy, manages portfolios worth about 3 billion euros of GBV—and this is demonstrated by the fact that today, when a credit institution puts up an asset for sale, up to 25-30 operators are invited to participate in the purchase. The increase in the number of operators has also induced an upward revision of prices: to make a space among many competitors, some have bought in the past at very aggressive levels, and the increase in the average value of transactions has benefited bank balance sheets. Now it remains to understand what 2022 will bring, but it is difficult to predict: I hope that the support interventions for the business system are abandoned only gradually; this would help the resilience of sectors most exposed so far, such as manufacturing, fashion, tourism, and catering."
-The system of loans and financing relies on real guarantees, in the vast majority of cases, real estate. In this case too, COVID left its mark: in 2021, 125,000 judicial auctions are estimated in Italy, a drop of 39 percent compared to pre-pandemic levels. The courts have suspended over 120,000 auctions, and there are operations valued at at least 13 billion euros blocked in the judicial courts. These too await the restart.
-***
-**Glossary of Terms**
-**NPL (Non-Performing Loans):** Loans that are not being repaid by the borrower, or distressed credits.
-**UTP (Unlikely to Pay):** Exposures for which the bank assesses that the debtor is unlikely to fully meet its contractual obligations.
-**Moratoria:** A temporary suspension of debt payments.
-**NPE Ratio:** Non-Performing Exposure ratio (a measure of bad debt relative to total loans).
-**GBV (Gross Book Value):** The total value of assets recorded on the balance sheet before any deductions.
-**Scheduled Provisioning (Calendar Provisioning):** The process of setting aside reserves (provisions) for potential losses based on a defined schedule.</t>
+          <t>Observation date: 2021-10-18 00:00:00. Last September 20, the CEO of Banco BPM, Giuseppe Castagna, expressed optimism regarding the resilience of the recovery phase. “We—referring to the moratoriums—have fallen from over 16 billion euros to 4.8 billion, which means that the clientele has resumed repaying loans. Nearly 75 percent of the clientele exposed for those 4.8 billion have good ratings, and we are confident. These are very encouraging figures.” However, despite Castagna’s optimism, concern for the stability of the system remains concrete. While it is true that credits under moratorium have fallen from 280 billion in March 2020 to 147 billion in December 2020, and then to 71 billion in September 2021, the expiration of the support measures is seen as the real great test for the Italian economy. Today, the economy sees GDP growing by over 6 percent annually, but it must face this sharp turn. The first half of 2022 seems destined to bring to light what has been held back until now. “This is a happy time for the Italian economy,” explains Ferruccio Ferrara, founder and president of Negentropy Capital Partners, who signed one of the earliest distressed credit acquisitions with PIMCO and Deutsche Bank back in 2011. After very difficult months, the rebound underway is bringing optimism, and this is a fantastic medicine for the economy. But the time will soon come when we will have to face the past and for businesses resume payments owed to banks and currently under moratorium. There are different levels of reactivity depending on the industrial sectors, but the underlying condition remains quite heavy. This is also because Italy entered the pandemic with a complicated financial situation and fractional growth compared to major European competitors—this cannot be forgotten. COVID extended the recovery times, and it is undeniable that over the last eighteen months, banking exposures have increased. Today, in Italy, the total amount of non-performing loans, or the combination of NPLs and UTPs—whose distinction is very subtle and often depends on the bank—stands at approximately 500 billion euros. This is a truly considerable figure, making Italy the first European market for this type of position, one of the first in the world. Of these 500 billion, about 180 billion are UTPs and about 120 billion are NPLs still within the banking perimeter. The remaining 200 billion have not disappeared. They have left the banking perimeter and therefore no longer represent a structural issue for the credit industry, which is also burdened by the needs imposed by calendar provisioning, but they are in specialized fund portfolios. From the perspective of the Italian economy, however, little changes... In 2021, the value of portfolios ceded by banks will be about 34 billion (1.5 billion only from MPS if the cession to UniCredit were to materialize), growing compared to 2020, as will UTPs, which will reach 11 billion. From here until the end of the year, NPLs worth 26 billion are ready to be ceded. Last month, Banca Ifis, in its usual September sector report, wrote: “In the two-year period 2022-2023, new distressed credit on households and businesses is expected to grow (about 70 billion euros over the two years), but without reaching the peak of 2013. The increase in the deterioration rate will be driven by the corporate component.” But the bank led by Frederick Geertman also highlighted the positive effect of government measures: “In 2021, the gross stock of distressed credits is expected to contract. This will reduce the NPE ratio below the 5 percent target required by the ECB. The incidence on employment is expected to increase starting in 2022 and will reach 5.9 percent in 2023,” precisely when the safety net provided by the executive will be behind us. In the distressed credit market, a significant role is played by public hands, both through the subsidiary Amco and through GACS, the public guarantees on the securitization of distressed assets, introduced by a decree in February 2016 and repeatedly extended. Based on the further 12-month extension granted by the European Union during 2021, Banca Ifis forecasts about 7 billion euros in new guaranteed operations, bringing the total transacted since 2016 to 94 billion euros. Seven are the services committed in GACS-assisted operations so far, with 80 percent of the value, or the gross book value (GBV), concentrated among the first four Italian operators: Dovalue, Prelios, Cerved, and Credito Fondiario. The operators “the attention of operators on the Italian market is very high,” emphasizes Ferrara, who, with Negentropy, manages portfolios worth about 3 billion euros of GBV—and this is demonstrated by the fact that today, when a credit institution puts up an asset for sale, up to 25-30 operators are invited to participate in the purchase. The increase in the number of operators has also led to an upward revision of prices: to make space among many competitors, some have bought in the past at very aggressive levels, and the increase in the average value of transactions has benefited banks' balance sheets. Now it remains to understand what 2022 will bring, but it is difficult to predict: I hope that the support measures for the business system are abandoned only gradually, as this would help the stability of sectors most exposed so far, such as manufacturing, fashion, tourism, and catering.” The system of loans and financing relies on real guarantees, in the vast majority of cases, real estate. In this case too, COVID left its mark: in 2021, 125,000 judicial auctions are estimated in Italy, a drop of 39 percent compared to pre-pandemic levels. The courts have suspended over 120,000 auctions, and there are operations for at least 13 billion euros blocked in the courts. These too await a restart. © Reproduction reserved. NPL refers to non-performing loans, or non-performing credits. UTP refers to unlikely to pay, meaning exposures for which the bank assesses it unlikely that the debtor will fully meet its contractual obligations. Past due are exposures or payments overdue for a period exceeding 90 days. It is the first stage of the crisis, which can evolve into UTP and then into NPL.</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>['On 2021-09-20, Giuseppe Castagna, CEO of BPM, expressed optimism regarding the resilience of the recovery phase.', 'Giuseppe Castagna stated that moratoriums dropped from over 16 billion euros to 4.8 billion euros.', 'The drop in moratoriums means that the clientele has resumed repaying loans.', 'Nearly 75 percent of the clientele exposed for 4.8 billion euros have good ratings.', 'Credits under moratorium fell from 280 billion euros in March 2020 to 147 billion euros in December 2020.', 'Credits under moratorium fell from 147 billion euros in December 2020 to 71 billion euros in September 2021.', 'The expiration of the support measures is viewed as a major test for the Italian economy.', 'On 2021-10-18, the economy sees GDP growing by over 6 percent annually.', 'The first half of 2022 is expected to reveal previously held back issues.', 'Ferruccio Ferrara, founder and president of Negentropy Capital Partners, signed one of the earliest distressed credit acquisition deals with Pimco and Deutsche Bank in 2011.', 'Businesses will soon have to resume payments owed to banks and currently under moratorium.', 'The total of non-performing credits (NPL and UTP combined) in Italy amounts to approximately 500 billion euros on 2021-10-18.', 'Of the 500 billion euros, about 180 billion euros are UTP within the banking perimeter.', 'The remaining 200 billion euros have left the banking perimeter.', 'The 200 billion euros are in the portfolios of specialized funds.', 'In 2021, the value of portfolios ceded by banks will be about 34 billion euros.', 'UTP is expected to reach 11 billion euros in 2021.', 'By the end of 2021, NPLs worth 26 billion euros are ready to be ceded.', 'Banca Ifis reported that new distressed credit on households and resident businesses is expected to grow by about 70 billion euros over the two years 2022-2023.', 'The expected growth of distressed credit will not reach the peak of 2013.', 'The increase in the deterioration rate will be driven by the corporate component.', 'Banca Ifis expects the gross distressed credit stock to contract in 2021.', 'The contraction of the distressed credit stock will reduce the NPE ratio below the 5 percent target required by the BCE.', 'The incidence on employment is expected to increase starting in 2022.', 'Gacs are public guarantees on the securitization of distressed assets.', 'Gacs were introduced by a decree in February 2016.', "Banca Ifis forecasts about 7 billion euros in new guaranteed operations based on the European Union's 12-month extension in 2021.", 'The total value transacted through Gacs since 2016 is 94 billion euros.', '80 percent of the Gross Book Value (GBV) in Gacs-assisted operations is concentrated among Dovalue, Prelios, Cerved, and Credito Fondiario.', 'Ferruccio Ferrara, with Negentropy, manages portfolios worth about 3 billion euros of GBV.', 'When a credit institution puts up an asset for sale on 2021-10-18, up to 25-30 operators are invited to participate in the purchase.', 'The increase in the number of operators has induced an upward revision of prices in the distressed credit market.', 'In 2021, 125,000 judicial auctions are estimated in Italy.', 'The number of judicial auctions in 2021 represents a 39 percent drop compared to pre-pandemic levels.', 'The courts have suspended over 120,000 auctions.', 'Operations valued at at least 13 billion euros are blocked in the judicial courts.']</t>
+          <t>['On September 20, Giuseppe Castagna, CEO of Banco BPM, expressed optimism regarding the resilience of the recovery phase.', 'The moratoriums fell from over 16 billion euros to 4.8 billion euros.', 'The reduction in moratoriums means that the clientele resumed repaying loans.', 'Nearly 75 percent of the clientele exposed for the 4.8 billion euros have good ratings.', 'Credits under moratorium fell from 280 billion euros in March 2020 to 147 billion euros in December 2020.', 'Credits under moratorium fell further to 71 billion euros in September 2021.', 'The expiration of the support measures is seen as the real great test for the Italian economy.', 'The economy sees GDP growing by over 6 percent annually.', 'The Italian economy must face a sharp turn.', 'The rebound underway is bringing optimism to the economy.', 'The time will soon come when businesses will have to resume payments owed to banks and currently under moratorium.', 'The underlying condition for payments remains quite heavy.', 'Italy entered the pandemic with a complicated financial situation.', 'Italy had fractional growth compared to major European competitors.', 'COVID extended the recovery times.', 'Over the last eighteen months, banking exposures have increased.', '2021-10-18, the total amount of non-performing loans (NPLs) and unlikely to pay (UTPs) in Italy stands at approximately 500 billion euros.', 'The 500 billion euros figure makes Italy the first European market for this type of position.', 'Of the 500 billion euros, about 180 billion euros are UTPs.', 'Of the 500 billion euros, about 120 billion euros are NPLs still within the banking perimeter.', 'The remaining 200 billion euros have left the banking perimeter.', 'The 200 billion euros are in specialized fund portfolios.', 'In 2021, the value of portfolios ceded by banks will be about 34 billion euros.', 'The cession from MPS to UniCredit is estimated at 1.5 billion euros.', 'UTPs are expected to reach 11 billion euros.', 'NPLs worth 26 billion euros are ready to be ceded from here until the end of the year.', 'Banca Ifis wrote a sector report in September.', 'Banca Ifis expects new distressed credit on households and businesses to grow by about 70 billion euros over the two years (2022-2023).', 'The expected growth of distressed credit will not reach the peak of 2013.', 'The increase in the deterioration rate will be driven by the corporate component.', 'Banca Ifis highlighted the positive effect of government measures.', 'In 2021, the gross stock of distressed credits is expected to contract according to Banca Ifis.', 'The contraction of distressed credits will reduce the Non-Performing Exposure (NPE) ratio below the 5 percent target required by the ECB.', 'The incidence on employment is expected to increase starting in 2022.', 'Public hands play a significant role in the distressed credit market.', 'Public guarantees on the securitization of distressed assets (GACS) were introduced by a decree in February 2016.', 'Banca Ifis forecasts about 7 billion euros in new guaranteed operations based on the further 12-month extension granted by the European Union during 2021.', 'The total transacted value since 2016 is forecast to reach 94 billion euros.', 'Seven services were committed in GACS-assisted operations so far.', '80 percent of the value, or the gross book value (GBV), is concentrated among the first four Italian operators: Dovalue, Prelios, Cerved, and Credito Fondiario.', "The operators' attention on the Italian market is very high.", 'When a credit institution puts up an asset for sale, up to 25-30 operators are invited to participate in the purchase.', 'The increase in the number of operators has led to an upward revision of prices.', "The increase in the average value of transactions has benefited banks' balance sheets.", 'The author hopes that the support measures for the business system are abandoned only gradually.', 'Gradual abandonment of support measures would help the stability of sectors such as manufacturing, fashion, tourism, and catering.', 'The system of loans and financing relies on real guarantees, in the vast majority of cases, real estate.', 'In 2021, 125,000 judicial auctions are estimated in Italy.', 'The 125,000 judicial auctions represent a drop of 39 percent compared to pre-pandemic levels.', 'Over 120,000 auctions have been suspended by the courts.', 'Operations for at least 13 billion euros are blocked in the courts.']</t>
         </is>
       </c>
     </row>
@@ -854,17 +802,17 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>I do not address the merits of the measure, but rather the methods of its disbursement. A letter is required: 1 sheet (plus envelope). An application is required: 4 sheets. The instructions: 2 sheets. Photocopies to be attached to the application: 2 sheets (or 4 if a power of attorney is needed). In the best-case scenario, a minimum of 9 sheets will be used for each application (plus envelope), which, multiplied by the estimated population of 1,300,000, results in 11,700,000 sheets (eleven million seven hundred thousand sheets), which, to give an idea, equals 23,400 reams of 500-sheet paper. I forgot the envelopes: 1,300,000. I wonder, hasn't the Ministry of Simplification been established? Regarding the foregone deductions on building renovations, Claudia Ceroni, Roma, are distracted by a VAT increase on a non-essential good (Sky); a much graver problem than the new decree passed last Friday is being overlooked. I am 30 years old, a building engineer. Given the incentives that we knew to be certain, I convinced my parents to renovate their house by improving the roof insulation and installing sanitary panels for sanitary water use, a condensing boiler, and thermostatic valves, for a total of approximately 10,000 euros. Together with my boyfriend, we spent about 50,000 euros on supplementary roof and window insulation that meets energy efficiency requirements for our new house, spending approximately 50,000 euros additionally, with the conviction that we could access the deduction. Now this deduction no longer exists, or at least it is not certain, or it will be reduced from the current 55% to 35%. I wish our Minister Tremonti and the Prime Minister's staff would answer these two simple questions of mine: who will reimburse us for this missed reimbursement that, at the time of the intervention, was considered certain? I believe we are not far from a scam, if by that one means what De Mauro cited: "a crime committed by those who derive illicit profit to the detriment of others, having misled them with artifices and tricks." It is enough to replace "artifices and tricks" with "laws and decrees," which makes the act even more serious. The 4% rate on mortgages set by the government in the financial package is expected to ensure that, by 2009, the interest rate on variable-rate mortgages will not exceed 4%. Heavens! Even an extreme left government would not have thought of it. Tito Boeri, in the newspaper on sale yesterday, asks (rhetorically, I presume) why such a measure is not also provided for fixed-rate mortgages. Simply because with the next ECB rate cut to 2.75%, or less, the Euribor will initially quote just over 3%, plus an average spread of 1%, and thus 4% will be the rate that banks will still have to apply to variable-rate mortgages. A virtually zero advantage for families. If we apply the principle also to fixed-rate mortgages, stipulated with interest rates well above 4%, we run the risk of actually helping the families! If we then consider that during 2009, a variable rate of 3.5% could also be reached. This 4% rate would be another way to help those who truly need it: the banks. The news about the mafias and the choices of TG1, Pino Caserta, TG1 editorial secretary, dear director, on page 19 of yesterday's Repubblica, headlines: "for TG1 the most important yo-yo of the fight against crime," because TG1 did not report, in Saturday's 8 PM edition, the review on the fight against mafias organized by 'politicamente scorretto' in Casalecchio di Reno (Bologna). The meeting was certainly relevant, but, upon closer inspection, even the national edition of your newspaper decided not to report on the conference on mafias. Repubblica limited itself to reporting the protest of Rita Borsellino. What the TG1 editorial secretary omits to say is that the conference on mafias was held a few hundred meters from the yo-yo championship: this is the reason for the controversy raised by Borsellino.</t>
+          <t>I am not addressing the merits of the provision itself, but rather the methods of its disbursement. A letter is required: 1 sheet (plus envelope). An application is required: 4 sheets. Instructions: 2 sheets. Photocopies to attach to the application: 2 sheets (or 4 if a power of attorney is needed). In the best-case scenario, each application will require a minimum of 9 sheets (plus envelope), which, multiplied by the estimated population of 1,300,000, amounts to 11,700,000 sheets (eleven million seven hundred thousand sheets). To give an idea, this equals 23,400 reams of 500-sheet paper. I forgot the envelopes: 1,300,000. I wonder if the Ministry of Simplification was not established? The lost tax deductions on structural renovations, which Claudia Ceroni in Rome was misled by an increase in VAT on a non-essential good (Sky), are causing us to overlook a much graver problem than the new decree passed last Friday. I am 30 years old, a structural engineer. Given the incentives we believed to be certain, I convinced my parents to renovate their home by improving the roof insulation and installing sanitary water panels, a condensing boiler, and thermostatic valves, for a total cost of about €10,000. Together with my boyfriend, we spent about €50,000 on supplementary roof and window insulation that meets energy efficiency requirements for our new home, spending an additional €50,000, with the conviction that we could access the tax deduction. Now, this deduction no longer exists, or at least it is not certain, or it will be reduced from the current 55% to 35%. I wish our Minister Tremonti and the Prime Minister's staff would answer my two simple questions: who will reimburse us for this missed refund that was considered certain at the time of the intervention? I believe we are not far from a scam, if by that what De Mauro cited: 'a crime committed by someone who obtains illicit profit to the detriment of others, having misled them with artifice and trickery.' It is enough to replace 'artifice and trickery' with 'laws and decrees,' which makes the act even more serious. The 4% mortgage rate set by the government in the maneuver is expected to ensure that, by 2009, the interest rate on variable-rate mortgages will not exceed 4%. Heavens! Not even an extreme left government would have thought of that. Tito Boeri, in the newspaper on sale yesterday, asks (rhetorically, I presume) why such a measure is not also provided for fixed-rate mortgages. Simply because with the next BCE rate cut to 2.75%, or less, the Euribor will initially be just over 3%, plus an average spread of 1%, and thus the 4% will be the rate that banks will still have to apply to variable-rate mortgages. The benefit for families is practically zero. If we apply the same principle to fixed-rate mortgages, stipulated with interest rates well above 4%, we run the risk of actually helping the families! If we then consider that during 2009, a variable rate of 3.5% could even be reached. This 4% rate would be another way to help those who truly need it: the banks. The news about the mafia and the choices of TG1, Pino Caserta, editor of TG1, dear director, on page 19 of yesterday's Repubblica, headlines: 'for TG1, the most important yo-yo in the fight against crime,' because TG1 failed to report, in Saturday's 8 PM edition, the review on the fight against the mafia organized by 'Politicamente Scorretto' in Casalecchio di Reno (Bologna). The meeting was certainly relevant, but, upon closer inspection, even your newspaper's national edition decided not to report on the mafia conference. Repubblica limited itself to reporting the protest of Rita Borsellino. What the editor of TG1 omits to say is that the mafia conference took place a few hundred meters from the yo-yo championship: this is the reason for the controversy raised by Borsellino.</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>Observation date: 2008-12-02 00:00:00. I do not address the merits of the measure, but rather the methods of its disbursement. A letter is required: 1 sheet (plus envelope). An application is required: 4 sheets. The instructions: 2 sheets. Photocopies to be attached to the application: 2 sheets (or 4 if a power of attorney is needed). In the best-case scenario, a minimum of 9 sheets will be used for each application (plus envelope), which, multiplied by the estimated population of 1,300,000, results in 11,700,000 sheets (eleven million seven hundred thousand sheets), which, to give an idea, equals 23,400 reams of 500-sheet paper. I forgot the envelopes: 1,300,000. I wonder, hasn't the Ministry of Simplification been established? Regarding the foregone deductions on building renovations, Claudia Ceroni, Roma, are distracted by a VAT increase on a non-essential good (Sky); a much graver problem than the new decree passed last Friday is being overlooked. I am 30 years old, a building engineer. Given the incentives that we knew to be certain, I convinced my parents to renovate their house by improving the roof insulation and installing sanitary panels for sanitary water use, a condensing boiler, and thermostatic valves, for a total of approximately 10,000 euros. Together with my boyfriend, we spent about 50,000 euros on supplementary roof and window insulation that meets energy efficiency requirements for our new house, spending approximately 50,000 euros additionally, with the conviction that we could access the deduction. Now this deduction no longer exists, or at least it is not certain, or it will be reduced from the current 55% to 35%. I wish our Minister Tremonti and the Prime Minister's staff would answer these two simple questions of mine: who will reimburse us for this missed reimbursement that, at the time of the intervention, was considered certain? I believe we are not far from a scam, if by that one means what De Mauro cited: "a crime committed by those who derive illicit profit to the detriment of others, having misled them with artifices and tricks." It is enough to replace "artifices and tricks" with "laws and decrees," which makes the act even more serious. The 4% rate on mortgages set by the government in the financial package is expected to ensure that, by 2009, the interest rate on variable-rate mortgages will not exceed 4%. Heavens! Even an extreme left government would not have thought of it. Tito Boeri, in the newspaper on sale yesterday, asks (rhetorically, I presume) why such a measure is not also provided for fixed-rate mortgages. Simply because with the next ECB rate cut to 2.75%, or less, the Euribor will initially quote just over 3%, plus an average spread of 1%, and thus 4% will be the rate that banks will still have to apply to variable-rate mortgages. A virtually zero advantage for families. If we apply the principle also to fixed-rate mortgages, stipulated with interest rates well above 4%, we run the risk of actually helping the families! If we then consider that during 2009, a variable rate of 3.5% could also be reached. This 4% rate would be another way to help those who truly need it: the banks. The news about the mafias and the choices of TG1, Pino Caserta, TG1 editorial secretary, dear director, on page 19 of yesterday's Repubblica, headlines: "for TG1 the most important yo-yo of the fight against crime," because TG1 did not report, in Saturday's 8 PM edition, the review on the fight against mafias organized by 'politicamente scorretto' in Casalecchio di Reno (Bologna). The meeting was certainly relevant, but, upon closer inspection, even the national edition of your newspaper decided not to report on the conference on mafias. Repubblica limited itself to reporting the protest of Rita Borsellino. What the TG1 editorial secretary omits to say is that the conference on mafias was held a few hundred meters from the yo-yo championship: this is the reason for the controversy raised by Borsellino.</t>
+          <t>Observation date: 2008-12-02 00:00:00. I am not addressing the merits of the provision itself, but rather the methods of its disbursement. A letter is required: 1 sheet (plus envelope). An application is required: 4 sheets. Instructions: 2 sheets. Photocopies to attach to the application: 2 sheets (or 4 if a power of attorney is needed). In the best-case scenario, each application will require a minimum of 9 sheets (plus envelope), which, multiplied by the estimated population of 1,300,000, amounts to 11,700,000 sheets (eleven million seven hundred thousand sheets). To give an idea, this equals 23,400 reams of 500-sheet paper. I forgot the envelopes: 1,300,000. I wonder if the Ministry of Simplification was not established? The lost tax deductions on structural renovations, which Claudia Ceroni in Rome was misled by an increase in VAT on a non-essential good (Sky), are causing us to overlook a much graver problem than the new decree passed last Friday. I am 30 years old, a structural engineer. Given the incentives we believed to be certain, I convinced my parents to renovate their home by improving the roof insulation and installing sanitary water panels, a condensing boiler, and thermostatic valves, for a total cost of about €10,000. Together with my boyfriend, we spent about €50,000 on supplementary roof and window insulation that meets energy efficiency requirements for our new home, spending an additional €50,000, with the conviction that we could access the tax deduction. Now, this deduction no longer exists, or at least it is not certain, or it will be reduced from the current 55% to 35%. I wish our Minister Tremonti and the Prime Minister's staff would answer my two simple questions: who will reimburse us for this missed refund that was considered certain at the time of the intervention? I believe we are not far from a scam, if by that what De Mauro cited: 'a crime committed by someone who obtains illicit profit to the detriment of others, having misled them with artifice and trickery.' It is enough to replace 'artifice and trickery' with 'laws and decrees,' which makes the act even more serious. The 4% mortgage rate set by the government in the maneuver is expected to ensure that, by 2009, the interest rate on variable-rate mortgages will not exceed 4%. Heavens! Not even an extreme left government would have thought of that. Tito Boeri, in the newspaper on sale yesterday, asks (rhetorically, I presume) why such a measure is not also provided for fixed-rate mortgages. Simply because with the next BCE rate cut to 2.75%, or less, the Euribor will initially be just over 3%, plus an average spread of 1%, and thus the 4% will be the rate that banks will still have to apply to variable-rate mortgages. The benefit for families is practically zero. If we apply the same principle to fixed-rate mortgages, stipulated with interest rates well above 4%, we run the risk of actually helping the families! If we then consider that during 2009, a variable rate of 3.5% could even be reached. This 4% rate would be another way to help those who truly need it: the banks. The news about the mafia and the choices of TG1, Pino Caserta, editor of TG1, dear director, on page 19 of yesterday's Repubblica, headlines: 'for TG1, the most important yo-yo in the fight against crime,' because TG1 failed to report, in Saturday's 8 PM edition, the review on the fight against the mafia organized by 'Politicamente Scorretto' in Casalecchio di Reno (Bologna). The meeting was certainly relevant, but, upon closer inspection, even your newspaper's national edition decided not to report on the mafia conference. Repubblica limited itself to reporting the protest of Rita Borsellino. What the editor of TG1 omits to say is that the mafia conference took place a few hundred meters from the yo-yo championship: this is the reason for the controversy raised by Borsellino.</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>['A letter requires 1 sheet plus an envelope.', 'An application requires 4 sheets.', 'The instructions require 2 sheets.', 'Photocopies require 2 sheets, or 4 sheets if a power of attorney is needed.', 'In the best-case scenario, a minimum of 9 sheets are used for each application plus an envelope.', 'The estimated population is 1,300,000.', 'The total estimated sheets needed is 11,700,000 sheets.', 'The total estimated reams needed is 23,400 reams of 500-sheet paper.', 'The number of envelopes needed is 1,300,000.', 'Claudia Ceroni, Roma, is distracted by a VAT increase on a non-essential good (Sky).', 'The VAT increase on a non-essential good (Sky) is a much graver problem than the new decree passed on 2008-12-01.', "The author, a 30-year-old building engineer, convinced the author's parents to renovate their house.", 'The parent renovation included improving roof insulation, installing sanitary panels for sanitary water use, a condensing boiler, and thermostatic valves.', 'The parent renovation cost was approximately 10,000 euros.', 'The author and boyfriend spent about 50,000 euros on supplementary roof and window insulation.', 'The deduction for building renovations was previously 55% but may be reduced to 35%.', 'The government set a 4% rate on mortgages in the financial package.', 'The 4% rate is expected to ensure that, by 2009, the interest rate on variable-rate mortgages will not exceed 4%.', 'Tito Boeri asked why the 4% measure was not provided for fixed-rate mortgages.', 'The next ECB rate cut is expected to be 2.75% or less.', 'The Euribor will initially quote just over 3% plus an average spread of 1%.', "The news headline in Repubblica on 2008-12-19 was: 'for TG1 the most important yo-yo of the fight against crime.'", "The headline was due to TG1 not reporting, in the 2008-11-29's 8 PM edition, the review on the fight against mafias organized by 'politicamente scorretto' in Casalecchio di Reno, Bologna.", 'The meeting on mafias was held a few hundred meters from the yo-yo championship.', 'Rita Borsellino raised a controversy regarding the location of the conference on mafias.']</t>
+          <t>['A letter requires 1 sheet plus an envelope.', 'An application requires 4 sheets.', 'Instructions require 2 sheets.', 'Photocopies require 2 sheets, or 4 sheets if a power of attorney is needed.', 'Each application requires a minimum of 9 sheets plus an envelope.', 'The estimated population is 1,300,000.', 'The total estimated sheets required is 11,700,000 sheets.', 'The total estimated reams required is 23,400 reams of 500-sheet paper.', 'Claudia Ceroni in Rome was misled by an increase in VAT on a non-essential good (Sky).', 'Lost tax deductions on structural renovations are causing the oversight of a graver problem than the new decree passed on 2008-11-25.', 'The structural engineer convinced the parents to renovate their home.', "The parents' renovation included improving roof insulation, installing sanitary water panels, a condensing boiler, and thermostatic valves.", "The total cost of the parents' renovation was about €10,000.", 'The structural engineer and the boyfriend spent an additional €50,000 on supplementary roof and window insulation.', 'The tax deduction for structural renovations is no longer certain, or it will be reduced from 55% to 35%.', "The structural engineer asked Minister Tremonti and the Prime Minister's staff who will reimburse the missed refund.", "De Mauro defined a scam as 'a crime committed by someone who obtains illicit profit to the detriment of others, having misled them with artifice and trickery.'", 'The government set a 4% mortgage rate in the maneuver.', 'The interest rate on variable-rate mortgages is expected not to exceed 4% by 2009.', 'The structural engineer stated that the benefit for families regarding the 4% mortgage rate is practically zero.', 'The structural engineer suggested applying the same principle to fixed-rate mortgages could help families.', 'A variable rate of 3.5% could be reached during 2009.', 'The news about the mafia and the choices of TG1 was published on page 19 of *Repubblica* on 2008-12-01.', "The headline on page 19 of *Repubblica* on 2008-12-01 was 'for TG1, the most important yo-yo in the fight against crime.'", "TG1 failed to report the review on the fight against the mafia organized by 'Politicamente Scorretto' in Casalecchio di Reno (Bologna) in the 8 PM edition on 2008-12-01.", 'The national edition of *Repubblica* decided not to report on the mafia conference.', '*Repubblica* limited its reporting to the protest of Rita Borsellino.', 'The editor of TG1 omitted that the mafia conference took place a few hundred meters from the yo-yo championship.', 'The proximity of the mafia conference to the yo-yo championship is the reason for the controversy raised by Borsellino.']</t>
         </is>
       </c>
     </row>
@@ -918,27 +866,17 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>A study by the Unione Nazionale Consumatori has ranked the cities with the largest annual increases, utilizing Istat data relating to last January. Consequently, Perugia and Terni finish in the top six most expensive cities, nearly reaching the podium. Specifically, in Perugia, the cost of electricity and gas saw an 85.8% growth, while Terni stopped at 85.4%. This minimal delta between the two provincial capitals indicates that the average utility expenditure is, in fact, uniform throughout the region. Specifically, considering the average expenditure of an Italian family, the average utility expenditure in Perugia is 1,157 euros on an annual basis; while that for a Terni family is 1,152 euros. It is a derby that finishes essentially tied (there is only a 5 euro difference), and winning it brings neither carousels nor parties with scarves and flags.
-Nationally, however, the survey compares the variation in electricity and gas prices over the last 3 years, comparing the free market with the regulated market. From June 2021, before the increases that started in July, to January 2023, electricity in the free market in Italy rose by 248.3% compared to 108.4% in the regulated market—more than double (+129%). Furthermore, considering the first useful gas data reported by Istat, December 2021, the free market since then increased by 141.1% compared to a 7.4% drop in the regulated market. In 3 years, from January 2020 to January 2023, free electricity jumped by 262.8%, compared to 115.8% in the regulated market.
-For electricity, gas, and other fuels—a category that includes gas, electricity (free and regulated market), heating oil, and solid fuels—if the increase in Italy in January was 67.3% compared to one year earlier, with an average utility expenditure for a family of 907.50 euros on an annual basis, in some cities it approached 90 percent.
-The comparison does not console the fact that Umbria is at the bottom of the podium, especially because the distance to the winner of the highest step is reduced. In Alessandria, expenses for electricity, gas, and heating oil soared by 88.6% in January 2022. Piemonte is fully stocked, with Vercelli recording an increase of 87.1% and Biella with an increase of 86.1%. On the other side of the ranking, the least affected city is Potenza with an increase of 35.2%. Aosta is second with an increase of 50.8%. At the bottom of the virtuous cities podium is Olbia-Tempio with an increase of 51%. Following are Napoli (+51.4%), Gorizia (+51.7%), Benevento (+53.1%), Caserta (+53.5%), then Avellino (+53.7%) and Trieste (+54.6%). Closing the top ten are Pordenone and Udine, tied at +54.7%.
-Another ranking, another study on the price run, comes from the CGIAG office of studies in Mestre, which indicates the weight of family purchasing power relative to inflation, which is accelerating. Over the two years 2022-2023, the loss of purchasing power in Umbria due to inflation could amount to nearly six thousand euros per family. The estimate is based on data from Banca d'Italia, Istat, and the European Commission. Given that bank deposits amounted to 14.5 billion euros at the end of 2021, in Umbria, the estimated loss of purchasing power in 2022 amounts to 1.2 billion euros, while in 2023, thanks to a slowdown in inflation, it amounts to 885 million, for a total of 2.1 billion euros. At the provincial level, the CGIAG data states that for Perugia, the loss of purchasing power could amount to over 1.6 billion euros (nearly 5,746 per family), while in Terni it is 536 million (5,251 per family). Here, the gap is clearer compared to the increases in electricity and gas bills.
-Luca Benedetti</t>
+          <t>According to a study by the National Consumers Union, which ranked cities based on the largest annual increases, the report analyzed Istat data from last January. Consequently, Perugia and Terni finished in the top six cities with the highest costs, nearly reaching the podium. Specifically, in Perugia, the cost of electricity and gas saw an 85.8% growth: while Terni recorded 85.4%. This minimal delta between the two city centers indicates that the cost of living is, in fact, uniform throughout the region. Considering the average expenditure of an Italian family, the cost of living in Perugia amounts to 1,157 euros on an annual basis; while for a family in Terni, it is 1,152 euros. A derby that essentially ends in a draw (there is only a 5 euro difference), and winning it neither leads to celebrations nor parades with scarves and flags. Nationally, however, the survey compares the variation in electricity and gas prices over the last three years, contrasting the free market with the regulated market. From June 2021, before the increases that began in July, electricity in the free market in Italy rose by 248.3% compared to 108.4% in the regulated market—more than double (+129%). Furthermore, considering the first available gas data from Istat, December 2021, the free market since then increased by 141.1% compared to a 7.4% decrease in the regulated market. In three years, from January 2020 to January 2023, free market electricity jumped by 262.8%, compared to 115.8% in the regulated market. For electricity, gas, and other fuels—a category that includes gas, electricity (free and regulated markets), heating oil, and solid fuels—if the increase in January was 67.3% compared to one year prior, the average family cost was 907.50 euros on an annual basis, with some cities approaching 90%. The comparison does little to console the fact that Umbria is at the foot of the podium, especially because the distance to the city at the top is reduced. In Alessandria, expenses for electricity, gas, and heating oil soared by 88.6% by January 2022. Piedmont is well-stocked, with Vercelli recording an increase of 87.1% and Biella with 86.1%. On the other side of the ranking, the least affected city is Potenza, with an increase of 35.2%. In second place is Aosta with an increase of 50.8%. At the bottom of the 'virtuous cities' podium is Olbia-Tempio with an increase of 51%. Following are Naples (+51.4%), Gorizia (+51.7%), Benevento (+53.1%), Caserta (+53.5%), then Avellino (+53.7%) and Trieste (+54.6%). Closing the top ten are Pordenone and Udine, tied at +54.7%. Another ranking, a study on price increases, comes from the CGIAR study office, which indicates the impact of family purchasing power relative to inflation, which is running wild. Over the two years 2022-2023, the loss of purchasing power in Umbria due to inflation could amount to nearly six million euros per family. The estimate is based on data from the Bank of Italy, Istat, and the European Commission. Against bank deposits, which amounted to 14.5 billion euros at the end of 2021, the estimated loss of purchasing power in Umbria in 2022 was 1.2 billion euros, while in 2023, thanks to a slowdown in inflation, it was 885 million euros, totaling 2.1 billion euros. At the provincial level, the CGIAR data states that for Perugia, the loss of purchasing power could amount to over 1.6 billion euros (nearly 5,746 per family), while in Terni, it is 536 million euros (5,251 per family). Here, the gap is clearer compared to the increases in electricity and gas bills.</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>Observation date: 2023-02-26 00:00:00. A study by the Unione Nazionale Consumatori has ranked the cities with the largest annual increases, utilizing Istat data relating to last January. Consequently, Perugia and Terni finish in the top six most expensive cities, nearly reaching the podium. Specifically, in Perugia, the cost of electricity and gas saw an 85.8% growth, while Terni stopped at 85.4%. This minimal delta between the two provincial capitals indicates that the average utility expenditure is, in fact, uniform throughout the region. Specifically, considering the average expenditure of an Italian family, the average utility expenditure in Perugia is 1,157 euros on an annual basis; while that for a Terni family is 1,152 euros. It is a derby that finishes essentially tied (there is only a 5 euro difference), and winning it brings neither carousels nor parties with scarves and flags.
-Nationally, however, the survey compares the variation in electricity and gas prices over the last 3 years, comparing the free market with the regulated market. From June 2021, before the increases that started in July, to January 2023, electricity in the free market in Italy rose by 248.3% compared to 108.4% in the regulated market—more than double (+129%). Furthermore, considering the first useful gas data reported by Istat, December 2021, the free market since then increased by 141.1% compared to a 7.4% drop in the regulated market. In 3 years, from January 2020 to January 2023, free electricity jumped by 262.8%, compared to 115.8% in the regulated market.
-For electricity, gas, and other fuels—a category that includes gas, electricity (free and regulated market), heating oil, and solid fuels—if the increase in Italy in January was 67.3% compared to one year earlier, with an average utility expenditure for a family of 907.50 euros on an annual basis, in some cities it approached 90 percent.
-The comparison does not console the fact that Umbria is at the bottom of the podium, especially because the distance to the winner of the highest step is reduced. In Alessandria, expenses for electricity, gas, and heating oil soared by 88.6% in January 2022. Piemonte is fully stocked, with Vercelli recording an increase of 87.1% and Biella with an increase of 86.1%. On the other side of the ranking, the least affected city is Potenza with an increase of 35.2%. Aosta is second with an increase of 50.8%. At the bottom of the virtuous cities podium is Olbia-Tempio with an increase of 51%. Following are Napoli (+51.4%), Gorizia (+51.7%), Benevento (+53.1%), Caserta (+53.5%), then Avellino (+53.7%) and Trieste (+54.6%). Closing the top ten are Pordenone and Udine, tied at +54.7%.
-Another ranking, another study on the price run, comes from the CGIAG office of studies in Mestre, which indicates the weight of family purchasing power relative to inflation, which is accelerating. Over the two years 2022-2023, the loss of purchasing power in Umbria due to inflation could amount to nearly six thousand euros per family. The estimate is based on data from Banca d'Italia, Istat, and the European Commission. Given that bank deposits amounted to 14.5 billion euros at the end of 2021, in Umbria, the estimated loss of purchasing power in 2022 amounts to 1.2 billion euros, while in 2023, thanks to a slowdown in inflation, it amounts to 885 million, for a total of 2.1 billion euros. At the provincial level, the CGIAG data states that for Perugia, the loss of purchasing power could amount to over 1.6 billion euros (nearly 5,746 per family), while in Terni it is 536 million (5,251 per family). Here, the gap is clearer compared to the increases in electricity and gas bills.
-Luca Benedetti</t>
+          <t>Observation date: 2023-02-26 00:00:00. According to a study by the National Consumers Union, which ranked cities based on the largest annual increases, the report analyzed Istat data from last January. Consequently, Perugia and Terni finished in the top six cities with the highest costs, nearly reaching the podium. Specifically, in Perugia, the cost of electricity and gas saw an 85.8% growth: while Terni recorded 85.4%. This minimal delta between the two city centers indicates that the cost of living is, in fact, uniform throughout the region. Considering the average expenditure of an Italian family, the cost of living in Perugia amounts to 1,157 euros on an annual basis; while for a family in Terni, it is 1,152 euros. A derby that essentially ends in a draw (there is only a 5 euro difference), and winning it neither leads to celebrations nor parades with scarves and flags. Nationally, however, the survey compares the variation in electricity and gas prices over the last three years, contrasting the free market with the regulated market. From June 2021, before the increases that began in July, electricity in the free market in Italy rose by 248.3% compared to 108.4% in the regulated market—more than double (+129%). Furthermore, considering the first available gas data from Istat, December 2021, the free market since then increased by 141.1% compared to a 7.4% decrease in the regulated market. In three years, from January 2020 to January 2023, free market electricity jumped by 262.8%, compared to 115.8% in the regulated market. For electricity, gas, and other fuels—a category that includes gas, electricity (free and regulated markets), heating oil, and solid fuels—if the increase in January was 67.3% compared to one year prior, the average family cost was 907.50 euros on an annual basis, with some cities approaching 90%. The comparison does little to console the fact that Umbria is at the foot of the podium, especially because the distance to the city at the top is reduced. In Alessandria, expenses for electricity, gas, and heating oil soared by 88.6% by January 2022. Piedmont is well-stocked, with Vercelli recording an increase of 87.1% and Biella with 86.1%. On the other side of the ranking, the least affected city is Potenza, with an increase of 35.2%. In second place is Aosta with an increase of 50.8%. At the bottom of the 'virtuous cities' podium is Olbia-Tempio with an increase of 51%. Following are Naples (+51.4%), Gorizia (+51.7%), Benevento (+53.1%), Caserta (+53.5%), then Avellino (+53.7%) and Trieste (+54.6%). Closing the top ten are Pordenone and Udine, tied at +54.7%. Another ranking, a study on price increases, comes from the CGIAR study office, which indicates the impact of family purchasing power relative to inflation, which is running wild. Over the two years 2022-2023, the loss of purchasing power in Umbria due to inflation could amount to nearly six million euros per family. The estimate is based on data from the Bank of Italy, Istat, and the European Commission. Against bank deposits, which amounted to 14.5 billion euros at the end of 2021, the estimated loss of purchasing power in Umbria in 2022 was 1.2 billion euros, while in 2023, thanks to a slowdown in inflation, it was 885 million euros, totaling 2.1 billion euros. At the provincial level, the CGIAR data states that for Perugia, the loss of purchasing power could amount to over 1.6 billion euros (nearly 5,746 per family), while in Terni, it is 536 million euros (5,251 per family). Here, the gap is clearer compared to the increases in electricity and gas bills.</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>['A study by the Unione Nazionale Consumatori utilized Istat data relating to January 2023 to rank cities by annual increases.', 'Perugia and Terni finished in the top six most expensive cities according to the Unione Nazionale Consumatori study.', 'In Perugia, the cost of electricity and gas saw an 85.8% growth.', 'The average utility expenditure for an Italian family in Perugia is 1,157 euros on an annual basis.', 'The survey comparing electricity and gas prices nationally compares the free market with the regulated market.', 'From June 2021 to January 2023, electricity in the free market in Italy rose by 248.3% compared to 108.4% in the regulated market.', 'The free market increase in electricity was more than double the regulated market increase (+129%).', 'Considering the first useful gas data reported by Istat in December 2021, the free market increased by 141.1% compared to a 7.4% drop in the regulated market.', 'In three years, from January 2020 to January 2023, free electricity jumped by 262.8% compared to 115.8% in the regulated market.', 'For electricity, gas, and other fuels, the increase in Italy in January was 67.3% compared to one year earlier.', 'In Alessandria, expenses for electricity, gas, and heating oil soared by 88.6% in January 2022.', 'Vercelli recorded an increase of 87.1% for electricity, gas, and heating oil.', 'Potenza was the least affected city with an increase of 35.2%.', 'Olbia-Tempio recorded an increase of 51%.', 'Benevento recorded an increase of 53.1%.', 'Trieste recorded an increase of 54.6%.', 'Pordenone and Udine were tied at an increase of 54.7%.', 'The CGIAG office of studies in Mestre conducted a study on the weight of family purchasing power relative to inflation.', 'Over the two years 2022-2023, the loss of purchasing power in Umbria due to inflation could amount to nearly six thousand euros per family.', "The estimate of purchasing power loss is based on data from Banca d'Italia, Istat, and the European Commission.", 'Bank deposits amounted to 14.5 billion euros in Umbria at the end of 2021.', 'The total estimated loss of purchasing power in Umbria over 2022 and 2023 is 2.1 billion euros.', 'The CGIAG data states that the loss of purchasing power for Perugia could amount to over 1.6 billion euros.']</t>
+          <t>['The National Consumers Union conducted a study ranking cities based on the largest annual increases.', 'The report analyzed Istat data from January 2023.', 'Perugia and Terni finished among the top six cities with the highest costs.', 'The cost of electricity and gas in Perugia saw an 85.8% growth.', 'Terni recorded an 85.4% growth in the cost of electricity and gas.', 'The average cost of living for an Italian family in Perugia is 1,157 euros annually.', 'The survey compares the variation in electricity and gas prices over the last three years.', 'The survey contrasts the free market with the regulated market for electricity and gas prices.', 'From June 2021, electricity in the regulated market in Italy rose by 108.4%.', 'The increase in the free market electricity price was more than double the increase in the regulated market electricity price (+129%).', 'According to Istat data from December 2021, the regulated market gas price decreased by 7.4%.', 'From January 2020 to January 2023, regulated market electricity jumped by 115.8%.', 'If the increase in electricity, gas, and other fuels in January was 67.3% compared to one year prior, the average family cost was 907.50 euros annually.', 'Expenses for electricity, gas, and heating oil in Alessandria soared by 88.6% by January 2022.', 'Vercelli recorded an increase of 87.1% in Piedmont.', 'Potenza was the least affected city, recording an increase of 35.2%.', 'Aosta was in second place with an increase of 50.8%.', "Olbia-Tempio was at the bottom of the 'virtuous cities' podium with an increase of 51%.", 'Benevento recorded an increase of 53.1%.', 'Avellino recorded an increase of 53.7%.', 'Trieste recorded an increase of 54.6%.', 'Pordenone and Udine tied for the top ten with an increase of 54.7%.', 'Over the two years 2022-2023, the loss of purchasing power in Umbria due to inflation could amount to nearly six million euros per family.', 'The estimate of purchasing power loss is based on data from the Bank of Italy, Istat, and the European Commission.', 'Bank deposits amounted to 14.5 billion euros at the end of 2021.', 'The total estimated loss of purchasing power in Umbria over 2022 and 2023 was 2.1 billion euros.', 'CGIAR data states that the loss of purchasing power for Perugia could amount to over 1.6 billion euros.', 'CGIAR data states that the loss of purchasing power for Perugia is nearly 5,746 euros per family.']</t>
         </is>
       </c>
     </row>
@@ -988,17 +926,17 @@
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
-          <t>... the closing of the major international stock exchanges. The performance of the Dow Jones (see page 5) and Glauco Maggi New York received a new stimulus package in Congress to boost the American economy, which is in a severe crisis. Yesterday, this effort received support from Federal Reserve President Ben Bernanke and conditional approval from President Bush. Regarding the future of the US economy, the central bank also factors in a further cut in interest rates, thanks to inflation being kept low by the recession. For Bernanke, who spoke before the House Budget Committee, the credit crisis "is hitting the economy" because Americans are having difficulty finding money for their activities. "With an economy likely to be weak for several quarters still, and the risk of a prolonged slowdown, the idea of a fiscal package seems appropriate in this context," the governor told the deputies, though refusing to define the ideal size of the intervention. An hour after these statements of technical support, political approval arrived for putting a second fiscal package on the agenda in the country. The Bush administration "is open to ideas that could stimulate the economy and help us exit this downward spiral faster," echoed the President's spokesperson, Dana Perino, Bernanke. But the okay will only come if the ideas are capable of "truly stimulating the economy." Congress, which is responsible for approving a second fiscal package after the one passed earlier this year, which yielded very limited benefits, according to the Fed governor, "should include measures to facilitate access to credit for consumers, homeowners, and generally for anyone interested in obtaining loans. Such actions could be particularly effective," Bernanke ventured, "in promoting economic growth and job creation." Wall Street, which had already started positively, expanded its gains after the promise of stimulus from the central bank and the availability of Bush. The Dow Jones index rose above 9,000 points, with a gain of 4.67%, as did the Nasdaq, which gained 3.43%, closing at 1,700 points. Meanwhile, the dollar strengthened against the euro, falling to 1.33 dollars from 1.34 at the start. Europe also rose, where Londra shone (+5.41%), followed by Parigi (+3.56%), Madrid (+2.99%), and Milano (+2.65%). Frankfurt was more cautious (+1.12%). Contributing to the boost in stock purchases was also Bernanke's mention of a new rate cut at the Fed meeting at the end of October. Federal bonds are expected to see a 100% reduction of 25 cents in yield, but for the 46% it could also be half a point, like the previous one done together by all the banks. The fate of the American budget, however, is no longer a problem for anyone, in these current global market conditions where public spending is dominating to build a barrier against the threat of depression. The newly awarded Nobel laureate in economics, Paul Krugman, wrote this in the New York Times, calling for massive injections of state money into banks, and Bernanke himself mentioned it in his speech: "the current deficit is large," he admitted, "but not inappropriate given the nature of the emergency we are facing and unavoidable given the loss of tax revenue." Bernanke is aware that "every fiscal action inevitably entails trade-offs" and could "weigh on future generations," but he accepted the inevitability of the intervention. Without defining the current state of the economy as a recession, the governor predicted that "the pace of economic activity will remain below potential growth for numerous quarters, and that the slowdown in investment and business spending extends to the major sectors."</t>
+          <t>The closing of major international exchanges. The performance of the Dow Jones (see page 5) gave the Dow Jones and New York a new package to vote on in Congress to stimulate the American economy, which is in a severe crisis. Yesterday, this package received support from the Federal Reserve Chairman, Ben Bernanke, and conditional approval from President Bush. Looking into the near future of the US economy, the central bank is also considering a further cut in rates, thanks to inflation being kept low by the recession. For Bernanke, who spoke before the House Budget Committee, the credit crisis 'is hitting the economy' because Americans are having difficulty finding money for their activities. 'With an economy probably destined to be weak for several quarters still, and the risk of a prolonged slowdown, the idea of a fiscal package seems appropriate in this juncture,' the governor told the deputies, though refusing to define the ideal size of the intervention. An hour after these statements of technical support, the political green light arrived for putting a second fiscal drug package on the agenda in the country. The Bush administration 'is open to ideas that could stimulate the economy and help us exit this downward spiral faster,' echoed the President's spokesperson, Dana Perino, repeating Bernanke's words. But the okay will only come if the ideas are 'truly capable of stimulating the economy.' The Congress, which is responsible for approving a second fiscal package after the one passed earlier this year, which yielded very limited benefits, according to the Fed governor, 'should include measures to facilitate access to credit for consumers, homeowners, and generally anyone interested in obtaining loans. Such actions could be particularly effective' in 'promoting economic growth and job creation.' Wall Street, which had already started positively, expanded its gains after the promise of stimulus from the central bank and the availability of Bush. The Dow Jones index rose above 9,000 points, with a gain of 4.67%, and the Nasdaq also gained 3.43% at 1,700 points, while the dollar strengthened against the euro, falling to $1.33 from $1.34 at the start. Europe also rose, with London leading (+5.41%), followed by Paris (+3.56%), Madrid (+2.99%), and Milan (+2.65%). Frankfurt was more cautious (+1.12%). Contributing to the boost in stock purchases was also Bernanke's mention of a new rate cut at the Fed meeting at the end of October. Federal bonds discount, at 100%, a reduction of 25 cents, but for the 46% it could also be half a point, like the previous one done together by all banks. The fate of the American budget, however, is no longer a problem for anyone, in these global times of clear moons where public spending is dominating to build a barrier against the threat of depression. The newly awarded Nobel laureate in economics, Paul Krugman, wrote this in the New York Times, calling for massive state injections of money into banks, and Bernanke himself mentioned this in his speech: 'the current deficit is large,' he admitted, 'but not inappropriate given the nature of the emergency we are facing and unavoidable given the loss of tax revenue.' Bernanke is aware that 'every fiscal action inevitably entails trade-offs' and could 'weigh on future generations,' but he accepted the inevitability of the intervention. Without defining the current state of the economy as a recession, the governor predicted that 'the pace of economic activity will remain below potential growth for numerous quarters, and that the slowdown in investment and business spending extends to major sectors.'</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>Observation date: 2008-10-21 00:00:00. ... the closing of the major international stock exchanges. The performance of the Dow Jones (see page 5) and Glauco Maggi New York received a new stimulus package in Congress to boost the American economy, which is in a severe crisis. Yesterday, this effort received support from Federal Reserve President Ben Bernanke and conditional approval from President Bush. Regarding the future of the US economy, the central bank also factors in a further cut in interest rates, thanks to inflation being kept low by the recession. For Bernanke, who spoke before the House Budget Committee, the credit crisis "is hitting the economy" because Americans are having difficulty finding money for their activities. "With an economy likely to be weak for several quarters still, and the risk of a prolonged slowdown, the idea of a fiscal package seems appropriate in this context," the governor told the deputies, though refusing to define the ideal size of the intervention. An hour after these statements of technical support, political approval arrived for putting a second fiscal package on the agenda in the country. The Bush administration "is open to ideas that could stimulate the economy and help us exit this downward spiral faster," echoed the President's spokesperson, Dana Perino, Bernanke. But the okay will only come if the ideas are capable of "truly stimulating the economy." Congress, which is responsible for approving a second fiscal package after the one passed earlier this year, which yielded very limited benefits, according to the Fed governor, "should include measures to facilitate access to credit for consumers, homeowners, and generally for anyone interested in obtaining loans. Such actions could be particularly effective," Bernanke ventured, "in promoting economic growth and job creation." Wall Street, which had already started positively, expanded its gains after the promise of stimulus from the central bank and the availability of Bush. The Dow Jones index rose above 9,000 points, with a gain of 4.67%, as did the Nasdaq, which gained 3.43%, closing at 1,700 points. Meanwhile, the dollar strengthened against the euro, falling to 1.33 dollars from 1.34 at the start. Europe also rose, where Londra shone (+5.41%), followed by Parigi (+3.56%), Madrid (+2.99%), and Milano (+2.65%). Frankfurt was more cautious (+1.12%). Contributing to the boost in stock purchases was also Bernanke's mention of a new rate cut at the Fed meeting at the end of October. Federal bonds are expected to see a 100% reduction of 25 cents in yield, but for the 46% it could also be half a point, like the previous one done together by all the banks. The fate of the American budget, however, is no longer a problem for anyone, in these current global market conditions where public spending is dominating to build a barrier against the threat of depression. The newly awarded Nobel laureate in economics, Paul Krugman, wrote this in the New York Times, calling for massive injections of state money into banks, and Bernanke himself mentioned it in his speech: "the current deficit is large," he admitted, "but not inappropriate given the nature of the emergency we are facing and unavoidable given the loss of tax revenue." Bernanke is aware that "every fiscal action inevitably entails trade-offs" and could "weigh on future generations," but he accepted the inevitability of the intervention. Without defining the current state of the economy as a recession, the governor predicted that "the pace of economic activity will remain below potential growth for numerous quarters, and that the slowdown in investment and business spending extends to the major sectors."</t>
+          <t>Observation date: 2008-10-21 00:00:00. The closing of major international exchanges. The performance of the Dow Jones (see page 5) gave the Dow Jones and New York a new package to vote on in Congress to stimulate the American economy, which is in a severe crisis. Yesterday, this package received support from the Federal Reserve Chairman, Ben Bernanke, and conditional approval from President Bush. Looking into the near future of the US economy, the central bank is also considering a further cut in rates, thanks to inflation being kept low by the recession. For Bernanke, who spoke before the House Budget Committee, the credit crisis 'is hitting the economy' because Americans are having difficulty finding money for their activities. 'With an economy probably destined to be weak for several quarters still, and the risk of a prolonged slowdown, the idea of a fiscal package seems appropriate in this juncture,' the governor told the deputies, though refusing to define the ideal size of the intervention. An hour after these statements of technical support, the political green light arrived for putting a second fiscal drug package on the agenda in the country. The Bush administration 'is open to ideas that could stimulate the economy and help us exit this downward spiral faster,' echoed the President's spokesperson, Dana Perino, repeating Bernanke's words. But the okay will only come if the ideas are 'truly capable of stimulating the economy.' The Congress, which is responsible for approving a second fiscal package after the one passed earlier this year, which yielded very limited benefits, according to the Fed governor, 'should include measures to facilitate access to credit for consumers, homeowners, and generally anyone interested in obtaining loans. Such actions could be particularly effective' in 'promoting economic growth and job creation.' Wall Street, which had already started positively, expanded its gains after the promise of stimulus from the central bank and the availability of Bush. The Dow Jones index rose above 9,000 points, with a gain of 4.67%, and the Nasdaq also gained 3.43% at 1,700 points, while the dollar strengthened against the euro, falling to $1.33 from $1.34 at the start. Europe also rose, with London leading (+5.41%), followed by Paris (+3.56%), Madrid (+2.99%), and Milan (+2.65%). Frankfurt was more cautious (+1.12%). Contributing to the boost in stock purchases was also Bernanke's mention of a new rate cut at the Fed meeting at the end of October. Federal bonds discount, at 100%, a reduction of 25 cents, but for the 46% it could also be half a point, like the previous one done together by all banks. The fate of the American budget, however, is no longer a problem for anyone, in these global times of clear moons where public spending is dominating to build a barrier against the threat of depression. The newly awarded Nobel laureate in economics, Paul Krugman, wrote this in the New York Times, calling for massive state injections of money into banks, and Bernanke himself mentioned this in his speech: 'the current deficit is large,' he admitted, 'but not inappropriate given the nature of the emergency we are facing and unavoidable given the loss of tax revenue.' Bernanke is aware that 'every fiscal action inevitably entails trade-offs' and could 'weigh on future generations,' but he accepted the inevitability of the intervention. Without defining the current state of the economy as a recession, the governor predicted that 'the pace of economic activity will remain below potential growth for numerous quarters, and that the slowdown in investment and business spending extends to major sectors.'</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>['The Dow Jones and Glauco Maggi New York received a new stimulus package in Congress.', 'The stimulus package aims to boost the American economy.', 'The American economy is in a severe crisis.', 'On 2008-10-20, the effort received support from Federal Reserve President Ben Bernanke.', 'On 2008-10-20, the effort received conditional approval from President Bush.', 'The central bank factors in a further cut in interest rates regarding the future of the US economy.', 'The recession is keeping inflation low.', 'Ben Bernanke spoke before the House Budget Committee.', 'Ben Bernanke stated that the credit crisis is hitting the economy.', 'The credit crisis is causing Americans to have difficulty finding money for their activities.', 'Ben Bernanke told the deputies that a fiscal package seems appropriate.', 'The economy is likely to be weak for several quarters.', 'There is a risk of a prolonged slowdown.', "Political approval arrived for putting a second fiscal package on the agenda in the country an hour after Ben Bernanke's statements.", "Dana Perino, the President's spokesperson, echoed Ben Bernanke's statement that the Bush administration is open to ideas that could stimulate the economy.", 'Dana Perino stated that the Bush administration is open to ideas that could help exit the downward spiral faster.', 'Congress is responsible for approving a second fiscal package.', 'The second fiscal package would follow the one passed on 2008-01-01.', 'Ben Bernanke stated that the first fiscal package yielded very limited benefits.', 'Ben Bernanke suggested that the second fiscal package should include measures to facilitate access to credit for consumers, homeowners, and anyone interested in obtaining loans.', 'Ben Bernanke believes that facilitating access to credit could promote economic growth and job creation.', 'Wall Street expanded its gains after the promise of stimulus from the central bank.', 'Wall Street expanded its gains after the availability of President Bush.', 'The Dow Jones index rose above 9,000 points.', 'The Dow Jones index gained 4.67%.', 'The Nasdaq gained 3.43%.', 'The Nasdaq closed at 1,700 points.', 'The dollar strengthened against the euro.', 'The dollar fell to 1.33 dollars from 1.34 at the start.', 'Londra rose by 5.41%.', 'Parigi rose by 3.56%.', 'Madrid rose by 2.99%.', 'Milano rose by 2.65%.', 'Frankfurt rose by 1.12%.', "Bernanke's mention of a new rate cut at the Fed meeting at the end of October contributed to the boost in stock purchases.", 'Federal bonds are expected to see a 100% reduction of 25 cents in yield.', 'For the 46%, the yield reduction could be half a point.', 'Paul Krugman wrote in the New York Times, calling for massive injections of state money into banks.', 'Ben Bernanke admitted that the current deficit is large.', 'Ben Bernanke stated that the current deficit is not inappropriate given the nature of the emergency.', 'Ben Bernanke stated that the current deficit is unavoidable given the loss of tax revenue.', 'Ben Bernanke is aware that every fiscal action entails trade-offs.', 'Ben Bernanke acknowledged that fiscal actions could weigh on future generations.', 'Ben Bernanke predicted that the pace of economic activity will remain below potential growth for numerous quarters.', 'Ben Bernanke predicted that the slowdown in investment and business spending extends to the major sectors.']</t>
+          <t>['The performance of the Dow Jones gave the Dow Jones and New York a new package to vote on in Congress.', 'The package was intended to stimulate the American economy.', 'The American economy was in a severe crisis.', 'On 2008-10-20, the package received support from Ben Bernanke.', 'On 2008-10-20, the package received conditional approval from President Bush.', 'The central bank is considering a further cut in rates for the US economy.', 'The recession kept inflation low.', 'Ben Bernanke stated that the credit crisis is hitting the economy.', 'The credit crisis is hitting the economy because Americans are having difficulty finding money for their activities.', 'Ben Bernanke told the deputies that a fiscal package seems appropriate.', 'Ben Bernanke stated the economy is probably destined to be weak for several quarters.', 'Ben Bernanke mentioned the risk of a prolonged slowdown.', "An hour after Ben Bernanke's statements, the political green light arrived for putting a second fiscal package on the agenda.", "Dana Perino, the President's spokesperson, stated the Bush administration is open to ideas that could stimulate the economy.", "Dana Perino repeated Ben Bernanke's words.", 'The Congress is responsible for approving a second fiscal package.', 'The first fiscal package passed earlier on 2008-01-01 yielded very limited benefits, according to Ben Bernanke.', 'Ben Bernanke stated the second fiscal package should include measures to facilitate access to credit for consumers, homeowners, and anyone interested in obtaining loans.', 'Such actions could be particularly effective in promoting economic growth and job creation.', 'Wall Street expanded its gains after the promise of stimulus from the central bank.', 'Wall Street expanded its gains after the availability of Bush.', 'The Dow Jones index rose above 9,000 points.', 'The Dow Jones index gained 4.67%.', 'The Nasdaq gained 3.43% at 1,700 points.', 'The dollar strengthened against the euro.', 'The dollar fell to $1.33 from $1.34 against the euro.', 'London rose by 5.41%.', 'Paris rose by 3.56%.', 'Madrid rose by 2.99%.', 'Milan rose by 2.65%.', 'Frankfurt rose by 1.12%.', "Bernanke's mention of a new rate cut at the Fed meeting at the end of October contributed to the boost in stock purchases.", 'Federal bonds discount was at 100%.', 'The discount reduction was 25 cents.', 'The discount could be half a point for the 46%.', 'Paul Krugman wrote in the New York Times calling for massive state injections of money into banks.', 'Ben Bernanke admitted that the current deficit is large.', 'Ben Bernanke stated the current deficit is not inappropriate given the nature of the emergency.', 'Ben Bernanke stated the deficit is unavoidable given the loss of tax revenue.', 'Ben Bernanke is aware that every fiscal action inevitably entails trade-offs.', 'Ben Bernanke acknowledged that fiscal actions could weigh on future generations.', 'Ben Bernanke predicted that the pace of economic activity will remain below potential growth for numerous quarters.', 'Ben Bernanke predicted that the slowdown in investment and business spending extends to major sectors.']</t>
         </is>
       </c>
     </row>
@@ -1048,17 +986,17 @@
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
-          <t>If, instead, there had been the capacity to generate income from those savings, even with a remuneration of one percentage point, families would have gained a total of 30 billion, nearly 2% of the Gross Domestic Product (GDP). "The savings rate of Italian families relative to disposable income has grown by 50% in the year, but, excluding savings invested in listed companies, its yield has remained rather low, close to zero. Given the consistency of financial assets held by families, every percentage point of remuneration can be estimated at around 30 billion euros, nearly 2% of GDP, the size of a good public budget maneuver from the past." The core theme of the annual report by CONSOB President Paolo Savona is the primary asset that the authority he leads intends to protect: savings. But this is now threatened by a shadow lengthening over international markets—one that is very difficult to control: the sirens of cryptocurrencies and Bitcoin. A phenomenon in strong growth and increasingly difficult to keep under control, much so that it has prompted Savona to issue a warning: the speculative effect they are triggering seems very similar to what happened before 2008 with subprime mortgages. "The diffusion of virtual instruments has stimulated the birth of the already remembered technological platforms," he said. "These new market segments are rapidly evolving, and the experience preceding the 2008 crisis seems to be repeating itself, when derivatives contracts developed to reach a size ten times the global GDP, assuming complex forms that received a high rating. With due distinctions, it is predictable that something analogous is happening in the market for virtual monetary and financial products, especially cryptocurrencies." Savona recalled how "a single Bitcoin recently had the ability to purchase a large-cylinder electric car and shortly after lost half of its purchasing power." For the president of CONSOB, "financial informatics is a prodigious lamp from which genius has emerged. The authorities will not be able to put it back, because it operates in the immaterial sphere controllable only by changing the information exchange protocol, thus fragmenting the unit of the global market and thereby reducing the international competitiveness rate." Traditional supervisory tools are no longer sufficient. Under current conditions, according to Savona, "the authorities can intervene by also utilizing the advantages of digitized techniques; their action will be more effective if they cooperate with each other." For Italy, the issue is even more delicate due to the constitutional norm that confers upon the "Republic the task of encouraging and protecting savings in all their forms and of regulating, coordinating, and controlling the exercise of credit." It would be inappropriate, he explained, "if the specification of 'savings in all their forms' and the credit to be protected were given content that also encompassed virtual instruments, without passing through specific regulation." These currencies are based on blockchain. "As far as is known about the state of hacking techniques, the original blockchain is impenetrable, while that used by other cryptocurrencies is not," he concluded. And once again, there is a call to proceed quickly with regulatory systems. "Without adequate safeguards (rules and bodies)—he said—there results a deterioration of market transparency, the foundation of legality and the rational choices of operators. Among the well-known negative effects is the shielding that these techniques allow to criminal activities, such as tax evasion, money laundering, the financing of terrorism, and the kidnapping of persons." Savona recalled CONSOB's activity in obscuring hundreds of websites in Italy that were illegally collecting savings. But in this context, it is somewhat like emptying the sea with your hands. Savona obviously hopes for an international solution. "The issue of cybersecurity encompasses political problems of even broader content, the solution of which cannot be achieved at the national level and requires close international cooperation, such as the birth of a 'global public good,' like the FMI, the ONU, and the WTO. The part of the Bretton Woods agreement addressing the problem of interchangeability between different national currencies did not withstand the test of international cooperation, but technological innovations applied to finance have revived the urgency of its relaunch in a contemporary context," he stated. The president of CONSOB also relaunched the proposal to unify the single text on finance and the single banking text, suggesting closer collaboration among Italian authorities. "To this end, it is necessary to activate in Italy formal consultation structures between governing bodies and independent authorities that impose a unitary direction to choices in the matter, also with a view to the position to be assumed regarding ongoing European and international initiatives—he explained. A first step would be adopting the recommendation from the European Committee for Systemic Risk of 2011, which would establish a single national counterparty responsible for macro-prudential stability. The Banca d’Italia would maintain a central role, justified by its participation in the Eurosystem around which European finance currently revolves, but strict coordination would be guaranteed among the three independent supervisory authorities (CONSOB, IVASS, and COVIP), with the participation of the Ministry of Economy." "To cope with economic and social difficulties, public debt has grown greatly, albeit in forms different from what an emergency state would have required. However, confidence in the reaction capabilities of the Italian economy has grown. This result is also the fruit of the decisions made by the BCE to purchase significant volumes of public bonds and by the European Commission to suspend, even if temporarily, the Stability Pact and to launch the Next Generation EU plan. We agree with the assessment that these decisions will structurally improve our real growth rate." Now, however, it is necessary to change pace. "However, for the continuation of the productive relaunch phase, it is necessary to integrate the decisions taken so far to incentivize corporate venture capital, thereby improving their financial leverage and making them more available to undertake new initiatives," said Savona, who believes that "the fiscal reform long requested offers an important opportunity," especially "by assigning it the task of considering productive demands on the same level as ethical ones in the assessments of distributive equity."</t>
+          <t xml:space="preserve">If there had been the ability to generate income from those savings, even with a remuneration of one percentage point, households would have collectively earned 30 billion, almost 2% of the gross domestic product. 'The savings rate of Italian households relative to disposable income has grown by 50% in the year, but, excluding savings invested in listed companies, its return has remained quite low, close to zero. Given the consistency of financial assets held by households, every percentage point of remuneration can be estimated at around 30 billion euros, almost 2% of GDP, the size of a good public budget maneuver in the past.' The core theme of the annual report by the President of Consob, Paolo Savona, is the primary asset that the authority he leads intends to protect: savings. But this has been focused on deposits for the last two years. And now it is threatened by a shadow lengthening over international markets, which is very difficult to control: these are the sirens of cryptocurrencies and Bitcoin. A phenomenon that is growing rapidly and becoming increasingly difficult to contain, much so that it has prompted Savona to sound the alarm: the speculative effect they are triggering seems very similar to what happened before 2008 with subprime mortgages. 'The spread of virtual instruments has stimulated the birth of the already remembered technological platforms,' he said. 'These new market segments are rapidly evolving, and the experience preceding the 2008 crisis seems to be repeating itself, when derivative contracts developed to reach a size ten times the global GDP, assuming complex forms that received high ratings. With due distinctions, it is predictable that something analogous is happening in the market for virtual monetary and financial products, especially crypto.' Savona recalled how 'a single Bitcoin recently had the ability to purchase a large electric car and shortly after lost half its purchasing power.' For the President of Consob, 'financial technology is a prodigious lamp from which genius has emerged. The authorities will not be able to put it back, because it operates in the immaterial sphere controllable only by changing the information exchange protocol, thus fragmenting the unit of the global market and reducing the international competitiveness rate.' Traditional supervisory tools are no longer sufficient. Under current conditions, according to Savona, 'the authorities can intervene by also utilizing the advantages of digitized techniques; their action will be more effective if they cooperate with each other.' For Italy, the issue is even more delicate due to the constitutional rule that assigns the 'Republic the task of encouraging and protecting savings in all their forms and of regulating, coordinating, and controlling the exercise of credit.' It would be inappropriate, he explained, 'if the specification of </t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>Observation date: 2021-06-14 00:00:00. If, instead, there had been the capacity to generate income from those savings, even with a remuneration of one percentage point, families would have gained a total of 30 billion, nearly 2% of the Gross Domestic Product (GDP). "The savings rate of Italian families relative to disposable income has grown by 50% in the year, but, excluding savings invested in listed companies, its yield has remained rather low, close to zero. Given the consistency of financial assets held by families, every percentage point of remuneration can be estimated at around 30 billion euros, nearly 2% of GDP, the size of a good public budget maneuver from the past." The core theme of the annual report by CONSOB President Paolo Savona is the primary asset that the authority he leads intends to protect: savings. But this is now threatened by a shadow lengthening over international markets—one that is very difficult to control: the sirens of cryptocurrencies and Bitcoin. A phenomenon in strong growth and increasingly difficult to keep under control, much so that it has prompted Savona to issue a warning: the speculative effect they are triggering seems very similar to what happened before 2008 with subprime mortgages. "The diffusion of virtual instruments has stimulated the birth of the already remembered technological platforms," he said. "These new market segments are rapidly evolving, and the experience preceding the 2008 crisis seems to be repeating itself, when derivatives contracts developed to reach a size ten times the global GDP, assuming complex forms that received a high rating. With due distinctions, it is predictable that something analogous is happening in the market for virtual monetary and financial products, especially cryptocurrencies." Savona recalled how "a single Bitcoin recently had the ability to purchase a large-cylinder electric car and shortly after lost half of its purchasing power." For the president of CONSOB, "financial informatics is a prodigious lamp from which genius has emerged. The authorities will not be able to put it back, because it operates in the immaterial sphere controllable only by changing the information exchange protocol, thus fragmenting the unit of the global market and thereby reducing the international competitiveness rate." Traditional supervisory tools are no longer sufficient. Under current conditions, according to Savona, "the authorities can intervene by also utilizing the advantages of digitized techniques; their action will be more effective if they cooperate with each other." For Italy, the issue is even more delicate due to the constitutional norm that confers upon the "Republic the task of encouraging and protecting savings in all their forms and of regulating, coordinating, and controlling the exercise of credit." It would be inappropriate, he explained, "if the specification of 'savings in all their forms' and the credit to be protected were given content that also encompassed virtual instruments, without passing through specific regulation." These currencies are based on blockchain. "As far as is known about the state of hacking techniques, the original blockchain is impenetrable, while that used by other cryptocurrencies is not," he concluded. And once again, there is a call to proceed quickly with regulatory systems. "Without adequate safeguards (rules and bodies)—he said—there results a deterioration of market transparency, the foundation of legality and the rational choices of operators. Among the well-known negative effects is the shielding that these techniques allow to criminal activities, such as tax evasion, money laundering, the financing of terrorism, and the kidnapping of persons." Savona recalled CONSOB's activity in obscuring hundreds of websites in Italy that were illegally collecting savings. But in this context, it is somewhat like emptying the sea with your hands. Savona obviously hopes for an international solution. "The issue of cybersecurity encompasses political problems of even broader content, the solution of which cannot be achieved at the national level and requires close international cooperation, such as the birth of a 'global public good,' like the FMI, the ONU, and the WTO. The part of the Bretton Woods agreement addressing the problem of interchangeability between different national currencies did not withstand the test of international cooperation, but technological innovations applied to finance have revived the urgency of its relaunch in a contemporary context," he stated. The president of CONSOB also relaunched the proposal to unify the single text on finance and the single banking text, suggesting closer collaboration among Italian authorities. "To this end, it is necessary to activate in Italy formal consultation structures between governing bodies and independent authorities that impose a unitary direction to choices in the matter, also with a view to the position to be assumed regarding ongoing European and international initiatives—he explained. A first step would be adopting the recommendation from the European Committee for Systemic Risk of 2011, which would establish a single national counterparty responsible for macro-prudential stability. The Banca d’Italia would maintain a central role, justified by its participation in the Eurosystem around which European finance currently revolves, but strict coordination would be guaranteed among the three independent supervisory authorities (CONSOB, IVASS, and COVIP), with the participation of the Ministry of Economy." "To cope with economic and social difficulties, public debt has grown greatly, albeit in forms different from what an emergency state would have required. However, confidence in the reaction capabilities of the Italian economy has grown. This result is also the fruit of the decisions made by the BCE to purchase significant volumes of public bonds and by the European Commission to suspend, even if temporarily, the Stability Pact and to launch the Next Generation EU plan. We agree with the assessment that these decisions will structurally improve our real growth rate." Now, however, it is necessary to change pace. "However, for the continuation of the productive relaunch phase, it is necessary to integrate the decisions taken so far to incentivize corporate venture capital, thereby improving their financial leverage and making them more available to undertake new initiatives," said Savona, who believes that "the fiscal reform long requested offers an important opportunity," especially "by assigning it the task of considering productive demands on the same level as ethical ones in the assessments of distributive equity."</t>
+          <t xml:space="preserve">Observation date: 2021-06-14 00:00:00. If there had been the ability to generate income from those savings, even with a remuneration of one percentage point, households would have collectively earned 30 billion, almost 2% of the gross domestic product. 'The savings rate of Italian households relative to disposable income has grown by 50% in the year, but, excluding savings invested in listed companies, its return has remained quite low, close to zero. Given the consistency of financial assets held by households, every percentage point of remuneration can be estimated at around 30 billion euros, almost 2% of GDP, the size of a good public budget maneuver in the past.' The core theme of the annual report by the President of Consob, Paolo Savona, is the primary asset that the authority he leads intends to protect: savings. But this has been focused on deposits for the last two years. And now it is threatened by a shadow lengthening over international markets, which is very difficult to control: these are the sirens of cryptocurrencies and Bitcoin. A phenomenon that is growing rapidly and becoming increasingly difficult to contain, much so that it has prompted Savona to sound the alarm: the speculative effect they are triggering seems very similar to what happened before 2008 with subprime mortgages. 'The spread of virtual instruments has stimulated the birth of the already remembered technological platforms,' he said. 'These new market segments are rapidly evolving, and the experience preceding the 2008 crisis seems to be repeating itself, when derivative contracts developed to reach a size ten times the global GDP, assuming complex forms that received high ratings. With due distinctions, it is predictable that something analogous is happening in the market for virtual monetary and financial products, especially crypto.' Savona recalled how 'a single Bitcoin recently had the ability to purchase a large electric car and shortly after lost half its purchasing power.' For the President of Consob, 'financial technology is a prodigious lamp from which genius has emerged. The authorities will not be able to put it back, because it operates in the immaterial sphere controllable only by changing the information exchange protocol, thus fragmenting the unit of the global market and reducing the international competitiveness rate.' Traditional supervisory tools are no longer sufficient. Under current conditions, according to Savona, 'the authorities can intervene by also utilizing the advantages of digitized techniques; their action will be more effective if they cooperate with each other.' For Italy, the issue is even more delicate due to the constitutional rule that assigns the 'Republic the task of encouraging and protecting savings in all their forms and of regulating, coordinating, and controlling the exercise of credit.' It would be inappropriate, he explained, 'if the specification of </t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>['If families had generated income from savings, even with a 1% remuneration, families would have gained 30 billion euros.', 'This gain of 30 billion euros represents nearly 2% of the Gross Domestic Product (GDP).', 'The savings rate of Italian families relative to disposable income grew by 50% in the year.', 'Excluding savings invested in listed companies, the yield of family savings remained low, close to zero.', 'For every percentage point of remuneration, the yield on family financial assets can be estimated at around 30 billion euros.', 'This estimated amount of 30 billion euros represents nearly 2% of GDP.', 'The core theme of the annual report by CONSOB President Paolo Savona is the protection of savings.', 'International markets are threatening savings with cryptocurrencies and Bitcoin.', 'Paolo Savona issued a warning regarding the speculative effect triggered by cryptocurrencies and Bitcoin.', 'Paolo Savona stated that the speculative effect triggered by cryptocurrencies and Bitcoin seems similar to what happened before 2008 with subprime mortgages.', 'Paolo Savona noted that the diffusion of virtual instruments stimulated the birth of already remembered technological platforms.', 'New market segments are rapidly evolving.', 'The experience preceding the 2008 crisis seems to be repeating itself in the market for virtual monetary and financial products, especially cryptocurrencies.', 'Derivatives contracts developed to reach a size ten times the global GDP during the 2008 crisis.', 'Something analogous is happening in the market for virtual monetary and financial products, especially cryptocurrencies.', 'A single Bitcoin recently had the ability to purchase a large-cylinder electric car.', 'A single Bitcoin shortly after lost half of its purchasing power.', 'Paolo Savona stated that financial informatics is a prodigious lamp from which genius has emerged.', 'The authorities will not be able to put financial informatics back.', 'Financial informatics operates in the immaterial sphere.', 'The immaterial sphere is controllable only by changing the information exchange protocol.', 'Changing the information exchange protocol fragments the unit of the global market.', 'Fragmenting the unit of the global market reduces the international competitiveness rate.', 'Traditional supervisory tools are no longer sufficient.', 'Paolo Savona suggested that the authorities can intervene by utilizing the advantages of digitized techniques.', "The authorities' action will be more effective if the authorities cooperate with each other.", 'The constitutional norm confers upon the Republic the task of encouraging and protecting savings in all their forms and of regulating, coordinating, and controlling the exercise of credit.', "Paolo Savona explained that it would be inappropriate if the specification of 'savings in all their forms' and the credit to be protected were given content that also encompassed virtual instruments without passing through specific regulation.", 'These cryptocurrencies are based on blockchain.', 'The original blockchain is impenetrable, according to the state of hacking techniques known.', 'The blockchain used by other cryptocurrencies is not impenetrable.', 'Paolo Savona called for proceeding quickly with regulatory systems.', 'Without adequate safeguards (rules and bodies), there results a deterioration of market transparency.', 'Market transparency is the foundation of legality and the rational choices of operators.', 'A well-known negative effect is that these techniques allow shielding for criminal activities.', 'Criminal activities include tax evasion, money laundering, the financing of terrorism, and the kidnapping of persons.', 'Paolo Savona hopes for an international solution regarding cybersecurity.', 'The issue of cybersecurity encompasses political problems of even broader content.', 'The solution to cybersecurity cannot be achieved at the national level.', 'The solution to cybersecurity requires close international cooperation.', "The relaunch of the Bretton Woods agreement's part addressing interchangeability between different national currencies is urgent in a contemporary context.", 'Paolo Savona relaunched the proposal to unify the single text on finance and the single banking text.', 'Paolo Savona suggested closer collaboration among Italian authorities.', 'It is necessary to activate formal consultation structures in Italy between governing bodies and independent authorities.', 'These structures must impose a unitary direction to choices in the matter.', 'A first step would be adopting the recommendation from the European Committee for Systemic Risk of 2011.', 'This recommendation would establish a single national counterparty responsible for macro-prudential stability.', 'The Banca d’Italia would maintain a central role due to its participation in the Eurosystem.', 'Strict coordination would be guaranteed among the three independent supervisory authorities (CONSOB, IVASS, and COVIP).', 'Public debt has grown greatly to cope with economic and social difficulties.', 'Confidence in the reaction capabilities of the Italian economy has grown.', 'The growth in confidence is a result of the decisions made by the BCE to purchase significant volumes of public bonds.', 'The growth in confidence is a result of the European Commission launching the Next Generation EU plan.', 'The decisions made by the BCE and the European Commission will structurally improve the real growth rate.', 'For the continuation of the productive relaunch phase, it is necessary to integrate decisions to incentivize corporate venture capital.', 'Incentivizing corporate venture capital will improve their financial leverage.', 'Improving financial leverage will make corporate venture capital more available to undertake new initiatives.', 'Paolo Savona believes that the fiscal reform offers an important opportunity.', 'The fiscal reform should consider productive demands on the same level as ethical ones in the assessments of distributive equity.']</t>
+          <t>['If households could generate income from savings with a 1% remuneration, households would have collectively earned 30 billion euros.', 'This amount (30 billion euros) represents almost 2% of the gross domestic product.', 'The savings rate of Italian households relative to disposable income grew by 50% in the year.', 'Excluding savings invested in listed companies, the return on savings remained low, close to zero.', 'Every percentage point of remuneration on financial assets held by households is estimated at around 30 billion euros.', 'The core theme of the annual report by the President of Consob, Paolo Savona, is protecting savings.', 'The authority led by Paolo Savona intends to protect savings.', 'The focus of the protection efforts has been on deposits for the last two years.', 'International markets are now threatened by a shadow that is difficult to control.', 'This threat involves cryptocurrencies and Bitcoin.', 'The phenomenon of cryptocurrencies and Bitcoin is growing rapidly and becoming increasingly difficult to contain.', 'The speculative effect triggered by cryptocurrencies and Bitcoin prompted Paolo Savona to sound the alarm.', 'The speculative effect is similar to what happened before 2008 with subprime mortgages.', 'The spread of virtual instruments stimulated the birth of technological platforms.', 'New market segments are rapidly evolving.', 'The experience preceding the 2008 crisis seems to be repeating itself.', 'During the experience preceding the 2008 crisis, derivative contracts reached a size ten times the global GDP.', 'Something analogous to the pre-2008 crisis is predictable in the market for virtual monetary and financial products, especially crypto.', 'Paolo Savona recalled that a single Bitcoin recently had the ability to purchase a large electric car.', 'Shortly after, the single Bitcoin lost half its purchasing power.', 'For the President of Consob, financial technology is a prodigious lamp from which genius has emerged.', 'The authorities will not be able to reverse financial technology.', 'Financial technology operates in the immaterial sphere.', 'Changing the information exchange protocol controls the immaterial sphere of financial technology.', 'This process fragments the unit of the global market and reduces the international competitiveness rate.', 'Traditional supervisory tools are no longer sufficient.', 'According to Paolo Savona, the authorities can intervene by utilizing the advantages of digitized techniques.', 'The action of the authorities will be more effective if the authorities cooperate with each other.', 'For Italy, the issue is delicate due to a constitutional rule.', 'The constitutional rule assigns the Republic the task of encouraging and protecting savings in all their forms.', 'The constitutional rule also assigns the Republic the task of regulating, coordinating, and controlling the exercise of credit.']</t>
         </is>
       </c>
     </row>
@@ -1112,29 +1050,17 @@
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr">
         <is>
-          <t>The financial crisis is beginning to affect businesses and families. For now, the credit provided by banks has not decreased, says the Governor of the Banca d'Italia, Mario Draghi, "however, the situation can change quickly." Consumption is falling. Following the drop in production in the second quarter, "negative signals are arriving for the coming quarters." To curb the negative effects, Silvio Berlusconi accepted the proposal from Confindustria to open a discussion forum among the government, businesses, and banks. He will convene it immediately upon his return from his trip to China: "We ask that the banks do not fail in their support for investments and consumption." The promise is to find "substantial funds" in the budget. Minister Claudio Scajola added: state guarantee schemes are being studied for corporate debts, similar to those implemented for banks.
-In his hearing before the Senate, Draghi first sought to reassure about Italian banks: "Thanks to rigorous laws and firm supervisory action, we do not have that extensive 'shadow banking system' where the crisis found its origin and sustenance elsewhere." Today, "the capitalization of the major Italian banks remains sufficient"; even if losses from the Lehman Brothers failure reached the worst-case scenario, "such a shock could be absorbed."
-However, banks suffered on the stock exchange due to a phrase from the Prime Minister that was partially misinterpreted. Again, and always in Napoli, like the first time with Eni and Enel, Berlusconi let slip comments about listed companies. According to the official clarification, he said: "Perhaps two or three banks, in addition to Unicredit, will benefit from increasing their capital, finding the means naturally in the market." At the initial reports from the news agencies, the quotes of the major banks fell, before recovering somewhat later.
-Market clarity was confirmed yesterday with the Euribor three-month rate falling below 5%, a reference point for variable-rate home mortgages. The Italian banks, the Governor assures, "have shared only a minimal portion of the errors and distortions" of the global financial system, originating mainly in the United States. Regarding European standards, "the Banca d'Italia has consistently given a severe interpretation."
-Draghi is well aware that public opinion tends to involve central banks in blame. He makes it clear that this may be justified in the USA, where there was a "regulatory capture" (in simple terms, Wall Street influenced the government and the Federal Reserve) and in other countries; it is not the case in the Euro area and especially not in Italy. "The alarms, over time, were not lacking," he recalls: "not least the person speaking about it repeatedly drew attention to the imbalances in the international financial system," in various interventions, especially in the autumn of 2006; the problem is that "in calm times, warnings often remain unheard." "Neither the timing, nor the precise mechanism, nor the magnitude of the crisis could be foreseen," he summarizes; "but the accumulating tensions could clearly be seen."
-The banks or other intermediaries that held Lehman Brothers titles for savers "will not leave them alone." New rules on transparency in relationships between banks and clients will be ready at the beginning of next year. Globally, to clean up, it will be necessary to better regulate derivatives and other innovative financial products. New rules must prevent banks from assuming risks too disproportionate to their capital.
-"All things considered, Italy is not doing badly" from the financial crisis, concludes the Governor; but the effects of the crisis on the real economy "add to pre-existing structural weaknesses." The same judgment comes from the International Monetary Fund, which confirms the forecast of a drop in gross product both in 2008 (-0.1%) and in 2009 (-0.2%). But responding with state aid would not be the right answer, warns the head of the IMF's European Department, Alessandro Leipold: "Liberalization is better."</t>
+          <t>Governor Stefano Lepri stated that the financial crisis is beginning to spread to businesses and families; for now, credit provided by banks has not decreased, said the Governor of the Bank of Italy, Mario Draghi, though, "the situation, however, can change quickly." Consumption is falling. Following the drop in product in the second quarter, "negative signals are arriving for the coming quarters." To curb the negative effects, Silvio Berlusconi accepted the Confindustria proposal to open a discussion forum among the government, businesses, and banks. He will convene it immediately upon his return from his trip to China: "We ask that the banks do not fail to provide their support for investments and consumption." The promise is to find "funds of significant magnitude" in the budget. Minister Claudio Scajola added: "State guarantee forms are being studied for corporate debts, as was done for banks." In his hearing before the Senate, Draghi first sought to reassure about Italian banks: "Thanks to rigorous laws and firm supervisory action, we do not have that extensive 'shadow banking system' where the crisis found its origin and sustenance elsewhere." Today, "the capitalization of the major Italian banks remains sufficient"; even if losses from the Lehman failure reached the worst-case scenario, "such a shock could be absorbed." However, banks suffered on the stock exchange due to a phrase from the Prime Minister that was partially misunderstood. Again, and always in Naples, like the first time with Eni and Enel, Berlusconi let slip comments about listed companies on the stock exchange. According to the official clarification, he said: "Perhaps two or three banks, in addition to UniCredit, will have advantages in increasing their capital, naturally finding the means in the market." At the initial reports from the news agencies, the quotes of the major banks fell, before recovering somewhat later. The clarity in the financial markets was confirmed yesterday with the Euribor rate falling below 5% for three months, a reference point for variable-rate home mortgages. The Governor assures that Italian banks "have shared only a minimal portion of the errors and distortions" of the global financial system, originating mainly in the United States. Regarding European standards, "the Bank of Italy has consistently given a severe interpretation." Draghi is well aware that public opinion tends to involve central banks in blame. He makes it clear that this may be justified in the US, where there was a "regulatory capture" (in simple terms, Wall Street influenced the government and the Federal Reserve) and in other countries; it is not the case in the Euro area, and especially not in Italy. "Alarms were not lacking over time," he recalls: "not least the person speaking had repeatedly drawn attention to the imbalances of the international financial system," in various interventions, especially in the autumn of 2006; the problem is that "in calm times, warnings often remain unheard." "Neither the timing, nor the precise mechanism, nor the magnitude of the crisis could be foreseen; but the accumulating tensions could clearly be seen." The banks or other intermediaries that sold Lehman Brothers securities to savers "will not leave them alone." New rules on transparency in relationships between banks and clients will be ready at the beginning of next year. Globally, cleaning up will require better regulation of derivatives and other innovative financial products. New rules must prevent banks from assuming risks too disproportionate to their capital. "All in all, Italy is not doing badly" from the financial crisis, concludes the Governor; but the effects of the crisis on the real economy "add to pre-existing structural weaknesses." The same judgment comes from the International Monetary Fund, which confirms the forecast of a drop in gross product both in 2008 (-0.1%) and in 2009 (-0.2%). But reacting with state aid would not be the right answer, warns the head of the IMF's European Department, Alessandro Leipold: "Liberalization is better."</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>Observation date: 2008-10-22 00:00:00. The financial crisis is beginning to affect businesses and families. For now, the credit provided by banks has not decreased, says the Governor of the Banca d'Italia, Mario Draghi, "however, the situation can change quickly." Consumption is falling. Following the drop in production in the second quarter, "negative signals are arriving for the coming quarters." To curb the negative effects, Silvio Berlusconi accepted the proposal from Confindustria to open a discussion forum among the government, businesses, and banks. He will convene it immediately upon his return from his trip to China: "We ask that the banks do not fail in their support for investments and consumption." The promise is to find "substantial funds" in the budget. Minister Claudio Scajola added: state guarantee schemes are being studied for corporate debts, similar to those implemented for banks.
-In his hearing before the Senate, Draghi first sought to reassure about Italian banks: "Thanks to rigorous laws and firm supervisory action, we do not have that extensive 'shadow banking system' where the crisis found its origin and sustenance elsewhere." Today, "the capitalization of the major Italian banks remains sufficient"; even if losses from the Lehman Brothers failure reached the worst-case scenario, "such a shock could be absorbed."
-However, banks suffered on the stock exchange due to a phrase from the Prime Minister that was partially misinterpreted. Again, and always in Napoli, like the first time with Eni and Enel, Berlusconi let slip comments about listed companies. According to the official clarification, he said: "Perhaps two or three banks, in addition to Unicredit, will benefit from increasing their capital, finding the means naturally in the market." At the initial reports from the news agencies, the quotes of the major banks fell, before recovering somewhat later.
-Market clarity was confirmed yesterday with the Euribor three-month rate falling below 5%, a reference point for variable-rate home mortgages. The Italian banks, the Governor assures, "have shared only a minimal portion of the errors and distortions" of the global financial system, originating mainly in the United States. Regarding European standards, "the Banca d'Italia has consistently given a severe interpretation."
-Draghi is well aware that public opinion tends to involve central banks in blame. He makes it clear that this may be justified in the USA, where there was a "regulatory capture" (in simple terms, Wall Street influenced the government and the Federal Reserve) and in other countries; it is not the case in the Euro area and especially not in Italy. "The alarms, over time, were not lacking," he recalls: "not least the person speaking about it repeatedly drew attention to the imbalances in the international financial system," in various interventions, especially in the autumn of 2006; the problem is that "in calm times, warnings often remain unheard." "Neither the timing, nor the precise mechanism, nor the magnitude of the crisis could be foreseen," he summarizes; "but the accumulating tensions could clearly be seen."
-The banks or other intermediaries that held Lehman Brothers titles for savers "will not leave them alone." New rules on transparency in relationships between banks and clients will be ready at the beginning of next year. Globally, to clean up, it will be necessary to better regulate derivatives and other innovative financial products. New rules must prevent banks from assuming risks too disproportionate to their capital.
-"All things considered, Italy is not doing badly" from the financial crisis, concludes the Governor; but the effects of the crisis on the real economy "add to pre-existing structural weaknesses." The same judgment comes from the International Monetary Fund, which confirms the forecast of a drop in gross product both in 2008 (-0.1%) and in 2009 (-0.2%). But responding with state aid would not be the right answer, warns the head of the IMF's European Department, Alessandro Leipold: "Liberalization is better."</t>
+          <t>Observation date: 2008-10-22 00:00:00. Governor Stefano Lepri stated that the financial crisis is beginning to spread to businesses and families; for now, credit provided by banks has not decreased, said the Governor of the Bank of Italy, Mario Draghi, though, "the situation, however, can change quickly." Consumption is falling. Following the drop in product in the second quarter, "negative signals are arriving for the coming quarters." To curb the negative effects, Silvio Berlusconi accepted the Confindustria proposal to open a discussion forum among the government, businesses, and banks. He will convene it immediately upon his return from his trip to China: "We ask that the banks do not fail to provide their support for investments and consumption." The promise is to find "funds of significant magnitude" in the budget. Minister Claudio Scajola added: "State guarantee forms are being studied for corporate debts, as was done for banks." In his hearing before the Senate, Draghi first sought to reassure about Italian banks: "Thanks to rigorous laws and firm supervisory action, we do not have that extensive 'shadow banking system' where the crisis found its origin and sustenance elsewhere." Today, "the capitalization of the major Italian banks remains sufficient"; even if losses from the Lehman failure reached the worst-case scenario, "such a shock could be absorbed." However, banks suffered on the stock exchange due to a phrase from the Prime Minister that was partially misunderstood. Again, and always in Naples, like the first time with Eni and Enel, Berlusconi let slip comments about listed companies on the stock exchange. According to the official clarification, he said: "Perhaps two or three banks, in addition to UniCredit, will have advantages in increasing their capital, naturally finding the means in the market." At the initial reports from the news agencies, the quotes of the major banks fell, before recovering somewhat later. The clarity in the financial markets was confirmed yesterday with the Euribor rate falling below 5% for three months, a reference point for variable-rate home mortgages. The Governor assures that Italian banks "have shared only a minimal portion of the errors and distortions" of the global financial system, originating mainly in the United States. Regarding European standards, "the Bank of Italy has consistently given a severe interpretation." Draghi is well aware that public opinion tends to involve central banks in blame. He makes it clear that this may be justified in the US, where there was a "regulatory capture" (in simple terms, Wall Street influenced the government and the Federal Reserve) and in other countries; it is not the case in the Euro area, and especially not in Italy. "Alarms were not lacking over time," he recalls: "not least the person speaking had repeatedly drawn attention to the imbalances of the international financial system," in various interventions, especially in the autumn of 2006; the problem is that "in calm times, warnings often remain unheard." "Neither the timing, nor the precise mechanism, nor the magnitude of the crisis could be foreseen; but the accumulating tensions could clearly be seen." The banks or other intermediaries that sold Lehman Brothers securities to savers "will not leave them alone." New rules on transparency in relationships between banks and clients will be ready at the beginning of next year. Globally, cleaning up will require better regulation of derivatives and other innovative financial products. New rules must prevent banks from assuming risks too disproportionate to their capital. "All in all, Italy is not doing badly" from the financial crisis, concludes the Governor; but the effects of the crisis on the real economy "add to pre-existing structural weaknesses." The same judgment comes from the International Monetary Fund, which confirms the forecast of a drop in gross product both in 2008 (-0.1%) and in 2009 (-0.2%). But reacting with state aid would not be the right answer, warns the head of the IMF's European Department, Alessandro Leipold: "Liberalization is better."</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>['The financial crisis was beginning to affect businesses and families on 2008-10-22.', "Mario Draghi, Governor of the Banca d'Italia, stated that the credit provided by banks had not decreased for now.", "Mario Draghi, Governor of the Banca d'Italia, warned that the situation could change quickly.", 'Consumption was falling.', 'Negative signals were arriving for the coming quarters following the drop in production in the second quarter.', 'Silvio Berlusconi accepted the proposal from Confindustria to open a discussion forum among the government, businesses, and banks.', 'Silvio Berlusconi will convene the forum immediately upon returning from the trip to China.', 'Silvio Berlusconi asked that the banks do not fail in their support for investments and consumption.', 'Minister Claudio Scajola stated that state guarantee schemes are being studied for corporate debts.', 'State guarantee schemes for corporate debts are similar to those implemented for banks.', "Mario Draghi, during the hearing before the Senate, stated that Italy does not have an extensive 'shadow banking system' where the crisis found its origin and sustenance.", 'Mario Draghi stated that the capitalization of the major Italian banks remains sufficient on 2008-10-22.', 'Mario Draghi stated that the major Italian banks could absorb a shock even if losses from the Lehman Brothers failure reached the worst-case scenario.', 'Banks suffered on the stock exchange due to a phrase from the Prime Minister that was partially misinterpreted.', 'Silvio Berlusconi made comments about listed companies in Napoli.', 'Silvio Berlusconi officially clarified that two or three banks, in addition to Unicredit, might benefit from increasing their capital.', 'Silvio Berlusconi stated that the means for increasing the capital of the banks would be found naturally in the market.', 'The quotes of the major banks fell according to initial reports from the news agencies.', 'The quotes of the major banks recovered somewhat later.', 'Market clarity was confirmed on 2008-10-21 with the Euribor three-month rate falling below 5%.', 'Mario Draghi assured that the Italian banks shared only a minimal portion of the errors and distortions of the global financial system.', "The global financial system's errors and distortions originated mainly in the United States.", "The Banca d'Italia consistently gave a severe interpretation regarding European standards.", 'Mario Draghi stated that public opinion tends to involve central banks in blame.', 'Mario Draghi explained that the blame might be justified in the USA because Wall Street influenced the government and the Federal Reserve.', 'Mario Draghi stated that the blame is not the case in the Euro area or in Italy.', 'Mario Draghi recalled that alarms about the international financial system were not lacking.', 'A person repeatedly drew attention to the imbalances in the international financial system in various interventions, especially in the autumn of 2006.', 'Mario Draghi noted that warnings often remain unheard during calm times.', 'Mario Draghi summarized that the timing, precise mechanism, or magnitude of the crisis could not be foreseen.', 'Mario Draghi summarized that the accumulating tensions of the crisis could clearly be seen.', 'The banks or other intermediaries that held Lehman Brothers titles for savers will not leave savers alone.', 'New rules on transparency in relationships between banks and clients will be ready at the beginning of 2009.', 'Globally, better regulation of derivatives and other innovative financial products will be necessary to clean up.', 'New rules must prevent banks from assuming risks disproportionate to their capital.', 'Mario Draghi concluded that Italy is not doing badly from the financial crisis.', 'The effects of the crisis on the real economy add to pre-existing structural weaknesses.', 'The International Monetary Fund confirmed a forecast of a drop in gross product of -0.1% in 2008.', "Alessandro Leipold, head of the IMF's European Department, warned that responding with state aid would not be the right answer.", 'Alessandro Leipold recommended that liberalization is better.']</t>
+          <t>['Stefano Lepri stated that the financial crisis is beginning to spread to businesses and families.', 'Mario Draghi, Governor of the Bank of Italy, stated that credit provided by banks has not decreased for now.', 'Mario Draghi stated that the situation can change quickly.', 'Consumption is falling.', 'Negative signals are arriving for the coming quarters following the drop in product in the second quarter.', 'Silvio Berlusconi accepted the Confindustria proposal.', 'The Confindustria proposal was to open a discussion forum among the government, businesses, and banks.', 'Silvio Berlusconi will convene the forum immediately upon his return from his trip to China.', 'Silvio Berlusconi asked that the banks do not fail to provide their support for investments and consumption.', 'The promise is to find funds of significant magnitude in the budget.', 'Minister Claudio Scajola added that state guarantee forms are being studied for corporate debts.', 'State guarantee forms were previously done for banks.', 'Mario Draghi sought to reassure about Italian banks during a hearing before the Senate.', "Mario Draghi stated that Italy does not have the extensive 'shadow banking system' where the crisis found its origin and sustenance elsewhere.", 'The capitalization of the major Italian banks remains sufficient on 2008-10-22.', 'A shock from Lehman failure losses could be absorbed even if losses reached the worst-case scenario.', 'Banks suffered on the stock exchange due to a phrase from the Prime Minister that was partially misunderstood.', 'Silvio Berlusconi let slip comments about listed companies on the stock exchange.', 'Silvio Berlusconi clarified that perhaps two or three banks, in addition to UniCredit, will have advantages in increasing their capital.', 'The quotes of the major banks fell at the initial reports from the news agencies.', 'The quotes of the major banks recovered somewhat later.', 'The clarity in the financial markets was confirmed on 2008-10-21.', 'The Euribor rate fell below 5% for three months on 2008-10-21.', 'Mario Draghi assures that Italian banks have shared only a minimal portion of the errors and distortions of the global financial system.', 'The global financial system errors and distortions originated mainly in the United States.', 'The Bank of Italy has consistently given a severe interpretation regarding European standards.', 'Mario Draghi is aware that public opinion tends to involve central banks in blame.', 'Mario Draghi stated that the situation (blame) may be justified in the US and other countries.', 'Mario Draghi stated that the situation (blame) is not the case in the Euro area or Italy.', 'Mario Draghi recalled that the person speaking had repeatedly drawn attention to the imbalances of the international financial system.', 'The person speaking drew attention to the imbalances of the international financial system in various interventions, especially in the autumn of 2006.', 'The banks or other intermediaries that sold Lehman Brothers securities to savers will not leave the savers alone.', 'New rules on transparency in relationships between banks and clients will be ready on 2009-10-22.', 'Cleaning up globally will require better regulation of derivatives and other innovative financial products.', 'New rules must prevent banks from assuming risks too disproportionate to their capital.', 'Mario Draghi concluded that Italy is not doing badly from the financial crisis.', 'The effects of the crisis on the real economy add to pre-existing structural weaknesses.', 'The International Monetary Fund confirmed the forecast of a drop in gross product in 2008 (-0.1%).', 'Alessandro Leipold warned that reacting with state aid would not be the right answer.', 'Alessandro Leipold recommended that liberalization is better.']</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1110,17 @@
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr">
         <is>
-          <t>The combination of falling mortgage applications, rising lending requirements, and an intensifying credit crunch is evident. Goldman Sachs explains in a report that this crunch is the most intense since the sovereign debt crisis. The interest rate increases by the European Central Bank (BCE) are beginning to impact households and businesses significantly. According to the latest bank lending survey from Frankfurt, in the fourth quarter of 2022, the contraction in residential mortgage demand, down 21%, was "the strongest ever recorded," and "the demand for consumer credit and other household loans decreased sharply in net terms, although to a lesser extent than mortgages for construction." This scenario, according to Goldman Sachs, represents "a substantial further tightening of credit standards" required of households and businesses, which are primarily weighed down by uncertain economic prospects but increasingly affected by the cost of funds and liquidity position. As the BCE explains, "the net fall in real estate mortgage demand was determined mainly by the general level of interest rates, lower consumer confidence, and the deterioration of real estate market prospects." In the first quarter of 2023, banking institutions anticipate a further net decline in lending to businesses. Regarding household loans, the Frankfurt survey notes that "banks estimate a persistent and sharp net decline in demand for the first quarter of 2023." This picture is also confirmed by Goldman Sachs, which anticipates a slowdown in credit provision and a reduction in demand for both personal loans and mortgages, "of equal magnitude" to what was observed in the last four months of the year. Unlike the crisis that hit the Euro area a decade ago, in this case, the phenomenon is spread homogeneously across the Euro area.</t>
+          <t>Mortgage applications are falling, lending requirements are rising, and the credit crunch is intensifying. Goldman Sachs explains in a report that this crunch is the most severe since the sovereign debt crisis. The interest rate hikes by the European Central Bank (ECB) are beginning to impact households and businesses consistently. According to the latest Frankfurt Bank Lending Survey, in the fourth quarter of 2022, the contraction in residential mortgage demand, down 21%, was 'the strongest ever recorded,' and 'consumer credit and other household loans decreased sharply in net terms, although to a lesser extent than housing mortgages.' This scenario, according to Goldman Sachs, represents 'a substantial further tightening of credit standards' required of households and businesses, primarily weighed down by uncertain economic prospects, but increasingly influenced by the cost of funds and liquidity position. [The text also mentions the ECB's hawkish stance for all of 2023, noting that the situation is destined to worsen in step with rising money costs.] As the ECB explains, 'the net fall in real estate mortgage demand was determined mainly by the general level of interest rates, lower consumer confidence, and the deterioration of real estate market prospects.' In the first quarter of 2023, banking institutions anticipate a further net decline in corporate lending demand. Regarding household loans, Frankfurt notes that 'banks estimate a persistent and sharp net decline in demand for the first quarter of 2023.' This picture is also confirmed by Goldman Sachs, which expects a slowdown in credit provision and a reduction in demand for both personal loans and mortgages, 'of equal magnitude' to what was observed in the last four months of the year. Unlike the crisis that hit the Eurozone a decade ago, this phenomenon is spread homogeneously across the Euro area.</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>Observation date: 2023-02-02 00:00:00. The combination of falling mortgage applications, rising lending requirements, and an intensifying credit crunch is evident. Goldman Sachs explains in a report that this crunch is the most intense since the sovereign debt crisis. The interest rate increases by the European Central Bank (BCE) are beginning to impact households and businesses significantly. According to the latest bank lending survey from Frankfurt, in the fourth quarter of 2022, the contraction in residential mortgage demand, down 21%, was "the strongest ever recorded," and "the demand for consumer credit and other household loans decreased sharply in net terms, although to a lesser extent than mortgages for construction." This scenario, according to Goldman Sachs, represents "a substantial further tightening of credit standards" required of households and businesses, which are primarily weighed down by uncertain economic prospects but increasingly affected by the cost of funds and liquidity position. As the BCE explains, "the net fall in real estate mortgage demand was determined mainly by the general level of interest rates, lower consumer confidence, and the deterioration of real estate market prospects." In the first quarter of 2023, banking institutions anticipate a further net decline in lending to businesses. Regarding household loans, the Frankfurt survey notes that "banks estimate a persistent and sharp net decline in demand for the first quarter of 2023." This picture is also confirmed by Goldman Sachs, which anticipates a slowdown in credit provision and a reduction in demand for both personal loans and mortgages, "of equal magnitude" to what was observed in the last four months of the year. Unlike the crisis that hit the Euro area a decade ago, in this case, the phenomenon is spread homogeneously across the Euro area.</t>
+          <t>Observation date: 2023-02-02 00:00:00. Mortgage applications are falling, lending requirements are rising, and the credit crunch is intensifying. Goldman Sachs explains in a report that this crunch is the most severe since the sovereign debt crisis. The interest rate hikes by the European Central Bank (ECB) are beginning to impact households and businesses consistently. According to the latest Frankfurt Bank Lending Survey, in the fourth quarter of 2022, the contraction in residential mortgage demand, down 21%, was 'the strongest ever recorded,' and 'consumer credit and other household loans decreased sharply in net terms, although to a lesser extent than housing mortgages.' This scenario, according to Goldman Sachs, represents 'a substantial further tightening of credit standards' required of households and businesses, primarily weighed down by uncertain economic prospects, but increasingly influenced by the cost of funds and liquidity position. [The text also mentions the ECB's hawkish stance for all of 2023, noting that the situation is destined to worsen in step with rising money costs.] As the ECB explains, 'the net fall in real estate mortgage demand was determined mainly by the general level of interest rates, lower consumer confidence, and the deterioration of real estate market prospects.' In the first quarter of 2023, banking institutions anticipate a further net decline in corporate lending demand. Regarding household loans, Frankfurt notes that 'banks estimate a persistent and sharp net decline in demand for the first quarter of 2023.' This picture is also confirmed by Goldman Sachs, which expects a slowdown in credit provision and a reduction in demand for both personal loans and mortgages, 'of equal magnitude' to what was observed in the last four months of the year. Unlike the crisis that hit the Eurozone a decade ago, this phenomenon is spread homogeneously across the Euro area.</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>['Falling mortgage applications are evident.', 'Rising lending requirements are evident.', 'An intensifying credit crunch is evident.', 'Goldman Sachs explained in a report that the credit crunch is the most intense since the sovereign debt crisis.', 'Interest rate increases by the European Central Bank (BCE) are beginning to impact households significantly.', 'The latest bank lending survey from Frankfurt reported data for the fourth quarter of 2022.', 'In the fourth quarter of 2022, the contraction in residential mortgage demand was down 21%.', 'The contraction in residential mortgage demand in the fourth quarter of 2022 was the strongest ever recorded.', 'The latest bank lending survey from Frankfurt noted that demand for consumer credit and other household loans decreased sharply in net terms.', 'The decrease in consumer credit and other household loans was to a lesser extent than the decrease in mortgages for construction.', 'Goldman Sachs stated that the scenario represents a substantial further tightening of credit standards.', 'Households are primarily weighed down by uncertain economic prospects.', 'Households are increasingly affected by the cost of funds and liquidity position.', 'The BCE explained that the net fall in real estate mortgage demand was determined mainly by the deterioration of real estate market prospects.', 'Banking institutions anticipate a further net decline in lending to businesses in the first quarter of 2023.', 'The Frankfurt survey noted that banks estimate a persistent and sharp net decline in demand for household loans in the first quarter of 2023.', 'Goldman Sachs confirmed the picture of declining credit provision.', 'Goldman Sachs anticipates a reduction in demand for personal loans.', 'The reduction in demand for personal loans and mortgages is anticipated to be of equal magnitude to what was observed in the last four months of the year.', 'The current phenomenon is spread homogeneously across the Euro area.', 'The current phenomenon differs from the crisis that hit the Euro area a decade ago.']</t>
+          <t>['Mortgage applications are falling.', 'Lending requirements are rising.', 'The credit crunch is intensifying.', 'Goldman Sachs explained in a report that the credit crunch is the most severe since the sovereign debt crisis.', 'The European Central Bank (ECB) interest rate hikes are beginning to impact households.', 'The Frankfurt Bank Lending Survey reported data for the fourth quarter of 2022.', 'In the fourth quarter of 2022, the contraction in residential mortgage demand was 21%.', 'The Frankfurt Bank Lending Survey stated that the contraction in residential mortgage demand in the fourth quarter of 2022 was the strongest ever recorded.', 'In the fourth quarter of 2022, consumer credit and other household loans decreased sharply in net terms.', 'The decrease in consumer credit and other household loans in the fourth quarter of 2022 was less than the decrease in housing mortgages.', 'Goldman Sachs stated that the scenario represents a substantial further tightening of credit standards.', 'The tightening of credit standards is required of households.', 'The tightening of credit standards is primarily weighed down by uncertain economic prospects.', 'The tightening of credit standards is increasingly influenced by the cost of funds and liquidity position.', 'The ECB maintained a hawkish stance for all of 2023.', 'The situation is destined to worsen with rising money costs.', 'The ECB explained that the net fall in real estate mortgage demand was determined mainly by the general level of interest rates.', 'The net fall in real estate mortgage demand was determined mainly by lower consumer confidence.', 'The net fall in real estate mortgage demand was determined mainly by the deterioration of real estate market prospects.', 'Banking institutions anticipate a further net decline in corporate lending demand in the first quarter of 2023.', 'Frankfurt noted that banks estimate a persistent and sharp net decline in household loan demand for the first quarter of 2023.', 'Goldman Sachs confirmed the picture of declining credit demand.', 'Goldman Sachs expects a slowdown in credit provision.', 'Goldman Sachs expects a reduction in demand for personal loans.', 'The expected reduction in personal loans and mortgages is of equal magnitude to what was observed in the last four months of the year.', 'The current phenomenon is spread homogeneously across the Euro area.', 'The current phenomenon differs from the crisis that hit the Eurozone a decade ago.']</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: added sentiment analysis during translation
+ added batch processing to TranslationService
+ handled edge cases like dirty sentiment values or missing column
</commit_message>
<xml_diff>
--- a/data/Annotazioni_1_with_factoids.xlsx
+++ b/data/Annotazioni_1_with_factoids.xlsx
@@ -542,17 +542,17 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Pensioners, beneficiaries of maintenance payments following divorce, and landlords can try to avoid being overwhelmed by the crazy run of prices. However, public and private employees (unless there are specific contractual agreements) and the self-employed will see their wages stagnate. In fact, as Istat explained a few days ago, with contractual wages growing by only 0.8% and an inflation rate of 5.2%, there will be a loss of purchasing power of nearly five points this year. The shield, however, is not for everyone, and, as stated, things will not go well for all. The law, for example, provides for the revaluation of maintenance payments in the event of separation or divorce, in order to protect the recipient by adjusting the amount owed to the economically weaker spouse or children according to the average cost of living. This revaluation must be carried out every year according to Istat indices and must be applied always and forever, regardless of whether the spouses agreed to it or if the judge ruled on the separation or divorce. For revaluation, the Consumer Price Index (CPI) for working-class families is used, referencing the index published by Istat relative to the month of the first payment of the maintenance payment decided by the court in the previous year. In case of failure to adjust, the rule also provides for the possibility of claiming back pay for the last 5 years. Even pensioners will have a protective shield. Since this year, the indexation mechanism has been reintroduced, revaluing pension amounts for different tiers and brackets. Thus, pensioners who receive a monthly allowance up to 4 times the social allowance (about 2,000 euros) will receive a full revaluation of the amount relative to inflation; pensioners who receive between 4 and 5 times the allowance will receive a 90% increase relative to inflation; and pensioners who receive more than 5 times the social allowance will receive a 75% increase relative to inflation. Istat has established that, for this year, the inflation index used for these adjustments, however, refers to 2021, and will be 1.9 percent. But in 2023, the allowances will recover the price growth recorded in 2022, and the revaluation, based on current estimates, could reach around 7%. Property owners can also link their rental payments to inflation, while, regarding severance pay, the rules provide that the TFR (end-of-service benefit), excluding the amount accrued in the current year, will be increased every year by applying a fixed rate of 1.5% and 75% of the increase in the CPI for working-class families (3/4 of the inflation rate), determined by Istat, relative to the month of December of the previous year. In case of applying the revaluation rate for fractions of a year, the increase in the Istat index is that resulting in the month the employment relationship ceases compared to that of December of the previous year. Example: if inflation is at 2%: 75% equals 1.5%, to which the fixed rate is added. Therefore, the TFR must be revalued by 3%, equal to 1.5% plus 1.5%. Michele di Branco</t>
+          <t>Pensioners, recipients of maintenance payments in case of divorce, and landlords can try to avoid being overwhelmed by the crazy run of prices. However, public and private employees (unless there are specific contractual agreements) and the self-employed will remain stuck with their salaries. In fact, as Istat explained a few days ago, with contractual wages growing by only 0.8% and an inflation rate of 5.2%, there will be a loss of purchasing power of nearly five points this year. The shield is not for everyone, though, and as mentioned, things will not be that bad. For instance, the law provides for the revaluation of maintenance payments in the event of separation or divorce, in order to protect the recipient by adjusting the amount owed to the economically weaker spouse or children according to the average cost of living. This revaluation must be carried out every year according to Istat indices and must always apply, regardless of whether the spouses agreed to it or if the judge ruled on the separation or divorce. For revaluation, the Consumer Price Index for working-class families is used, taking as reference the index published by Istat relative to the month of the first payment of the previous year's maintenance payment decided by the court. In case of non-adjustment, the rule also provides for the possibility of claiming arrears for the last 5 years. Even pensioners will have a protective shield. Since this year, the mechanism of indexation has been reintroduced, revaluing pension amounts for specific brackets and tiers. Thus, pensioners who receive a monthly allowance up to 4 times the social minimum (about 2,000 euros) will receive a full revaluation of the amount relative to inflation; pensioners who receive between 4 and 5 times the social minimum will receive a 90% increase relative to inflation; and pensioners who receive more than 5 times the social minimum will receive a 75% increase relative to inflation. Istat has established that, for this year, the inflation index used for the adjustments mentioned is based on 2021, and will be 1.9 percent. However, in 2023, the allowances will recover the price growth recorded in 2022, and the revaluation, based on current estimates, could reach around 7%. Property owners can also link their rental income to inflation, while, regarding liquidations, the rules provide that the TFR (end-of-service benefit), excluding the amount accrued in the current year, will be increased every year by applying a fixed rate of 1.5% and 75% of the increase in the Consumer Price Index for working-class families (3/4 of the inflation rate), determined by Istat, compared to the month of December of the previous year. In case of applying the revaluation rate for partial years, the Istat index increase is that resulting in the month of the termination of the employment relationship compared to that of December of the previous year. Example: if inflation is at 2%: 75% is equal to 1.5%, to which the fixed rate is added. Therefore, the TFR must be revalued by 3%, equal to 1.5% plus 1.5%. Michele di Branco</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>Observation date: 2022-07-02 00:00:00. Pensioners, beneficiaries of maintenance payments following divorce, and landlords can try to avoid being overwhelmed by the crazy run of prices. However, public and private employees (unless there are specific contractual agreements) and the self-employed will see their wages stagnate. In fact, as Istat explained a few days ago, with contractual wages growing by only 0.8% and an inflation rate of 5.2%, there will be a loss of purchasing power of nearly five points this year. The shield, however, is not for everyone, and, as stated, things will not go well for all. The law, for example, provides for the revaluation of maintenance payments in the event of separation or divorce, in order to protect the recipient by adjusting the amount owed to the economically weaker spouse or children according to the average cost of living. This revaluation must be carried out every year according to Istat indices and must be applied always and forever, regardless of whether the spouses agreed to it or if the judge ruled on the separation or divorce. For revaluation, the Consumer Price Index (CPI) for working-class families is used, referencing the index published by Istat relative to the month of the first payment of the maintenance payment decided by the court in the previous year. In case of failure to adjust, the rule also provides for the possibility of claiming back pay for the last 5 years. Even pensioners will have a protective shield. Since this year, the indexation mechanism has been reintroduced, revaluing pension amounts for different tiers and brackets. Thus, pensioners who receive a monthly allowance up to 4 times the social allowance (about 2,000 euros) will receive a full revaluation of the amount relative to inflation; pensioners who receive between 4 and 5 times the allowance will receive a 90% increase relative to inflation; and pensioners who receive more than 5 times the social allowance will receive a 75% increase relative to inflation. Istat has established that, for this year, the inflation index used for these adjustments, however, refers to 2021, and will be 1.9 percent. But in 2023, the allowances will recover the price growth recorded in 2022, and the revaluation, based on current estimates, could reach around 7%. Property owners can also link their rental payments to inflation, while, regarding severance pay, the rules provide that the TFR (end-of-service benefit), excluding the amount accrued in the current year, will be increased every year by applying a fixed rate of 1.5% and 75% of the increase in the CPI for working-class families (3/4 of the inflation rate), determined by Istat, relative to the month of December of the previous year. In case of applying the revaluation rate for fractions of a year, the increase in the Istat index is that resulting in the month the employment relationship ceases compared to that of December of the previous year. Example: if inflation is at 2%: 75% equals 1.5%, to which the fixed rate is added. Therefore, the TFR must be revalued by 3%, equal to 1.5% plus 1.5%. Michele di Branco</t>
+          <t>Observation date: 2022-07-02 00:00:00. Pensioners, recipients of maintenance payments in case of divorce, and landlords can try to avoid being overwhelmed by the crazy run of prices. However, public and private employees (unless there are specific contractual agreements) and the self-employed will remain stuck with their salaries. In fact, as Istat explained a few days ago, with contractual wages growing by only 0.8% and an inflation rate of 5.2%, there will be a loss of purchasing power of nearly five points this year. The shield is not for everyone, though, and as mentioned, things will not be that bad. For instance, the law provides for the revaluation of maintenance payments in the event of separation or divorce, in order to protect the recipient by adjusting the amount owed to the economically weaker spouse or children according to the average cost of living. This revaluation must be carried out every year according to Istat indices and must always apply, regardless of whether the spouses agreed to it or if the judge ruled on the separation or divorce. For revaluation, the Consumer Price Index for working-class families is used, taking as reference the index published by Istat relative to the month of the first payment of the previous year's maintenance payment decided by the court. In case of non-adjustment, the rule also provides for the possibility of claiming arrears for the last 5 years. Even pensioners will have a protective shield. Since this year, the mechanism of indexation has been reintroduced, revaluing pension amounts for specific brackets and tiers. Thus, pensioners who receive a monthly allowance up to 4 times the social minimum (about 2,000 euros) will receive a full revaluation of the amount relative to inflation; pensioners who receive between 4 and 5 times the social minimum will receive a 90% increase relative to inflation; and pensioners who receive more than 5 times the social minimum will receive a 75% increase relative to inflation. Istat has established that, for this year, the inflation index used for the adjustments mentioned is based on 2021, and will be 1.9 percent. However, in 2023, the allowances will recover the price growth recorded in 2022, and the revaluation, based on current estimates, could reach around 7%. Property owners can also link their rental income to inflation, while, regarding liquidations, the rules provide that the TFR (end-of-service benefit), excluding the amount accrued in the current year, will be increased every year by applying a fixed rate of 1.5% and 75% of the increase in the Consumer Price Index for working-class families (3/4 of the inflation rate), determined by Istat, compared to the month of December of the previous year. In case of applying the revaluation rate for partial years, the Istat index increase is that resulting in the month of the termination of the employment relationship compared to that of December of the previous year. Example: if inflation is at 2%: 75% is equal to 1.5%, to which the fixed rate is added. Therefore, the TFR must be revalued by 3%, equal to 1.5% plus 1.5%. Michele di Branco</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>['Public and private employees (unless there are specific contractual agreements) and the self-employed will see their wages stagnate.', 'Istat explained on 2022-06-28 that contractual wages grew by 0.8%.', 'Istat explained on 2022-06-28 that the inflation rate was 5.2%.', 'The combination of 0.8% wage growth and 5.2% inflation will result in a loss of purchasing power of nearly five points in 2022.', 'The law provides for the revaluation of maintenance payments following separation or divorce.', 'The revaluation protects the recipient by adjusting the amount owed to the economically weaker spouse or children according to the average cost of living.', 'The revaluation of maintenance payments must be carried out every year according to Istat indices.', 'The revaluation must be applied always and forever, regardless of whether the spouses agreed to it or if the judge ruled on the separation or divorce.', 'The Consumer Price Index (CPI) for working-class families is used for maintenance revaluation.', 'The CPI references the index published by Istat relative to the month of the first payment of the maintenance payment decided by the court in the previous year.', 'If adjustment fails, the rule allows claiming back pay for the last 5 years.', 'The indexation mechanism for pensions was reintroduced in 2022.', 'Pensioners receiving a monthly allowance up to 4 times the social allowance (about 2,000 euros) will receive a full revaluation of the amount relative to inflation.', 'Pensioners receiving between 4 and 5 times the social allowance will receive a 90% increase relative to inflation.', 'Istat established that the inflation index used for pension adjustments in 2022 refers to 2021 and will be 1.9 percent.', 'The allowances will recover the price growth recorded in 2022 in 2023.', 'The revaluation for pensions could reach around 7% based on current estimates.', 'Property owners can link their rental payments to inflation.', 'Rules regarding severance pay state that the TFR (end-of-service benefit), excluding the amount accrued in the current year, will be increased every year.', 'The TFR increase is calculated by applying a fixed rate of 1.5% and 75% of the increase in the CPI for working-class families (3/4 of the inflation rate), determined by Istat.', 'The TFR calculation references the month of December of the previous year.', 'If applying the revaluation rate for fractions of a year, the increase in the Istat index compares the month the employment relationship ceases to December of the previous year.']</t>
+          <t>['Public and private employees (unless there are specific contractual agreements) and the self-employed will remain stuck with their salaries.', 'Istat explained that contractual wages grew by 0.8%.', 'Istat explained that the inflation rate is 5.2%.', 'The combination of 0.8% wage growth and 5.2% inflation will result in a loss of purchasing power of nearly five points on 2022-01-01.', 'The law provides for the revaluation of maintenance payments in the event of separation or divorce.', 'The revaluation protects the recipient by adjusting the amount owed to the economically weaker spouse or children according to the average cost of living.', 'The revaluation must be carried out every year according to Istat indices.', 'The revaluation applies regardless of whether the spouses agreed to it.', 'The revaluation applies regardless of whether the judge ruled on the separation or divorce.', 'The Consumer Price Index for working-class families is used for revaluation.', "The index used for revaluation is published by Istat relative to the month of the first payment of the previous year's maintenance payment decided by the court.", 'If there is non-adjustment, the rule allows claiming arrears for the last 5 years.', 'Since 2022-07-02, the mechanism of indexation has been reintroduced.', 'The indexation mechanism revalues pension amounts for specific brackets and tiers.', 'Pensioners receiving a monthly allowance up to 4 times the social minimum (about 2,000 euros) will receive a full revaluation relative to inflation.', 'Pensioners receiving between 4 and 5 times the social minimum will receive a 90% increase relative to inflation.', 'Istat established that the inflation index used for the adjustments mentioned for on 2022-01-01 will be 1.9 percent.', 'In 2023, the allowances will recover the price growth recorded in 2022.', 'The revaluation, based on current estimates, could reach around 7%.', 'Property owners can link their rental income to inflation.', 'The rules regarding liquidations state that the TFR (end-of-service benefit), excluding the amount accrued in the current year, will be increased every year.', 'The TFR increase applies by applying a fixed rate of 1.5%.', 'The TFR increase also applies by applying 75% of the increase in the Consumer Price Index for working-class families (3/4 of the inflation rate).', 'Istat determines the TFR increase rate by comparing it to the month of December of the previous year.', 'When applying the revaluation rate for partial years, the Istat index increase is calculated from the month of the termination of the employment relationship compared to December of the previous year.', 'If inflation is at 2%, 75% equals 1.5%.', 'The TFR must be revalued by 3% (1.5% plus 1.5%) if inflation is at 2%.']</t>
         </is>
       </c>
     </row>
@@ -610,17 +610,17 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>The government's move on the IMU property tax is triggered, which returns in a disguised form this December, serving as an advance payment for a 'service tax.' The Treasury is scrambling for 3 billion [euros] to avoid the planned VAT increase in October, but this 'makeup operation' concerning the housing tax is expected to arrive in November. And now, alarm bells are ringing at the Quirinale [Prime Minister's residence]. The stability of the Finance Law is at risk. The President's consultations with Secretaries Alfano and Epifani take place while the PDL threatens another crisis. In Germany, Angela Merkel has seen a clear winner in the popular vote. However, an electoral law that many insist on exporting here will not allow her to govern alone. A new, large coalition thus looms on the horizon. The last one, the series, in 2005, resulted from an agreement signed after weeks of negotiations. The legislative program was over 300 pages, exceeding in length even Prodi's 2006 electoral manifesto. Like that, it remained dead letter. Our great coalition was born from a half-hour investiture speech by the acting president. Everything and more was promised, denying any budgetary constraints. Then came the same decision paralysis, albeit more animated than in Germany: furious arguments broadcast live on TV as soon as they had to confront budgetary constraints. Those do not forgive. Unlike the Germans, we cannot afford decision paralysis. The current government now acts only in the realm of dreams or in that of accounting tricks. The update note to the Stability Pact, presented a few days ago by our executive, proposes macroeconomic scenarios straight out of a late summer dream. We should grow in the next three years at a rate double the potential rate, shattering the estimates of international organizations, without having done anything to make such a sharp change of pace possible. These scenarios contemplate the coexistence of high inflation (a GDP deflator of 2 percent), a further drop in household consumption, and rising unemployment. It is difficult to understand how these three phenomena can materialize simultaneously. Perhaps they will be used to draw tables in which the public debt-to-GDP ratio never rises above 130 percent. But these unrealistic scenarios cannot convince institutional fund managers to invest in our country. On the contrary, they risk weakening our negotiating position at the community level. We are already hearing the objections in Brussels: 'If things are destined to go so well, why should we grant you the room for maneuver you ask for?' To the false optimism has been added accounting engineering. They plan to revalue the shares held by banks at the Bank of Italy, a legacy from when banks were public. The banks are pleased to see their equity position strengthened. The Treasury is pleased to receive a contribution from the realized capital gains. The taxpayers, however, are less pleased, as they will one day have to repurchase these shares because a central bank cannot be owned by private banks. They risk paying a very high price because the price will presumably be very high. This would be in the interest of both the banks and the Treasury. And there are no market references, so much so that a special commission of experts has been established. While they bury their heads in the sand with dreams and accounting engineering, the country risks ending, day after day, in the hands of the Troika, without us even realizing it. It was difficult to return from a debt of 120 percent. It is much more difficult to do so from a debt of 130 percent and rising. If this government does not want to be remembered for ceding national sovereignty, it must find a program agreement on the basis of which to open negotiations with Brussels. The agreement should be enshrined in the Stability Law. Its philosophy is to address emergencies with long-term reforms. For example, the refinancing of the temporary layoff fund should contemplate the gradual phasing out of this institution, with wage supplements for those working less than 5 euros per hour, a way to facilitate labor mobility and increase employment. Every new access to the temporary fund must be blocked, starting with that requested for former party employees by a very large parliamentary coalition. They will be able, like other workers, to access ordinary social safety nets. Another example: the VAT increase could be avoided, possibly restricted only to luxury goods, with a cut to the tax wedge, given that indirect taxes increase the difference between labor costs and purchasing power of wages. There should then be spending cut measures, which could be implemented gradually, but with already approved interventions. One could start by dismantling the bureaucracy created by the Lega's federalism, which has created duplications, uncontrolled local spending, and an excess of centers of power. Some examples: how to justify the sponsorship offered by the Sardinia region to the Cagliari football team? What are 45 port authorities for? And can the staffing levels of the prefectures be reduced, and the provinces truly abolished? It is unnecessary to point out that cutting these waste items is politically costly. The steering committee should really serve to protect the government from the fierce attacks it will face from those affected by the cuts. With these measures included in the Stability Law, it is possible to open negotiations with Brussels that also contemplate deficits exceeding 3 percent in the coming years. But it will require a cohesive government, not a collection whose survival is questioned every day.</t>
+          <t>The government's move on the IMU (municipal property tax) is underway, which returns in a disguised form by December as an advance payment for the "service tax." The Treasury is hunting for 3 billion euros to avoid the VAT increase scheduled for October, but the 'makeover' operation concerning the housing tax is expected by November. And now, alarm bells ring in the Quirinale (Presidential Palace). The stability of the financial law is at risk. Consultations between President Napolitano and Secretaries Alfano and Epifani, while the PDL threatens another crisis. In Germany, the elections had a clear popular winner: Angela Merkel. But an electoral law that many insist on exporting to us will not allow her to govern alone. Thus, a new Grand Coalition looms on the horizon—the last one occurred in 2005, stemming from an agreement signed after weeks of negotiations. The legislative program was over 300 pages, exceeding in length even Prodi's 2006 electoral manifesto. Like that, it remained dead letter. Our great coalition was born from a half-hour investiture speech by the acting president. Everything and more was promised, denying any budgetary constraints. Then came the same decision paralysis, albeit more animated than in Germany: furious arguments live on TV as soon as they encountered budgetary constraints. Those do not forgive. Unlike the Germans, we cannot afford decision paralysis. The current government now acts only in the realm of dreams or in that of accounting tricks. The update to the Stability Pact (DEF) presented a few days ago by our executive proposes macroeconomic scenarios straight out of a dream late summer. We should grow in the next three years at a rate double the potential rate, shattering the estimates of international organizations, without having done anything to make such a sharp change of pace possible. These scenarios contemplate the coexistence of high inflation (a 2% GDP deflator), a further decline in household consumption, and rising unemployment. It is difficult to understand how these three phenomena can materialize simultaneously. Perhaps they will be used to draw tables in which the public debt-to-GDP ratio never rises above 130 percent, but these unrealistic scenarios cannot convince institutional fund managers to invest in our country. On the contrary, they risk weakening our negotiating position at the community level. We are already hearing objections from Brussels: "If things are destined to go so well, why should we grant you the maneuvering room you ask for?" To the false optimism has been added the accounting engineering. They plan to revalue the shares held by banks at the Bank of Italy, a relic from when banks were public. The banks are pleased to see their equity position strengthened. The Treasury is pleased to receive a contribution from the realized capital gains. The taxpayers, however, are less pleased, as they will eventually have to repurchase these shares because a central bank cannot be owned by private banks. They risk paying a very high price because the price will presumably be very elevated. This would be in the interest of both the banks and the Treasury. And there are no market references, so an ad hoc commission of experts has been established. While they bury their heads in the sand with dreams and accounting engineering, the country risks ending, day after day, in the hands of the Troika, without us even realizing it. It was difficult to return from a debt of 120 percent. It is much harder to do so from a debt of 130 percent and rising. If this government does not want to be remembered for ceding national sovereignty, it must find a program agreement on the basis of which to open negotiations with Brussels. The agreement should be enshrined in the Stability Law. Its philosophy is to address emergencies with long-term reforms. For example, the refinancing of the temporary layoff fund should contemplate the gradual phasing out of this institution, with wage supplements for those working less than 5 euros an hour, a way to facilitate labor mobility and increase employment. New access to the temporary layoff fund must be blocked, starting with that requested for former party employees by a very large parliamentary coalition. They will be able, like other workers, to access ordinary social safety nets. Another example: the VAT increase could be limited possibly only to luxury goods, coupled with a reduction of the tax wedge, given that indirect taxes increase the difference between labor costs and the purchasing power of wages. There should then be spending cut measures, which could be implemented gradually, but with already approved interventions. We can start by dismantling the bureaucracy created by the Lega's federalism, which has created duplications, uncontrolled local spending, and an excess of centers of power. Some examples: how to justify the sponsorship offered by the Sardinia region to the Cagliari football team? What are 45 port authorities for? And cannot the staffing levels of the prefectures be reduced, and the provinces abolished for good? Needless to say, cutting these wastes is politically costly. The steering committee should really serve to protect the government from the fierce attacks it will face from those affected by the cuts. With these measures included in the Stability Law, it is possible to open negotiations with Brussels that also contemplate deficits above 3 percent in the coming years. But it will require a cohesive government, not a coalition whose survival is questioned every day.</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Observation date: 2013-09-25 00:00:00. The government's move on the IMU property tax is triggered, which returns in a disguised form this December, serving as an advance payment for a 'service tax.' The Treasury is scrambling for 3 billion [euros] to avoid the planned VAT increase in October, but this 'makeup operation' concerning the housing tax is expected to arrive in November. And now, alarm bells are ringing at the Quirinale [Prime Minister's residence]. The stability of the Finance Law is at risk. The President's consultations with Secretaries Alfano and Epifani take place while the PDL threatens another crisis. In Germany, Angela Merkel has seen a clear winner in the popular vote. However, an electoral law that many insist on exporting here will not allow her to govern alone. A new, large coalition thus looms on the horizon. The last one, the series, in 2005, resulted from an agreement signed after weeks of negotiations. The legislative program was over 300 pages, exceeding in length even Prodi's 2006 electoral manifesto. Like that, it remained dead letter. Our great coalition was born from a half-hour investiture speech by the acting president. Everything and more was promised, denying any budgetary constraints. Then came the same decision paralysis, albeit more animated than in Germany: furious arguments broadcast live on TV as soon as they had to confront budgetary constraints. Those do not forgive. Unlike the Germans, we cannot afford decision paralysis. The current government now acts only in the realm of dreams or in that of accounting tricks. The update note to the Stability Pact, presented a few days ago by our executive, proposes macroeconomic scenarios straight out of a late summer dream. We should grow in the next three years at a rate double the potential rate, shattering the estimates of international organizations, without having done anything to make such a sharp change of pace possible. These scenarios contemplate the coexistence of high inflation (a GDP deflator of 2 percent), a further drop in household consumption, and rising unemployment. It is difficult to understand how these three phenomena can materialize simultaneously. Perhaps they will be used to draw tables in which the public debt-to-GDP ratio never rises above 130 percent. But these unrealistic scenarios cannot convince institutional fund managers to invest in our country. On the contrary, they risk weakening our negotiating position at the community level. We are already hearing the objections in Brussels: 'If things are destined to go so well, why should we grant you the room for maneuver you ask for?' To the false optimism has been added accounting engineering. They plan to revalue the shares held by banks at the Bank of Italy, a legacy from when banks were public. The banks are pleased to see their equity position strengthened. The Treasury is pleased to receive a contribution from the realized capital gains. The taxpayers, however, are less pleased, as they will one day have to repurchase these shares because a central bank cannot be owned by private banks. They risk paying a very high price because the price will presumably be very high. This would be in the interest of both the banks and the Treasury. And there are no market references, so much so that a special commission of experts has been established. While they bury their heads in the sand with dreams and accounting engineering, the country risks ending, day after day, in the hands of the Troika, without us even realizing it. It was difficult to return from a debt of 120 percent. It is much more difficult to do so from a debt of 130 percent and rising. If this government does not want to be remembered for ceding national sovereignty, it must find a program agreement on the basis of which to open negotiations with Brussels. The agreement should be enshrined in the Stability Law. Its philosophy is to address emergencies with long-term reforms. For example, the refinancing of the temporary layoff fund should contemplate the gradual phasing out of this institution, with wage supplements for those working less than 5 euros per hour, a way to facilitate labor mobility and increase employment. Every new access to the temporary fund must be blocked, starting with that requested for former party employees by a very large parliamentary coalition. They will be able, like other workers, to access ordinary social safety nets. Another example: the VAT increase could be avoided, possibly restricted only to luxury goods, with a cut to the tax wedge, given that indirect taxes increase the difference between labor costs and purchasing power of wages. There should then be spending cut measures, which could be implemented gradually, but with already approved interventions. One could start by dismantling the bureaucracy created by the Lega's federalism, which has created duplications, uncontrolled local spending, and an excess of centers of power. Some examples: how to justify the sponsorship offered by the Sardinia region to the Cagliari football team? What are 45 port authorities for? And can the staffing levels of the prefectures be reduced, and the provinces truly abolished? It is unnecessary to point out that cutting these waste items is politically costly. The steering committee should really serve to protect the government from the fierce attacks it will face from those affected by the cuts. With these measures included in the Stability Law, it is possible to open negotiations with Brussels that also contemplate deficits exceeding 3 percent in the coming years. But it will require a cohesive government, not a collection whose survival is questioned every day.</t>
+          <t>Observation date: 2013-09-25 00:00:00. The government's move on the IMU (municipal property tax) is underway, which returns in a disguised form by December as an advance payment for the "service tax." The Treasury is hunting for 3 billion euros to avoid the VAT increase scheduled for October, but the 'makeover' operation concerning the housing tax is expected by November. And now, alarm bells ring in the Quirinale (Presidential Palace). The stability of the financial law is at risk. Consultations between President Napolitano and Secretaries Alfano and Epifani, while the PDL threatens another crisis. In Germany, the elections had a clear popular winner: Angela Merkel. But an electoral law that many insist on exporting to us will not allow her to govern alone. Thus, a new Grand Coalition looms on the horizon—the last one occurred in 2005, stemming from an agreement signed after weeks of negotiations. The legislative program was over 300 pages, exceeding in length even Prodi's 2006 electoral manifesto. Like that, it remained dead letter. Our great coalition was born from a half-hour investiture speech by the acting president. Everything and more was promised, denying any budgetary constraints. Then came the same decision paralysis, albeit more animated than in Germany: furious arguments live on TV as soon as they encountered budgetary constraints. Those do not forgive. Unlike the Germans, we cannot afford decision paralysis. The current government now acts only in the realm of dreams or in that of accounting tricks. The update to the Stability Pact (DEF) presented a few days ago by our executive proposes macroeconomic scenarios straight out of a dream late summer. We should grow in the next three years at a rate double the potential rate, shattering the estimates of international organizations, without having done anything to make such a sharp change of pace possible. These scenarios contemplate the coexistence of high inflation (a 2% GDP deflator), a further decline in household consumption, and rising unemployment. It is difficult to understand how these three phenomena can materialize simultaneously. Perhaps they will be used to draw tables in which the public debt-to-GDP ratio never rises above 130 percent, but these unrealistic scenarios cannot convince institutional fund managers to invest in our country. On the contrary, they risk weakening our negotiating position at the community level. We are already hearing objections from Brussels: "If things are destined to go so well, why should we grant you the maneuvering room you ask for?" To the false optimism has been added the accounting engineering. They plan to revalue the shares held by banks at the Bank of Italy, a relic from when banks were public. The banks are pleased to see their equity position strengthened. The Treasury is pleased to receive a contribution from the realized capital gains. The taxpayers, however, are less pleased, as they will eventually have to repurchase these shares because a central bank cannot be owned by private banks. They risk paying a very high price because the price will presumably be very elevated. This would be in the interest of both the banks and the Treasury. And there are no market references, so an ad hoc commission of experts has been established. While they bury their heads in the sand with dreams and accounting engineering, the country risks ending, day after day, in the hands of the Troika, without us even realizing it. It was difficult to return from a debt of 120 percent. It is much harder to do so from a debt of 130 percent and rising. If this government does not want to be remembered for ceding national sovereignty, it must find a program agreement on the basis of which to open negotiations with Brussels. The agreement should be enshrined in the Stability Law. Its philosophy is to address emergencies with long-term reforms. For example, the refinancing of the temporary layoff fund should contemplate the gradual phasing out of this institution, with wage supplements for those working less than 5 euros an hour, a way to facilitate labor mobility and increase employment. New access to the temporary layoff fund must be blocked, starting with that requested for former party employees by a very large parliamentary coalition. They will be able, like other workers, to access ordinary social safety nets. Another example: the VAT increase could be limited possibly only to luxury goods, coupled with a reduction of the tax wedge, given that indirect taxes increase the difference between labor costs and the purchasing power of wages. There should then be spending cut measures, which could be implemented gradually, but with already approved interventions. We can start by dismantling the bureaucracy created by the Lega's federalism, which has created duplications, uncontrolled local spending, and an excess of centers of power. Some examples: how to justify the sponsorship offered by the Sardinia region to the Cagliari football team? What are 45 port authorities for? And cannot the staffing levels of the prefectures be reduced, and the provinces abolished for good? Needless to say, cutting these wastes is politically costly. The steering committee should really serve to protect the government from the fierce attacks it will face from those affected by the cuts. With these measures included in the Stability Law, it is possible to open negotiations with Brussels that also contemplate deficits above 3 percent in the coming years. But it will require a cohesive government, not a coalition whose survival is questioned every day.</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>["The government's move on the IMU property tax is triggered.", 'The move on the IMU property tax returns in a disguised form in December 2013.', "The disguised form serves as an advance payment for a 'service tax.'", 'The Treasury is scrambling for 3 billion euros.', 'The Treasury needs the money to avoid the planned VAT increase in October 2013.', "A 'makeup operation' concerning the housing tax is expected to arrive in November 2013.", "Alarm bells are ringing at the Quirinale [Prime Minister's residence].", 'The stability of the Finance Law is at risk.', "The President's consultations with Secretaries Alfano and Epifani take place.", 'The PDL threatens another crisis.', 'In Germany, Angela Merkel saw a clear winner in the popular vote.', 'An electoral law that many insist on exporting here will not allow Angela Merkel to govern alone.', 'A new, large coalition looms on the horizon.', 'The last coalition in 2005 resulted from an agreement signed after weeks of negotiations.', 'The legislative program from 2005 was over 300 pages.', "The legislative program from 2005 exceeded in length even Prodi's 2006 electoral manifesto.", 'The legislative program from 2005 remained a dead letter.', 'The great coalition was born from a half-hour investiture speech by the acting president.', 'The current government acts only in the realm of dreams or in that of accounting tricks.', 'The executive presented an update note to the Stability Pact a few days ago.', 'The update note to the Stability Pact proposes macroeconomic scenarios.', 'The scenarios propose growth in the next three years at a rate double the potential rate.', 'The scenarios contemplate the coexistence of high inflation (a GDP deflator of 2 percent).', 'The scenarios contemplate a further drop in household consumption.', 'The scenarios contemplate rising unemployment.', 'The scenarios might be used to draw tables where the public debt-to-GDP ratio never rises above 130 percent.', 'The unrealistic scenarios cannot convince institutional fund managers to invest in the country.', 'The scenarios risk weakening the negotiating position of the country at the community level.', 'The plan involves revaluing the shares held by banks at the Bank of Italy.', 'The banks are pleased to see their equity position strengthened.', 'The Treasury is pleased to receive a contribution from the realized capital gains.', 'The taxpayers will one day have to repurchase these shares.', 'A central bank cannot be owned by private banks.', 'The taxpayers risk paying a very high price.', 'A special commission of experts has been established because there are no market references.', 'The country risks ending in the hands of the Troika.', 'It was difficult to return from a debt of 120 percent.', 'It is much more difficult to return from a debt of 130 percent and rising.', 'The government must find a program agreement to open negotiations with Brussels.', 'The program agreement should be enshrined in the Stability Law.', 'The philosophy of the Stability Law is to address emergencies with long-term reforms.', 'Refinancing the temporary layoff fund should contemplate the gradual phasing out of this institution.', 'The phasing out should include wage supplements for those working less than 5 euros per hour.', 'This measure aims to facilitate labor mobility and increase employment.', 'Every new access to the temporary fund must be blocked.', 'The blocking must start with the access requested for former party employees by a very large parliamentary coalition.', 'Former party employees will be able to access ordinary social safety nets.', 'The VAT increase could be restricted only to luxury goods.', 'The VAT increase could involve a cut to the tax wedge.', 'Indirect taxes increase the difference between labor costs and purchasing power of wages.', 'Spending cut measures should be implemented.', "Dismantling the bureaucracy created by the Lega's federalism is a potential spending cut measure.", 'The steering committee should protect the government from fierce attacks.', 'The measures included in the Stability Law make it possible to open negotiations with Brussels.', 'These negotiations can contemplate deficits exceeding 3 percent in the coming years.']</t>
+          <t>["The government's move on the IMU (municipal property tax) is underway.", "The IMU move will return in a disguised form by December 2013 as an advance payment for the 'service tax'.", 'The Treasury is hunting for 3 billion euros.', 'The Treasury needs 3 billion euros to avoid the VAT increase scheduled for October 2013.', "The 'makeover' operation concerning the housing tax is expected by November 2013.", 'Alarm bells are ringing in the Quirinale (Presidential Palace).', 'The stability of the financial law is at risk.', 'In Germany, Angela Merkel was the clear popular winner in the elections.', 'An electoral law that many insist on exporting to Italy will not allow Angela Merkel to govern alone.', 'A new Grand Coalition looms on the horizon.', 'The last Grand Coalition occurred in 2005.', "The legislative program from the 2005 Grand Coalition exceeded the length of Prodi's 2006 electoral manifesto.", 'The current government acts only in the realm of dreams or in the realm of accounting tricks.', 'The update to the Stability Pact (DEF) was presented a few days ago by the executive.', "The executive's update proposes macroeconomic scenarios for the next three years.", 'The proposed scenarios suggest a growth rate double the potential rate.', 'The proposed scenarios contemplate high inflation, specifically a 2% GDP deflator.', 'The proposed scenarios contemplate a further decline in household consumption.', 'The proposed scenarios contemplate rising unemployment.', 'International organizations shattered the estimates of the proposed growth rate.', "The proposed scenarios risk weakening Italy's negotiating position at the community level.", 'Brussels has already heard objections regarding the proposed scenarios.', 'The false optimism has been added to by accounting engineering.', 'The government plans to revalue the shares held by banks at the Bank of Italy.', 'The banks are pleased to see their equity position strengthened.', 'The Treasury is pleased to receive a contribution from the realized capital gains.', 'Taxpayers will eventually have to repurchase the shares.', 'A central bank cannot be owned by private banks.', 'An ad hoc commission of experts has been established because there are no market references.', 'The country risks ending in the hands of the Troika.', 'It was difficult to return from a debt of 120 percent.', 'It is much harder to return from a debt of 130 percent and rising.', 'The government must find a program agreement to open negotiations with Brussels.', 'The program agreement should be enshrined in the Stability Law.', 'The philosophy of the Stability Law is to address emergencies with long-term reforms.', 'The refinancing of the temporary layoff fund should contemplate the gradual phasing out of this institution.', 'Wage supplements for those working less than 5 euros an hour should be implemented.', 'This measure aims to facilitate labor mobility and increase employment.', 'New access to the temporary layoff fund must be blocked.', 'The blocking of new access must start with the request for former party employees by a very large parliamentary coalition.', 'Former party employees will be able to access ordinary social safety nets.', 'The VAT increase could be limited possibly only to luxury goods.', 'The VAT increase could be coupled with a reduction of the tax wedge.', 'Indirect taxes increase the difference between labor costs and the purchasing power of wages.', 'Spending cut measures should be implemented.', 'Spending cut measures should be approved interventions.', "Italy can start by dismantling the bureaucracy created by the Lega's federalism.", "The Lega's federalism created duplications and uncontrolled local spending.", "The Lega's federalism created an excess of centers of power.", 'The staffing levels of the prefectures can be reduced.', 'The provinces can be abolished for good.', 'The steering committee should protect the government from fierce attacks from those affected by the cuts.', 'Including these measures in the Stability Law makes it possible to open negotiations with Brussels.', 'These negotiations can also contemplate deficits above 3 percent in the coming years.', 'Opening negotiations requires a cohesive government.']</t>
         </is>
       </c>
     </row>
@@ -674,17 +674,17 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>It is useless to delude oneself: the recovery will be timid, weak, and fraught with 'downside risks.' Small businesses, especially those in the south, are left on the sidelines; consumption is languishing. Furthermore, unemployment is increasing even in 2015, and inflation continues to decline. The Bank of Italy's economic bulletin, the first of the new year, is more cautious than ever. Its quarterly release coincides this time with two major pieces of news regarding GDP. The first: the EU Commissioner, Olli Rehn, is confident in the country's ability to recover, calling for increased dismissals and a spending review, and suggesting the hypothesis that Italy could obtain more 'flexibility' regarding budgetary rules—a condition essential for freeing up resources for investment. For the record: yesterday, the Commissioner held a breakfast meeting with the Minister of Economy, Fabrizio Saccomanni, on these and other topics. The second piece of news reveals that the EU is revising the calculation of GDP, moving investments in research and development from the expenditure category—thus a liability—to the investment category. According to extrapolations, the benefit will be between 1% and 2%, with non-negligible effects even for the deficit-to-GDP and debt-to-GDP ratios, and thus, for the country's fiscal consolidation and relations with Brussels. The Bank of Italy's document, naturally, remains anchored only on technical-analytical grounds. Thus, the macro projections elaborated by these economists place year-end GDP growth at 0.7%, before rising to 1% in 2015. These are therefore estimates considerably more contained than those of the government (1% and 1.7%, respectively). They are small upward jumps, within an overall sluggish European context. The effects on the labor market are not yet visible: this year the unemployment rate will remain stuck at 12.8%, and next year it will rise to 12.9%. Only the recovery of domestic demand can extend the recovery to the labor market, warns the Bank of Italy. However, at the moment, risks to growth 'remain oriented downwards'; the recovery of investments can be 'delayed,' especially 'if access to credit conditions remain restrictive for longer than anticipated, or if public administration commercial debt payments register delays.' And weighing on everything is the risk of generalized deflation: this danger is judged to be 'modest.' But the fall in inflation could be 'more accentuated and persistent' than expected, 'especially if the weakness of demand were to reflect on expectations.' In short, as the President of the ECB recently recalled, 'it is still too early to celebrate victory'; it is better to keep one's feet on the ground. The general picture, in fact, remains unclear. While business confidence is certainly improving, industrial activity is regaining momentum after having decreased 'almost without interruption' since the summer of 2011. But the underlying picture is very varied depending on the type of business and its location: small businesses, especially in the south, remain on the margins of the process. Similarly, while it is true that the decline in household consumption attenuated in the third quarter of 2013, it is also true that Italians are not spending today. Consumption continues to be constrained by both weak disposable income and difficult labor market conditions. The Bank of Italy also notes that 'the recovery of confidence, which began in early 2013, stopped in the fourth quarter.' Via Nazionale, meanwhile, is changing its internal organization: under the board, 8 departments, services, and divisions. © reproduction reserved.</t>
+          <t>It is useless to imagine: the recovery will be timid, sluggish, and fraught with 'downside risks.' Small businesses, especially those in the south, are left on the sidelines; consumption is languishing. Furthermore, the number of unemployed people is increasing even in 2015, and inflation continues to decline. The Bank of Italy's economic bulletin, the first of the new year, is more cautious than ever. Its quarterly release coincides this time with two major pieces of news regarding GDP. The first: the EU Commissioner, Olli Rehn, is confident in the country's ability to recover, calling for structural reforms and spending reviews and suggesting the hypothesis that Italy could obtain more 'flexibility' regarding budgetary rules—a condition essential for freeing up resources for investment. For the record: yesterday there was a breakfast meeting between the Commissioner and the Minister of Economy, Fabrizio Saccomanni, on these and other topics. The second piece of news reveals that the EU is revising the calculation of GDP, moving investments in research and development from the expenditure category—thus a liability—to the investment category itself. According to extrapolations, the benefit will be between 1% and 2%, with non-negligible effects also for the deficit-to-GDP and debt-to-GDP ratios, and thus, for the country's finances and relations with Brussels. The Bank of Italy's document, obviously, remains anchored only on the technical-analytical ground. Thus, the macro projections elaborated by these economists place the year-end GDP growth at 0.7%, before rising to 1% in 2015. These are therefore estimates much more contained than those of the government (1% and 1.7%, respectively). They are small upward jumps, in a European context that is also slowing down. The effects on employment are not yet visible: this year the unemployment rate will remain stuck at 12.8%, and next year it will rise to 12.9%. Only the recovery of domestic demand can extend the recovery to the labor market, warns the Bank of Italy. At the moment, however, the risks to growth 'remain oriented downwards'; the recovery of investments can be 'delayed,' especially 'if access to credit conditions remain restrictive for longer than anticipated or if public administration commercial debt payments register delays.' And everything is weighed down by the risk of generalized deflation: this danger is judged 'moderate.' But the fall in inflation could be 'more accentuated and persistent' than expected, 'especially if the weakness of demand were to reflect on expectations.' In short, as the President of the ECB recently recalled, 'it is still too early to celebrate victory'; it is better to keep one's feet on the ground. The general picture, in fact, remains unclear. While business confidence is certainly improving, industrial activity is recovering after having decreased 'almost without interruption' since the summer of 2011. But the underlying picture is very varied depending on the type of business and its location: small businesses, especially in the south, remain on the margins of the process. Similarly, while it is true that the decline in family consumption attenuated in the third quarter of 2013, it is also true that today Italians are not spending. Consumption continues to be constrained by both the weakness of disposable income and the difficult conditions of the labor market. The Bank of Italy also notes that 'the recovery of confidence, which began in early 2013, stopped in the fourth quarter.' Meanwhile, Via Nazionale is changing its internal organization: under the board, 8 departments, services, and divisions. © reproduction reserved.</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>Observation date: 2014-01-18 00:00:00. It is useless to delude oneself: the recovery will be timid, weak, and fraught with 'downside risks.' Small businesses, especially those in the south, are left on the sidelines; consumption is languishing. Furthermore, unemployment is increasing even in 2015, and inflation continues to decline. The Bank of Italy's economic bulletin, the first of the new year, is more cautious than ever. Its quarterly release coincides this time with two major pieces of news regarding GDP. The first: the EU Commissioner, Olli Rehn, is confident in the country's ability to recover, calling for increased dismissals and a spending review, and suggesting the hypothesis that Italy could obtain more 'flexibility' regarding budgetary rules—a condition essential for freeing up resources for investment. For the record: yesterday, the Commissioner held a breakfast meeting with the Minister of Economy, Fabrizio Saccomanni, on these and other topics. The second piece of news reveals that the EU is revising the calculation of GDP, moving investments in research and development from the expenditure category—thus a liability—to the investment category. According to extrapolations, the benefit will be between 1% and 2%, with non-negligible effects even for the deficit-to-GDP and debt-to-GDP ratios, and thus, for the country's fiscal consolidation and relations with Brussels. The Bank of Italy's document, naturally, remains anchored only on technical-analytical grounds. Thus, the macro projections elaborated by these economists place year-end GDP growth at 0.7%, before rising to 1% in 2015. These are therefore estimates considerably more contained than those of the government (1% and 1.7%, respectively). They are small upward jumps, within an overall sluggish European context. The effects on the labor market are not yet visible: this year the unemployment rate will remain stuck at 12.8%, and next year it will rise to 12.9%. Only the recovery of domestic demand can extend the recovery to the labor market, warns the Bank of Italy. However, at the moment, risks to growth 'remain oriented downwards'; the recovery of investments can be 'delayed,' especially 'if access to credit conditions remain restrictive for longer than anticipated, or if public administration commercial debt payments register delays.' And weighing on everything is the risk of generalized deflation: this danger is judged to be 'modest.' But the fall in inflation could be 'more accentuated and persistent' than expected, 'especially if the weakness of demand were to reflect on expectations.' In short, as the President of the ECB recently recalled, 'it is still too early to celebrate victory'; it is better to keep one's feet on the ground. The general picture, in fact, remains unclear. While business confidence is certainly improving, industrial activity is regaining momentum after having decreased 'almost without interruption' since the summer of 2011. But the underlying picture is very varied depending on the type of business and its location: small businesses, especially in the south, remain on the margins of the process. Similarly, while it is true that the decline in household consumption attenuated in the third quarter of 2013, it is also true that Italians are not spending today. Consumption continues to be constrained by both weak disposable income and difficult labor market conditions. The Bank of Italy also notes that 'the recovery of confidence, which began in early 2013, stopped in the fourth quarter.' Via Nazionale, meanwhile, is changing its internal organization: under the board, 8 departments, services, and divisions. © reproduction reserved.</t>
+          <t>Observation date: 2014-01-18 00:00:00. It is useless to imagine: the recovery will be timid, sluggish, and fraught with 'downside risks.' Small businesses, especially those in the south, are left on the sidelines; consumption is languishing. Furthermore, the number of unemployed people is increasing even in 2015, and inflation continues to decline. The Bank of Italy's economic bulletin, the first of the new year, is more cautious than ever. Its quarterly release coincides this time with two major pieces of news regarding GDP. The first: the EU Commissioner, Olli Rehn, is confident in the country's ability to recover, calling for structural reforms and spending reviews and suggesting the hypothesis that Italy could obtain more 'flexibility' regarding budgetary rules—a condition essential for freeing up resources for investment. For the record: yesterday there was a breakfast meeting between the Commissioner and the Minister of Economy, Fabrizio Saccomanni, on these and other topics. The second piece of news reveals that the EU is revising the calculation of GDP, moving investments in research and development from the expenditure category—thus a liability—to the investment category itself. According to extrapolations, the benefit will be between 1% and 2%, with non-negligible effects also for the deficit-to-GDP and debt-to-GDP ratios, and thus, for the country's finances and relations with Brussels. The Bank of Italy's document, obviously, remains anchored only on the technical-analytical ground. Thus, the macro projections elaborated by these economists place the year-end GDP growth at 0.7%, before rising to 1% in 2015. These are therefore estimates much more contained than those of the government (1% and 1.7%, respectively). They are small upward jumps, in a European context that is also slowing down. The effects on employment are not yet visible: this year the unemployment rate will remain stuck at 12.8%, and next year it will rise to 12.9%. Only the recovery of domestic demand can extend the recovery to the labor market, warns the Bank of Italy. At the moment, however, the risks to growth 'remain oriented downwards'; the recovery of investments can be 'delayed,' especially 'if access to credit conditions remain restrictive for longer than anticipated or if public administration commercial debt payments register delays.' And everything is weighed down by the risk of generalized deflation: this danger is judged 'moderate.' But the fall in inflation could be 'more accentuated and persistent' than expected, 'especially if the weakness of demand were to reflect on expectations.' In short, as the President of the ECB recently recalled, 'it is still too early to celebrate victory'; it is better to keep one's feet on the ground. The general picture, in fact, remains unclear. While business confidence is certainly improving, industrial activity is recovering after having decreased 'almost without interruption' since the summer of 2011. But the underlying picture is very varied depending on the type of business and its location: small businesses, especially in the south, remain on the margins of the process. Similarly, while it is true that the decline in family consumption attenuated in the third quarter of 2013, it is also true that today Italians are not spending. Consumption continues to be constrained by both the weakness of disposable income and the difficult conditions of the labor market. The Bank of Italy also notes that 'the recovery of confidence, which began in early 2013, stopped in the fourth quarter.' Meanwhile, Via Nazionale is changing its internal organization: under the board, 8 departments, services, and divisions. © reproduction reserved.</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>['Small businesses, especially those in the south, are left on the sidelines.', 'Consumption is languishing.', 'Unemployment is increasing in 2015.', 'Inflation continues to decline.', "The Bank of Italy's economic bulletin, released on 2014-01-18, is more cautious than ever.", "The Bank of Italy's quarterly release coincides with two major pieces of news regarding GDP.", "Olli Rehn, the EU Commissioner, is confident in Italy's ability to recover.", 'Olli Rehn, the EU Commissioner, called for increased dismissals and a spending review.', "Olli Rehn, the EU Commissioner, suggested that Italy could obtain more 'flexibility' regarding budgetary rules.", 'On 2014-01-17, Olli Rehn, the Commissioner, held a breakfast meeting with Fabrizio Saccomanni, the Minister of Economy.', 'The EU is revising the calculation of GDP.', 'The EU is moving investments in research and development from the expenditure category to the investment category.', 'Extrapolations suggest the benefit of the GDP revision will be between 1% and 2%.', 'The GDP revision will have non-negligible effects on the deficit-to-GDP ratio.', 'Macro projections elaborated by the economists place year-end GDP growth at 0.7%.', "The macro projections are considerably more contained than the government's estimates for year-end GDP growth.", 'The government estimates GDP growth at 1.7% in 2015.', 'The unemployment rate is projected to remain stuck at 12.8% in 2014.', 'The Bank of Italy warns that only the recovery of domestic demand can extend the recovery to the labor market.', 'Risks to growth remain oriented downwards.', 'The recovery of investments can be delayed if access to credit conditions remain restrictive for longer than anticipated.', 'The recovery of investments can be delayed if public administration commercial debt payments register delays.', 'The risk of generalized deflation is judged to be modest.', 'The fall in inflation could be more accentuated and persistent than expected if the weakness of demand reflects on expectations.', 'Business confidence is improving.', 'Industrial activity is regaining momentum after decreasing since the summer of 2011.', 'The underlying picture is varied depending on the type of business and its location.', 'Small businesses, especially in the south, remain on the margins of the process.', 'The decline in household consumption attenuated in the third quarter of 2013.', 'Italians are not spending on 2014-01-18.', 'Weak disposable income constrains consumption.', 'Difficult labor market conditions constrain consumption.', 'The Bank of Italy notes that the recovery of confidence, which began in early 2013, stopped in the fourth quarter.', 'Via Nazionale is changing its internal organization.', 'Via Nazionale will have 8 departments, services, and divisions under the board.']</t>
+          <t>["The recovery is expected to be timid, sluggish, and fraught with 'downside risks.'", 'Small businesses, especially those in the south, are left on the sidelines.', 'Consumption is languishing.', 'The number of unemployed people is increasing in 2015.', 'Inflation continues to decline.', "The Bank of Italy's economic bulletin, published on 2014-01-18, is more cautious than ever.", "The Bank of Italy's quarterly release coincides with two major pieces of news regarding GDP.", "Olli Rehn, the EU Commissioner, is confident in Italy's ability to recover.", 'Olli Rehn, the EU Commissioner, called for structural reforms and spending reviews.', "Olli Rehn, the EU Commissioner, suggested that Italy could obtain more 'flexibility' regarding budgetary rules.", 'A breakfast meeting occurred between Olli Rehn, the EU Commissioner, and Fabrizio Saccomanni, the Minister of Economy, on 2014-01-17.', 'The EU is revising the calculation of GDP.', 'The EU is moving investments in research and development from the expenditure category to the investment category.', 'The benefit of the GDP revision is estimated to be between 1% and 2%.', 'The GDP revision will have non-negligible effects on the deficit-to-GDP ratio.', "The Bank of Italy's macro projections place the year-end GDP growth at 0.7%.", "The Bank of Italy's macro projections estimate GDP growth will rise to 1% in 2015.", "The Bank of Italy's estimates are more contained than the government's estimates.", 'The government projected GDP growth of 1% for the year-end.', 'The unemployment rate is projected to remain at 12.8% in 2014.', 'The Bank of Italy warns that only the recovery of domestic demand can extend the recovery to the labor market.', 'Risks to growth remain oriented downwards.', 'The recovery of investments can be delayed if access to credit conditions remain restrictive for longer than anticipated.', 'The recovery of investments can be delayed if public administration commercial debt payments register delays.', 'The risk of generalized deflation is judged moderate.', 'The fall in inflation could be more accentuated and persistent than expected if the weakness of demand reflects on expectations.', 'Industrial activity is recovering after having decreased since the summer of 2011.', 'The underlying economic picture is varied depending on the type of business and its location.', 'Small businesses, especially in the south, remain on the margins of the process.', 'The decline in family consumption attenuated in the third quarter of 2013.', 'Consumption is constrained by the weakness of disposable income.', 'Consumption is constrained by the difficult conditions of the labor market.', 'The Bank of Italy noted that the recovery of confidence, which began in early 2013, stopped in the fourth quarter.', 'Via Nazionale is changing its internal organization.', "Via Nazionale's internal organization includes 8 departments, services, and divisions under the board."]</t>
         </is>
       </c>
     </row>
@@ -738,17 +738,17 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Last September 20, the CEO of Banco BPM, Giuseppe Castagna, expressed optimism regarding the resilience of the recovery phase. “We—referring to the moratoriums—have fallen from over 16 billion euros to 4.8 billion, which means that the clientele has resumed repaying loans. Nearly 75 percent of the clientele exposed for those 4.8 billion have good ratings, and we are confident. These are very encouraging figures.” However, despite Castagna’s optimism, concern for the stability of the system remains concrete. While it is true that credits under moratorium have fallen from 280 billion in March 2020 to 147 billion in December 2020, and then to 71 billion in September 2021, the expiration of the support measures is seen as the real great test for the Italian economy. Today, the economy sees GDP growing by over 6 percent annually, but it must face this sharp turn. The first half of 2022 seems destined to bring to light what has been held back until now. “This is a happy time for the Italian economy,” explains Ferruccio Ferrara, founder and president of Negentropy Capital Partners, who signed one of the earliest distressed credit acquisitions with PIMCO and Deutsche Bank back in 2011. After very difficult months, the rebound underway is bringing optimism, and this is a fantastic medicine for the economy. But the time will soon come when we will have to face the past and for businesses resume payments owed to banks and currently under moratorium. There are different levels of reactivity depending on the industrial sectors, but the underlying condition remains quite heavy. This is also because Italy entered the pandemic with a complicated financial situation and fractional growth compared to major European competitors—this cannot be forgotten. COVID extended the recovery times, and it is undeniable that over the last eighteen months, banking exposures have increased. Today, in Italy, the total amount of non-performing loans, or the combination of NPLs and UTPs—whose distinction is very subtle and often depends on the bank—stands at approximately 500 billion euros. This is a truly considerable figure, making Italy the first European market for this type of position, one of the first in the world. Of these 500 billion, about 180 billion are UTPs and about 120 billion are NPLs still within the banking perimeter. The remaining 200 billion have not disappeared. They have left the banking perimeter and therefore no longer represent a structural issue for the credit industry, which is also burdened by the needs imposed by calendar provisioning, but they are in specialized fund portfolios. From the perspective of the Italian economy, however, little changes... In 2021, the value of portfolios ceded by banks will be about 34 billion (1.5 billion only from MPS if the cession to UniCredit were to materialize), growing compared to 2020, as will UTPs, which will reach 11 billion. From here until the end of the year, NPLs worth 26 billion are ready to be ceded. Last month, Banca Ifis, in its usual September sector report, wrote: “In the two-year period 2022-2023, new distressed credit on households and businesses is expected to grow (about 70 billion euros over the two years), but without reaching the peak of 2013. The increase in the deterioration rate will be driven by the corporate component.” But the bank led by Frederick Geertman also highlighted the positive effect of government measures: “In 2021, the gross stock of distressed credits is expected to contract. This will reduce the NPE ratio below the 5 percent target required by the ECB. The incidence on employment is expected to increase starting in 2022 and will reach 5.9 percent in 2023,” precisely when the safety net provided by the executive will be behind us. In the distressed credit market, a significant role is played by public hands, both through the subsidiary Amco and through GACS, the public guarantees on the securitization of distressed assets, introduced by a decree in February 2016 and repeatedly extended. Based on the further 12-month extension granted by the European Union during 2021, Banca Ifis forecasts about 7 billion euros in new guaranteed operations, bringing the total transacted since 2016 to 94 billion euros. Seven are the services committed in GACS-assisted operations so far, with 80 percent of the value, or the gross book value (GBV), concentrated among the first four Italian operators: Dovalue, Prelios, Cerved, and Credito Fondiario. The operators “the attention of operators on the Italian market is very high,” emphasizes Ferrara, who, with Negentropy, manages portfolios worth about 3 billion euros of GBV—and this is demonstrated by the fact that today, when a credit institution puts up an asset for sale, up to 25-30 operators are invited to participate in the purchase. The increase in the number of operators has also led to an upward revision of prices: to make space among many competitors, some have bought in the past at very aggressive levels, and the increase in the average value of transactions has benefited banks' balance sheets. Now it remains to understand what 2022 will bring, but it is difficult to predict: I hope that the support measures for the business system are abandoned only gradually, as this would help the stability of sectors most exposed so far, such as manufacturing, fashion, tourism, and catering.” The system of loans and financing relies on real guarantees, in the vast majority of cases, real estate. In this case too, COVID left its mark: in 2021, 125,000 judicial auctions are estimated in Italy, a drop of 39 percent compared to pre-pandemic levels. The courts have suspended over 120,000 auctions, and there are operations for at least 13 billion euros blocked in the courts. These too await a restart. © Reproduction reserved. NPL refers to non-performing loans, or non-performing credits. UTP refers to unlikely to pay, meaning exposures for which the bank assesses it unlikely that the debtor will fully meet its contractual obligations. Past due are exposures or payments overdue for a period exceeding 90 days. It is the first stage of the crisis, which can evolve into UTP and then into NPL.</t>
+          <t>The optimism observed on September 20th, on these pages, saw the CEO of Banco BPM, Giuseppe Castagna, express confidence regarding the recovery phase. “We—said Castagna, referring to the moratoriums—have dropped from over 16 billion euros to 4.8 billion, which means that the clientele has resumed repaying loans. Nearly 75 percent of the clientele exposed for those 4.8 billion have good ratings, and we are confident. These are very comforting figures.” However, despite Castagna's optimism, concern for the system's stability remains concrete. While it is true that moratorium loans have fallen from 280 billion in March 2020 to 147 billion in December 2020, and then to 71 billion in September 2021, the expiration of support measures is seen as the real major test for the Italian economy, which today sees GDP growing by over 6 percent annually, but which must face this elbow curve. The first half of 2022 thus seems destined to bring to light what has been held back until now. “This is a happy moment for the Italian economy,” explains Ferruccio Ferrara, founder and president of Negentropy Capital Partners, who signed one of the very first distressed credit acquisitions with Pimco and Deutsche Bank back in 2011. After very heavy months, the rebound underway is bringing back optimism, and this is a fantastic medicine for the economy. But the time will soon come when we will have to account for the past and for businesses to resume payments owed to banks and currently under moratorium. There are diverse reactivities depending on the industrial sectors, but the underlying condition remains quite heavy. This is also because Italy entered the pandemic with a complicated financial situation and fractional growth compared to major European competitors, which must not be forgotten. COVID extended the recovery times, and it is undeniable that over the last eighteen months, banking exposures have increased. Today, in Italy, the total of non-performing loans, or the set of NPL and UTP, whose distinction is moreover very subtle and often depends on the bank, amounts to approximately 500 billion euros. This is a truly considerable figure that makes Italy the first European market for this type of position, one of the first in the world. Of these 500 billion, about 180 billion are UTP and about 120 billion are NPL still within the banking perimeter. The remaining 200 billion have not disappeared. They have left the banks' perimeter and therefore no longer represent a structural issue for the credit industry, also burdened by the needs imposed by calendar provisioning, but are in specialized funds' portfolios. From the perspective of the Italian economy, little changes, however... In 2021, the value of portfolios ceded by banks will be about 34 billion (1.5 billion only from MPS if the cession to Unicredit were to materialize), growing compared to 2020, as will UTP, which will reach 11 billion. By the end of the year, NPLs worth 26 billion are ready to be ceded. Last month, Banca Ifis, in its usual September report on the sector, wrote: “In the two-year period 2022-2023, new distressed credit on households and businesses residing is expected to grow (about 70 billion euros over the two years), without reaching the peak of 2013. The increase in the deterioration rate will be driven by the corporate component.” But the bank led by Frederick Geertman also highlighted the positive effect of government measures: “In 2021, the gross distressed credit stock is expected to contract. This will reduce the NPE ratio below the 5 percent target required by the BCE. The incidence on employment is expected to increase starting in 2022 and reach 5.9% in 2023,” when the protection network established by the executive will finally be left behind. In the distressed credit market, an important role is played by public hands, both through the controlled entity Amco and through GACS, the public guarantees on the securitization of distressed assets, introduced with a decree in February 2016 and repeatedly extended. Based on the further 12-month extension granted by the European Union during 2021, Banca Ifis forecasts about 7 billion euros in new guaranteed operations, bringing the total transacted since 2016 to 94 billion euros. Seven are the services committed in the GACS-assisted operations so far carried out, with 80 percent of the value, or the gross book value (GBV), concentrated among the first four Italian operators: Dovale, Prelios, Cerved, and Credito Fondiario. The operators “the attention of operators on the Italian market is very high,” emphasizes Ferrara, who, with Negentropy, controls portfolios worth about 3 billion euros of GBV—and this is demonstrated by the fact that today when a credit institution puts up an asset for sale, up to 25-30 operators are invited to participate in the purchase. The increase in the number of operators has also induced an upward revision of prices: to make space among many competitors, some have bought in the past at very aggressive levels, and the increase in the average value of transactions has benefited banks' balance sheets. Now it remains to understand how 2022 will be, but it is difficult to make a prediction: I hope that the support measures for the business system are abandoned only gradually, as this would help the stability of sectors most exposed until now, such as manufacturing, fashion, tourism, and catering.” The system of loans and financing is based on real guarantees, in the vast majority of cases, real estate. In this case too, COVID left its mark: in 2021, 125 thousand judicial auctions are estimated in Italy, a drop of 39 percent compared to before the pandemic. The courts have in fact suspended over 120 thousand auctions, and there are operations for at least 13 billion euros blocked in the courts, also awaiting recovery. © reserved reproduction NPL refers to non-performing loans, or non-performing credits, meaning loans that are not repaid to banks by businesses, thus finding themselves in a situation of insolvency. UTP refers to unlikely to pay, meaning exposures for which the bank assesses it unlikely that the debtor will fully meet its contractual obligations. Past due are exposures or payments overdue for a period exceeding 90 days. It is the first step of the crisis, which can evolve into UTP and then into NPL.</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>Observation date: 2021-10-18 00:00:00. Last September 20, the CEO of Banco BPM, Giuseppe Castagna, expressed optimism regarding the resilience of the recovery phase. “We—referring to the moratoriums—have fallen from over 16 billion euros to 4.8 billion, which means that the clientele has resumed repaying loans. Nearly 75 percent of the clientele exposed for those 4.8 billion have good ratings, and we are confident. These are very encouraging figures.” However, despite Castagna’s optimism, concern for the stability of the system remains concrete. While it is true that credits under moratorium have fallen from 280 billion in March 2020 to 147 billion in December 2020, and then to 71 billion in September 2021, the expiration of the support measures is seen as the real great test for the Italian economy. Today, the economy sees GDP growing by over 6 percent annually, but it must face this sharp turn. The first half of 2022 seems destined to bring to light what has been held back until now. “This is a happy time for the Italian economy,” explains Ferruccio Ferrara, founder and president of Negentropy Capital Partners, who signed one of the earliest distressed credit acquisitions with PIMCO and Deutsche Bank back in 2011. After very difficult months, the rebound underway is bringing optimism, and this is a fantastic medicine for the economy. But the time will soon come when we will have to face the past and for businesses resume payments owed to banks and currently under moratorium. There are different levels of reactivity depending on the industrial sectors, but the underlying condition remains quite heavy. This is also because Italy entered the pandemic with a complicated financial situation and fractional growth compared to major European competitors—this cannot be forgotten. COVID extended the recovery times, and it is undeniable that over the last eighteen months, banking exposures have increased. Today, in Italy, the total amount of non-performing loans, or the combination of NPLs and UTPs—whose distinction is very subtle and often depends on the bank—stands at approximately 500 billion euros. This is a truly considerable figure, making Italy the first European market for this type of position, one of the first in the world. Of these 500 billion, about 180 billion are UTPs and about 120 billion are NPLs still within the banking perimeter. The remaining 200 billion have not disappeared. They have left the banking perimeter and therefore no longer represent a structural issue for the credit industry, which is also burdened by the needs imposed by calendar provisioning, but they are in specialized fund portfolios. From the perspective of the Italian economy, however, little changes... In 2021, the value of portfolios ceded by banks will be about 34 billion (1.5 billion only from MPS if the cession to UniCredit were to materialize), growing compared to 2020, as will UTPs, which will reach 11 billion. From here until the end of the year, NPLs worth 26 billion are ready to be ceded. Last month, Banca Ifis, in its usual September sector report, wrote: “In the two-year period 2022-2023, new distressed credit on households and businesses is expected to grow (about 70 billion euros over the two years), but without reaching the peak of 2013. The increase in the deterioration rate will be driven by the corporate component.” But the bank led by Frederick Geertman also highlighted the positive effect of government measures: “In 2021, the gross stock of distressed credits is expected to contract. This will reduce the NPE ratio below the 5 percent target required by the ECB. The incidence on employment is expected to increase starting in 2022 and will reach 5.9 percent in 2023,” precisely when the safety net provided by the executive will be behind us. In the distressed credit market, a significant role is played by public hands, both through the subsidiary Amco and through GACS, the public guarantees on the securitization of distressed assets, introduced by a decree in February 2016 and repeatedly extended. Based on the further 12-month extension granted by the European Union during 2021, Banca Ifis forecasts about 7 billion euros in new guaranteed operations, bringing the total transacted since 2016 to 94 billion euros. Seven are the services committed in GACS-assisted operations so far, with 80 percent of the value, or the gross book value (GBV), concentrated among the first four Italian operators: Dovalue, Prelios, Cerved, and Credito Fondiario. The operators “the attention of operators on the Italian market is very high,” emphasizes Ferrara, who, with Negentropy, manages portfolios worth about 3 billion euros of GBV—and this is demonstrated by the fact that today, when a credit institution puts up an asset for sale, up to 25-30 operators are invited to participate in the purchase. The increase in the number of operators has also led to an upward revision of prices: to make space among many competitors, some have bought in the past at very aggressive levels, and the increase in the average value of transactions has benefited banks' balance sheets. Now it remains to understand what 2022 will bring, but it is difficult to predict: I hope that the support measures for the business system are abandoned only gradually, as this would help the stability of sectors most exposed so far, such as manufacturing, fashion, tourism, and catering.” The system of loans and financing relies on real guarantees, in the vast majority of cases, real estate. In this case too, COVID left its mark: in 2021, 125,000 judicial auctions are estimated in Italy, a drop of 39 percent compared to pre-pandemic levels. The courts have suspended over 120,000 auctions, and there are operations for at least 13 billion euros blocked in the courts. These too await a restart. © Reproduction reserved. NPL refers to non-performing loans, or non-performing credits. UTP refers to unlikely to pay, meaning exposures for which the bank assesses it unlikely that the debtor will fully meet its contractual obligations. Past due are exposures or payments overdue for a period exceeding 90 days. It is the first stage of the crisis, which can evolve into UTP and then into NPL.</t>
+          <t>Observation date: 2021-10-18 00:00:00. The optimism observed on September 20th, on these pages, saw the CEO of Banco BPM, Giuseppe Castagna, express confidence regarding the recovery phase. “We—said Castagna, referring to the moratoriums—have dropped from over 16 billion euros to 4.8 billion, which means that the clientele has resumed repaying loans. Nearly 75 percent of the clientele exposed for those 4.8 billion have good ratings, and we are confident. These are very comforting figures.” However, despite Castagna's optimism, concern for the system's stability remains concrete. While it is true that moratorium loans have fallen from 280 billion in March 2020 to 147 billion in December 2020, and then to 71 billion in September 2021, the expiration of support measures is seen as the real major test for the Italian economy, which today sees GDP growing by over 6 percent annually, but which must face this elbow curve. The first half of 2022 thus seems destined to bring to light what has been held back until now. “This is a happy moment for the Italian economy,” explains Ferruccio Ferrara, founder and president of Negentropy Capital Partners, who signed one of the very first distressed credit acquisitions with Pimco and Deutsche Bank back in 2011. After very heavy months, the rebound underway is bringing back optimism, and this is a fantastic medicine for the economy. But the time will soon come when we will have to account for the past and for businesses to resume payments owed to banks and currently under moratorium. There are diverse reactivities depending on the industrial sectors, but the underlying condition remains quite heavy. This is also because Italy entered the pandemic with a complicated financial situation and fractional growth compared to major European competitors, which must not be forgotten. COVID extended the recovery times, and it is undeniable that over the last eighteen months, banking exposures have increased. Today, in Italy, the total of non-performing loans, or the set of NPL and UTP, whose distinction is moreover very subtle and often depends on the bank, amounts to approximately 500 billion euros. This is a truly considerable figure that makes Italy the first European market for this type of position, one of the first in the world. Of these 500 billion, about 180 billion are UTP and about 120 billion are NPL still within the banking perimeter. The remaining 200 billion have not disappeared. They have left the banks' perimeter and therefore no longer represent a structural issue for the credit industry, also burdened by the needs imposed by calendar provisioning, but are in specialized funds' portfolios. From the perspective of the Italian economy, little changes, however... In 2021, the value of portfolios ceded by banks will be about 34 billion (1.5 billion only from MPS if the cession to Unicredit were to materialize), growing compared to 2020, as will UTP, which will reach 11 billion. By the end of the year, NPLs worth 26 billion are ready to be ceded. Last month, Banca Ifis, in its usual September report on the sector, wrote: “In the two-year period 2022-2023, new distressed credit on households and businesses residing is expected to grow (about 70 billion euros over the two years), without reaching the peak of 2013. The increase in the deterioration rate will be driven by the corporate component.” But the bank led by Frederick Geertman also highlighted the positive effect of government measures: “In 2021, the gross distressed credit stock is expected to contract. This will reduce the NPE ratio below the 5 percent target required by the BCE. The incidence on employment is expected to increase starting in 2022 and reach 5.9% in 2023,” when the protection network established by the executive will finally be left behind. In the distressed credit market, an important role is played by public hands, both through the controlled entity Amco and through GACS, the public guarantees on the securitization of distressed assets, introduced with a decree in February 2016 and repeatedly extended. Based on the further 12-month extension granted by the European Union during 2021, Banca Ifis forecasts about 7 billion euros in new guaranteed operations, bringing the total transacted since 2016 to 94 billion euros. Seven are the services committed in the GACS-assisted operations so far carried out, with 80 percent of the value, or the gross book value (GBV), concentrated among the first four Italian operators: Dovale, Prelios, Cerved, and Credito Fondiario. The operators “the attention of operators on the Italian market is very high,” emphasizes Ferrara, who, with Negentropy, controls portfolios worth about 3 billion euros of GBV—and this is demonstrated by the fact that today when a credit institution puts up an asset for sale, up to 25-30 operators are invited to participate in the purchase. The increase in the number of operators has also induced an upward revision of prices: to make space among many competitors, some have bought in the past at very aggressive levels, and the increase in the average value of transactions has benefited banks' balance sheets. Now it remains to understand how 2022 will be, but it is difficult to make a prediction: I hope that the support measures for the business system are abandoned only gradually, as this would help the stability of sectors most exposed until now, such as manufacturing, fashion, tourism, and catering.” The system of loans and financing is based on real guarantees, in the vast majority of cases, real estate. In this case too, COVID left its mark: in 2021, 125 thousand judicial auctions are estimated in Italy, a drop of 39 percent compared to before the pandemic. The courts have in fact suspended over 120 thousand auctions, and there are operations for at least 13 billion euros blocked in the courts, also awaiting recovery. © reserved reproduction NPL refers to non-performing loans, or non-performing credits, meaning loans that are not repaid to banks by businesses, thus finding themselves in a situation of insolvency. UTP refers to unlikely to pay, meaning exposures for which the bank assesses it unlikely that the debtor will fully meet its contractual obligations. Past due are exposures or payments overdue for a period exceeding 90 days. It is the first step of the crisis, which can evolve into UTP and then into NPL.</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>['On September 20, Giuseppe Castagna, CEO of Banco BPM, expressed optimism regarding the resilience of the recovery phase.', 'The moratoriums fell from over 16 billion euros to 4.8 billion euros.', 'The reduction in moratoriums means that the clientele resumed repaying loans.', 'Nearly 75 percent of the clientele exposed for the 4.8 billion euros have good ratings.', 'Credits under moratorium fell from 280 billion euros in March 2020 to 147 billion euros in December 2020.', 'Credits under moratorium fell further to 71 billion euros in September 2021.', 'The expiration of the support measures is seen as the real great test for the Italian economy.', 'The economy sees GDP growing by over 6 percent annually.', 'The Italian economy must face a sharp turn.', 'The rebound underway is bringing optimism to the economy.', 'The time will soon come when businesses will have to resume payments owed to banks and currently under moratorium.', 'The underlying condition for payments remains quite heavy.', 'Italy entered the pandemic with a complicated financial situation.', 'Italy had fractional growth compared to major European competitors.', 'COVID extended the recovery times.', 'Over the last eighteen months, banking exposures have increased.', '2021-10-18, the total amount of non-performing loans (NPLs) and unlikely to pay (UTPs) in Italy stands at approximately 500 billion euros.', 'The 500 billion euros figure makes Italy the first European market for this type of position.', 'Of the 500 billion euros, about 180 billion euros are UTPs.', 'Of the 500 billion euros, about 120 billion euros are NPLs still within the banking perimeter.', 'The remaining 200 billion euros have left the banking perimeter.', 'The 200 billion euros are in specialized fund portfolios.', 'In 2021, the value of portfolios ceded by banks will be about 34 billion euros.', 'The cession from MPS to UniCredit is estimated at 1.5 billion euros.', 'UTPs are expected to reach 11 billion euros.', 'NPLs worth 26 billion euros are ready to be ceded from here until the end of the year.', 'Banca Ifis wrote a sector report in September.', 'Banca Ifis expects new distressed credit on households and businesses to grow by about 70 billion euros over the two years (2022-2023).', 'The expected growth of distressed credit will not reach the peak of 2013.', 'The increase in the deterioration rate will be driven by the corporate component.', 'Banca Ifis highlighted the positive effect of government measures.', 'In 2021, the gross stock of distressed credits is expected to contract according to Banca Ifis.', 'The contraction of distressed credits will reduce the Non-Performing Exposure (NPE) ratio below the 5 percent target required by the ECB.', 'The incidence on employment is expected to increase starting in 2022.', 'Public hands play a significant role in the distressed credit market.', 'Public guarantees on the securitization of distressed assets (GACS) were introduced by a decree in February 2016.', 'Banca Ifis forecasts about 7 billion euros in new guaranteed operations based on the further 12-month extension granted by the European Union during 2021.', 'The total transacted value since 2016 is forecast to reach 94 billion euros.', 'Seven services were committed in GACS-assisted operations so far.', '80 percent of the value, or the gross book value (GBV), is concentrated among the first four Italian operators: Dovalue, Prelios, Cerved, and Credito Fondiario.', "The operators' attention on the Italian market is very high.", 'When a credit institution puts up an asset for sale, up to 25-30 operators are invited to participate in the purchase.', 'The increase in the number of operators has led to an upward revision of prices.', "The increase in the average value of transactions has benefited banks' balance sheets.", 'The author hopes that the support measures for the business system are abandoned only gradually.', 'Gradual abandonment of support measures would help the stability of sectors such as manufacturing, fashion, tourism, and catering.', 'The system of loans and financing relies on real guarantees, in the vast majority of cases, real estate.', 'In 2021, 125,000 judicial auctions are estimated in Italy.', 'The 125,000 judicial auctions represent a drop of 39 percent compared to pre-pandemic levels.', 'Over 120,000 auctions have been suspended by the courts.', 'Operations for at least 13 billion euros are blocked in the courts.']</t>
+          <t>['Giuseppe Castagna, CEO of Banco BPM, expressed confidence regarding the recovery phase on September 20th.', 'Giuseppe Castagna stated that moratoriums dropped from over 16 billion euros to 4.8 billion euros.', 'Giuseppe Castagna stated that the clientele resumed repaying loans due to the drop in moratoriums.', 'Nearly 75 percent of the clientele exposed for 4.8 billion euros have good ratings.', 'Moratorium loans fell from 280 billion euros in March 2020 to 147 billion euros in December 2020.', 'Moratorium loans fell from 147 billion euros in December 2020 to 71 billion euros in September 2021.', "On 2021-10-18, the Italian economy's GDP sees growth of over 6 percent annually.", 'Banking exposures increased over the last eighteen months.', 'On 2021-10-18, the total of non-performing loans (NPL) and unlikely to pay (UTP) in Italy amounts to approximately 500 billion euros.', 'Of the 500 billion euros, about 180 billion euros are UTP.', 'Of the 500 billion euros, about 120 billion euros are NPL within the banking perimeter.', "The remaining 200 billion euros are in specialized funds' portfolios.", 'In 2021, the value of portfolios ceded by banks will be about 34 billion euros.', 'The value of portfolios ceded by banks will grow compared to 2020.', 'UTP will reach 11 billion euros by the end of 2021.', 'By the end of 2021, NPLs worth 26 billion euros are ready to be ceded.', 'Banca Ifis wrote that new distressed credit on households and businesses residing is expected to grow by about 70 billion euros over the two years 2022-2023.', 'Banca Ifis expects the gross distressed credit stock to contract in 2021.', 'The contraction of the gross distressed credit stock will reduce the NPE ratio below the 5 percent target required by the BCE.', 'The incidence on employment is expected to increase starting in 2022 and reach 5.9% in 2023.', 'GACS is public guarantees on the securitization of distressed assets, introduced with a decree in February 2016.', 'Banca Ifis forecasts about 7 billion euros in new guaranteed operations.', 'The total transacted amount since 2016 is expected to reach 94 billion euros.', 'Seven services have been committed in GACS-assisted operations so far.', '80 percent of the gross book value (GBV) is concentrated among the first four Italian operators: Dovale, Prelios, Cerved, and Credito Fondiario.', 'Negentropy controls portfolios worth about 3 billion euros of GBV.']</t>
         </is>
       </c>
     </row>
@@ -802,17 +802,17 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>I am not addressing the merits of the provision itself, but rather the methods of its disbursement. A letter is required: 1 sheet (plus envelope). An application is required: 4 sheets. Instructions: 2 sheets. Photocopies to attach to the application: 2 sheets (or 4 if a power of attorney is needed). In the best-case scenario, each application will require a minimum of 9 sheets (plus envelope), which, multiplied by the estimated population of 1,300,000, amounts to 11,700,000 sheets (eleven million seven hundred thousand sheets). To give an idea, this equals 23,400 reams of 500-sheet paper. I forgot the envelopes: 1,300,000. I wonder if the Ministry of Simplification was not established? The lost tax deductions on structural renovations, which Claudia Ceroni in Rome was misled by an increase in VAT on a non-essential good (Sky), are causing us to overlook a much graver problem than the new decree passed last Friday. I am 30 years old, a structural engineer. Given the incentives we believed to be certain, I convinced my parents to renovate their home by improving the roof insulation and installing sanitary water panels, a condensing boiler, and thermostatic valves, for a total cost of about €10,000. Together with my boyfriend, we spent about €50,000 on supplementary roof and window insulation that meets energy efficiency requirements for our new home, spending an additional €50,000, with the conviction that we could access the tax deduction. Now, this deduction no longer exists, or at least it is not certain, or it will be reduced from the current 55% to 35%. I wish our Minister Tremonti and the Prime Minister's staff would answer my two simple questions: who will reimburse us for this missed refund that was considered certain at the time of the intervention? I believe we are not far from a scam, if by that what De Mauro cited: 'a crime committed by someone who obtains illicit profit to the detriment of others, having misled them with artifice and trickery.' It is enough to replace 'artifice and trickery' with 'laws and decrees,' which makes the act even more serious. The 4% mortgage rate set by the government in the maneuver is expected to ensure that, by 2009, the interest rate on variable-rate mortgages will not exceed 4%. Heavens! Not even an extreme left government would have thought of that. Tito Boeri, in the newspaper on sale yesterday, asks (rhetorically, I presume) why such a measure is not also provided for fixed-rate mortgages. Simply because with the next BCE rate cut to 2.75%, or less, the Euribor will initially be just over 3%, plus an average spread of 1%, and thus the 4% will be the rate that banks will still have to apply to variable-rate mortgages. The benefit for families is practically zero. If we apply the same principle to fixed-rate mortgages, stipulated with interest rates well above 4%, we run the risk of actually helping the families! If we then consider that during 2009, a variable rate of 3.5% could even be reached. This 4% rate would be another way to help those who truly need it: the banks. The news about the mafia and the choices of TG1, Pino Caserta, editor of TG1, dear director, on page 19 of yesterday's Repubblica, headlines: 'for TG1, the most important yo-yo in the fight against crime,' because TG1 failed to report, in Saturday's 8 PM edition, the review on the fight against the mafia organized by 'Politicamente Scorretto' in Casalecchio di Reno (Bologna). The meeting was certainly relevant, but, upon closer inspection, even your newspaper's national edition decided not to report on the mafia conference. Repubblica limited itself to reporting the protest of Rita Borsellino. What the editor of TG1 omits to say is that the mafia conference took place a few hundred meters from the yo-yo championship: this is the reason for the controversy raised by Borsellino.</t>
+          <t>I am not addressing the merits of the provision, but rather the methods of its disbursement. A letter is required: 1 sheet (plus envelope). An application is required: 4 sheets. Instructions: 2 sheets. Photocopies to attach to the application: 2 sheets (or 4 if a power of attorney is needed). In the best-case scenario, each application will require a minimum of 9 sheets (plus envelope), which, multiplied by the estimated population of 1.3 million, results in 11.7 million sheets (eleven million seven hundred thousand sheets), which, to give an idea, equals 23,400 reams of 500-sheet paper. I forgot the envelopes: 1.3 million. I wonder if the Ministry of Simplification has not been established? The lost deductions on building renovations, concerning Claudio Ceroni in Rome, are being overshadowed by an increase in VAT on a non-essential good (Sky). A much graver problem is being overlooked than the new decree passed last Friday. I am 30 years old, a structural engineer. Given the incentives that we believed to be certain, I convinced my parents to renovate their home by improving the roof insulation and installing sanitary panels for sanitary water, a condensing boiler, and thermostatic valves, for a total of about 10,000 euros. Together with my boyfriend, we spent about 50,000 euros on supplementary roof insulation and windows that meet energy efficiency requirements, for our new house, spending an additional 50,000 euros, with the conviction that we could access the deduction. Now that this deduction no longer exists, or at least is not certain, or will be reduced from the current 55% to 35%. I would like our Minister Tremonti and the Prime Minister's staff to answer these two simple questions: who will reimburse us for this lost reimbursement, which was considered certain at the time of the intervention? I believe we are not far from a scam, if by that one means what De Mauro cited: 'a crime committed by those who obtain illicit profit at the expense of others, having misled them with artifice and trickery.' Simply replacing 'artifice and trickery' with 'laws and decrees' makes the act even more serious. The 4% rate on mortgages set by the government in the fiscal package is expected that, by 2009, the interest rate on variable-rate mortgages will not exceed 4%. Heavens! Even a far-left government would not have thought of that. Tito Boeri, in the newspaper on sale yesterday, asks (rhetorically, I presume) why such a measure is not also provided for fixed-rate mortgages. Simply because with the next ECB rate cut to 2.75%, if not less, the Euribor will initially be just over 3%, plus an average spread of 1%, and thus 4% will be the rate that banks will still have to apply to variable-rate mortgages. Virtually zero advantage for families. If we apply the same principle to fixed-rate mortgages, stipulated with interest rates well above 4%, we run the risk of actually helping the families! If we then consider that during 2009, a variable rate of 3.5% could also be reached. This 4% rate would be another way to help those who truly need it: the banks. The news about the mafia and the choices of TG1 (Pino Caserta, TG1 editorial secretary, to the kind director, on page 19 of yesterday's Repubblica) titles: 'For TG1, the most important yo-yo in the fight against crime,' because TG1 did not report, in Saturday's 8 PM edition, the review on the fight against the mafia organized by 'Politicamente Scorretto' in Casalecchio di Reno (Bologna). The meeting was certainly relevant, but, clearly, even the national edition of your newspaper decided not to report on the mafia conference. Repubblica limited itself to reporting the protest of Rita Borsellino. What the TG1 editorial secretary omits to say is that the mafia conference took place a few hundred meters from the yo-yo championship: this is the reason for the controversy raised by Borsellino. 2lette_13563977rb1</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>Observation date: 2008-12-02 00:00:00. I am not addressing the merits of the provision itself, but rather the methods of its disbursement. A letter is required: 1 sheet (plus envelope). An application is required: 4 sheets. Instructions: 2 sheets. Photocopies to attach to the application: 2 sheets (or 4 if a power of attorney is needed). In the best-case scenario, each application will require a minimum of 9 sheets (plus envelope), which, multiplied by the estimated population of 1,300,000, amounts to 11,700,000 sheets (eleven million seven hundred thousand sheets). To give an idea, this equals 23,400 reams of 500-sheet paper. I forgot the envelopes: 1,300,000. I wonder if the Ministry of Simplification was not established? The lost tax deductions on structural renovations, which Claudia Ceroni in Rome was misled by an increase in VAT on a non-essential good (Sky), are causing us to overlook a much graver problem than the new decree passed last Friday. I am 30 years old, a structural engineer. Given the incentives we believed to be certain, I convinced my parents to renovate their home by improving the roof insulation and installing sanitary water panels, a condensing boiler, and thermostatic valves, for a total cost of about €10,000. Together with my boyfriend, we spent about €50,000 on supplementary roof and window insulation that meets energy efficiency requirements for our new home, spending an additional €50,000, with the conviction that we could access the tax deduction. Now, this deduction no longer exists, or at least it is not certain, or it will be reduced from the current 55% to 35%. I wish our Minister Tremonti and the Prime Minister's staff would answer my two simple questions: who will reimburse us for this missed refund that was considered certain at the time of the intervention? I believe we are not far from a scam, if by that what De Mauro cited: 'a crime committed by someone who obtains illicit profit to the detriment of others, having misled them with artifice and trickery.' It is enough to replace 'artifice and trickery' with 'laws and decrees,' which makes the act even more serious. The 4% mortgage rate set by the government in the maneuver is expected to ensure that, by 2009, the interest rate on variable-rate mortgages will not exceed 4%. Heavens! Not even an extreme left government would have thought of that. Tito Boeri, in the newspaper on sale yesterday, asks (rhetorically, I presume) why such a measure is not also provided for fixed-rate mortgages. Simply because with the next BCE rate cut to 2.75%, or less, the Euribor will initially be just over 3%, plus an average spread of 1%, and thus the 4% will be the rate that banks will still have to apply to variable-rate mortgages. The benefit for families is practically zero. If we apply the same principle to fixed-rate mortgages, stipulated with interest rates well above 4%, we run the risk of actually helping the families! If we then consider that during 2009, a variable rate of 3.5% could even be reached. This 4% rate would be another way to help those who truly need it: the banks. The news about the mafia and the choices of TG1, Pino Caserta, editor of TG1, dear director, on page 19 of yesterday's Repubblica, headlines: 'for TG1, the most important yo-yo in the fight against crime,' because TG1 failed to report, in Saturday's 8 PM edition, the review on the fight against the mafia organized by 'Politicamente Scorretto' in Casalecchio di Reno (Bologna). The meeting was certainly relevant, but, upon closer inspection, even your newspaper's national edition decided not to report on the mafia conference. Repubblica limited itself to reporting the protest of Rita Borsellino. What the editor of TG1 omits to say is that the mafia conference took place a few hundred meters from the yo-yo championship: this is the reason for the controversy raised by Borsellino.</t>
+          <t>Observation date: 2008-12-02 00:00:00. I am not addressing the merits of the provision, but rather the methods of its disbursement. A letter is required: 1 sheet (plus envelope). An application is required: 4 sheets. Instructions: 2 sheets. Photocopies to attach to the application: 2 sheets (or 4 if a power of attorney is needed). In the best-case scenario, each application will require a minimum of 9 sheets (plus envelope), which, multiplied by the estimated population of 1.3 million, results in 11.7 million sheets (eleven million seven hundred thousand sheets), which, to give an idea, equals 23,400 reams of 500-sheet paper. I forgot the envelopes: 1.3 million. I wonder if the Ministry of Simplification has not been established? The lost deductions on building renovations, concerning Claudio Ceroni in Rome, are being overshadowed by an increase in VAT on a non-essential good (Sky). A much graver problem is being overlooked than the new decree passed last Friday. I am 30 years old, a structural engineer. Given the incentives that we believed to be certain, I convinced my parents to renovate their home by improving the roof insulation and installing sanitary panels for sanitary water, a condensing boiler, and thermostatic valves, for a total of about 10,000 euros. Together with my boyfriend, we spent about 50,000 euros on supplementary roof insulation and windows that meet energy efficiency requirements, for our new house, spending an additional 50,000 euros, with the conviction that we could access the deduction. Now that this deduction no longer exists, or at least is not certain, or will be reduced from the current 55% to 35%. I would like our Minister Tremonti and the Prime Minister's staff to answer these two simple questions: who will reimburse us for this lost reimbursement, which was considered certain at the time of the intervention? I believe we are not far from a scam, if by that one means what De Mauro cited: 'a crime committed by those who obtain illicit profit at the expense of others, having misled them with artifice and trickery.' Simply replacing 'artifice and trickery' with 'laws and decrees' makes the act even more serious. The 4% rate on mortgages set by the government in the fiscal package is expected that, by 2009, the interest rate on variable-rate mortgages will not exceed 4%. Heavens! Even a far-left government would not have thought of that. Tito Boeri, in the newspaper on sale yesterday, asks (rhetorically, I presume) why such a measure is not also provided for fixed-rate mortgages. Simply because with the next ECB rate cut to 2.75%, if not less, the Euribor will initially be just over 3%, plus an average spread of 1%, and thus 4% will be the rate that banks will still have to apply to variable-rate mortgages. Virtually zero advantage for families. If we apply the same principle to fixed-rate mortgages, stipulated with interest rates well above 4%, we run the risk of actually helping the families! If we then consider that during 2009, a variable rate of 3.5% could also be reached. This 4% rate would be another way to help those who truly need it: the banks. The news about the mafia and the choices of TG1 (Pino Caserta, TG1 editorial secretary, to the kind director, on page 19 of yesterday's Repubblica) titles: 'For TG1, the most important yo-yo in the fight against crime,' because TG1 did not report, in Saturday's 8 PM edition, the review on the fight against the mafia organized by 'Politicamente Scorretto' in Casalecchio di Reno (Bologna). The meeting was certainly relevant, but, clearly, even the national edition of your newspaper decided not to report on the mafia conference. Repubblica limited itself to reporting the protest of Rita Borsellino. What the TG1 editorial secretary omits to say is that the mafia conference took place a few hundred meters from the yo-yo championship: this is the reason for the controversy raised by Borsellino. 2lette_13563977rb1</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>['A letter requires 1 sheet plus an envelope.', 'An application requires 4 sheets.', 'Instructions require 2 sheets.', 'Photocopies require 2 sheets, or 4 sheets if a power of attorney is needed.', 'Each application requires a minimum of 9 sheets plus an envelope.', 'The estimated population is 1,300,000.', 'The total estimated sheets required is 11,700,000 sheets.', 'The total estimated reams required is 23,400 reams of 500-sheet paper.', 'Claudia Ceroni in Rome was misled by an increase in VAT on a non-essential good (Sky).', 'Lost tax deductions on structural renovations are causing the oversight of a graver problem than the new decree passed on 2008-11-25.', 'The structural engineer convinced the parents to renovate their home.', "The parents' renovation included improving roof insulation, installing sanitary water panels, a condensing boiler, and thermostatic valves.", "The total cost of the parents' renovation was about €10,000.", 'The structural engineer and the boyfriend spent an additional €50,000 on supplementary roof and window insulation.', 'The tax deduction for structural renovations is no longer certain, or it will be reduced from 55% to 35%.', "The structural engineer asked Minister Tremonti and the Prime Minister's staff who will reimburse the missed refund.", "De Mauro defined a scam as 'a crime committed by someone who obtains illicit profit to the detriment of others, having misled them with artifice and trickery.'", 'The government set a 4% mortgage rate in the maneuver.', 'The interest rate on variable-rate mortgages is expected not to exceed 4% by 2009.', 'The structural engineer stated that the benefit for families regarding the 4% mortgage rate is practically zero.', 'The structural engineer suggested applying the same principle to fixed-rate mortgages could help families.', 'A variable rate of 3.5% could be reached during 2009.', 'The news about the mafia and the choices of TG1 was published on page 19 of *Repubblica* on 2008-12-01.', "The headline on page 19 of *Repubblica* on 2008-12-01 was 'for TG1, the most important yo-yo in the fight against crime.'", "TG1 failed to report the review on the fight against the mafia organized by 'Politicamente Scorretto' in Casalecchio di Reno (Bologna) in the 8 PM edition on 2008-12-01.", 'The national edition of *Repubblica* decided not to report on the mafia conference.', '*Repubblica* limited its reporting to the protest of Rita Borsellino.', 'The editor of TG1 omitted that the mafia conference took place a few hundred meters from the yo-yo championship.', 'The proximity of the mafia conference to the yo-yo championship is the reason for the controversy raised by Borsellino.']</t>
+          <t>['A letter requires 1 sheet plus an envelope.', 'An application requires 4 sheets.', 'Instructions require 2 sheets.', 'Photocopies attached to the application require 2 sheets (or 4 sheets if a power of attorney is needed).', 'Each application requires a minimum of 9 sheets plus an envelope.', 'The estimated population is 1.3 million.', 'The total required sheets for the estimated population is 11.7 million sheets.', '11.7 million sheets equals 23,400 reams of 500-sheet paper.', 'The required envelopes total 1.3 million.', 'Lost deductions on building renovations concern Claudio Ceroni in Rome.', 'An increase in VAT on a non-essential good (Sky) is overshadowing the lost deductions.', "The renovation of the parents' home cost about 10,000 euros.", 'The renovation included improving roof insulation, installing sanitary panels for sanitary water, a condensing boiler, and thermostatic valves.', 'The speaker and boyfriend spent about 50,000 euros on supplementary roof insulation and windows for their new house.', 'The speaker and boyfriend spent an additional 50,000 euros on the new house.', 'The deduction for renovations is no longer certain.', 'The deduction may be reduced from 55% to 35%.', 'The government set a 4% rate on mortgages in the fiscal package.', 'The 4% rate is expected to keep the interest rate on variable-rate mortgages below 4% by 2009.', 'Tito Boeri asked in the newspaper on sale on 2008-12-01 why the measure was not provided for fixed-rate mortgages.', 'The next ECB rate cut is expected to be 2.75%.', 'The Euribor will initially be just over 3% plus an average spread of 1%.', 'A variable rate of 3.5% could be reached during 2009.', 'Pino Caserta, TG1 editorial secretary, wrote to the kind director on page 19 of the newspaper on sale on 2008-12-01.', "Pino Caserta titled the article 'For TG1, the most important yo-yo in the fight against crime.'", "TG1 did not report the review on the fight against the mafia organized by 'Politicamente Scorretto' in Casalecchio di Reno (Bologna) in the 2008-11-29's 8 PM edition.", 'The national edition of the newspaper decided not to report on the mafia conference.', 'Repubblica limited itself to reporting the protest of Rita Borsellino.', 'The mafia conference took place a few hundred meters from the yo-yo championship.']</t>
         </is>
       </c>
     </row>
@@ -866,17 +866,17 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>According to a study by the National Consumers Union, which ranked cities based on the largest annual increases, the report analyzed Istat data from last January. Consequently, Perugia and Terni finished in the top six cities with the highest costs, nearly reaching the podium. Specifically, in Perugia, the cost of electricity and gas saw an 85.8% growth: while Terni recorded 85.4%. This minimal delta between the two city centers indicates that the cost of living is, in fact, uniform throughout the region. Considering the average expenditure of an Italian family, the cost of living in Perugia amounts to 1,157 euros on an annual basis; while for a family in Terni, it is 1,152 euros. A derby that essentially ends in a draw (there is only a 5 euro difference), and winning it neither leads to celebrations nor parades with scarves and flags. Nationally, however, the survey compares the variation in electricity and gas prices over the last three years, contrasting the free market with the regulated market. From June 2021, before the increases that began in July, electricity in the free market in Italy rose by 248.3% compared to 108.4% in the regulated market—more than double (+129%). Furthermore, considering the first available gas data from Istat, December 2021, the free market since then increased by 141.1% compared to a 7.4% decrease in the regulated market. In three years, from January 2020 to January 2023, free market electricity jumped by 262.8%, compared to 115.8% in the regulated market. For electricity, gas, and other fuels—a category that includes gas, electricity (free and regulated markets), heating oil, and solid fuels—if the increase in January was 67.3% compared to one year prior, the average family cost was 907.50 euros on an annual basis, with some cities approaching 90%. The comparison does little to console the fact that Umbria is at the foot of the podium, especially because the distance to the city at the top is reduced. In Alessandria, expenses for electricity, gas, and heating oil soared by 88.6% by January 2022. Piedmont is well-stocked, with Vercelli recording an increase of 87.1% and Biella with 86.1%. On the other side of the ranking, the least affected city is Potenza, with an increase of 35.2%. In second place is Aosta with an increase of 50.8%. At the bottom of the 'virtuous cities' podium is Olbia-Tempio with an increase of 51%. Following are Naples (+51.4%), Gorizia (+51.7%), Benevento (+53.1%), Caserta (+53.5%), then Avellino (+53.7%) and Trieste (+54.6%). Closing the top ten are Pordenone and Udine, tied at +54.7%. Another ranking, a study on price increases, comes from the CGIAR study office, which indicates the impact of family purchasing power relative to inflation, which is running wild. Over the two years 2022-2023, the loss of purchasing power in Umbria due to inflation could amount to nearly six million euros per family. The estimate is based on data from the Bank of Italy, Istat, and the European Commission. Against bank deposits, which amounted to 14.5 billion euros at the end of 2021, the estimated loss of purchasing power in Umbria in 2022 was 1.2 billion euros, while in 2023, thanks to a slowdown in inflation, it was 885 million euros, totaling 2.1 billion euros. At the provincial level, the CGIAR data states that for Perugia, the loss of purchasing power could amount to over 1.6 billion euros (nearly 5,746 per family), while in Terni, it is 536 million euros (5,251 per family). Here, the gap is clearer compared to the increases in electricity and gas bills.</t>
+          <t>A study by the National Consumers Union placed a ranking of cities based on the largest annual increases, elaborating data from ISTAT regarding last January. Consequently, Perugia and Terni finished in the top six of the most expensive cities, nearly reaching the podium. Specifically, in Perugia, the cost of electricity and gas saw an 85.8% growth: while Terni stopped at 85.4%. A minimal delta between the two city capitals indicates that the cost of living is, in fact, uniform throughout the region. Considering how much an average Italian family spends, the cost of living in Perugia is 1,157 euros on an annual basis; while for a family in Terni, it is 1,152 euros. A derby that ends essentially in a draw (there is only a 5 euro difference), and winning it brings neither carousels nor parties with scarves and flags. Nationally, however, the survey compares the variation in electricity and gas prices over the last 3 years, comparing the free market with the regulated market. From June 2021, before the increases that started in July, electricity in the free market in Italy rose by 248.3% versus 108.4% in the regulated market, more than double (+129%). Furthermore, considering the first useful gas data detected by ISTAT, December 2021, the free market since then increased by 141.1% versus a 7.4% drop in the regulated market. In 3 years, from January 2020 to January 2023, free electricity jumped by 262.8%, compared to 115.8% in the regulated market. For electrical energy, gas, and other fuels—a category that includes gas, electricity (free and regulated market), heating oil, and solid fuels—if the increase in January was 67.3% compared to one year prior, the cost of living for a family averaged 907.50 euros on an annual basis, with some cities approaching 90 percent. The comparison does not console the fact that Umbria is at the foot of the podium, especially because the distance to the city that achieved the highest step is reduced. In Alessandria, expenses for electricity, gas, and kerosene soared by 88.6% in January 2022. Piedmont is fully loaded, with Vercelli entering with +87.1% and Biella with +86.1%. On the other side of the ranking, the least affected city is Potenza with +35.2%. In second place, Aosta with +50.8%. At the bottom of the podium of virtuous cities, Olbia-Tempio with +51%. Following are Naples (+51.4%), Gorizia (+51.7%), Benevento (+53.1%), Caserta (+53.5%), then Avellino (+53.7%) and Trieste (+54.6%). Closing the top ten are Pordenone and Udine, tied at +54.7%. Another ranking, a different study on price increases, comes from the CGIAR study office in Mestre, which indicates the weight of families' purchasing power relative to inflation, which is running wild. Over two years, 2022-2023, the loss of purchasing power in Umbria due to inflation could amount to nearly six thousand euros per family. The estimate is based on data from Banca d'Italia, ISTAT, and the European Commission. Faced with bank deposits that amounted to 14.5 billion euros at the end of 2021, in Umbria, the estimated loss of purchasing power in 2022 amounts to 1.2 billion euros, while in 2023, due to a slowdown in inflation, it amounts to 885 million, for a total of 2.1 billion euros. At the provincial level, the CGIAR data states that for Perugia, the loss of purchasing power could amount to over 1.6 billion euros (nearly 5,746 per family), while in Terni, it is 536 million (5,251 per family). Here, the gap is clearer compared to the increases in electricity and gas bills. Luca Benedetti.</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>Observation date: 2023-02-26 00:00:00. According to a study by the National Consumers Union, which ranked cities based on the largest annual increases, the report analyzed Istat data from last January. Consequently, Perugia and Terni finished in the top six cities with the highest costs, nearly reaching the podium. Specifically, in Perugia, the cost of electricity and gas saw an 85.8% growth: while Terni recorded 85.4%. This minimal delta between the two city centers indicates that the cost of living is, in fact, uniform throughout the region. Considering the average expenditure of an Italian family, the cost of living in Perugia amounts to 1,157 euros on an annual basis; while for a family in Terni, it is 1,152 euros. A derby that essentially ends in a draw (there is only a 5 euro difference), and winning it neither leads to celebrations nor parades with scarves and flags. Nationally, however, the survey compares the variation in electricity and gas prices over the last three years, contrasting the free market with the regulated market. From June 2021, before the increases that began in July, electricity in the free market in Italy rose by 248.3% compared to 108.4% in the regulated market—more than double (+129%). Furthermore, considering the first available gas data from Istat, December 2021, the free market since then increased by 141.1% compared to a 7.4% decrease in the regulated market. In three years, from January 2020 to January 2023, free market electricity jumped by 262.8%, compared to 115.8% in the regulated market. For electricity, gas, and other fuels—a category that includes gas, electricity (free and regulated markets), heating oil, and solid fuels—if the increase in January was 67.3% compared to one year prior, the average family cost was 907.50 euros on an annual basis, with some cities approaching 90%. The comparison does little to console the fact that Umbria is at the foot of the podium, especially because the distance to the city at the top is reduced. In Alessandria, expenses for electricity, gas, and heating oil soared by 88.6% by January 2022. Piedmont is well-stocked, with Vercelli recording an increase of 87.1% and Biella with 86.1%. On the other side of the ranking, the least affected city is Potenza, with an increase of 35.2%. In second place is Aosta with an increase of 50.8%. At the bottom of the 'virtuous cities' podium is Olbia-Tempio with an increase of 51%. Following are Naples (+51.4%), Gorizia (+51.7%), Benevento (+53.1%), Caserta (+53.5%), then Avellino (+53.7%) and Trieste (+54.6%). Closing the top ten are Pordenone and Udine, tied at +54.7%. Another ranking, a study on price increases, comes from the CGIAR study office, which indicates the impact of family purchasing power relative to inflation, which is running wild. Over the two years 2022-2023, the loss of purchasing power in Umbria due to inflation could amount to nearly six million euros per family. The estimate is based on data from the Bank of Italy, Istat, and the European Commission. Against bank deposits, which amounted to 14.5 billion euros at the end of 2021, the estimated loss of purchasing power in Umbria in 2022 was 1.2 billion euros, while in 2023, thanks to a slowdown in inflation, it was 885 million euros, totaling 2.1 billion euros. At the provincial level, the CGIAR data states that for Perugia, the loss of purchasing power could amount to over 1.6 billion euros (nearly 5,746 per family), while in Terni, it is 536 million euros (5,251 per family). Here, the gap is clearer compared to the increases in electricity and gas bills.</t>
+          <t>Observation date: 2023-02-26 00:00:00. A study by the National Consumers Union placed a ranking of cities based on the largest annual increases, elaborating data from ISTAT regarding last January. Consequently, Perugia and Terni finished in the top six of the most expensive cities, nearly reaching the podium. Specifically, in Perugia, the cost of electricity and gas saw an 85.8% growth: while Terni stopped at 85.4%. A minimal delta between the two city capitals indicates that the cost of living is, in fact, uniform throughout the region. Considering how much an average Italian family spends, the cost of living in Perugia is 1,157 euros on an annual basis; while for a family in Terni, it is 1,152 euros. A derby that ends essentially in a draw (there is only a 5 euro difference), and winning it brings neither carousels nor parties with scarves and flags. Nationally, however, the survey compares the variation in electricity and gas prices over the last 3 years, comparing the free market with the regulated market. From June 2021, before the increases that started in July, electricity in the free market in Italy rose by 248.3% versus 108.4% in the regulated market, more than double (+129%). Furthermore, considering the first useful gas data detected by ISTAT, December 2021, the free market since then increased by 141.1% versus a 7.4% drop in the regulated market. In 3 years, from January 2020 to January 2023, free electricity jumped by 262.8%, compared to 115.8% in the regulated market. For electrical energy, gas, and other fuels—a category that includes gas, electricity (free and regulated market), heating oil, and solid fuels—if the increase in January was 67.3% compared to one year prior, the cost of living for a family averaged 907.50 euros on an annual basis, with some cities approaching 90 percent. The comparison does not console the fact that Umbria is at the foot of the podium, especially because the distance to the city that achieved the highest step is reduced. In Alessandria, expenses for electricity, gas, and kerosene soared by 88.6% in January 2022. Piedmont is fully loaded, with Vercelli entering with +87.1% and Biella with +86.1%. On the other side of the ranking, the least affected city is Potenza with +35.2%. In second place, Aosta with +50.8%. At the bottom of the podium of virtuous cities, Olbia-Tempio with +51%. Following are Naples (+51.4%), Gorizia (+51.7%), Benevento (+53.1%), Caserta (+53.5%), then Avellino (+53.7%) and Trieste (+54.6%). Closing the top ten are Pordenone and Udine, tied at +54.7%. Another ranking, a different study on price increases, comes from the CGIAR study office in Mestre, which indicates the weight of families' purchasing power relative to inflation, which is running wild. Over two years, 2022-2023, the loss of purchasing power in Umbria due to inflation could amount to nearly six thousand euros per family. The estimate is based on data from Banca d'Italia, ISTAT, and the European Commission. Faced with bank deposits that amounted to 14.5 billion euros at the end of 2021, in Umbria, the estimated loss of purchasing power in 2022 amounts to 1.2 billion euros, while in 2023, due to a slowdown in inflation, it amounts to 885 million, for a total of 2.1 billion euros. At the provincial level, the CGIAR data states that for Perugia, the loss of purchasing power could amount to over 1.6 billion euros (nearly 5,746 per family), while in Terni, it is 536 million (5,251 per family). Here, the gap is clearer compared to the increases in electricity and gas bills. Luca Benedetti.</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>['The National Consumers Union conducted a study ranking cities based on the largest annual increases.', 'The report analyzed Istat data from January 2023.', 'Perugia and Terni finished among the top six cities with the highest costs.', 'The cost of electricity and gas in Perugia saw an 85.8% growth.', 'Terni recorded an 85.4% growth in the cost of electricity and gas.', 'The average cost of living for an Italian family in Perugia is 1,157 euros annually.', 'The survey compares the variation in electricity and gas prices over the last three years.', 'The survey contrasts the free market with the regulated market for electricity and gas prices.', 'From June 2021, electricity in the regulated market in Italy rose by 108.4%.', 'The increase in the free market electricity price was more than double the increase in the regulated market electricity price (+129%).', 'According to Istat data from December 2021, the regulated market gas price decreased by 7.4%.', 'From January 2020 to January 2023, regulated market electricity jumped by 115.8%.', 'If the increase in electricity, gas, and other fuels in January was 67.3% compared to one year prior, the average family cost was 907.50 euros annually.', 'Expenses for electricity, gas, and heating oil in Alessandria soared by 88.6% by January 2022.', 'Vercelli recorded an increase of 87.1% in Piedmont.', 'Potenza was the least affected city, recording an increase of 35.2%.', 'Aosta was in second place with an increase of 50.8%.', "Olbia-Tempio was at the bottom of the 'virtuous cities' podium with an increase of 51%.", 'Benevento recorded an increase of 53.1%.', 'Avellino recorded an increase of 53.7%.', 'Trieste recorded an increase of 54.6%.', 'Pordenone and Udine tied for the top ten with an increase of 54.7%.', 'Over the two years 2022-2023, the loss of purchasing power in Umbria due to inflation could amount to nearly six million euros per family.', 'The estimate of purchasing power loss is based on data from the Bank of Italy, Istat, and the European Commission.', 'Bank deposits amounted to 14.5 billion euros at the end of 2021.', 'The total estimated loss of purchasing power in Umbria over 2022 and 2023 was 2.1 billion euros.', 'CGIAR data states that the loss of purchasing power for Perugia could amount to over 1.6 billion euros.', 'CGIAR data states that the loss of purchasing power for Perugia is nearly 5,746 euros per family.']</t>
+          <t>['A study by the National Consumers Union placed a ranking of cities based on the largest annual increases.', 'The National Consumers Union elaborated data from ISTAT regarding January 2023.', 'Perugia and Terni finished in the top six of the most expensive cities.', 'In Perugia, the cost of electricity and gas saw an 85.8% growth.', 'Terni saw an 85.4% growth in the cost of electricity and gas.', 'A minimal delta between Perugia and Terni indicates that the cost of living is uniform throughout the region.', 'The cost of living for an average Italian family in Perugia is 1,157 euros annually.', 'The survey compares the variation in electricity and gas prices over the last 3 years.', 'The survey compares the free market with the regulated market for electricity and gas prices.', 'From June 2021, electricity in the regulated market in Italy rose by 108.4%.', 'The free market increase (248.3%) was more than double the regulated market increase (108.4%).', 'According to ISTAT, the regulated market gas dropped by 7.4% since December 2021.', 'From January 2020 to January 2023, regulated electricity jumped by 115.8%.', 'If the increase in electrical energy, gas, and other fuels in January was 67.3% compared to one year prior, the cost of living for a family averaged 907.50 euros annually.', 'In Alessandria, expenses for electricity, gas, and kerosene soared by 88.6% in January 2022.', 'Vercelli saw an increase of 87.1%.', 'Potenza was the least affected city with a +35.2% increase.', 'Olbia-Tempio saw a +51% increase.', 'Naples saw a +51.4% increase.', 'Gorizia saw a +51.7% increase.', 'Benevento saw a +53.1% increase.', 'Caserta saw a +53.5% increase.', 'Trieste saw a +54.6% increase.', 'Pordenone and Udine were tied at a +54.7% increase.', 'Over two years (2022-2023), the loss of purchasing power in Umbria due to inflation could amount to nearly six thousand euros per family.', "The estimate of purchasing power loss is based on data from Banca d'Italia, ISTAT, and the European Commission.", 'Umbria had bank deposits amounting to 14.5 billion euros at the end of 2021.', 'The total estimated loss of purchasing power in Umbria over 2022 and 2023 is 2.1 billion euros.', 'CGIAR data states that the loss of purchasing power for Perugia could amount to over 1.6 billion euros.', 'CGIAR data states that the loss of purchasing power for Perugia is nearly 5,746 euros per family.']</t>
         </is>
       </c>
     </row>
@@ -926,17 +926,17 @@
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
-          <t>The closing of major international exchanges. The performance of the Dow Jones (see page 5) gave the Dow Jones and New York a new package to vote on in Congress to stimulate the American economy, which is in a severe crisis. Yesterday, this package received support from the Federal Reserve Chairman, Ben Bernanke, and conditional approval from President Bush. Looking into the near future of the US economy, the central bank is also considering a further cut in rates, thanks to inflation being kept low by the recession. For Bernanke, who spoke before the House Budget Committee, the credit crisis 'is hitting the economy' because Americans are having difficulty finding money for their activities. 'With an economy probably destined to be weak for several quarters still, and the risk of a prolonged slowdown, the idea of a fiscal package seems appropriate in this juncture,' the governor told the deputies, though refusing to define the ideal size of the intervention. An hour after these statements of technical support, the political green light arrived for putting a second fiscal drug package on the agenda in the country. The Bush administration 'is open to ideas that could stimulate the economy and help us exit this downward spiral faster,' echoed the President's spokesperson, Dana Perino, repeating Bernanke's words. But the okay will only come if the ideas are 'truly capable of stimulating the economy.' The Congress, which is responsible for approving a second fiscal package after the one passed earlier this year, which yielded very limited benefits, according to the Fed governor, 'should include measures to facilitate access to credit for consumers, homeowners, and generally anyone interested in obtaining loans. Such actions could be particularly effective' in 'promoting economic growth and job creation.' Wall Street, which had already started positively, expanded its gains after the promise of stimulus from the central bank and the availability of Bush. The Dow Jones index rose above 9,000 points, with a gain of 4.67%, and the Nasdaq also gained 3.43% at 1,700 points, while the dollar strengthened against the euro, falling to $1.33 from $1.34 at the start. Europe also rose, with London leading (+5.41%), followed by Paris (+3.56%), Madrid (+2.99%), and Milan (+2.65%). Frankfurt was more cautious (+1.12%). Contributing to the boost in stock purchases was also Bernanke's mention of a new rate cut at the Fed meeting at the end of October. Federal bonds discount, at 100%, a reduction of 25 cents, but for the 46% it could also be half a point, like the previous one done together by all banks. The fate of the American budget, however, is no longer a problem for anyone, in these global times of clear moons where public spending is dominating to build a barrier against the threat of depression. The newly awarded Nobel laureate in economics, Paul Krugman, wrote this in the New York Times, calling for massive state injections of money into banks, and Bernanke himself mentioned this in his speech: 'the current deficit is large,' he admitted, 'but not inappropriate given the nature of the emergency we are facing and unavoidable given the loss of tax revenue.' Bernanke is aware that 'every fiscal action inevitably entails trade-offs' and could 'weigh on future generations,' but he accepted the inevitability of the intervention. Without defining the current state of the economy as a recession, the governor predicted that 'the pace of economic activity will remain below potential growth for numerous quarters, and that the slowdown in investment and business spending extends to major sectors.'</t>
+          <t>The closing of major international stock exchanges. The performance of the Dow Jones (see page 5) showed that New York has a new package to vote in Congress to stimulate the American economy in a severe crisis, which yesterday received support from Federal Reserve Chairman Ben Bernanke, and a conditional green light from President Bush. Regarding the near future of the US economy, the central bank is also considering a further rate cut, thanks to inflation kept low by the recession. For Bernanke, who spoke before the House Budget Committee, the credit crisis "is hitting the economy" because Americans are having difficulty finding money for their activities. "With an economy likely to remain weak for several more quarters and the risk of a prolonged slowdown, the idea of a fiscal package seems appropriate in this context," the governor told the deputies, though refusing to define the ideal extent of the intervention. An hour after these technical statements of support, the political green light arrived for putting a second fiscal law on the agenda. The Bush administration, through the presidential spokesperson Dana Perino, echoed Bernanke: "is open to ideas that could stimulate the economy and help us exit this downward spiral faster." But the okay will only come if the ideas are "truly capable of stimulating the economy." The Congress, which is responsible for approving a second fiscal package after the one passed earlier this year which provided very limited benefits, according to the Fed governor, "should include measures to facilitate access to credit for consumers, homeowners, and generally anyone interested in loans. Such actions could be particularly effective," Bernanke ventured, "in promoting economic growth and job creation." Wall Street, which had already started positively, expanded its gains after the promise of stimulus from the central bank and the availability of Bush. The Dow Jones index rose above 9,000 points, with a gain of 4.67%, and the Nasdaq also gained 3.43% to 1,700 points, while the dollar strengthened against the euro, falling to $1.33 from $1.34 at the start. Europe also ran up, with London shining (+5.41%), followed by Paris (+3.56%), Madrid (+2.99%), and Milan (+2.65%). Frankfurt was more cautious (+1.12%). Contributing to the boost in stock purchases was also Bernanke's mention of a new rate cut at the Fed meeting at the end of October. Federal bonds discount, at 100%, a reduction of 25 cents, but for the 46% it could also be half a point, like the previous one done together by all the banks. The fate of the American budget, however, is no longer a problem for anyone, in these global times of clarity where the use of public spending is dominant to build a barrier against the threat of depression. The newly awarded Nobel laureate in economics Paul Krugman wrote this in the New York Times, calling for massive injections of state money into banks, and Bernanke himself mentioned it in his speech: "the current deficit is large," he admitted, "but not inappropriate given the nature of the emergency we are facing and unavoidable given the loss of tax revenue." Bernanke is aware that "every fiscal action inevitably entails trade-offs" and may "weigh on future generations," but he accepted the inevitability of the intervention. Without defining a recession, the governor predicted that "the pace of economic activity will remain below the growth potential for numerous quarters, and that the slowdown in investment and business spending extends to major sectors."</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>Observation date: 2008-10-21 00:00:00. The closing of major international exchanges. The performance of the Dow Jones (see page 5) gave the Dow Jones and New York a new package to vote on in Congress to stimulate the American economy, which is in a severe crisis. Yesterday, this package received support from the Federal Reserve Chairman, Ben Bernanke, and conditional approval from President Bush. Looking into the near future of the US economy, the central bank is also considering a further cut in rates, thanks to inflation being kept low by the recession. For Bernanke, who spoke before the House Budget Committee, the credit crisis 'is hitting the economy' because Americans are having difficulty finding money for their activities. 'With an economy probably destined to be weak for several quarters still, and the risk of a prolonged slowdown, the idea of a fiscal package seems appropriate in this juncture,' the governor told the deputies, though refusing to define the ideal size of the intervention. An hour after these statements of technical support, the political green light arrived for putting a second fiscal drug package on the agenda in the country. The Bush administration 'is open to ideas that could stimulate the economy and help us exit this downward spiral faster,' echoed the President's spokesperson, Dana Perino, repeating Bernanke's words. But the okay will only come if the ideas are 'truly capable of stimulating the economy.' The Congress, which is responsible for approving a second fiscal package after the one passed earlier this year, which yielded very limited benefits, according to the Fed governor, 'should include measures to facilitate access to credit for consumers, homeowners, and generally anyone interested in obtaining loans. Such actions could be particularly effective' in 'promoting economic growth and job creation.' Wall Street, which had already started positively, expanded its gains after the promise of stimulus from the central bank and the availability of Bush. The Dow Jones index rose above 9,000 points, with a gain of 4.67%, and the Nasdaq also gained 3.43% at 1,700 points, while the dollar strengthened against the euro, falling to $1.33 from $1.34 at the start. Europe also rose, with London leading (+5.41%), followed by Paris (+3.56%), Madrid (+2.99%), and Milan (+2.65%). Frankfurt was more cautious (+1.12%). Contributing to the boost in stock purchases was also Bernanke's mention of a new rate cut at the Fed meeting at the end of October. Federal bonds discount, at 100%, a reduction of 25 cents, but for the 46% it could also be half a point, like the previous one done together by all banks. The fate of the American budget, however, is no longer a problem for anyone, in these global times of clear moons where public spending is dominating to build a barrier against the threat of depression. The newly awarded Nobel laureate in economics, Paul Krugman, wrote this in the New York Times, calling for massive state injections of money into banks, and Bernanke himself mentioned this in his speech: 'the current deficit is large,' he admitted, 'but not inappropriate given the nature of the emergency we are facing and unavoidable given the loss of tax revenue.' Bernanke is aware that 'every fiscal action inevitably entails trade-offs' and could 'weigh on future generations,' but he accepted the inevitability of the intervention. Without defining the current state of the economy as a recession, the governor predicted that 'the pace of economic activity will remain below potential growth for numerous quarters, and that the slowdown in investment and business spending extends to major sectors.'</t>
+          <t>Observation date: 2008-10-21 00:00:00. The closing of major international stock exchanges. The performance of the Dow Jones (see page 5) showed that New York has a new package to vote in Congress to stimulate the American economy in a severe crisis, which yesterday received support from Federal Reserve Chairman Ben Bernanke, and a conditional green light from President Bush. Regarding the near future of the US economy, the central bank is also considering a further rate cut, thanks to inflation kept low by the recession. For Bernanke, who spoke before the House Budget Committee, the credit crisis "is hitting the economy" because Americans are having difficulty finding money for their activities. "With an economy likely to remain weak for several more quarters and the risk of a prolonged slowdown, the idea of a fiscal package seems appropriate in this context," the governor told the deputies, though refusing to define the ideal extent of the intervention. An hour after these technical statements of support, the political green light arrived for putting a second fiscal law on the agenda. The Bush administration, through the presidential spokesperson Dana Perino, echoed Bernanke: "is open to ideas that could stimulate the economy and help us exit this downward spiral faster." But the okay will only come if the ideas are "truly capable of stimulating the economy." The Congress, which is responsible for approving a second fiscal package after the one passed earlier this year which provided very limited benefits, according to the Fed governor, "should include measures to facilitate access to credit for consumers, homeowners, and generally anyone interested in loans. Such actions could be particularly effective," Bernanke ventured, "in promoting economic growth and job creation." Wall Street, which had already started positively, expanded its gains after the promise of stimulus from the central bank and the availability of Bush. The Dow Jones index rose above 9,000 points, with a gain of 4.67%, and the Nasdaq also gained 3.43% to 1,700 points, while the dollar strengthened against the euro, falling to $1.33 from $1.34 at the start. Europe also ran up, with London shining (+5.41%), followed by Paris (+3.56%), Madrid (+2.99%), and Milan (+2.65%). Frankfurt was more cautious (+1.12%). Contributing to the boost in stock purchases was also Bernanke's mention of a new rate cut at the Fed meeting at the end of October. Federal bonds discount, at 100%, a reduction of 25 cents, but for the 46% it could also be half a point, like the previous one done together by all the banks. The fate of the American budget, however, is no longer a problem for anyone, in these global times of clarity where the use of public spending is dominant to build a barrier against the threat of depression. The newly awarded Nobel laureate in economics Paul Krugman wrote this in the New York Times, calling for massive injections of state money into banks, and Bernanke himself mentioned it in his speech: "the current deficit is large," he admitted, "but not inappropriate given the nature of the emergency we are facing and unavoidable given the loss of tax revenue." Bernanke is aware that "every fiscal action inevitably entails trade-offs" and may "weigh on future generations," but he accepted the inevitability of the intervention. Without defining a recession, the governor predicted that "the pace of economic activity will remain below the growth potential for numerous quarters, and that the slowdown in investment and business spending extends to major sectors."</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>['The performance of the Dow Jones gave the Dow Jones and New York a new package to vote on in Congress.', 'The package was intended to stimulate the American economy.', 'The American economy was in a severe crisis.', 'On 2008-10-20, the package received support from Ben Bernanke.', 'On 2008-10-20, the package received conditional approval from President Bush.', 'The central bank is considering a further cut in rates for the US economy.', 'The recession kept inflation low.', 'Ben Bernanke stated that the credit crisis is hitting the economy.', 'The credit crisis is hitting the economy because Americans are having difficulty finding money for their activities.', 'Ben Bernanke told the deputies that a fiscal package seems appropriate.', 'Ben Bernanke stated the economy is probably destined to be weak for several quarters.', 'Ben Bernanke mentioned the risk of a prolonged slowdown.', "An hour after Ben Bernanke's statements, the political green light arrived for putting a second fiscal package on the agenda.", "Dana Perino, the President's spokesperson, stated the Bush administration is open to ideas that could stimulate the economy.", "Dana Perino repeated Ben Bernanke's words.", 'The Congress is responsible for approving a second fiscal package.', 'The first fiscal package passed earlier on 2008-01-01 yielded very limited benefits, according to Ben Bernanke.', 'Ben Bernanke stated the second fiscal package should include measures to facilitate access to credit for consumers, homeowners, and anyone interested in obtaining loans.', 'Such actions could be particularly effective in promoting economic growth and job creation.', 'Wall Street expanded its gains after the promise of stimulus from the central bank.', 'Wall Street expanded its gains after the availability of Bush.', 'The Dow Jones index rose above 9,000 points.', 'The Dow Jones index gained 4.67%.', 'The Nasdaq gained 3.43% at 1,700 points.', 'The dollar strengthened against the euro.', 'The dollar fell to $1.33 from $1.34 against the euro.', 'London rose by 5.41%.', 'Paris rose by 3.56%.', 'Madrid rose by 2.99%.', 'Milan rose by 2.65%.', 'Frankfurt rose by 1.12%.', "Bernanke's mention of a new rate cut at the Fed meeting at the end of October contributed to the boost in stock purchases.", 'Federal bonds discount was at 100%.', 'The discount reduction was 25 cents.', 'The discount could be half a point for the 46%.', 'Paul Krugman wrote in the New York Times calling for massive state injections of money into banks.', 'Ben Bernanke admitted that the current deficit is large.', 'Ben Bernanke stated the current deficit is not inappropriate given the nature of the emergency.', 'Ben Bernanke stated the deficit is unavoidable given the loss of tax revenue.', 'Ben Bernanke is aware that every fiscal action inevitably entails trade-offs.', 'Ben Bernanke acknowledged that fiscal actions could weigh on future generations.', 'Ben Bernanke predicted that the pace of economic activity will remain below potential growth for numerous quarters.', 'Ben Bernanke predicted that the slowdown in investment and business spending extends to major sectors.']</t>
+          <t>['New York has a new package to vote in Congress to stimulate the American economy in a severe crisis.', 'The package received support from Federal Reserve Chairman Ben Bernanke on 2008-10-20.', 'The package received a conditional green light from President Bush on 2008-10-20.', 'The central bank is considering a further rate cut for the US economy.', 'The recession kept inflation low.', 'Ben Bernanke spoke before the House Budget Committee.', 'Ben Bernanke stated that the credit crisis is hitting the economy.', 'Ben Bernanke stated that Americans are having difficulty finding money for their activities.', 'Ben Bernanke told the deputies that the idea of a fiscal package seems appropriate because the economy is likely to remain weak for several more quarters and there is a risk of a prolonged slowdown.', 'The political green light arrived for putting a second fiscal law on the agenda an hour after the technical statements of support.', 'The Bush administration, through Dana Perino, echoed Ben Bernanke.', 'The Bush administration stated that the administration is open to ideas that could stimulate the economy and help the US exit the downward spiral faster.', 'The Bush administration stated that the ideas must be truly capable of stimulating the economy.', 'The Congress is responsible for approving a second fiscal package.', 'The first fiscal package was passed on 2008-01-01.', 'The first fiscal package provided very limited benefits.', 'Ben Bernanke suggested that the second fiscal package should include measures to facilitate access to credit for consumers, homeowners, and generally anyone interested in loans.', 'Wall Street expanded its gains after the promise of stimulus from the central bank and the availability of Bush.', 'The Dow Jones index rose above 9,000 points.', 'The Dow Jones index gained 4.67%.', 'The Nasdaq gained 3.43% to 1,700 points.', 'The dollar strengthened against the euro.', 'The dollar fell to $1.33 from $1.34 at the start.', 'London gained 5.41%.', 'Paris gained 3.56%.', 'Madrid gained 2.99%.', 'Milan gained 2.65%.', 'Frankfurt gained 1.12%.', "Bernanke's mention of a new rate cut at the Fed meeting at the end of October contributed to the boost in stock purchases.", 'Federal bonds discount was at 100%.', 'A reduction of 25 cents was possible for federal bonds discount.', 'For the 46% (of bonds), the discount could be half a point.', 'Paul Krugman wrote in the New York Times calling for massive injections of state money into banks.', 'Ben Bernanke admitted that the current deficit is large.', 'Ben Bernanke stated that the current deficit is not inappropriate given the nature of the emergency.', 'Ben Bernanke stated that the current deficit is unavoidable given the loss of tax revenue.', 'Ben Bernanke is aware that every fiscal action inevitably entails trade-offs.', 'Ben Bernanke predicted that the pace of economic activity will remain below the growth potential for numerous quarters.', 'Ben Bernanke predicted that the slowdown in investment and business spending extends to major sectors.']</t>
         </is>
       </c>
     </row>
@@ -986,17 +986,17 @@
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
-          <t xml:space="preserve">If there had been the ability to generate income from those savings, even with a remuneration of one percentage point, households would have collectively earned 30 billion, almost 2% of the gross domestic product. 'The savings rate of Italian households relative to disposable income has grown by 50% in the year, but, excluding savings invested in listed companies, its return has remained quite low, close to zero. Given the consistency of financial assets held by households, every percentage point of remuneration can be estimated at around 30 billion euros, almost 2% of GDP, the size of a good public budget maneuver in the past.' The core theme of the annual report by the President of Consob, Paolo Savona, is the primary asset that the authority he leads intends to protect: savings. But this has been focused on deposits for the last two years. And now it is threatened by a shadow lengthening over international markets, which is very difficult to control: these are the sirens of cryptocurrencies and Bitcoin. A phenomenon that is growing rapidly and becoming increasingly difficult to contain, much so that it has prompted Savona to sound the alarm: the speculative effect they are triggering seems very similar to what happened before 2008 with subprime mortgages. 'The spread of virtual instruments has stimulated the birth of the already remembered technological platforms,' he said. 'These new market segments are rapidly evolving, and the experience preceding the 2008 crisis seems to be repeating itself, when derivative contracts developed to reach a size ten times the global GDP, assuming complex forms that received high ratings. With due distinctions, it is predictable that something analogous is happening in the market for virtual monetary and financial products, especially crypto.' Savona recalled how 'a single Bitcoin recently had the ability to purchase a large electric car and shortly after lost half its purchasing power.' For the President of Consob, 'financial technology is a prodigious lamp from which genius has emerged. The authorities will not be able to put it back, because it operates in the immaterial sphere controllable only by changing the information exchange protocol, thus fragmenting the unit of the global market and reducing the international competitiveness rate.' Traditional supervisory tools are no longer sufficient. Under current conditions, according to Savona, 'the authorities can intervene by also utilizing the advantages of digitized techniques; their action will be more effective if they cooperate with each other.' For Italy, the issue is even more delicate due to the constitutional rule that assigns the 'Republic the task of encouraging and protecting savings in all their forms and of regulating, coordinating, and controlling the exercise of credit.' It would be inappropriate, he explained, 'if the specification of </t>
+          <t xml:space="preserve">If only there were a way to reinvest that savings, even with a one percent remuneration, families would have collectively earned 30 billion, almost 2% of the gross domestic product. 'The savings rate of Italian families relative to disposable income has grown by 50% in the year, but excluding savings invested in listed companies, its return has remained rather low, close to zero. Given the consistency of financial assets held by families, every percentage point of remuneration can be estimated at around 30 billion euros, almost 2% of GDP, the size of a good public budget maneuver in the past.' The central theme of the annual report by the President of Consob, Paolo Savona, is the main asset that the authority he leads intends to protect: savings. But this has been stable regarding deposits over the last two years. And now it is threatened by a shadow lengthening over international markets, one that is very difficult to control: these are the sirens of cryptocurrencies and Bitcoin. A rapidly growing and increasingly difficult phenomenon to keep under control, much so that it has prompted Savona to issue an alarm: the speculative effect they are triggering seems very similar to what happened before 2008 with subprime mortgages. 'The diffusion of virtual instruments has stimulated the birth of the already remembered technological platforms,' he said. 'These new market segments are rapidly evolving, and the experience preceding the 2008 crisis seems to be repeating itself, when derivatives contracts developed to reach a size ten times the global GDP, assuming complex forms that received a high rating. With due distinctions, it is predictable that something analogous is happening in the market for virtual monetary and financial products, especially crypto.' Savona recalled how 'a single Bitcoin recently had the ability to purchase a large electric car and shortly after lost half of its purchasing power.' For the Consob President, 'financial computing is a prodigious lamp from which genius has emerged. The authorities will not be able to put it back, because it operates in the immaterial sphere controllable only by changing the information exchange protocol, thus fragmenting the unit of the global market and reducing the international competitiveness rate.' Traditional supervisory tools are no longer sufficient. Under current conditions, according to Savona, 'the authorities can intervene by also utilizing the advantages of digitized techniques; their action will be more effective if they cooperate with each other.' For Italy, the issue is even more delicate due to the constitutional norm that gives the 'Republic the task of encouraging and protecting savings in all their forms and of regulating, coordinating, and controlling the exercise of credit.' It would be inappropriate, he explained, 'if the specification of </t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Observation date: 2021-06-14 00:00:00. If there had been the ability to generate income from those savings, even with a remuneration of one percentage point, households would have collectively earned 30 billion, almost 2% of the gross domestic product. 'The savings rate of Italian households relative to disposable income has grown by 50% in the year, but, excluding savings invested in listed companies, its return has remained quite low, close to zero. Given the consistency of financial assets held by households, every percentage point of remuneration can be estimated at around 30 billion euros, almost 2% of GDP, the size of a good public budget maneuver in the past.' The core theme of the annual report by the President of Consob, Paolo Savona, is the primary asset that the authority he leads intends to protect: savings. But this has been focused on deposits for the last two years. And now it is threatened by a shadow lengthening over international markets, which is very difficult to control: these are the sirens of cryptocurrencies and Bitcoin. A phenomenon that is growing rapidly and becoming increasingly difficult to contain, much so that it has prompted Savona to sound the alarm: the speculative effect they are triggering seems very similar to what happened before 2008 with subprime mortgages. 'The spread of virtual instruments has stimulated the birth of the already remembered technological platforms,' he said. 'These new market segments are rapidly evolving, and the experience preceding the 2008 crisis seems to be repeating itself, when derivative contracts developed to reach a size ten times the global GDP, assuming complex forms that received high ratings. With due distinctions, it is predictable that something analogous is happening in the market for virtual monetary and financial products, especially crypto.' Savona recalled how 'a single Bitcoin recently had the ability to purchase a large electric car and shortly after lost half its purchasing power.' For the President of Consob, 'financial technology is a prodigious lamp from which genius has emerged. The authorities will not be able to put it back, because it operates in the immaterial sphere controllable only by changing the information exchange protocol, thus fragmenting the unit of the global market and reducing the international competitiveness rate.' Traditional supervisory tools are no longer sufficient. Under current conditions, according to Savona, 'the authorities can intervene by also utilizing the advantages of digitized techniques; their action will be more effective if they cooperate with each other.' For Italy, the issue is even more delicate due to the constitutional rule that assigns the 'Republic the task of encouraging and protecting savings in all their forms and of regulating, coordinating, and controlling the exercise of credit.' It would be inappropriate, he explained, 'if the specification of </t>
+          <t xml:space="preserve">Observation date: 2021-06-14 00:00:00. If only there were a way to reinvest that savings, even with a one percent remuneration, families would have collectively earned 30 billion, almost 2% of the gross domestic product. 'The savings rate of Italian families relative to disposable income has grown by 50% in the year, but excluding savings invested in listed companies, its return has remained rather low, close to zero. Given the consistency of financial assets held by families, every percentage point of remuneration can be estimated at around 30 billion euros, almost 2% of GDP, the size of a good public budget maneuver in the past.' The central theme of the annual report by the President of Consob, Paolo Savona, is the main asset that the authority he leads intends to protect: savings. But this has been stable regarding deposits over the last two years. And now it is threatened by a shadow lengthening over international markets, one that is very difficult to control: these are the sirens of cryptocurrencies and Bitcoin. A rapidly growing and increasingly difficult phenomenon to keep under control, much so that it has prompted Savona to issue an alarm: the speculative effect they are triggering seems very similar to what happened before 2008 with subprime mortgages. 'The diffusion of virtual instruments has stimulated the birth of the already remembered technological platforms,' he said. 'These new market segments are rapidly evolving, and the experience preceding the 2008 crisis seems to be repeating itself, when derivatives contracts developed to reach a size ten times the global GDP, assuming complex forms that received a high rating. With due distinctions, it is predictable that something analogous is happening in the market for virtual monetary and financial products, especially crypto.' Savona recalled how 'a single Bitcoin recently had the ability to purchase a large electric car and shortly after lost half of its purchasing power.' For the Consob President, 'financial computing is a prodigious lamp from which genius has emerged. The authorities will not be able to put it back, because it operates in the immaterial sphere controllable only by changing the information exchange protocol, thus fragmenting the unit of the global market and reducing the international competitiveness rate.' Traditional supervisory tools are no longer sufficient. Under current conditions, according to Savona, 'the authorities can intervene by also utilizing the advantages of digitized techniques; their action will be more effective if they cooperate with each other.' For Italy, the issue is even more delicate due to the constitutional norm that gives the 'Republic the task of encouraging and protecting savings in all their forms and of regulating, coordinating, and controlling the exercise of credit.' It would be inappropriate, he explained, 'if the specification of </t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>['If households could generate income from savings with a 1% remuneration, households would have collectively earned 30 billion euros.', 'This amount (30 billion euros) represents almost 2% of the gross domestic product.', 'The savings rate of Italian households relative to disposable income grew by 50% in the year.', 'Excluding savings invested in listed companies, the return on savings remained low, close to zero.', 'Every percentage point of remuneration on financial assets held by households is estimated at around 30 billion euros.', 'The core theme of the annual report by the President of Consob, Paolo Savona, is protecting savings.', 'The authority led by Paolo Savona intends to protect savings.', 'The focus of the protection efforts has been on deposits for the last two years.', 'International markets are now threatened by a shadow that is difficult to control.', 'This threat involves cryptocurrencies and Bitcoin.', 'The phenomenon of cryptocurrencies and Bitcoin is growing rapidly and becoming increasingly difficult to contain.', 'The speculative effect triggered by cryptocurrencies and Bitcoin prompted Paolo Savona to sound the alarm.', 'The speculative effect is similar to what happened before 2008 with subprime mortgages.', 'The spread of virtual instruments stimulated the birth of technological platforms.', 'New market segments are rapidly evolving.', 'The experience preceding the 2008 crisis seems to be repeating itself.', 'During the experience preceding the 2008 crisis, derivative contracts reached a size ten times the global GDP.', 'Something analogous to the pre-2008 crisis is predictable in the market for virtual monetary and financial products, especially crypto.', 'Paolo Savona recalled that a single Bitcoin recently had the ability to purchase a large electric car.', 'Shortly after, the single Bitcoin lost half its purchasing power.', 'For the President of Consob, financial technology is a prodigious lamp from which genius has emerged.', 'The authorities will not be able to reverse financial technology.', 'Financial technology operates in the immaterial sphere.', 'Changing the information exchange protocol controls the immaterial sphere of financial technology.', 'This process fragments the unit of the global market and reduces the international competitiveness rate.', 'Traditional supervisory tools are no longer sufficient.', 'According to Paolo Savona, the authorities can intervene by utilizing the advantages of digitized techniques.', 'The action of the authorities will be more effective if the authorities cooperate with each other.', 'For Italy, the issue is delicate due to a constitutional rule.', 'The constitutional rule assigns the Republic the task of encouraging and protecting savings in all their forms.', 'The constitutional rule also assigns the Republic the task of regulating, coordinating, and controlling the exercise of credit.']</t>
+          <t>['If savings could be reinvested with a one percent remuneration, families would have collectively earned 30 billion euros.', '30 billion euros represents almost 2% of the gross domestic product.', 'The savings rate of Italian families relative to disposable income grew by 50% in the year.', 'Excluding savings invested in listed companies, the return on savings remained low, close to zero.', 'Every percentage point of remuneration on financial assets held by families is estimated at around 30 billion euros.', 'The central theme of the annual report by the President of Consob, Paolo Savona, is savings.', 'The authority led by Paolo Savona intends to protect savings.', 'Savings regarding deposits have been stable over the last two years.', 'International markets are now threatened by cryptocurrencies and Bitcoin.', 'The phenomenon of cryptocurrencies and Bitcoin is rapidly growing and increasingly difficult to control.', 'The speculative effect triggered by cryptocurrencies and Bitcoin prompted Paolo Savona to issue an alarm.', 'The speculative effect triggered by cryptocurrencies and Bitcoin seems similar to what happened before 2008 with subprime mortgages.', 'The diffusion of virtual instruments stimulated the birth of technological platforms.', 'New market segments are rapidly evolving.', 'The experience preceding the 2008 crisis involved derivatives contracts reaching a size ten times the global GDP.', 'Something analogous to the pre-2008 crisis is predictable in the market for virtual monetary and financial products, especially crypto.', 'Paolo Savona recalled that a single Bitcoin recently had the ability to purchase a large electric car.', 'A single Bitcoin shortly after lost half of its purchasing power.', 'Paolo Savona stated that financial computing is a prodigious lamp from which genius has emerged.', 'Authorities will not be able to reverse financial computing.', 'Financial computing operates in the immaterial sphere.', 'Changing the information exchange protocol controls the immaterial sphere of financial computing.', 'This process fragments the unit of the global market and reduces the international competitiveness rate.', 'Traditional supervisory tools are no longer sufficient.', 'Paolo Savona stated that authorities can intervene by utilizing the advantages of digitized techniques.', 'The action of the authorities will be more effective if the authorities cooperate with each other.', 'The constitutional norm gives the Republic the task of encouraging and protecting savings in all their forms.', 'The constitutional norm requires the Republic to regulate, coordinate, and control the exercise of credit.']</t>
         </is>
       </c>
     </row>
@@ -1050,17 +1050,17 @@
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr">
         <is>
-          <t>Governor Stefano Lepri stated that the financial crisis is beginning to spread to businesses and families; for now, credit provided by banks has not decreased, said the Governor of the Bank of Italy, Mario Draghi, though, "the situation, however, can change quickly." Consumption is falling. Following the drop in product in the second quarter, "negative signals are arriving for the coming quarters." To curb the negative effects, Silvio Berlusconi accepted the Confindustria proposal to open a discussion forum among the government, businesses, and banks. He will convene it immediately upon his return from his trip to China: "We ask that the banks do not fail to provide their support for investments and consumption." The promise is to find "funds of significant magnitude" in the budget. Minister Claudio Scajola added: "State guarantee forms are being studied for corporate debts, as was done for banks." In his hearing before the Senate, Draghi first sought to reassure about Italian banks: "Thanks to rigorous laws and firm supervisory action, we do not have that extensive 'shadow banking system' where the crisis found its origin and sustenance elsewhere." Today, "the capitalization of the major Italian banks remains sufficient"; even if losses from the Lehman failure reached the worst-case scenario, "such a shock could be absorbed." However, banks suffered on the stock exchange due to a phrase from the Prime Minister that was partially misunderstood. Again, and always in Naples, like the first time with Eni and Enel, Berlusconi let slip comments about listed companies on the stock exchange. According to the official clarification, he said: "Perhaps two or three banks, in addition to UniCredit, will have advantages in increasing their capital, naturally finding the means in the market." At the initial reports from the news agencies, the quotes of the major banks fell, before recovering somewhat later. The clarity in the financial markets was confirmed yesterday with the Euribor rate falling below 5% for three months, a reference point for variable-rate home mortgages. The Governor assures that Italian banks "have shared only a minimal portion of the errors and distortions" of the global financial system, originating mainly in the United States. Regarding European standards, "the Bank of Italy has consistently given a severe interpretation." Draghi is well aware that public opinion tends to involve central banks in blame. He makes it clear that this may be justified in the US, where there was a "regulatory capture" (in simple terms, Wall Street influenced the government and the Federal Reserve) and in other countries; it is not the case in the Euro area, and especially not in Italy. "Alarms were not lacking over time," he recalls: "not least the person speaking had repeatedly drawn attention to the imbalances of the international financial system," in various interventions, especially in the autumn of 2006; the problem is that "in calm times, warnings often remain unheard." "Neither the timing, nor the precise mechanism, nor the magnitude of the crisis could be foreseen; but the accumulating tensions could clearly be seen." The banks or other intermediaries that sold Lehman Brothers securities to savers "will not leave them alone." New rules on transparency in relationships between banks and clients will be ready at the beginning of next year. Globally, cleaning up will require better regulation of derivatives and other innovative financial products. New rules must prevent banks from assuming risks too disproportionate to their capital. "All in all, Italy is not doing badly" from the financial crisis, concludes the Governor; but the effects of the crisis on the real economy "add to pre-existing structural weaknesses." The same judgment comes from the International Monetary Fund, which confirms the forecast of a drop in gross product both in 2008 (-0.1%) and in 2009 (-0.2%). But reacting with state aid would not be the right answer, warns the head of the IMF's European Department, Alessandro Leipold: "Liberalization is better."</t>
+          <t>The words of Governor Stefano Lepri: Rome, the financial crisis is beginning to affect businesses and families; for now, the credit provided by banks has not decreased, says the Governor of the Bank of Italy, Mario Draghi, 'however, the situation can change quickly.' Consumption is falling. Following the drop in product in the second quarter, 'negative signs are coming for the coming quarters.' To curb the negative effects, Silvio Berlusconi accepted the proposal from Confindustria to open a discussion table among the government, businesses, and banks. He will convene it as soon as he returns from his trip to China: 'We ask that the banks do not fail in their support for investments and consumption.' The promise is to find 'funds of significant magnitude' in the budget. And Minister Claudio Scajola added: state guarantee forms are being studied for corporate debts, as was done for banks. In his hearing before the Senate, Draghi first wanted to reassure about Italian banks: 'Thanks to rigorous laws and firm supervisory action, we do not have that extensive ''shadow banking system'' where elsewhere the crisis found its origin and sustenance.' Today, 'the capitalization of the major Italian banks remains sufficient'; even if losses from the Lehman failure reached the worst hypothesis, 'such a shock could be absorbed.' However, banks suffered on the stock exchange due to a phrase by the Prime Minister that was partially misunderstood. Again, and always in Naples, like the first time on Eni and Enel, Berlusconi let slip comments about listed companies. According to the official clarification, he said: 'Perhaps two or three banks, besides Unicredit, will have advantages in increasing their capital, finding the means naturally in the market.' To the initial headlines of the news agencies, the quotes of the major banks fell, only to recover somewhat later. The clarity on the financial markets was confirmed yesterday with the Euribor rate at three months below 5%, the reference point for variable-rate home mortgages. Italian banks, the Governor assures, 'have shared only minimally the errors and distortions' of the global financial system, originating mainly in the United States. Regarding European standards, 'the Bank of Italy has constantly given a severe interpretation.' Draghi is well aware that public opinion tends to involve central banks in blame. He makes it clear that this can be justified in the USA, where there was a 'regulatory capture' (in plain words, Wall Street influenced the government and the Federal Reserve) and in other countries; it is not the case in the Euro area and especially in Italy. 'Alarms, over time, were not lacking,' he recalls: 'not least those who speak of it had repeatedly drawn attention to the imbalances of the international financial system,' in various interventions, especially in the autumn of 2006; the problem is that 'in calm times, warnings often remain unheard.' 'Neither the moment, nor the precise mechanism, nor the magnitude of the crisis could be foreseen,' he summarizes; 'but the tensions that were accumulating could clearly be seen.' The banks or other intermediaries that passed Lehman Brothers titles to savers 'will not leave them alone.' New rules on transparency in relationships between banks and clients will be ready at the beginning of next year. Globally, to clean up, it will be necessary to better regulate derivatives and other innovative financial products. New rules must prevent banks from assuming risks too disproportionate to their capital. 'All things considered, Italy is not doing badly' from the financial crisis, concludes the Governor; but the effects of the crisis on the real economy 'add to pre-existing structural weaknesses.' The same judgment comes from the International Monetary Fund, which confirms the forecast of a drop in gross product both in 2008 (-0.1%) and in 2009 (-0.2%). But reacting with state aid would not be the right answer, warns the head of the European Department at the IMF, Alessandro Leipold: 'Liberalizations are better.'</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>Observation date: 2008-10-22 00:00:00. Governor Stefano Lepri stated that the financial crisis is beginning to spread to businesses and families; for now, credit provided by banks has not decreased, said the Governor of the Bank of Italy, Mario Draghi, though, "the situation, however, can change quickly." Consumption is falling. Following the drop in product in the second quarter, "negative signals are arriving for the coming quarters." To curb the negative effects, Silvio Berlusconi accepted the Confindustria proposal to open a discussion forum among the government, businesses, and banks. He will convene it immediately upon his return from his trip to China: "We ask that the banks do not fail to provide their support for investments and consumption." The promise is to find "funds of significant magnitude" in the budget. Minister Claudio Scajola added: "State guarantee forms are being studied for corporate debts, as was done for banks." In his hearing before the Senate, Draghi first sought to reassure about Italian banks: "Thanks to rigorous laws and firm supervisory action, we do not have that extensive 'shadow banking system' where the crisis found its origin and sustenance elsewhere." Today, "the capitalization of the major Italian banks remains sufficient"; even if losses from the Lehman failure reached the worst-case scenario, "such a shock could be absorbed." However, banks suffered on the stock exchange due to a phrase from the Prime Minister that was partially misunderstood. Again, and always in Naples, like the first time with Eni and Enel, Berlusconi let slip comments about listed companies on the stock exchange. According to the official clarification, he said: "Perhaps two or three banks, in addition to UniCredit, will have advantages in increasing their capital, naturally finding the means in the market." At the initial reports from the news agencies, the quotes of the major banks fell, before recovering somewhat later. The clarity in the financial markets was confirmed yesterday with the Euribor rate falling below 5% for three months, a reference point for variable-rate home mortgages. The Governor assures that Italian banks "have shared only a minimal portion of the errors and distortions" of the global financial system, originating mainly in the United States. Regarding European standards, "the Bank of Italy has consistently given a severe interpretation." Draghi is well aware that public opinion tends to involve central banks in blame. He makes it clear that this may be justified in the US, where there was a "regulatory capture" (in simple terms, Wall Street influenced the government and the Federal Reserve) and in other countries; it is not the case in the Euro area, and especially not in Italy. "Alarms were not lacking over time," he recalls: "not least the person speaking had repeatedly drawn attention to the imbalances of the international financial system," in various interventions, especially in the autumn of 2006; the problem is that "in calm times, warnings often remain unheard." "Neither the timing, nor the precise mechanism, nor the magnitude of the crisis could be foreseen; but the accumulating tensions could clearly be seen." The banks or other intermediaries that sold Lehman Brothers securities to savers "will not leave them alone." New rules on transparency in relationships between banks and clients will be ready at the beginning of next year. Globally, cleaning up will require better regulation of derivatives and other innovative financial products. New rules must prevent banks from assuming risks too disproportionate to their capital. "All in all, Italy is not doing badly" from the financial crisis, concludes the Governor; but the effects of the crisis on the real economy "add to pre-existing structural weaknesses." The same judgment comes from the International Monetary Fund, which confirms the forecast of a drop in gross product both in 2008 (-0.1%) and in 2009 (-0.2%). But reacting with state aid would not be the right answer, warns the head of the IMF's European Department, Alessandro Leipold: "Liberalization is better."</t>
+          <t>Observation date: 2008-10-22 00:00:00. The words of Governor Stefano Lepri: Rome, the financial crisis is beginning to affect businesses and families; for now, the credit provided by banks has not decreased, says the Governor of the Bank of Italy, Mario Draghi, 'however, the situation can change quickly.' Consumption is falling. Following the drop in product in the second quarter, 'negative signs are coming for the coming quarters.' To curb the negative effects, Silvio Berlusconi accepted the proposal from Confindustria to open a discussion table among the government, businesses, and banks. He will convene it as soon as he returns from his trip to China: 'We ask that the banks do not fail in their support for investments and consumption.' The promise is to find 'funds of significant magnitude' in the budget. And Minister Claudio Scajola added: state guarantee forms are being studied for corporate debts, as was done for banks. In his hearing before the Senate, Draghi first wanted to reassure about Italian banks: 'Thanks to rigorous laws and firm supervisory action, we do not have that extensive ''shadow banking system'' where elsewhere the crisis found its origin and sustenance.' Today, 'the capitalization of the major Italian banks remains sufficient'; even if losses from the Lehman failure reached the worst hypothesis, 'such a shock could be absorbed.' However, banks suffered on the stock exchange due to a phrase by the Prime Minister that was partially misunderstood. Again, and always in Naples, like the first time on Eni and Enel, Berlusconi let slip comments about listed companies. According to the official clarification, he said: 'Perhaps two or three banks, besides Unicredit, will have advantages in increasing their capital, finding the means naturally in the market.' To the initial headlines of the news agencies, the quotes of the major banks fell, only to recover somewhat later. The clarity on the financial markets was confirmed yesterday with the Euribor rate at three months below 5%, the reference point for variable-rate home mortgages. Italian banks, the Governor assures, 'have shared only minimally the errors and distortions' of the global financial system, originating mainly in the United States. Regarding European standards, 'the Bank of Italy has constantly given a severe interpretation.' Draghi is well aware that public opinion tends to involve central banks in blame. He makes it clear that this can be justified in the USA, where there was a 'regulatory capture' (in plain words, Wall Street influenced the government and the Federal Reserve) and in other countries; it is not the case in the Euro area and especially in Italy. 'Alarms, over time, were not lacking,' he recalls: 'not least those who speak of it had repeatedly drawn attention to the imbalances of the international financial system,' in various interventions, especially in the autumn of 2006; the problem is that 'in calm times, warnings often remain unheard.' 'Neither the moment, nor the precise mechanism, nor the magnitude of the crisis could be foreseen,' he summarizes; 'but the tensions that were accumulating could clearly be seen.' The banks or other intermediaries that passed Lehman Brothers titles to savers 'will not leave them alone.' New rules on transparency in relationships between banks and clients will be ready at the beginning of next year. Globally, to clean up, it will be necessary to better regulate derivatives and other innovative financial products. New rules must prevent banks from assuming risks too disproportionate to their capital. 'All things considered, Italy is not doing badly' from the financial crisis, concludes the Governor; but the effects of the crisis on the real economy 'add to pre-existing structural weaknesses.' The same judgment comes from the International Monetary Fund, which confirms the forecast of a drop in gross product both in 2008 (-0.1%) and in 2009 (-0.2%). But reacting with state aid would not be the right answer, warns the head of the European Department at the IMF, Alessandro Leipold: 'Liberalizations are better.'</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>['Stefano Lepri stated that the financial crisis is beginning to spread to businesses and families.', 'Mario Draghi, Governor of the Bank of Italy, stated that credit provided by banks has not decreased for now.', 'Mario Draghi stated that the situation can change quickly.', 'Consumption is falling.', 'Negative signals are arriving for the coming quarters following the drop in product in the second quarter.', 'Silvio Berlusconi accepted the Confindustria proposal.', 'The Confindustria proposal was to open a discussion forum among the government, businesses, and banks.', 'Silvio Berlusconi will convene the forum immediately upon his return from his trip to China.', 'Silvio Berlusconi asked that the banks do not fail to provide their support for investments and consumption.', 'The promise is to find funds of significant magnitude in the budget.', 'Minister Claudio Scajola added that state guarantee forms are being studied for corporate debts.', 'State guarantee forms were previously done for banks.', 'Mario Draghi sought to reassure about Italian banks during a hearing before the Senate.', "Mario Draghi stated that Italy does not have the extensive 'shadow banking system' where the crisis found its origin and sustenance elsewhere.", 'The capitalization of the major Italian banks remains sufficient on 2008-10-22.', 'A shock from Lehman failure losses could be absorbed even if losses reached the worst-case scenario.', 'Banks suffered on the stock exchange due to a phrase from the Prime Minister that was partially misunderstood.', 'Silvio Berlusconi let slip comments about listed companies on the stock exchange.', 'Silvio Berlusconi clarified that perhaps two or three banks, in addition to UniCredit, will have advantages in increasing their capital.', 'The quotes of the major banks fell at the initial reports from the news agencies.', 'The quotes of the major banks recovered somewhat later.', 'The clarity in the financial markets was confirmed on 2008-10-21.', 'The Euribor rate fell below 5% for three months on 2008-10-21.', 'Mario Draghi assures that Italian banks have shared only a minimal portion of the errors and distortions of the global financial system.', 'The global financial system errors and distortions originated mainly in the United States.', 'The Bank of Italy has consistently given a severe interpretation regarding European standards.', 'Mario Draghi is aware that public opinion tends to involve central banks in blame.', 'Mario Draghi stated that the situation (blame) may be justified in the US and other countries.', 'Mario Draghi stated that the situation (blame) is not the case in the Euro area or Italy.', 'Mario Draghi recalled that the person speaking had repeatedly drawn attention to the imbalances of the international financial system.', 'The person speaking drew attention to the imbalances of the international financial system in various interventions, especially in the autumn of 2006.', 'The banks or other intermediaries that sold Lehman Brothers securities to savers will not leave the savers alone.', 'New rules on transparency in relationships between banks and clients will be ready on 2009-10-22.', 'Cleaning up globally will require better regulation of derivatives and other innovative financial products.', 'New rules must prevent banks from assuming risks too disproportionate to their capital.', 'Mario Draghi concluded that Italy is not doing badly from the financial crisis.', 'The effects of the crisis on the real economy add to pre-existing structural weaknesses.', 'The International Monetary Fund confirmed the forecast of a drop in gross product in 2008 (-0.1%).', 'Alessandro Leipold warned that reacting with state aid would not be the right answer.', 'Alessandro Leipold recommended that liberalization is better.']</t>
+          <t>['Mario Draghi, Governor of the Bank of Italy, stated that the financial crisis is beginning to affect businesses and families.', 'Mario Draghi stated that the credit provided by banks has not decreased for now.', 'Mario Draghi stated that the situation can change quickly.', 'Consumption is falling.', 'A drop in product occurred in the second quarter.', 'Negative signs are coming for the coming quarters.', 'Silvio Berlusconi accepted the proposal from Confindustria.', 'The proposal was to open a discussion table among the government, businesses, and banks.', 'Silvio Berlusconi will convene the discussion table after returning from the trip to China.', 'Silvio Berlusconi asked that the banks do not fail in their support for investments and consumption.', 'The promise is to find funds of significant magnitude in the budget.', 'Minister Claudio Scajola added that state guarantee forms are being studied for corporate debts.', 'Minister Claudio Scajola noted that state guarantee forms were previously done for banks.', 'Mario Draghi reassured the Senate about Italian banks.', 'Mario Draghi stated that Italy does not have an extensive "shadow banking system."', 'Mario Draghi stated that the capitalization of the major Italian banks remains sufficient on 2008-10-22.', 'Mario Draghi stated that the Italian banking system could absorb losses from the Lehman failure, even in the worst hypothesis.', 'Banks suffered on the stock exchange due to a phrase by the Prime Minister that was partially misunderstood.', 'Silvio Berlusconi made comments about listed companies in Naples.', 'The official clarification from Silvio Berlusconi stated that two or three banks, besides Unicredit, might benefit from increasing their capital.', 'The quotes of the major banks fell following the initial headlines of the news agencies.', 'The quotes of the major banks recovered somewhat later.', 'The Euribor rate at three months was confirmed on 2008-10-21 to be below 5%.', 'Mario Draghi assured that Italian banks shared only minimally the errors and distortions of the global financial system.', "Mario Draghi stated that the global financial system's errors and distortions originated mainly in the United States.", 'Mario Draghi stated that the Bank of Italy has constantly given a severe interpretation regarding European standards.', 'Mario Draghi stated that the situation of regulatory capture (Wall Street influencing the government and the Federal Reserve) is justified in the USA and other countries.', 'Mario Draghi stated that the situation of regulatory capture is not the case in the Euro area or Italy.', 'Mario Draghi recalled that warnings about the imbalances of the international financial system were repeatedly drawn in various interventions, especially in the autumn of 2006.', 'Mario Draghi summarized that the tensions accumulating could clearly be seen, even if the moment, mechanism, or magnitude of the crisis could not be foreseen.', 'New rules on transparency in relationships between banks and clients will be ready at the beginning of 2009.', 'Globally, better regulation of derivatives and other innovative financial products will be necessary.', 'New rules must prevent banks from assuming risks too disproportionate to their capital.', 'Mario Draghi concluded that Italy is not doing badly from the financial crisis.', 'Mario Draghi noted that the effects of the crisis on the real economy add to pre-existing structural weaknesses.', 'The International Monetary Fund confirmed a forecast of a drop in gross product in 2008 (-0.1%).', 'Alessandro Leipold warned that reacting with state aid would not be the right answer.', 'Alessandro Leipold advised that liberalizations are better.']</t>
         </is>
       </c>
     </row>
@@ -1110,17 +1110,17 @@
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr">
         <is>
-          <t>Mortgage applications are falling, lending requirements are rising, and the credit crunch is intensifying. Goldman Sachs explains in a report that this crunch is the most severe since the sovereign debt crisis. The interest rate hikes by the European Central Bank (ECB) are beginning to impact households and businesses consistently. According to the latest Frankfurt Bank Lending Survey, in the fourth quarter of 2022, the contraction in residential mortgage demand, down 21%, was 'the strongest ever recorded,' and 'consumer credit and other household loans decreased sharply in net terms, although to a lesser extent than housing mortgages.' This scenario, according to Goldman Sachs, represents 'a substantial further tightening of credit standards' required of households and businesses, primarily weighed down by uncertain economic prospects, but increasingly influenced by the cost of funds and liquidity position. [The text also mentions the ECB's hawkish stance for all of 2023, noting that the situation is destined to worsen in step with rising money costs.] As the ECB explains, 'the net fall in real estate mortgage demand was determined mainly by the general level of interest rates, lower consumer confidence, and the deterioration of real estate market prospects.' In the first quarter of 2023, banking institutions anticipate a further net decline in corporate lending demand. Regarding household loans, Frankfurt notes that 'banks estimate a persistent and sharp net decline in demand for the first quarter of 2023.' This picture is also confirmed by Goldman Sachs, which expects a slowdown in credit provision and a reduction in demand for both personal loans and mortgages, 'of equal magnitude' to what was observed in the last four months of the year. Unlike the crisis that hit the Eurozone a decade ago, this phenomenon is spread homogeneously across the Euro area.</t>
+          <t>Mortgage applications are falling, requirements to obtain them are rising, and credit tightening is intensifying. Goldman Sachs explains in a report that this tightening is the most intense since the sovereign debt crisis. The increase in interest rates by the European Central Bank (BCE) is beginning to consistently impact households and businesses. According to the latest bank lending survey from Frankfurt, in the fourth quarter of 2022, the contraction in residential mortgage demand, down 21%, was "the strongest ever recorded," and "demand for consumer credit and other household loans decreased sharply in net terms, albeit less so than housing mortgages." This scenario, according to Goldman Sachs, represents "a substantial further tightening of credit standards" required of households and businesses, primarily weighed down by uncertain economic prospects, but increasingly influenced by the cost of funds and liquidity position. The Fed's hawkish stance for all of 2023, and the BCE rates—today is the day of the hawks—the situation is destined to worsen in step with rising money costs. As the BCE explains, "the net decline in residential mortgage demand was determined mainly by the general level of interest rates, lower consumer confidence, and the deterioration of real estate market prospects." In the first quarter of 2023, banking institutions predict a further net decline in corporate lending demand. Regarding household loans, Frankfurt notes, "banks estimate a persistent and sharp net decline in demand for the first quarter of 2023." This picture is also confirmed by Goldman Sachs, which anticipates a slowdown in credit provision and a reduction in demand, for both personal loans and mortgages, "of equal magnitude" compared to what was observed in the last four months of the year. Unlike the crisis that hit the Eurozone a decade ago, in this case the phenomenon is spread homogeneously across the Euro area.</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>Observation date: 2023-02-02 00:00:00. Mortgage applications are falling, lending requirements are rising, and the credit crunch is intensifying. Goldman Sachs explains in a report that this crunch is the most severe since the sovereign debt crisis. The interest rate hikes by the European Central Bank (ECB) are beginning to impact households and businesses consistently. According to the latest Frankfurt Bank Lending Survey, in the fourth quarter of 2022, the contraction in residential mortgage demand, down 21%, was 'the strongest ever recorded,' and 'consumer credit and other household loans decreased sharply in net terms, although to a lesser extent than housing mortgages.' This scenario, according to Goldman Sachs, represents 'a substantial further tightening of credit standards' required of households and businesses, primarily weighed down by uncertain economic prospects, but increasingly influenced by the cost of funds and liquidity position. [The text also mentions the ECB's hawkish stance for all of 2023, noting that the situation is destined to worsen in step with rising money costs.] As the ECB explains, 'the net fall in real estate mortgage demand was determined mainly by the general level of interest rates, lower consumer confidence, and the deterioration of real estate market prospects.' In the first quarter of 2023, banking institutions anticipate a further net decline in corporate lending demand. Regarding household loans, Frankfurt notes that 'banks estimate a persistent and sharp net decline in demand for the first quarter of 2023.' This picture is also confirmed by Goldman Sachs, which expects a slowdown in credit provision and a reduction in demand for both personal loans and mortgages, 'of equal magnitude' to what was observed in the last four months of the year. Unlike the crisis that hit the Eurozone a decade ago, this phenomenon is spread homogeneously across the Euro area.</t>
+          <t>Observation date: 2023-02-02 00:00:00. Mortgage applications are falling, requirements to obtain them are rising, and credit tightening is intensifying. Goldman Sachs explains in a report that this tightening is the most intense since the sovereign debt crisis. The increase in interest rates by the European Central Bank (BCE) is beginning to consistently impact households and businesses. According to the latest bank lending survey from Frankfurt, in the fourth quarter of 2022, the contraction in residential mortgage demand, down 21%, was "the strongest ever recorded," and "demand for consumer credit and other household loans decreased sharply in net terms, albeit less so than housing mortgages." This scenario, according to Goldman Sachs, represents "a substantial further tightening of credit standards" required of households and businesses, primarily weighed down by uncertain economic prospects, but increasingly influenced by the cost of funds and liquidity position. The Fed's hawkish stance for all of 2023, and the BCE rates—today is the day of the hawks—the situation is destined to worsen in step with rising money costs. As the BCE explains, "the net decline in residential mortgage demand was determined mainly by the general level of interest rates, lower consumer confidence, and the deterioration of real estate market prospects." In the first quarter of 2023, banking institutions predict a further net decline in corporate lending demand. Regarding household loans, Frankfurt notes, "banks estimate a persistent and sharp net decline in demand for the first quarter of 2023." This picture is also confirmed by Goldman Sachs, which anticipates a slowdown in credit provision and a reduction in demand, for both personal loans and mortgages, "of equal magnitude" compared to what was observed in the last four months of the year. Unlike the crisis that hit the Eurozone a decade ago, in this case the phenomenon is spread homogeneously across the Euro area.</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>['Mortgage applications are falling.', 'Lending requirements are rising.', 'The credit crunch is intensifying.', 'Goldman Sachs explained in a report that the credit crunch is the most severe since the sovereign debt crisis.', 'The European Central Bank (ECB) interest rate hikes are beginning to impact households.', 'The Frankfurt Bank Lending Survey reported data for the fourth quarter of 2022.', 'In the fourth quarter of 2022, the contraction in residential mortgage demand was 21%.', 'The Frankfurt Bank Lending Survey stated that the contraction in residential mortgage demand in the fourth quarter of 2022 was the strongest ever recorded.', 'In the fourth quarter of 2022, consumer credit and other household loans decreased sharply in net terms.', 'The decrease in consumer credit and other household loans in the fourth quarter of 2022 was less than the decrease in housing mortgages.', 'Goldman Sachs stated that the scenario represents a substantial further tightening of credit standards.', 'The tightening of credit standards is required of households.', 'The tightening of credit standards is primarily weighed down by uncertain economic prospects.', 'The tightening of credit standards is increasingly influenced by the cost of funds and liquidity position.', 'The ECB maintained a hawkish stance for all of 2023.', 'The situation is destined to worsen with rising money costs.', 'The ECB explained that the net fall in real estate mortgage demand was determined mainly by the general level of interest rates.', 'The net fall in real estate mortgage demand was determined mainly by lower consumer confidence.', 'The net fall in real estate mortgage demand was determined mainly by the deterioration of real estate market prospects.', 'Banking institutions anticipate a further net decline in corporate lending demand in the first quarter of 2023.', 'Frankfurt noted that banks estimate a persistent and sharp net decline in household loan demand for the first quarter of 2023.', 'Goldman Sachs confirmed the picture of declining credit demand.', 'Goldman Sachs expects a slowdown in credit provision.', 'Goldman Sachs expects a reduction in demand for personal loans.', 'The expected reduction in personal loans and mortgages is of equal magnitude to what was observed in the last four months of the year.', 'The current phenomenon is spread homogeneously across the Euro area.', 'The current phenomenon differs from the crisis that hit the Eurozone a decade ago.']</t>
+          <t>['Mortgage applications are falling.', 'Requirements to obtain mortgages are rising.', 'Credit tightening is intensifying.', 'Goldman Sachs explained in a report that the current credit tightening is the most intense since the sovereign debt crisis.', 'The increase in interest rates by the European Central Bank (BCE) is beginning to consistently impact households.', 'In the fourth quarter of 2022, the bank lending survey from Frankfurt reported that the contraction in residential mortgage demand was the strongest ever recorded.', 'In the fourth quarter of 2022, demand for consumer credit and other household loans decreased sharply in net terms.', 'In the fourth quarter of 2022, the decrease in demand for consumer credit and other household loans was less than the decrease in housing mortgages.', 'Goldman Sachs stated that the scenario represents a substantial further tightening of credit standards required of households and businesses.', 'The tightening of credit standards is primarily weighed down by uncertain economic prospects.', 'The tightening of credit standards is increasingly influenced by the cost of funds and liquidity position.', "The Fed's hawkish stance is projected for all of 2023.", 'The situation is destined to worsen in step with rising money costs.', 'The BCE explained that the net decline in residential mortgage demand was determined mainly by the deterioration of real estate market prospects.', 'In the first quarter of 2023, banking institutions predict a further net decline in corporate lending demand.', 'Frankfurt noted that banks estimate a persistent and sharp net decline in demand for household loans in the first quarter of 2023.', 'Goldman Sachs anticipates a slowdown in credit provision and a reduction in demand for personal loans and mortgages.', 'Goldman Sachs anticipates this reduction in demand for personal loans and mortgages will be of equal magnitude compared to the last four months of the year.', 'The current phenomenon is spread homogeneously across the Euro area.']</t>
         </is>
       </c>
     </row>

</xml_diff>